<commit_message>
chore: refresh daily snapshot (2026-09-13)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>37.93036529680365</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.77716048631313</v>
+        <v>34.76965869272961</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.45400029158803</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09066884030775024</v>
+        <v>0.09090415962969911</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1144356089853538</v>
+        <v>0.1146979601428062</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.535</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.19478598519915</v>
+        <v>24.18264317759899</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.09069562800033</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1380551171993909</v>
+        <v>0.1386265677321155</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2236321448597434</v>
+        <v>0.2242597789543264</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>16.65590863952334</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.1895278702949</v>
+        <v>20.207596394201</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.130520105868131</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1750223805862554</v>
+        <v>-0.1757600303070632</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2894614358948004</v>
+        <v>0.2901656708796634</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.37936507936508</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.76311457721979</v>
+        <v>22.77500684011763</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.561015029393565</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1047198303979128</v>
+        <v>-0.1051873124592303</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1772913545578569</v>
+        <v>0.17771891846736</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>27.45786163522012</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.39580978400739</v>
+        <v>16.37410678350809</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>17.45129729444267</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6746877401568017</v>
+        <v>0.6769074489532174</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9278215828328569</v>
+        <v>0.9303402776833312</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>24.08138238573021</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>19.6096367335396</v>
+        <v>19.60576870666489</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>7.232693044219446</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2280381688326893</v>
+        <v>0.2282804487815804</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2699368436425558</v>
+        <v>0.2705509847826661</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>309.6949152542373</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>174.1146800786864</v>
+        <v>173.9867834554464</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.92913075462029</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7786835384258184</v>
+        <v>0.7799910378453681</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1211920138920415</v>
+        <v>0.1215655287458917</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>44.91191066997519</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.87640520950526</v>
+        <v>19.80286514742586</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>19.32793571781289</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.259559019681158</v>
+        <v>1.26795013426697</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8532388312558883</v>
+        <v>0.8564104257536831</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>45.44299347061778</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.91850143588716</v>
+        <v>39.91873039403847</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.36670388957958</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1383942742340534</v>
+        <v>0.1383877448518331</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.113636913092201</v>
+        <v>0.1136368918037924</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>23.96284829721363</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.65000478588037</v>
+        <v>20.64675644835125</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.662887440086743</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1604282200262945</v>
+        <v>0.1606107892616311</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1424463232227213</v>
+        <v>0.1427745098118778</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.8402369442784</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.00736252076394</v>
+        <v>23.00733563970968</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.863781900610106</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4419074792823298</v>
+        <v>-0.4419068272244138</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06134979061163781</v>
+        <v>0.06139523027282179</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.31513327601032</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.22574077908948</v>
+        <v>14.22510989720509</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.207043060749312</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07657896441654222</v>
+        <v>0.07662671056196224</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2895840775374785</v>
+        <v>-0.2895318430660836</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.47408666100255</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.80613921732385</v>
+        <v>24.7979651085753</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.54683598532188</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2688023067701726</v>
+        <v>0.2692205397981868</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1369119287200737</v>
+        <v>0.1372179948816117</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.25700164744646</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.70505128511245</v>
+        <v>25.69509642969269</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.2291172602115</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2159867452024704</v>
+        <v>0.2164578456816593</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1557212564532875</v>
+        <v>0.1560881955092015</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>24.37721046878015</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.51984944825355</v>
+        <v>17.51388894681446</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7648217780058605</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3914052481318653</v>
+        <v>0.3918787850492815</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01022441291752063</v>
+        <v>0.01030287783379724</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.36679536679537</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.0124804236027</v>
+        <v>15.01583088487154</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.905675647260843</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4232688245975917</v>
+        <v>0.4229512526224855</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08263869576574012</v>
+        <v>0.08247725756777813</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>30.7028901734104</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.37989743854772</v>
+        <v>21.37408831167713</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.535559653636819</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4360634919629423</v>
+        <v>0.4364537904822234</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08812494365126411</v>
+        <v>0.08833454717187483</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>38.68231046931408</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.58434948169261</v>
+        <v>34.57399762391755</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.158822939769515</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1184917758765638</v>
+        <v>0.1188266653479055</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05057354649804369</v>
+        <v>0.05069788025443667</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.52148148148148</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.57591250953377</v>
+        <v>20.57258134369886</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.967932970378711</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04595514155251146</v>
+        <v>0.04612450532724499</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02511544798896215</v>
+        <v>0.02519525344873941</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>130.997461928934</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>38.36558989914167</v>
+        <v>38.30146529942742</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>20.37529543638785</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.414451915722133</v>
+        <v>2.420168416660871</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8858346653687155</v>
+        <v>0.8883604343143967</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>53.64296081277213</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.029973940036</v>
+        <v>35.00133660233855</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.1291333350506</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5313445823453273</v>
+        <v>0.5325974954107349</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2856372264178451</v>
+        <v>0.2864551702816613</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>78.82022471910109</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>84.60281007648415</v>
+        <v>84.14062311047331</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.769598026490771</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.06834980247293654</v>
+        <v>-0.06323221999897422</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1520990995166605</v>
+        <v>0.152523701668509</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.67915904936015</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.21483560557174</v>
+        <v>14.2131694053763</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.574385513112933</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1030137445426695</v>
+        <v>0.1031430500947468</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3824139070636855</v>
+        <v>-0.3823711015222546</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>21.24803493449782</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.86679928185745</v>
+        <v>18.86344951193065</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.317246492032939</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1262130166895976</v>
+        <v>0.1264130095112761</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04567790493352519</v>
+        <v>0.04578542708088928</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>37.36180904522614</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>25.61307332702475</v>
+        <v>25.59658996630991</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.18353233445217</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4587007411486659</v>
+        <v>0.4596400963722727</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2268454687601291</v>
+        <v>0.2273126002782788</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.23311897106109</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.92738052268832</v>
+        <v>15.92478333473714</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.672409379667902</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08198074043077996</v>
+        <v>0.0821572016914065</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3275865696303093</v>
+        <v>-0.3274869152039972</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>82.31677018633542</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.00741457457604</v>
+        <v>27.99208426195769</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.300687677165355</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.939106355824045</v>
+        <v>1.940716004424403</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2439425326806988</v>
+        <v>0.2445053550059697</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.62790697674419</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.492394090000051</v>
+        <v>9.493088068672243</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.480351620195931</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.858658482724666</v>
+        <v>2.858376400996264</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04999892076274981</v>
+        <v>-0.05010572930318846</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.917142991467138</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003951832075846838</v>
+        <v>0.003950478887045561</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.799454886225326</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2002.410782521819</v>
+        <v>2003.097026674181</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2585.694770015227</v>
+        <v>2585.930107902172</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-98.18831168831169</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>138.2729550294376</v>
+        <v>137.6590676676727</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>119.2881818090498</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.174644104217029</v>
+        <v>4.184692245707556</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
         <v>27.93555117653877</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6626937242120312</v>
+        <v>0.662234378283926</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.07436022855125</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.15454312586895</v>
+        <v>41.18378280047808</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.12456964192115</v>
+        <v>41.15666372328758</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
         <v>-22.07874015748031</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-79.96238534891215</v>
+        <v>-80.68007820889312</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.946562733600997</v>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02035935925193311</v>
+        <v>0.02043303423553744</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
         <v>19.69011522134627</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.72766832562197</v>
+        <v>16.72171575281377</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.608047814399391</v>
@@ -5200,10 +5200,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1770986151839637</v>
+        <v>0.1775176370901419</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.005192089385952725</v>
+        <v>0.005425181638038401</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>
@@ -5302,13 +5302,13 @@
         <v>23.1712962962963</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.79024564414526</v>
+        <v>16.77375562030881</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.025642900929268</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.627550747068279</v>
+        <v>6.669635475948002</v>
       </c>
       <c r="P39" s="6" t="n">
         <v>0.5043164488017432</v>
@@ -5326,16 +5326,16 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3800451040081179</v>
+        <v>0.3814018053441572</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4179780294298492</v>
+        <v>0.4198565143825406</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
       </c>
       <c r="X39" s="4" t="n">
-        <v>0.4248105529048555</v>
+        <v>0.425824021246188</v>
       </c>
       <c r="Y39" s="4" t="n">
         <v>0.7443888710868384</v>
@@ -5353,7 +5353,7 @@
         <v>1.170812813065623</v>
       </c>
       <c r="AD39" s="6" t="n">
-        <v>2.320539913090065</v>
+        <v>2.335275265081172</v>
       </c>
       <c r="AE39" s="6" t="n">
         <v>0.5141842451501851</v>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12 10:41 ET</t>
+          <t>2026-09-13 11:21 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-14)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>332.27</v>
+        <v>334.17001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2260432752552346</v>
+        <v>0.233054123310785</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.03569666540906058</v>
+        <v>-0.0301825173404533</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>235.03</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4880167778120</v>
+        <v>4908073951738</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>37.93036529680365</v>
+        <v>38.14726141552512</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.76965869272961</v>
+        <v>34.94378705930419</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.45400029158803</v>
+        <v>10.5137792091178</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.40440810128349</v>
+        <v>45.66404282435966</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.158983384068999</v>
+        <v>1.165610765474377</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.2305044817967</v>
+        <v>29.3961335169569</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.54988888319556</v>
+        <v>10.60966780072533</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02800784854422664</v>
+        <v>0.0278486023935314</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09090415962969911</v>
+        <v>0.0916750766247576</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1146979601428062</v>
+        <v>0.1170296262044463</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003190176663556746</v>
+        <v>0.003172038089234878</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3113031219292596</v>
+        <v>0.3090034763209347</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.3125421036337848</v>
+        <v>0.2978607153938829</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>14847202025.02401</v>
+        <v>13711498421.73662</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>495.63</v>
+        <v>508.12</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.0479764820938462</v>
+        <v>0.07438575163231675</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.1049086180741169</v>
+        <v>-0.08235209130968724</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3680325346500</v>
+        <v>3773070466000</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.535</v>
+        <v>28.23444444444445</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.18264317759899</v>
+        <v>24.77961551573403</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.09069562800033</v>
+        <v>11.37242165647799</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.323109110349083</v>
+        <v>8.534532841154917</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8746035962877013</v>
+        <v>0.8968202887342083</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.25470750389121</v>
+        <v>18.70520930644423</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.41577284918289</v>
+        <v>11.69749887766055</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01820137995780858</v>
+        <v>0.01775048193070232</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1386265677321155</v>
+        <v>0.1394222168829355</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2242597789543264</v>
+        <v>0.2251284786170114</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007344188204910922</v>
+        <v>0.007163662127056601</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5625067965786378</v>
+        <v>0.558727690336572</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4360525535827411</v>
+        <v>0.4353830518384593</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>13121876129.73938</v>
+        <v>12385142545.40151</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>338.5</v>
+        <v>347</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.07409172316590706</v>
+        <v>0.1010630072040466</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1715817038251634</v>
+        <v>-0.1507794718680404</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4096564670311</v>
+        <v>4199432616242</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.65590863952334</v>
+        <v>17.05486544190665</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.207596394201</v>
+        <v>20.73358038065668</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.130520105868131</v>
+        <v>9.349222133898973</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.364059689607794</v>
+        <v>6.516497179443543</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1481219642614271</v>
+        <v>0.1516699103088885</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.72985430859732</v>
+        <v>13.03057162050983</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.258013568029408</v>
+        <v>9.47671559606025</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01308601100055534</v>
+        <v>0.01277989599936413</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1757600303070632</v>
+        <v>-0.1774278668329795</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2901656708796634</v>
+        <v>0.2894117866894625</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002540620384047267</v>
+        <v>0.002478386167146974</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7789901606449278</v>
+        <v>0.7751385826763244</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3823461763573922</v>
+        <v>0.379213207556274</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8841449226.603495</v>
+        <v>8490362029.198562</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>256.78</v>
+        <v>254.78</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1336865342163354</v>
+        <v>0.1248565121412804</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1059192200557104</v>
+        <v>-0.112883008356546</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2762208138000</v>
+        <v>2740693938000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.37936507936508</v>
+        <v>20.22063492063492</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.77500684011763</v>
+        <v>22.60942955443562</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.561015029393565</v>
+        <v>3.533279107363862</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>5.006935354048076</v>
+        <v>4.967937493201841</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2306902747562646</v>
+        <v>0.228893481588913</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.44591132178727</v>
+        <v>11.36099673163069</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.747972279806106</v>
+        <v>3.720166933328177</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004208589439757852</v>
+        <v>-0.004241709831146357</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1051873124592303</v>
+        <v>-0.105654794520548</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.17771891846736</v>
+        <v>0.1781464823768628</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8296038041177198</v>
+        <v>0.831056140105345</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4652561170535028</v>
+        <v>0.4600153326456301</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>10365039248.01656</v>
+        <v>9344931571.26368</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>218.29</v>
+        <v>212.025</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1558908813608786</v>
+        <v>0.1227164053348313</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.07715396973027822</v>
+        <v>-0.1036399763253572</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5287202090000</v>
+        <v>5135457525000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>27.45786163522012</v>
+        <v>26.66981132075471</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.37410678350809</v>
+        <v>15.88313975964608</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.45129729444267</v>
+        <v>16.95043890629074</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>23.06027975753764</v>
+        <v>22.39844159417252</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.220410045779318</v>
+        <v>0.2140841997176229</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>22.69733890536532</v>
+        <v>22.04793370480213</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>17.50548435648532</v>
+        <v>17.0046259683334</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02402140070269189</v>
+        <v>0.02473119471472992</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6769074489532174</v>
+        <v>0.6791271577496334</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9303402776833312</v>
+        <v>0.9328589725338055</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002382152182875991</v>
+        <v>0.002452540973941752</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.322780447691964</v>
+        <v>1.327160397548167</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4084395360415243</v>
+        <v>0.4148400572918929</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27448909421.48951</v>
+        <v>27055168487.89567</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>648.03</v>
+        <v>663.325</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.003659189192663836</v>
+        <v>0.01985674788015412</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.1805386949924127</v>
+        <v>-0.1611975214972179</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1650847721957</v>
+        <v>1689811529045</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>24.08138238573021</v>
+        <v>24.64781865477518</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>19.60576870666489</v>
+        <v>20.06455222816985</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7.232693044219446</v>
+        <v>7.40281864570993</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>6.308605701685546</v>
+        <v>6.456995151232098</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-4.936683389074689</v>
+        <v>-5.052802824228906</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>16.32269614798453</v>
+        <v>16.68535705175956</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.657038493029512</v>
+        <v>7.827164094519996</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02482118699078128</v>
+        <v>0.02425076651060896</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2282804487815804</v>
+        <v>0.2284260508026987</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2705509847826661</v>
+        <v>0.2710650922747215</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003240590713392899</v>
+        <v>0.00316586891795123</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7840031621567214</v>
+        <v>0.7806994346944971</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4197310775348115</v>
+        <v>0.4169714993952099</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10201000387.61983</v>
+        <v>9992239438.008711</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>365.44</v>
+        <v>362.48</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.165795434770463</v>
+        <v>-0.1725523456534518</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.267405729406812</v>
+        <v>-0.2733396146983942</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1443322599663</v>
+        <v>1431631939377</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>309.6949152542373</v>
+        <v>307.1526271186441</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>173.9867834554464</v>
+        <v>172.4508465322345</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.92913075462029</v>
+        <v>13.8147864043853</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.61911717976467</v>
+        <v>13.5073177335421</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.243991406063495</v>
+        <v>-8.176316412031507</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>119.5082806503991</v>
+        <v>118.5232251775856</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.87241335723178</v>
+        <v>13.75806900699679</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.003992177494723192</v>
+        <v>0.004025220563815595</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7799910378453681</v>
+        <v>0.7811024607596293</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1215655287458917</v>
+        <v>0.1218155461162014</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.552710352419476</v>
+        <v>1.545780564140041</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5738652948790913</v>
+        <v>0.5740456608731275</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12812720116.62303</v>
+        <v>12684958207.25491</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>361.99</v>
+        <v>346.73999</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.04133825753598597</v>
+        <v>-0.002531514669893653</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2687070707070707</v>
+        <v>-0.2995151717171718</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1722196384200</v>
+        <v>1649643242739</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>44.91191066997519</v>
+        <v>43.01984987593052</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.80286514742586</v>
+        <v>18.94683586278015</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>19.32793571781289</v>
+        <v>18.51368336706545</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>17.30609228608687</v>
+        <v>16.57701667509279</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4468957447853964</v>
+        <v>0.4280688032208926</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>33.63068297265752</v>
+        <v>32.24245149989476</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.72571808448554</v>
+        <v>18.9114657337381</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02287950454518205</v>
+        <v>0.02388577055883724</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.26795013426697</v>
+        <v>1.270555895849621</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8564104257536831</v>
+        <v>0.8585251496160557</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.0070167684190171</v>
+        <v>0.007325373689951367</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.591136790691581</v>
+        <v>1.600700056177729</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3916057238939792</v>
+        <v>0.4025682119619466</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8616347746.350199</v>
+        <v>8505683809.747202</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>904.77</v>
+        <v>916</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.05882972498537153</v>
+        <v>0.07197191339964881</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1748563611491109</v>
+        <v>-0.1646146830825354</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,31 +1724,31 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>401246494830</v>
+        <v>406226764000</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>45.44299347061778</v>
+        <v>46.00703164239076</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.91873039403847</v>
+        <v>40.41420144449886</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.36670388957958</v>
+        <v>1.383667410341739</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.98627869259005</v>
+        <v>12.13505231430362</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.584721851008112</v>
+        <v>3.62921539786181</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>26.98911505390463</v>
+        <v>27.33329398756047</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.330210448112485</v>
+        <v>1.347173968874644</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02194660916285617</v>
+        <v>0.0216775475679884</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006123103109077445</v>
+        <v>0.006048034934497817</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1861953189174849</v>
+        <v>-0.1891268944090583</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1839168874187742</v>
+        <v>0.1860969081064974</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1722789357.552694</v>
+        <v>1692630979.817741</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>77.40000000000001</v>
+        <v>80.69</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1493570522346479</v>
+        <v>-0.1131992318451388</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3801057184046132</v>
+        <v>-0.353756206951786</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>322288955923</v>
+        <v>335988318519</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>23.96284829721363</v>
+        <v>24.98142414860681</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.64675644835125</v>
+        <v>21.52099162675565</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.662887440086743</v>
+        <v>6.946103198183928</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.75389669001632</v>
+        <v>11.21100676895888</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.7042739560522543</v>
+        <v>0.7342101487578345</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10.70361875953483</v>
+        <v>11.15135368720985</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.770598660029434</v>
+        <v>7.05381441812662</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03411413204809534</v>
+        <v>0.03272318528353318</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1606107892616311</v>
+        <v>0.1607933584969679</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1427745098118778</v>
+        <v>0.1431026964010345</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.09961480082447288</v>
+        <v>0.09790870291220452</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3634172639823042</v>
+        <v>0.3765823731261873</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2211242125.649261</v>
+        <v>2172210566.412371</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>510.37</v>
+        <v>512.91</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.02721141940303728</v>
+        <v>0.03232362624372875</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.05089820359281438</v>
+        <v>-0.04617473128277616</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1100793369280</v>
+        <v>1106271777411</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.8402369442784</v>
+        <v>12.9058746933681</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.00733563970968</v>
+        <v>23.1218111084785</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.863781900610106</v>
+        <v>2.878421209734147</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.466288622551745</v>
+        <v>1.473784113882457</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.353715828819828</v>
+        <v>0.3555239816539139</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.5582072300494</v>
+        <v>15.63180881811172</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.094517537634492</v>
+        <v>3.109156846758534</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02198047246656578</v>
+        <v>0.02186868238871257</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4419068272244138</v>
+        <v>-0.4418311509933723</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06139523027282179</v>
+        <v>0.0615833586816934</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06432354147288388</v>
+        <v>0.05690917823923999</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1406752297569992</v>
+        <v>0.1400473515421361</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2108686234.881185</v>
+        <v>2075894072.081889</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>356.23</v>
+        <v>350.54</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.09447581410756301</v>
+        <v>0.07699394177151042</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.02802182810368348</v>
+        <v>-0.04354706684856746</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>954521847300</v>
+        <v>939275435400</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.31513327601032</v>
+        <v>15.07050730868444</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.22510989720509</v>
+        <v>13.99727393438135</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.207043060749312</v>
+        <v>3.155817518218746</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.651959169563105</v>
+        <v>2.609599885744184</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.8018888817171094</v>
+        <v>0.78908044970136</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.20804902640618</v>
+        <v>20.0443906762559</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.325178482560737</v>
+        <v>6.273952940030171</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1702779254972009</v>
+        <v>-0.1730418936494206</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07662671056196224</v>
+        <v>0.07667445670738182</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2895318430660836</v>
+        <v>-0.2894796085946888</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01684305083794178</v>
+        <v>0.01711644890740001</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7724829929363041</v>
+        <v>0.7707282381692373</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1682573598779749</v>
+        <v>0.171074244059474</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>1996875316.184591</v>
+        <v>1947689584.188324</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>370.45</v>
+        <v>376.08</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.0691814484346045</v>
+        <v>0.08543058206852772</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.03921466919106775</v>
+        <v>-0.02461291075550487</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>691647639315</v>
+        <v>702159115113</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.47408666100255</v>
+        <v>31.95242141036533</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.7979651085753</v>
+        <v>25.16654507899095</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.54683598532188</v>
+        <v>15.78311263965564</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.15003476462562</v>
+        <v>20.45626960259253</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.122430186021555</v>
+        <v>2.154686312212137</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.16477556240979</v>
+        <v>24.52601948975875</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.8053101806105</v>
+        <v>16.04158683494425</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03038107672977968</v>
+        <v>0.02992626535456758</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2692205397981868</v>
+        <v>0.2696387728262006</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1372179948816117</v>
+        <v>0.1375240610011503</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007234444594412202</v>
+        <v>0.007126143373750267</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3161428791341334</v>
+        <v>0.3065458064898975</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1902203688985791</v>
+        <v>0.1931196194254112</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2295279806.026103</v>
+        <v>2225464739.478773</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>569.1900000000001</v>
+        <v>575.01</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.01076127193479715</v>
+        <v>0.02109636320952157</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05390445796349852</v>
+        <v>-0.04423057744090952</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>499200120840</v>
+        <v>504304470360</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.25700164744646</v>
+        <v>31.57660626029654</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.69509642969269</v>
+        <v>25.94778138848124</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.2291172602115</v>
+        <v>14.37461079041131</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>89.47167706291215</v>
+        <v>90.38653003029764</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.381447840668392</v>
+        <v>1.395573223111319</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.17562492494122</v>
+        <v>23.40642387230964</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.60970044865034</v>
+        <v>14.75519397885015</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03294870997291243</v>
+        <v>0.0326152175257509</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2164578456816593</v>
+        <v>0.2169289461608479</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1560881955092015</v>
+        <v>0.1564551345566814</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005920694319998594</v>
+        <v>0.005860767638823673</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3037572295055846</v>
+        <v>0.2947684382098303</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2087301167230023</v>
+        <v>0.2091536729951674</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1597794977.672933</v>
+        <v>1526338069.898275</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>379.09</v>
+        <v>383.59</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1269025174734455</v>
+        <v>0.1402794499396951</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1787834149300291</v>
+        <v>-0.1690351371257746</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>344268462112</v>
+        <v>348355108605</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.37721046878015</v>
+        <v>24.66658092727156</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.51388894681446</v>
+        <v>17.71576097379578</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7648217780058605</v>
+        <v>0.7739006120578766</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.488723909616341</v>
+        <v>3.530136918646581</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7386358420109492</v>
+        <v>-0.7474038424568836</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.09961813888134</v>
+        <v>15.25901840263168</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8642221721151048</v>
+        <v>0.8733453990011751</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.0686005330116958</v>
+        <v>0.06779187319321366</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3918787850492815</v>
+        <v>0.3923523219666978</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01030287783379724</v>
+        <v>0.01038134275007363</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02360916932654515</v>
+        <v>0.02361896816913893</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.436475309780648</v>
+        <v>0.4262510099876727</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2272317203020928</v>
+        <v>0.2274706885088772</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1791619278.642578</v>
+        <v>1761291428.937432</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>166.02</v>
+        <v>165.245</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3536078103103009</v>
+        <v>0.3472890170746035</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.05889688793152303</v>
+        <v>-0.063290062921603</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>688063249200</v>
+        <v>684851272463</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.36679536679537</v>
+        <v>21.26705276705277</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.01583088487154</v>
+        <v>14.94907161018081</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.905675647260843</v>
+        <v>1.89677968332964</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.671534979643766</v>
+        <v>2.659063954410517</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.092165379665381</v>
+        <v>2.082398916773918</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>10.02218237660982</v>
+        <v>9.977462895412462</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.993694259125907</v>
+        <v>1.984798295194704</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04440434805306558</v>
+        <v>0.04461260601899614</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4229512526224855</v>
+        <v>0.4226336806473794</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08247725756777813</v>
+        <v>0.08231581936981591</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02481628719431394</v>
+        <v>0.02493267572392508</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.547064655600945</v>
+        <v>-0.5450501269668325</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2306851828723931</v>
+        <v>0.2307829930272591</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2252779834.290212</v>
+        <v>2205824710.227472</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>265.58</v>
+        <v>267.7</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2808294776100182</v>
+        <v>0.2910537358091794</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.05511082648450571</v>
+        <v>-0.04756822143949913</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>640020821321</v>
+        <v>645129805963</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>30.7028901734104</v>
+        <v>30.94797687861271</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.37408831167713</v>
+        <v>21.5388552700378</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.535559653636819</v>
+        <v>6.587729946828825</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.626622706570476</v>
+        <v>7.687502442009626</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.801502585944636</v>
+        <v>-3.831848189838765</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.8219738325922</v>
+        <v>19.97343193297166</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.827750935075412</v>
+        <v>6.879921228267418</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02923029904150114</v>
+        <v>0.02899881516414226</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4364537904822234</v>
+        <v>0.4368440890015042</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08833454717187483</v>
+        <v>0.08854415069248511</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01988101513668198</v>
+        <v>0.01972357116174823</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.166496328835057</v>
+        <v>-0.1748754776236435</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2227528347813669</v>
+        <v>0.2116056571777831</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1697427104.77061</v>
+        <v>1652666672.513288</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>107.15</v>
+        <v>109.165</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.04975170299706777</v>
+        <v>-0.03188189134554265</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2072358686001775</v>
+        <v>-0.1923276117194436</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>852708272000</v>
+        <v>868743803200</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.68231046931408</v>
+        <v>39.40974729241878</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.57399762391755</v>
+        <v>35.2136357103365</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.158822939769515</v>
+        <v>1.180615083713851</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.675574624890572</v>
+        <v>8.838722388485108</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.354085986215958</v>
+        <v>9.52999343616673</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.35750769158944</v>
+        <v>21.7318285487523</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.243387519025875</v>
+        <v>1.265179662970211</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01584246388077727</v>
+        <v>0.01555003897609384</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1188266653479055</v>
+        <v>0.1191615548192475</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05069788025443667</v>
+        <v>0.05082221401082943</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009122725151656555</v>
+        <v>0.008954335180689782</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.04357380101997047</v>
+        <v>-0.05815779045644878</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3087826617573923</v>
+        <v>0.3117912557655074</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2781691745.647964</v>
+        <v>2730355064.764832</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>145.27</v>
+        <v>146.19</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.02454338725332006</v>
+        <v>0.03103185642295614</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1314200298953662</v>
+        <v>-0.1259192825112108</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>345337142278</v>
+        <v>347524174500</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.52148148148148</v>
+        <v>21.65777777777778</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.57258134369886</v>
+        <v>20.69951704521253</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.967932970378711</v>
+        <v>3.993062028908907</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.479655594630922</v>
+        <v>6.520691480547218</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.53764232804254</v>
+        <v>20.66770793650816</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.42830254436812</v>
+        <v>17.53120233838336</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.256148799039434</v>
+        <v>4.28127785756963</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04607960758298587</v>
+        <v>0.04578962031316184</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04612450532724499</v>
+        <v>0.04629386910197875</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02519525344873941</v>
+        <v>0.02527505890851667</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02953534797274042</v>
+        <v>0.02934947670839319</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.0406028465259391</v>
+        <v>-0.04614514794490439</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1635680009252458</v>
+        <v>0.160865359695334</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1298280859.599813</v>
+        <v>1271783359.64692</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>308.74</v>
+        <v>310.20001</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1072234299314409</v>
+        <v>-0.1030015515869899</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2765319273579379</v>
+        <v>-0.2731106971294669</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,37 +3110,37 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>307849902580</v>
+        <v>309305705572</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>21.56005586592179</v>
+        <v>21.66201187150838</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>20.57412154818365</v>
+        <v>20.67141513891231</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.819701982432496</v>
+        <v>1.828307239632099</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>18.46828910152254</v>
+        <v>18.55562435698381</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.395600558659249</v>
+        <v>-7.430573839645349</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.40171033159105</v>
+        <v>15.46258438519757</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.177211321818698</v>
+        <v>2.1858165790183</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04905312580398088</v>
+        <v>0.04882224843564936</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04792108938547468</v>
+        <v>0.0479210893854749</v>
       </c>
       <c r="V21" s="4" t="n">
         <v>0.01423568777486173</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03009004340221545</v>
+        <v>0.02994841940849711</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7194471644235487</v>
+        <v>0.7080513697226719</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.251315174403697</v>
+        <v>0.2497970071062758</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1239314204.777323</v>
+        <v>1199809742.470005</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>516.13</v>
+        <v>494.125</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.309616490717519</v>
+        <v>1.211146898021417</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.1173191045439776</v>
+        <v>-0.1549518581225523</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.85</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>841601578000</v>
+        <v>805720225000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>130.997461928934</v>
+        <v>125.4124365482233</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>38.30146529942742</v>
+        <v>36.60731156027715</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>20.37529543638785</v>
+        <v>19.50660271153613</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>12.52243291086517</v>
+        <v>11.98854389801262</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.057594188050109</v>
+        <v>1.012504074884739</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>78.44668576226908</v>
+        <v>75.09892004105244</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>20.35568521970706</v>
+        <v>19.48699249485534</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.009984534510936956</v>
+        <v>0.01042917844094084</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.420168416660871</v>
+        <v>2.42588491759961</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8883604343143967</v>
+        <v>0.8908862032600786</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.533602493189448</v>
+        <v>2.54426273472138</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.672303867425101</v>
+        <v>0.6751876786133827</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10307044310.83171</v>
+        <v>10128306494.24566</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1698.3</v>
+        <v>1596.773</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4592963938606747</v>
+        <v>0.3720573989955196</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1508330166603332</v>
+        <v>-0.2015975319506391</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>833.92</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>654555374115</v>
+        <v>615425041743</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>53.64296081277213</v>
+        <v>50.35558962264151</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.00133660233855</v>
+        <v>32.88202121349596</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.1291333350506</v>
+        <v>15.14070077783596</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.10606724275385</v>
+        <v>24.50622390746561</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.651672374875111</v>
+        <v>3.427889004623443</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>40.93697402252889</v>
+        <v>38.40744733449237</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.9964463348383</v>
+        <v>15.00801377762366</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01755329173835631</v>
+        <v>0.01869922581994628</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5325974954107349</v>
+        <v>0.5314018957561457</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2864551702816613</v>
+        <v>0.2852182160662287</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004581051639875169</v>
+        <v>0.004872326874264533</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.687285180894966</v>
+        <v>1.694667569641459</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4028885051083511</v>
+        <v>0.424706163478566</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2050948937.47111</v>
+        <v>2020619636.414062</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>210.45</v>
+        <v>210.64999</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.07604163826481103</v>
+        <v>-0.07516360342155404</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.1725968154118341</v>
+        <v>-0.1718105366620798</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>166333366500</v>
+        <v>166491435676</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>78.82022471910109</v>
+        <v>78.89512734082395</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>84.14062311047331</v>
+        <v>83.76298271958655</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.769598026490771</v>
+        <v>1.771279702920368</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>27.291044772</v>
+        <v>27.31697936950037</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4218516503027515</v>
+        <v>0.4222525346531628</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>29.49415345323741</v>
+        <v>29.51689721956835</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.180800750039896</v>
+        <v>2.182482426469493</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001262524798354274</v>
+        <v>-0.001261326140575</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.06323221999897422</v>
+        <v>-0.05811463752501189</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.152523701668509</v>
+        <v>0.1529483038203574</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.223650238997503</v>
+        <v>1.242856591853039</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3374332140188102</v>
+        <v>0.3372040913177615</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1168522708.489583</v>
+        <v>1127510266.767813</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>1029.18</v>
+        <v>993.79</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.1255987595112515</v>
+        <v>0.08689324628800277</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1081551833204794</v>
+        <v>-0.1388226934375515</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>303615304260</v>
+        <v>293175006530</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>15.67915904936015</v>
+        <v>15.14000609384522</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.2131694053763</v>
+        <v>13.72281831984176</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.574385513112933</v>
+        <v>2.485861150699102</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.516309967248374</v>
+        <v>2.429782625344218</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3674977625374731</v>
+        <v>0.3548607643289953</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>27.33804683400759</v>
+        <v>27.00547913643169</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.27696400841127</v>
+        <v>7.188439645997439</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1367355315015635</v>
+        <v>-0.1416048403694735</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1031430500947468</v>
+        <v>0.1032723556468242</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3823711015222546</v>
+        <v>-0.3823282959808237</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01748965195592608</v>
+        <v>0.01811247849143179</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.561111812045423</v>
+        <v>1.56460922709919</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3182777581679786</v>
+        <v>0.3262811020805543</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1824376179.444377</v>
+        <v>1804383991.244456</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>243.29</v>
+        <v>249.94</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.1653859348198972</v>
+        <v>-0.1425728987993139</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.2682127173193768</v>
+        <v>-0.2482103110148589</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>229211780860</v>
+        <v>235476971960</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>21.24803493449782</v>
+        <v>21.82882096069869</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.86344951193065</v>
+        <v>19.37561604161878</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.317246492032939</v>
+        <v>3.407918896044691</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.637300330895159</v>
+        <v>6.81872187391153</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2590118987170374</v>
+        <v>0.2660916353542535</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.71233468096911</v>
+        <v>18.09857419148018</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.158093417369785</v>
+        <v>4.248765821381537</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.05946902008638755</v>
+        <v>0.05788676441072748</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1264130095112761</v>
+        <v>0.1266130023329546</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04578542708088928</v>
+        <v>0.04589294922825382</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02770356364832094</v>
+        <v>0.02696647195326879</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.9033016742139656</v>
+        <v>0.9001586591133746</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3321552392656185</v>
+        <v>0.3284580294484706</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1234853481.073049</v>
+        <v>1200885175.557023</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1115.25</v>
+        <v>1145.4698</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.0322948046220759</v>
+        <v>0.06026677730687147</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1372374579352493</v>
+        <v>-0.1138592813213167</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1050276650250</v>
+        <v>1078735874922</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>37.36180904522614</v>
+        <v>38.37419765494138</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>25.59658996630991</v>
+        <v>26.27326956641244</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.18353233445217</v>
+        <v>13.5407649822383</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>29.37657841140529</v>
+        <v>30.1725921520706</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.3960506466077799</v>
+        <v>0.4067823850792955</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>31.13765764172915</v>
+        <v>31.94597463423085</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>13.76117041754429</v>
+        <v>14.11840306533042</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01909392158268635</v>
+        <v>0.01859018548117725</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4596400963722727</v>
+        <v>0.4605794515958792</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2273126002782788</v>
+        <v>0.227779731796429</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3937,16 +3937,16 @@
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005998655010087425</v>
+        <v>0.005840398411202111</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3463582056680412</v>
+        <v>0.3418951356085352</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3219499093209016</v>
+        <v>0.328599026128182</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3192849885.978597</v>
+        <v>3123879242.694877</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>214.38</v>
+        <v>208.45</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1785596877039992</v>
+        <v>0.1459593567585533</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.07694294940796553</v>
+        <v>-0.102475780409042</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>338137286400</v>
+        <v>328784011187</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>17.23311897106109</v>
+        <v>16.75361655948553</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.92478333473714</v>
+        <v>15.48176079312228</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.672409379667902</v>
+        <v>2.598051044503632</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>3.050173252307163</v>
+        <v>2.965303796426275</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4384380410586198</v>
+        <v>0.4262387346900449</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.94041252598221</v>
+        <v>23.61981806010836</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.552713499672012</v>
+        <v>5.478355164507741</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.0463835271376922</v>
+        <v>-0.04771106143087023</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.0821572016914065</v>
+        <v>0.08215188074267821</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3274869152039972</v>
+        <v>-0.3275002082938857</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.019358149081071</v>
+        <v>0.01990885104341569</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.369518247912609</v>
+        <v>1.373229260772864</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2705377143985447</v>
+        <v>0.2779897535596553</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>884303144.0093485</v>
+        <v>868968590.9007822</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>975.26</v>
+        <v>926.12</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.091940772564329</v>
+        <v>1.936148502232509</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2229003984063745</v>
+        <v>-0.2620557768924303</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,40 +4120,40 @@
         <v>154.65</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1101448891400</v>
+        <v>1045950666800</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>21.76433831733988</v>
+        <v>20.66621066726177</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.267436501124496</v>
+        <v>5.951641913357892</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>12.20117521545517</v>
+        <v>11.58556045739637</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.92185854414042</v>
+        <v>10.37079217664112</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03102056379243497</v>
+        <v>0.02945540990055924</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.84335427676821</v>
+        <v>15.0316661487139</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.9949253539225</v>
+        <v>11.38040027693467</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02376142933580332</v>
+        <v>0.02502167228932509</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.472606114706539</v>
+        <v>2.472354514621996</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.765110056317434</v>
+        <v>1.764909716313137</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005434448249697517</v>
+        <v>0.0005722800501014988</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.884074907778928</v>
+        <v>2.883347275231924</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8406891342442575</v>
+        <v>0.8248513252611771</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>27580450013.27393</v>
+        <v>26663728391.69365</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>132.53</v>
+        <v>142.41</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.1011868243949805</v>
+        <v>-0.03418105834218044</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.319402647823095</v>
+        <v>-0.2686646878177542</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>137017730860</v>
+        <v>147232287420</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>82.31677018633542</v>
+        <v>88.45341614906833</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.99208426195769</v>
+        <v>30.06241544274229</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.300687677165355</v>
+        <v>9.994046118653271</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>10.93827820389901</v>
+        <v>11.75371764141898</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>131.7068322981395</v>
+        <v>141.5254658385124</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>40.97670703926627</v>
+        <v>43.90138793063915</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>9.704570381482487</v>
+        <v>10.39722661485202</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03342633082049568</v>
+        <v>0.03110949307241409</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.940716004424403</v>
+        <v>1.94232565302476</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2445053550059697</v>
+        <v>0.2450681773312406</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.7425686691485414</v>
+        <v>0.7207905166666362</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6075948118380816</v>
+        <v>0.6285644861216921</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2252923509.665476</v>
+        <v>2225653407.549097</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.72</v>
+        <v>27.7899</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.100873695950755</v>
+        <v>0.1036497086256092</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.05100992810681282</v>
+        <v>-0.04861691201643281</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>157988476800</v>
+        <v>158386867656</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.62790697674419</v>
+        <v>36.72026955602537</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.493088068672243</v>
+        <v>9.51772209731608</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.480351620195931</v>
+        <v>2.486606186510927</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.85439934264585</v>
+        <v>1.859075479516375</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6126260547437744</v>
+        <v>-0.6141708801848491</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.44347883396705</v>
+        <v>17.47282480988593</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.457147651343883</v>
+        <v>3.46296377166541</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06953671699681833</v>
+        <v>0.06937404337418766</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.858376400996264</v>
+        <v>2.858094319267862</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05010572930318846</v>
+        <v>-0.05021253784362711</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06204906204906205</v>
+        <v>0.06189298989920799</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3541261297162214</v>
+        <v>0.3493970084106297</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2146777093459052</v>
+        <v>0.2087004289670491</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>999586815.2629089</v>
+        <v>974752994.2939217</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>190.07</v>
+        <v>176.64</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.1313017452200826</v>
+        <v>0.05136602449453043</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.04903187071596549</v>
+        <v>-0.1162255466052935</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1349221191324</v>
+        <v>1253887679462</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.917142991467138</v>
+        <v>7.414675307130095</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003950478887045561</v>
+        <v>0.00366847881386825</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.799454886225326</v>
+        <v>6.3679221533799</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.927298446329551</v>
+        <v>4.614583589084575</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01771757741788015</v>
+        <v>0.01659311748241866</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.998062425067403</v>
+        <v>7.488190590983496</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.769202581976064</v>
+        <v>6.337669849130638</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07089086128968651</v>
+        <v>0.07569489726394341</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2003.097026674181</v>
+        <v>2020.185260522643</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2585.930107902172</v>
+        <v>2609.025817305346</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.578365865207555</v>
+        <v>1.698369565217391</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.9937298607955094</v>
+        <v>0.9828267271293428</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3435314431.302287</v>
+        <v>3297475706.806618</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>568.53</v>
+        <v>544.33</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.5229842448194917</v>
+        <v>0.4581570259838426</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1537591354955867</v>
+        <v>-0.1897801527172053</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>301.37</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>71657946460</v>
+        <v>68607760359</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.820053339756524</v>
+        <v>1.825324155626536</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.3986133560350327</v>
+        <v>0.41033915708003</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3961573225.916544</v>
+        <v>3816249805.74646</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>151.21</v>
+        <v>152.04</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.06051567028842098</v>
+        <v>-0.0553587891716919</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.329861726644212</v>
+        <v>-0.3261833008331856</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1977201613485</v>
+        <v>1988054581802</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-98.18831168831169</v>
+        <v>-98.74025974025975</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>137.6590676676727</v>
+        <v>137.802885451069</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>119.2881818090498</v>
+        <v>119.9587390112217</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.969561089102686</v>
+        <v>7.008739231591524</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9818831168831168</v>
+        <v>-0.9874025974025975</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>461.4935477525798</v>
+        <v>464.1608109217663</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>116.0207308286576</v>
+        <v>116.6912880308296</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01437536759334413</v>
+        <v>-0.01429501074437222</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.184692245707556</v>
+        <v>4.195423725844542</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.457810540572236</v>
+        <v>3.441642708883008</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.783814195599935</v>
+        <v>0.7835565208528544</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>14188247188.11424</v>
+        <v>14192963950.06558</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>764.29</v>
+        <v>762.13</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1187406050018327</v>
+        <v>0.1155788735820786</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01934896134056996</v>
+        <v>-0.02212043060420599</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>814150923750</v>
+        <v>811850009181</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9952270977144121</v>
+        <v>0.9952897736453762</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1151986111457538</v>
+        <v>0.1151115487778224</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>30936755297.01904</v>
+        <v>29891923999.91215</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>433.24</v>
+        <v>420.435</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3555271107172935</v>
+        <v>0.3154626553282829</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.09553235908141966</v>
+        <v>-0.1222651356993737</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>257.98</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2246990595200</v>
+        <v>2180577718800</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.93555117653877</v>
+        <v>27.58780572620842</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.662234378283926</v>
+        <v>0.6422159848404414</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.07436022855125</v>
+        <v>13.89916072363153</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.714817505368815</v>
+        <v>9.59388616712771</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5247819590387496</v>
+        <v>0.5182494035320432</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.51345021489235</v>
+        <v>18.27477474575392</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.58978081708063</v>
+        <v>13.41458131216091</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01789632973916031</v>
+        <v>0.01812191372746905</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.18378280047808</v>
+        <v>41.95720813156435</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.15666372328758</v>
+        <v>41.93251569219548</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.253900840180962</v>
+        <v>0.2616337840569886</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.161816965705875</v>
+        <v>2.179047823951394</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3552040270120096</v>
+        <v>0.3630682379655741</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4139233405.578207</v>
+        <v>4086501824.133639</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.04</v>
+        <v>28.1228</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.01648545159974102</v>
+        <v>-0.01358120749818814</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.06533333333333335</v>
+        <v>-0.06257333333333326</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>70300113124</v>
+        <v>70507704043</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.07874015748031</v>
+        <v>-22.14393700787402</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-80.68007820889312</v>
+        <v>-81.65117073184392</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.946562733600997</v>
+        <v>1.952310786183026</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.14411474511237</v>
+        <v>2.150446153846154</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.164306903497528</v>
+        <v>0.164792089360923</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.35605175603306</v>
+        <v>16.3903643046281</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.739972674068946</v>
+        <v>2.745720726650976</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03100990742582123</v>
+        <v>0.03091860711661381</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02043303423553744</v>
+        <v>0.02050670921914222</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2915347672171608</v>
+        <v>0.2531405301144675</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.1902322332709558</v>
+        <v>0.1891923299751187</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>532577590.4036903</v>
+        <v>503867970.4693958</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>324.69</v>
+        <v>327.07</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1288868874797695</v>
+        <v>-0.1225015685361674</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1620686985470593</v>
+        <v>-0.155926604557537</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>219266403900</v>
+        <v>220873641700</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>19.69011522134627</v>
+        <v>19.83444511825349</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.72171575281377</v>
+        <v>16.83829513817301</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.608047814399391</v>
+        <v>2.627164984001998</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.421815052508752</v>
+        <v>6.46888739789965</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.220959109795273</v>
+        <v>1.229908823926638</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.426969903737259</v>
+        <v>9.491977095130238</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.772262247094787</v>
+        <v>2.791379416697394</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06864708743462911</v>
+        <v>0.06814756113110258</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1775176370901419</v>
+        <v>0.1779366589963201</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.005425181638038401</v>
+        <v>0.005658273890123855</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01090270719763467</v>
+        <v>0.01082337114379185</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9685305146415542</v>
+        <v>0.96112052940579</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.222332815308943</v>
+        <v>0.2216990654609904</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>780674338.0948893</v>
+        <v>765001632.2843527</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>150.15</v>
+        <v>143.56</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2327934451531496</v>
+        <v>-0.266465714193714</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.544309559939302</v>
+        <v>-0.564309559939302</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>329.5</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>432502570500</v>
+        <v>413520273200</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>23.1712962962963</v>
+        <v>22.15432098765432</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.77375562030881</v>
+        <v>16.02329270350585</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.025642900929268</v>
+        <v>5.761180784931106</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.669635475948002</v>
+        <v>6.376908883963337</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.5043164488017432</v>
+        <v>0.4821822803195354</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>14.71897433812355</v>
+        <v>14.21287421547978</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.69138540897502</v>
+        <v>7.426923292976859</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.06640422961370585</v>
+        <v>-0.06945245943506501</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3814018053441572</v>
+        <v>0.3826322340605446</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4198565143825406</v>
+        <v>0.4214263744375701</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01332001332001332</v>
+        <v>0.0139314572304263</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.030285433679443</v>
+        <v>2.074118099546188</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5780162656733132</v>
+        <v>0.5850709403993845</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4228908166.034698</v>
+        <v>4196707225.397536</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13 11:21 ET</t>
+          <t>2026-09-14 13:18 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-15)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -446,7 +446,7 @@
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="23" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,55 +699,55 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>333.08</v>
+        <v>329.64999</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2290320947482876</v>
+        <v>0.2163756987614149</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.03334590939431759</v>
+        <v>-0.04330037437966161</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>235.03</v>
+        <v>236.32</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4892064536480</v>
+        <v>4841686815755</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.02283105022831</v>
+        <v>37.63127739726028</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.82980592337726</v>
+        <v>34.4557922898374</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.47948480790364</v>
+        <v>10.37156870110299</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.51509390066965</v>
+        <v>45.04638600097518</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.161808726534753</v>
+        <v>1.149844587138507</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.30111425566516</v>
+        <v>29.00211184166637</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.57537339951116</v>
+        <v>10.46745729271051</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02793973770802866</v>
+        <v>0.02823045050233924</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.0916750766247576</v>
+        <v>0.09216114030149503</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1170296262044463</v>
+        <v>0.117919601370001</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003182418638165006</v>
+        <v>0.003215531721993985</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3089528812044592</v>
+        <v>0.3091698218796033</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2976224928133763</v>
+        <v>0.2956148449247202</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13912657866.93765</v>
+        <v>13293888719.37706</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>505.41</v>
+        <v>501.7073</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.06865563790539486</v>
+        <v>0.06082652643060737</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.08724626164848659</v>
+        <v>-0.09393321534349497</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3752947225500</v>
+        <v>3725452641515</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.07833333333333</v>
+        <v>27.87262777777778</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.64745626585675</v>
+        <v>24.45461871090728</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.30954235487691</v>
+        <v>11.22668716309717</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.487344542222081</v>
+        <v>8.425165142058875</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8918616782675931</v>
+        <v>0.8853277825470466</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.60466041904597</v>
+        <v>18.46904471879683</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.63461957605947</v>
+        <v>11.54981087515331</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.0178491718574794</v>
+        <v>0.01798403163448161</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1391980182648402</v>
+        <v>0.1397694687975646</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2248874130489094</v>
+        <v>0.2255150471434921</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007202073564037118</v>
+        <v>0.007255226304261469</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5569011303466421</v>
+        <v>0.5562011142553257</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4340989304501802</v>
+        <v>0.4348274611586234</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>12567165071.80573</v>
+        <v>11582425696.22803</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>349.39</v>
+        <v>343.66</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.1086466976571234</v>
+        <v>0.09046487912317769</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1449303737059788</v>
+        <v>-0.1589535253664863</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4228356662216</v>
+        <v>4159011564547</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>17.16534260178749</v>
+        <v>16.88828699106256</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.87638515618916</v>
+        <v>20.55242197065229</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.409784187807546</v>
+        <v>9.257906444063909</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.558709421059206</v>
+        <v>6.452849183581066</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1526523901172095</v>
+        <v>0.1501885184571042</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>13.11384500493733</v>
+        <v>12.90501170215935</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.537277649968823</v>
+        <v>9.385399906225187</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01269764366126457</v>
+        <v>0.01290595095857692</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1777626982179659</v>
+        <v>-0.1782823934240892</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2888869437375823</v>
+        <v>0.2899304626314998</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.00246143278285011</v>
+        <v>0.002502473374847233</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.770142024141324</v>
+        <v>0.7724142410527388</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3825682892334387</v>
+        <v>0.3684584056345456</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8698173074.388248</v>
+        <v>8312541467.382883</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>253.54</v>
+        <v>249.49</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1193818984547461</v>
+        <v>0.1015011037527593</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1172005571030641</v>
+        <v>-0.1313022284122562</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2727355134000</v>
+        <v>2683788879000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.12222222222222</v>
+        <v>19.80079365079365</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.4993907262407</v>
+        <v>22.15156853341933</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.516082835705446</v>
+        <v>3.459917593595297</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.943758819477176</v>
+        <v>4.864788151263551</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2277794698251551</v>
+        <v>0.2241409636612682</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.30869314991909</v>
+        <v>11.13717043508388</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.703040086117987</v>
+        <v>3.646874844007839</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004262371209044022</v>
+        <v>-0.004331562773421865</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.105654794520548</v>
+        <v>-0.1061222765818658</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1781464823768628</v>
+        <v>0.1785740462863659</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8318374772658809</v>
+        <v>0.8345785311076686</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4606663575162792</v>
+        <v>0.4596911307758973</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>9478337928.275068</v>
+        <v>8741121385.194023</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>210.96</v>
+        <v>212.27</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1170770091707865</v>
+        <v>0.1240137312129448</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.1081423860657816</v>
+        <v>-0.1026042107043206</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5109662160000</v>
+        <v>5141391670000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>26.53584905660377</v>
+        <v>26.7006289308176</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>15.8033588666192</v>
+        <v>15.87557250715581</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>16.86529697757857</v>
+        <v>16.97002554716819</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>22.28593438842888</v>
+        <v>22.42432353352199</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2130088563727378</v>
+        <v>0.2143315791725495</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>21.93754000350927</v>
+        <v>22.06992952021466</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>16.91948403962122</v>
+        <v>17.02159039769746</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02485604645141549</v>
+        <v>0.02470646785478988</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6791271577496334</v>
+        <v>0.6818687274920301</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9328589725338057</v>
+        <v>0.9361767872730502</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002464922260144103</v>
+        <v>0.00244971027465021</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.329315524502224</v>
+        <v>1.327525487399058</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4171953561352091</v>
+        <v>0.4130089407334011</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27437808210.02829</v>
+        <v>26835566161.85361</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>665.6</v>
+        <v>668.025</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.02335454172393714</v>
+        <v>0.02708295933763982</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.1583206879109762</v>
+        <v>-0.1552541729893778</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1695607060992</v>
+        <v>1701784715924</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>24.73429951690822</v>
+        <v>24.82441471571907</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>20.1333674489426</v>
+        <v>20.20271885011575</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7.428792633416284</v>
+        <v>7.455858171480145</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>6.479650564081755</v>
+        <v>6.503258065010088</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.07053140096618</v>
+        <v>-5.089005016722404</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>16.7407264363419</v>
+        <v>16.79842270550657</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.853138082226351</v>
+        <v>7.880203620290211</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.0241659762704853</v>
+        <v>0.02407825127149041</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2285227287304716</v>
+        <v>0.2287660339131454</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2711651259227765</v>
+        <v>0.271779256228301</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003155048076923077</v>
+        <v>0.003143594925339621</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7765247561934626</v>
+        <v>0.7749251316420632</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4182632984941506</v>
+        <v>0.4138640761944271</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10178323576.6413</v>
+        <v>9868792832.16403</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>358.97</v>
+        <v>360.355</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1805647636261851</v>
+        <v>-0.177403168500192</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2803760800272638</v>
+        <v>-0.2775995830242768</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1417769028024</v>
+        <v>1423239151165</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>304.2118644067797</v>
+        <v>305.3898220338983</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>170.780954479354</v>
+        <v>171.3141249024022</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.68251988558083</v>
+        <v>13.73550064222778</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.37799500333878</v>
+        <v>13.42979676748256</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.09803413702554</v>
+        <v>-8.129391037240389</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>117.383773530429</v>
+        <v>117.8631831741769</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.62580248819232</v>
+        <v>13.68145192695355</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.00406413166468358</v>
+        <v>0.004047669016651527</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7812985372649175</v>
+        <v>0.7826307212430914</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1219390435997418</v>
+        <v>0.1223280851497379</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.546711064330438</v>
+        <v>1.538872399802141</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5751696838324828</v>
+        <v>0.5751269196894302</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12819667448.53803</v>
+        <v>12579569948.95085</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>344.72</v>
+        <v>339.815</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-0.008342428968189375</v>
+        <v>-0.0224526644808114</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.3035959595959595</v>
+        <v>-0.3135050505050505</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1640032977600</v>
+        <v>1616697047700</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>42.76923076923077</v>
+        <v>42.1575682382134</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>18.83645800017926</v>
+        <v>18.59967808038237</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.40582889208116</v>
+        <v>18.14259862856886</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.4804445781924</v>
+        <v>16.24475012538871</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4255750190403653</v>
+        <v>0.4194886740535094</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>32.05856873122477</v>
+        <v>31.60978336873122</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>18.80361125875381</v>
+        <v>18.54038099524151</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02402573639565575</v>
+        <v>0.02437432487804365</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.270555895849621</v>
+        <v>1.266575155549506</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8585251496160557</v>
+        <v>0.8524380480254286</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007368298909259689</v>
+        <v>0.00747465532716331</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.603839698015839</v>
+        <v>1.605031466464408</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.4063188828354903</v>
+        <v>0.3888980769216379</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8718298436.112564</v>
+        <v>8604532715.337473</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>918.91</v>
+        <v>907.97</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.07537741369221762</v>
+        <v>0.06257460503218248</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1619607843137255</v>
+        <v>-0.171937984496124</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,31 +1724,31 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>407517287890</v>
+        <v>402665627630</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>46.15318935208438</v>
+        <v>45.60371672526369</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.54259153860747</v>
+        <v>40.05991537725069</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.388063122311274</v>
+        <v>1.371537662192127</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.17360362678683</v>
+        <v>12.02867188844788</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.640744892193446</v>
+        <v>3.597400332747367</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.42248015825847</v>
+        <v>27.0871891935038</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.351569680844179</v>
+        <v>1.335044220725032</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02160889920914712</v>
+        <v>0.02186926172921724</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006028882045031614</v>
+        <v>0.00610152317807857</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1908042222803441</v>
+        <v>-0.1892386300769955</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1874983102170152</v>
+        <v>0.1726876444671286</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1727701780.661401</v>
+        <v>1679329850.192424</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>80.31999999999999</v>
+        <v>77.82859999999999</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1172656128615882</v>
+        <v>-0.1446466443869447</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3567195258689733</v>
+        <v>-0.3766730738427039</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>334447660720</v>
+        <v>324073620606</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>24.86687306501548</v>
+        <v>24.09554179566564</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.42230818516562</v>
+        <v>20.75455762698772</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.9142521858865</v>
+        <v>6.699782964064823</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>11.15959925248205</v>
+        <v>10.8134460455892</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.7308434644717966</v>
+        <v>0.7081738503360268</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>11.10100051906985</v>
+        <v>10.76194678079623</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7.021963405829191</v>
+        <v>6.807494184007513</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03287392704834823</v>
+        <v>0.03392626644353429</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1607933584969676</v>
+        <v>0.1609759277323042</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1431026964010345</v>
+        <v>0.1434269861448505</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.09470983751137689</v>
+        <v>0.1001273037800634</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3738594083527357</v>
+        <v>0.3823242582324036</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2207519621.929148</v>
+        <v>2152766013.596189</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>514.95</v>
+        <v>515.41998</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.03642949315515032</v>
+        <v>0.03737541243506692</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.04238107635660349</v>
+        <v>-0.04150708520846502</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1110671758745</v>
+        <v>1111685443075</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.94483626351116</v>
+        <v>12.96914202743653</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.21377362560879</v>
+        <v>23.23493301977915</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.887110881105938</v>
+        <v>2.892531840790045</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.478233323602297</v>
+        <v>1.481008916082471</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3565972736916762</v>
+        <v>0.3572668355906716</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.67549760200748</v>
+        <v>15.70275238829495</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.117846518130324</v>
+        <v>3.123267477814431</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02180286168728554</v>
+        <v>0.02176200044851258</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4423639830264056</v>
+        <v>-0.4418257192135512</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06056996350464527</v>
+        <v>0.06163788923813973</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.05495250038840038</v>
+        <v>0.05420570709557663</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1410426740836873</v>
+        <v>0.1394374697778777</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2109431408.5975</v>
+        <v>2052405133.490605</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>350.13</v>
+        <v>343.58499</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.07573426380001957</v>
+        <v>0.05562547131176165</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.04466575716234655</v>
+        <v>-0.0625239017735334</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>938176836300</v>
+        <v>920639420454</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.05288048151333</v>
+        <v>14.77149613069647</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.98090238673174</v>
+        <v>13.71894780439785</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.152126398282448</v>
+        <v>3.093203520274969</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.60654763506479</v>
+        <v>2.557823291902253</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7881575222626153</v>
+        <v>0.7734244488807034</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.03259807106054</v>
+        <v>19.84434782471018</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.270261820093874</v>
+        <v>6.211338942086395</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1732445246047693</v>
+        <v>-0.1765446844299602</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07667445670738182</v>
+        <v>0.07672223419067215</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2894796085946888</v>
+        <v>-0.2894273564515862</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01713649216005484</v>
+        <v>0.01746292816807859</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7722642455725528</v>
+        <v>0.7774690338025343</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1717842435974667</v>
+        <v>0.1761580139505628</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2015473213.400635</v>
+        <v>1989747020.048416</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>375.28</v>
+        <v>374.875</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.08312164656104293</v>
+        <v>0.08195274796037899</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.02668776097725456</v>
+        <v>-0.02773815390201517</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>700665477344</v>
+        <v>699909323224</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.88445199660153</v>
+        <v>31.8500424808836</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.11301062870593</v>
+        <v>25.05682103741701</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.74953869232153</v>
+        <v>15.73254188149613</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.41275488316561</v>
+        <v>20.39072555645574</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.150102848455038</v>
+        <v>2.147782469928007</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.47468820345041</v>
+        <v>24.44870173977593</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>16.00801288761014</v>
+        <v>15.99101607678475</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.02999006042035009</v>
+        <v>0.03002246048560632</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2696387728262009</v>
+        <v>0.2711126616310333</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1375240610011503</v>
+        <v>0.1378301271625042</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007141334470262205</v>
+        <v>0.007149049683227743</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3051853919994814</v>
+        <v>0.3043837886111914</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1922583442671653</v>
+        <v>0.1804852376382017</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2277087061.263021</v>
+        <v>2227520172.995125</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>574.42</v>
+        <v>572.57001</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.02004864777101845</v>
+        <v>0.01676345610309293</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.04521126292344013</v>
+        <v>-0.04828627705195965</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>503787019120</v>
+        <v>502164508944</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.54420647995606</v>
+        <v>31.44261449752883</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.9211571714777</v>
+        <v>25.82767643578532</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.35986144628452</v>
+        <v>14.31361368594476</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>90.293787203707</v>
+        <v>90.00298499732669</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.394141268533772</v>
+        <v>1.389651265738997</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.3830267281606</v>
+        <v>23.30966309206005</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.74044463472337</v>
+        <v>14.6941968743836</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03264871736618159</v>
+        <v>0.03275420645435186</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2169289461608479</v>
+        <v>0.2174000466400365</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1564551345566814</v>
+        <v>0.1568220736126735</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005866787368127851</v>
+        <v>0.005885743125107094</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2935817535320609</v>
+        <v>0.2932120098584461</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2089175877623677</v>
+        <v>0.1966852027236337</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1558005584.737655</v>
+        <v>1502088672.713576</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>383.55</v>
+        <v>376.91</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1401605438733284</v>
+        <v>0.1204221368564626</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1691217884840345</v>
+        <v>-0.1835059139552012</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>348318786154</v>
+        <v>342288707312</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.6640087454183</v>
+        <v>24.23638351231432</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.71391360958151</v>
+        <v>17.39397073555487</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7738199186322142</v>
+        <v>0.760403408507339</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.529768803010757</v>
+        <v>3.468569578554958</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.747325904675142</v>
+        <v>-0.7343687484605945</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.25683290587276</v>
+        <v>15.02242075332842</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8732203127414585</v>
+        <v>0.8598038026165832</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.0678028315979442</v>
+        <v>0.06899914051299065</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3923523219666976</v>
+        <v>0.3933784229481845</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01038134275007363</v>
+        <v>0.01030214158350229</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02362143136488072</v>
+        <v>0.02403756865034093</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4244573418377957</v>
+        <v>0.4292037814150745</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2274900484914662</v>
+        <v>0.2279204356412717</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1786599094.704653</v>
+        <v>1765890067.196583</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>165.07</v>
+        <v>169.015</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.345862192795575</v>
+        <v>0.3780268886856732</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.0642820701774276</v>
+        <v>-0.04191939232469821</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>684126012200</v>
+        <v>700475904370</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.24453024453024</v>
+        <v>21.75225225225225</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.93324004171107</v>
+        <v>15.29337721023762</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.894770985985709</v>
+        <v>1.94005401974741</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.656247916454622</v>
+        <v>2.719729457803223</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.080193586443587</v>
+        <v>2.129908033033034</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.96736529342151</v>
+        <v>10.1941349112426</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.982789597850773</v>
+        <v>2.027900459757381</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04465990103453049</v>
+        <v>0.04362136014065058</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4226336806473792</v>
+        <v>0.422331506849315</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08231581936981591</v>
+        <v>0.08215438117185392</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02495910825710305</v>
+        <v>0.02437653462710411</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5434105106913146</v>
+        <v>-0.5496265863345695</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2310004784818244</v>
+        <v>0.235769764287829</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2246422120.522645</v>
+        <v>2195624573.778361</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>266.32</v>
+        <v>264.25299</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2843983224531217</v>
+        <v>0.2744296224813065</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.0524780303838901</v>
+        <v>-0.05983210588109722</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>641804146149</v>
+        <v>636822863766</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>30.78843930635838</v>
+        <v>30.54947861271677</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.42782194813772</v>
+        <v>21.35042362672566</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.553770038997641</v>
+        <v>6.502903774836872</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.647873180261501</v>
+        <v>7.588515151039767</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.812094919379379</v>
+        <v>-3.782507812442963</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.87484128272856</v>
+        <v>19.72716897207399</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.845961320436235</v>
+        <v>6.795095056275465</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02914907937608865</v>
+        <v>0.02937708594406598</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4368440890015042</v>
+        <v>0.430860536859609</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08854415069248511</v>
+        <v>0.08875387185717587</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01982577350555723</v>
+        <v>0.01998085243992887</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1737476460406477</v>
+        <v>-0.170768375962891</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2111034178170654</v>
+        <v>0.2108267922654884</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1680843383.236509</v>
+        <v>1625599304.065869</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>109.08</v>
+        <v>108.3937</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.03263570474027211</v>
+        <v>-0.03872208277324563</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.1929564960047351</v>
+        <v>-0.1980341817105653</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>868067366400</v>
+        <v>862605736096</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>39.37906137184116</v>
+        <v>39.13129963898917</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>35.18621704102511</v>
+        <v>34.95437599517003</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.179695812133072</v>
+        <v>1.17227350524027</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.831840224760276</v>
+        <v>8.776272825179666</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.522573022645233</v>
+        <v>9.462659730882843</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.7160383388968</v>
+        <v>21.5885463268517</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.264260391389433</v>
+        <v>1.25683808449663</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01556215625985776</v>
+        <v>0.01566068881148337</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1191615548192475</v>
+        <v>0.119496444290589</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.0508222140108292</v>
+        <v>0.05094654776722218</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.008961312797946461</v>
+        <v>0.009018051787142611</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.06001157526822717</v>
+        <v>-0.0572910695089674</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3114822793533726</v>
+        <v>0.3067937513722329</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2780804758.730911</v>
+        <v>2718864815.912511</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>146.13</v>
+        <v>146.8</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.03060869539015365</v>
+        <v>0.03533399358978029</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1262780269058297</v>
+        <v>-0.1222720478325858</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>347381541964</v>
+        <v>348974271952</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.64888888888889</v>
+        <v>21.74962962962963</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.69102145028324</v>
+        <v>20.78252485599786</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.991423177268131</v>
+        <v>4.009996829223734</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.518015227117894</v>
+        <v>6.548346099316896</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.65922539682562</v>
+        <v>20.75536084656106</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.52449148226216</v>
+        <v>17.60054785174555</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.279639005928854</v>
+        <v>4.298212657884457</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04580842122477855</v>
+        <v>0.04559624408132944</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04629386910197875</v>
+        <v>0.04653451783807983</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02527505890851667</v>
+        <v>0.0254247114288122</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02936152740710327</v>
+        <v>0.0292275204359673</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.04674076747521385</v>
+        <v>-0.04847916959282902</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.160764734967262</v>
+        <v>0.1503064794297618</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1296332418.248112</v>
+        <v>1266167775.389949</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>310.87</v>
+        <v>305.975</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.101064156451341</v>
+        <v>-0.1152189187448099</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2715407147041593</v>
+        <v>-0.2830111306385471</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,31 +3110,31 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>309973761790</v>
+        <v>305092874075</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>21.70879888268156</v>
+        <v>21.36696927374302</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>20.7160625953354</v>
+        <v>20.38986474284347</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.832256122558755</v>
+        <v>1.803405176118362</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>18.59570199193597</v>
+        <v>18.30289161701872</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.446622872547778</v>
+        <v>-7.329367367156067</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.4905189960276</v>
+        <v>15.28642584465816</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.189765461944957</v>
+        <v>2.160914515504563</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04871702660507948</v>
+        <v>0.04949640349937432</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.0298838742882877</v>
+        <v>0.03036195767628074</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7058868672376516</v>
+        <v>0.7093609924436535</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2502242802873501</v>
+        <v>0.246540985956761</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1226694079.953125</v>
+        <v>1204944344.503112</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>493.41</v>
+        <v>503.7806</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.207947363425748</v>
+        <v>1.254354487170996</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.1561746447078138</v>
+        <v>-0.1384389376293332</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.85</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>804554346000</v>
+        <v>821464646360</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>125.2309644670051</v>
+        <v>127.8630964467005</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36.55434069710366</v>
+        <v>37.26047429516517</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>19.47837661300085</v>
+        <v>19.88777742065125</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.97119644769725</v>
+        <v>12.22280968999167</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.01103897918316</v>
+        <v>1.032289219019233</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>74.9901423773092</v>
+        <v>76.56789012502333</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>19.45876639632006</v>
+        <v>19.86816720397047</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01044429135430958</v>
+        <v>0.01022928988756195</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.425884917599611</v>
+        <v>2.431601418538349</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8908862032600786</v>
+        <v>0.8934119722057594</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.545669055146133</v>
+        <v>2.540662423834458</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6757380094899845</v>
+        <v>0.6645158515052284</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10291128789.90689</v>
+        <v>10050294689.56701</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -3347,55 +3347,55 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1575.15</v>
+        <v>1591.82</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.3534774273035635</v>
+        <v>0.3678014400726015</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.2124092481849637</v>
+        <v>-0.2040740814816296</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>833.92</v>
+        <v>861.1799999999999</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>607091148524</v>
+        <v>613516066434</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>50.35558780841799</v>
+        <v>50.0290293904209</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>32.43674317792082</v>
+        <v>32.76890300288574</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.14070024513481</v>
+        <v>15.04251206029297</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>24.50622302454937</v>
+        <v>24.34729898512742</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.427888881122619</v>
+        <v>3.405658856237435</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>38.40744597124126</v>
+        <v>38.15616971349922</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.00801324492251</v>
+        <v>14.90982506008067</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01869922647784843</v>
+        <v>0.01882128342541458</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5524242841585354</v>
+        <v>0.5267227403375445</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3028611080328747</v>
+        <v>0.2824150857016017</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004939212138526489</v>
+        <v>0.004887487278712418</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.701372357510302</v>
+        <v>1.698471322134239</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4376047884782998</v>
+        <v>0.4375226644691245</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2066909334.696265</v>
+        <v>2040826459.700114</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>210.27</v>
+        <v>210.27991</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.07683190913728588</v>
+        <v>-0.07678840033536238</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.1733045016709258</v>
+        <v>-0.1732655396107725</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>166191099900</v>
+        <v>166198930275</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>78.75280898876402</v>
+        <v>78.7565205992509</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>83.61188327826393</v>
+        <v>83.16396587710337</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.768084471514442</v>
+        <v>1.76816777780733</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>27.26770246713443</v>
+        <v>27.26898759069675</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4214908363466836</v>
+        <v>0.4215107011594871</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>29.47368343884892</v>
+        <v>29.47481011151079</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.179287195063567</v>
+        <v>2.179370501356455</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001263605572899876</v>
+        <v>-0.001263546038789328</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.058114637525012</v>
+        <v>-0.05299705505104968</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1529483038203576</v>
+        <v>0.1533729156417385</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.242098762420381</v>
+        <v>1.238902943540715</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3371627648070844</v>
+        <v>0.3345804216929615</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1139446719.053749</v>
+        <v>1059990284.618443</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>988.45</v>
+        <v>957.33</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.08105296822606012</v>
+        <v>0.04701749008230482</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1434501165521365</v>
+        <v>-0.1704174212948119</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>291599669150</v>
+        <v>282419051310</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>15.05865326020719</v>
+        <v>14.5845521023766</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.64908055851598</v>
+        <v>13.21780872300822</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.472503702400434</v>
+        <v>2.394660295835912</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.416726507633899</v>
+        <v>2.340639169966271</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3529539666337912</v>
+        <v>0.3418416924250365</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.95529796929252</v>
+        <v>26.66285641098334</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.175082197698771</v>
+        <v>7.09723879113425</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1423698460324539</v>
+        <v>-0.1469978735762789</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1032723556468242</v>
+        <v>0.1034016611989015</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3823282959808239</v>
+        <v>-0.382285490439393</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.0182103293034549</v>
+        <v>0.01880229387985334</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.568896240889311</v>
+        <v>1.576163907424641</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3297536656376204</v>
+        <v>0.3163673996164783</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1844065424.760997</v>
+        <v>1814797433.898621</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>249.09</v>
+        <v>250.2</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.1454888507718697</v>
+        <v>-0.1416809605488851</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.2507670095650604</v>
+        <v>-0.247428262046562</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>234676158060</v>
+        <v>235721926800</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>21.75458515283843</v>
+        <v>21.85152838427948</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>19.30972313277915</v>
+        <v>19.3923290539268</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.396329190268753</v>
+        <v>3.411463982517331</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.795532654127483</v>
+        <v>6.825815047021944</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2651867066111507</v>
+        <v>0.2663684370874378</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>18.04920523149005</v>
+        <v>18.11367528512422</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.237176115605598</v>
+        <v>4.252310907854176</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.05808429843356708</v>
+        <v>0.05782661029902968</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1266130023329546</v>
+        <v>0.1268129951546333</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04589294922825382</v>
+        <v>0.04600047137561836</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02705849291420772</v>
+        <v>0.02693844924060752</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8971252793196376</v>
+        <v>0.8934888010026703</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3271665812957038</v>
+        <v>0.3168137635713446</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1220828464.444655</v>
+        <v>1174690553.0539</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1137.75</v>
+        <v>1145.35999</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.05312119610739008</v>
+        <v>0.06016513526024903</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.119831354194871</v>
+        <v>-0.1139442308436159</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,52 +3868,52 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1071465822750</v>
+        <v>1078632457965</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.11557788944724</v>
+        <v>38.3191699565072</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.09620301572835</v>
+        <v>26.25381288957396</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.44950810448147</v>
+        <v>13.53946684731717</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>29.96924643584521</v>
+        <v>30.16969966870332</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4040409084761278</v>
+        <v>0.4050808331259123</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>31.73948599039991</v>
+        <v>25.97057273015924</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.02714618757359</v>
+        <v>14.11710493040929</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.0187163226061006</v>
+        <v>0.01859196786812317</v>
       </c>
       <c r="T27" s="4" t="n">
-        <v>0.4470491333778837</v>
+        <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.460579451595879</v>
+        <v>0.4595658968730096</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.227779731796429</v>
+        <v>0.228246464557607</v>
       </c>
       <c r="W27" s="4" t="n">
-        <v>0.1877209505000597</v>
+        <v>0.1877328985191485</v>
       </c>
       <c r="X27" s="4" t="n">
-        <v>0.9257633748190075</v>
+        <v>0.9258222975894521</v>
       </c>
       <c r="Y27" s="4" t="n">
-        <v>0.8401195996274436</v>
+        <v>0.8339940099766776</v>
       </c>
       <c r="Z27" s="4" t="n">
-        <v>0.4392022674723658</v>
+        <v>0.4971832329556723</v>
       </c>
       <c r="AA27" s="5" t="n">
         <v>8972000000</v>
@@ -3931,22 +3931,22 @@
         <v>0.3859069600725315</v>
       </c>
       <c r="AF27" s="6" t="n">
-        <v>1.307032492615315</v>
+        <v>1.062653562653563</v>
       </c>
       <c r="AG27" s="6" t="n">
-        <v>33.16107129385138</v>
+        <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005880026367831246</v>
+        <v>0.005840958352316812</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3407250759735089</v>
+        <v>0.3386164667011203</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.325820700942637</v>
+        <v>0.3250479851309561</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3162895450.557251</v>
+        <v>3079033823.923071</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>206.6</v>
+        <v>200.99001</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1357889331077817</v>
+        <v>0.1049478655528673</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1104413347685683</v>
+        <v>-0.1345962970936491</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>325866048000</v>
+        <v>317017515864</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>16.60771704180064</v>
+        <v>16.15675321543408</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.34435970189044</v>
+        <v>14.92526753704531</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.57542577590908</v>
+        <v>2.505492937302911</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.939480333644276</v>
+        <v>2.859662060280573</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4225268181859822</v>
+        <v>0.4110535789567702</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.52226966981293</v>
+        <v>23.21645587542168</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.455729895913191</v>
+        <v>5.384799773775182</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04813020594278052</v>
+        <v>-0.04949330728452513</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08233366295203282</v>
+        <v>0.08251012421265891</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3273872607776852</v>
+        <v>-0.3272876063513729</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02008712487899323</v>
+        <v>0.02064779239525387</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.378066152786705</v>
+        <v>1.384843569200202</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2838600492330827</v>
+        <v>0.2702874908851359</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>901055652.0337336</v>
+        <v>888563291.6675527</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>924.03</v>
+        <v>925.46</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>1.929522416660805</v>
+        <v>1.934056054157234</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2637211155378486</v>
+        <v>-0.2625816733067728</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,37 +4120,37 @@
         <v>154.65</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1043590241700</v>
+        <v>1045205269400</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>20.62106672617719</v>
+        <v>20.65297924570408</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.938210682417066</v>
+        <v>5.945241031966287</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.56025258324656</v>
+        <v>11.57814286948623</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.34813788173623</v>
+        <v>10.36415233707955</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.02939106654750906</v>
+        <v>0.02943655124515192</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>14.99679925233371</v>
+        <v>15.02042942381412</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.35400272171389</v>
+        <v>11.37189300795356</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02507880866858819</v>
+        <v>0.02504005745687068</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.472606114706539</v>
+        <v>2.473867440303503</v>
       </c>
       <c r="V29" s="4" t="n">
         <v>1.765110056317434</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005735744510459617</v>
+        <v>0.0005726881766905107</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.885442363676178</v>
+        <v>2.881697109418158</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8256190424097433</v>
+        <v>0.8123940601083595</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>26915220454.49057</v>
+        <v>26055014840.47032</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>142.35</v>
+        <v>146.26</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.03458797594978857</v>
+        <v>-0.008070511853994211</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2689728130809446</v>
+        <v>-0.2488933167630415</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>147170255700</v>
+        <v>151212656120</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>88.41614906832298</v>
+        <v>90.84472049689441</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>30.04974958411884</v>
+        <v>30.85835527126522</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.98983543985881</v>
+        <v>10.26423134129785</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.74876558005753</v>
+        <v>12.07147491211249</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>141.4658385093198</v>
+        <v>145.3515527950342</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>43.88657371739753</v>
+        <v>45.04518662080825</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.39371814417594</v>
+        <v>10.66811404561499</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.0311204188524081</v>
+        <v>0.03028847000984748</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.94232565302476</v>
+        <v>1.943926197566579</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2450681773312404</v>
+        <v>0.2456309996565116</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.711253205813258</v>
+        <v>0.7006968259160118</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6283435425653637</v>
+        <v>0.6291368994173632</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2258920226.575495</v>
+        <v>2194783123.786512</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.72</v>
+        <v>27.47</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.100873695950755</v>
+        <v>0.09094518137688445</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.05100992810681282</v>
+        <v>-0.05956864087641223</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>157988476800</v>
+        <v>156563616800</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.62790697674419</v>
+        <v>36.29756871035941</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.493782148823916</v>
+        <v>9.408847936443443</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.480351620195931</v>
+        <v>2.457981926651595</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.85439934264585</v>
+        <v>1.837674961849982</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6126260547437744</v>
+        <v>-0.6071009279874272</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.44347883396705</v>
+        <v>17.33060969581749</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.457147651343883</v>
+        <v>3.434777957799548</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06953671699681833</v>
+        <v>0.07016955934298523</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.858094319267862</v>
+        <v>2.85781223753946</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05021253784362711</v>
+        <v>-0.05031934638406588</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06204906204906205</v>
+        <v>0.06261376046596287</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3496282390178725</v>
+        <v>0.3495117154943911</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2088043753876717</v>
+        <v>0.209183226316025</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>988001149.972362</v>
+        <v>966922991.4588209</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>175.63</v>
+        <v>173.175</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.04535447736624998</v>
+        <v>0.03074225142572651</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.1212788312403063</v>
+        <v>-0.1335618151798669</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1246718145063</v>
+        <v>1229291207489</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.414675307130095</v>
+        <v>7.38409031764871</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003647503023548917</v>
+        <v>0.003598314060420221</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.3679221533799</v>
+        <v>6.341654943554526</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.614583589084575</v>
+        <v>4.595548771687055</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01659311748241866</v>
+        <v>0.01652467209504274</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.488190590983496</v>
+        <v>7.457154914126215</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.337669849130638</v>
+        <v>6.311402639305264</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07569489726394341</v>
+        <v>0.07600842642420826</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2031.808543066217</v>
+        <v>2051.097230441963</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2624.035360523716</v>
+        <v>2653.390795539407</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.70813642316233</v>
+        <v>1.73235166738848</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.9855001700845949</v>
+        <v>0.9147973844433476</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3333796407.208734</v>
+        <v>3243135688.615308</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>541.5</v>
+        <v>541.96</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.4505759917150454</v>
+        <v>0.451808244635062</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1939925278716342</v>
+        <v>-0.1933078308500662</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>301.37</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>68251065042</v>
+        <v>68309043786</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.828293058381121</v>
+        <v>1.827574172251887</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.4137902024091694</v>
+        <v>0.4040591364180168</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3886308062.686564</v>
+        <v>3799367435.75175</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>148.15</v>
+        <v>144.5801</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.07952778621274759</v>
+        <v>-0.1017079668134842</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3434231519234178</v>
+        <v>-0.3592443715653253</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1937189465232</v>
+        <v>1890509933191</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-96.20129870129871</v>
+        <v>-93.88318181818181</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>134.2771473268606</v>
+        <v>130.4648730500136</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>116.874175881267</v>
+        <v>114.0579145213273</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.828519776142866</v>
+        <v>6.663976186882977</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9620129870129871</v>
+        <v>-0.9388318181818182</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>451.8914003436525</v>
+        <v>440.6892088291337</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>113.6067249008748</v>
+        <v>110.7904635409351</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01467228709949444</v>
+        <v>-0.01503456792317652</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.194740387198083</v>
+        <v>4.204788528688608</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.461529722776998</v>
+        <v>3.471652279223203</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7855766027896656</v>
+        <v>0.7839797738368991</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>14309271538.60899</v>
+        <v>14218060076.60062</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>760.88</v>
+        <v>757.21</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1137491678993505</v>
+        <v>0.1083771520148606</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.02372429013177313</v>
+        <v>-0.02843322170471019</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>810518461399</v>
+        <v>806609037109</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9951782597768953</v>
+        <v>0.9952684723030731</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1154451686121067</v>
+        <v>0.1152769646468357</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>30486148873.09041</v>
+        <v>29338901279.6058</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>418.01</v>
+        <v>413.69</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3078752828707778</v>
+        <v>0.2943588090495732</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1273277661795408</v>
+        <v>-0.1363465553235909</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>257.98</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2168000504800</v>
+        <v>2145594911200</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.58780572620842</v>
+        <v>27.64576330126348</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6385117885598318</v>
+        <v>0.6311629187197041</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.89916072363153</v>
+        <v>13.92836064111815</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.59388616712771</v>
+        <v>9.614041390167893</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5182494035320432</v>
+        <v>0.5193381627831609</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.27477474575392</v>
+        <v>18.31455399061033</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.41458131216091</v>
+        <v>13.44378122964753</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01812191372746905</v>
+        <v>0.01808392229407813</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.20641563788966</v>
+        <v>42.80131101070088</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.18157995035575</v>
+        <v>42.78428010529495</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2631515992440372</v>
+        <v>0.2658995866470062</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.182358245656101</v>
+        <v>2.182894938145429</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3662558302635321</v>
+        <v>0.3625210639033964</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4177058875.66307</v>
+        <v>4058432163.025561</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.1</v>
+        <v>27.87</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.01438092688847081</v>
+        <v>-0.0224482716150064</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.06333333333333324</v>
+        <v>-0.07099999999999995</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>70450541326</v>
+        <v>69873899885</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.1259842519685</v>
+        <v>-21.94488188976378</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-81.58497367135612</v>
+        <v>-81.65673422767294</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.950727989090406</v>
+        <v>1.934761176381005</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.148702722455692</v>
+        <v>2.131115475972958</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1646584874565099</v>
+        <v>0.1633107489470793</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.38091592165289</v>
+        <v>16.28560328677686</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.744137929558355</v>
+        <v>2.728171116848955</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03094369410040947</v>
+        <v>0.03119906007232875</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02050670921914222</v>
+        <v>0.02058038420274655</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2528902568169814</v>
+        <v>0.2399821929974742</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.1891631311488362</v>
+        <v>0.1904242206290057</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>513505897.7286453</v>
+        <v>505854941.2946819</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>327.78</v>
+        <v>322.32999</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1205967044815636</v>
+        <v>-0.1352185751100595</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1540942992077216</v>
+        <v>-0.1681592041084932</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>221353111800</v>
+        <v>217672663232</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>19.87750151607035</v>
+        <v>19.54699757428745</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.87484752618812</v>
+        <v>16.58836791902805</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.632868005185969</v>
+        <v>2.589091185422193</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.482929988331389</v>
+        <v>6.375138075262544</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.232578696629692</v>
+        <v>1.212084565741844</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.511369996764278</v>
+        <v>9.362508624494419</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.797082437881365</v>
+        <v>2.753305618117588</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06799994758420197</v>
+        <v>0.06914970293700716</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1779366589963201</v>
+        <v>0.1783556809024982</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.005658273890123855</v>
+        <v>0.005891366142209531</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01079992678015742</v>
+        <v>0.01098253376919721</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9585179028789104</v>
+        <v>0.9614939136553785</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2223319342377628</v>
+        <v>0.2234581573750339</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>780789981.0595449</v>
+        <v>755198188.8363749</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>144.72</v>
+        <v>143.91499</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2605385773064524</v>
+        <v>-0.2646518570181891</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5607890743550834</v>
+        <v>-0.5632322003034902</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>329.5</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>416861618400</v>
+        <v>414542820711</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>22.33333333333333</v>
+        <v>22.20910339506172</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.15276483735976</v>
+        <v>16.04313808826583</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.807732538278279</v>
+        <v>5.775426957256503</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.428435871323309</v>
+        <v>6.392677474689989</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4860784313725492</v>
+        <v>0.4833746033042848</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>14.30196012477671</v>
+        <v>14.15972483327147</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.473475046324031</v>
+        <v>7.441169465302256</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.06889576476297632</v>
+        <v>-0.06928114193544857</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3826322340605446</v>
+        <v>0.3843366100118382</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4214263744375701</v>
+        <v>0.4232963938119607</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5338,10 +5338,10 @@
         <v>0.425824021246188</v>
       </c>
       <c r="Y39" s="4" t="n">
-        <v>0.7443888710868384</v>
+        <v>0.6394666815275089</v>
       </c>
       <c r="Z39" s="4" t="n">
-        <v>0.3249369575212115</v>
+        <v>0.3236273458071527</v>
       </c>
       <c r="AA39" s="5" t="n">
         <v>-23686000000</v>
@@ -5359,22 +5359,22 @@
         <v>0.5141842451501851</v>
       </c>
       <c r="AF39" s="6" t="n">
-        <v>3.187724958007839</v>
+        <v>3.169724284199364</v>
       </c>
       <c r="AG39" s="6" t="n">
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01381978993919292</v>
+        <v>0.0138970929991379</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.074229586262845</v>
+        <v>2.068944190557603</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5811597887336338</v>
+        <v>0.5570941813061446</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4282412869.755261</v>
+        <v>4122497288.122352</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 18:42 ET</t>
+          <t>2026-09-15 11:57 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-16)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,7 +442,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -699,55 +699,55 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>331.34</v>
+        <v>333.02</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2226116676891365</v>
+        <v>0.2288107007117652</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.03839568157413598</v>
+        <v>-0.03352003946948379</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>236.32</v>
+        <v>236.65</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4866508537040</v>
+        <v>4891183295120</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>37.82420091324201</v>
+        <v>38.01598173515982</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.632436109932</v>
+        <v>34.8004258678435</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.42474029137382</v>
+        <v>10.47759706595433</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.27732440569197</v>
+        <v>45.50689495256697</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.15573947234906</v>
+        <v>1.16159944190766</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.14943400068848</v>
+        <v>29.29588390204527</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.52062888298134</v>
+        <v>10.57348565756186</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02808646054140818</v>
+        <v>0.02794477159266767</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09216114030149503</v>
+        <v>0.09239989991868391</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1179196013700008</v>
+        <v>0.118190305206118</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003199130802197139</v>
+        <v>0.003182992012491742</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3085138427277651</v>
+        <v>0.3072398750722112</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2948156993843422</v>
+        <v>0.2950645760019249</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13507548538.13052</v>
+        <v>12936506731.42503</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>497.12</v>
+        <v>494.6302</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.05112698742709854</v>
+        <v>0.04586247187090287</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.1022177273712346</v>
+        <v>-0.1067142237954201</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3691389416000</v>
+        <v>3672901281610</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.61777777777777</v>
+        <v>27.47945555555555</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.23102086329266</v>
+        <v>24.08985946621722</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.1240373072484</v>
+        <v>11.06832313745521</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.348130663875747</v>
+        <v>8.306319480002802</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8772328950760488</v>
+        <v>0.8728393191544196</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.30802343881765</v>
+        <v>18.21713587189607</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.44911452843096</v>
+        <v>11.39227703494767</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01814682561250536</v>
+        <v>0.01824002173255826</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1397694687975644</v>
+        <v>0.1407063455098934</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2255150471434921</v>
+        <v>0.226123141342697</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007322175732217573</v>
+        <v>0.007359033071575492</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5579241349035604</v>
+        <v>0.554309862636615</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4370350965003246</v>
+        <v>0.4338715710278684</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>11776456198.26951</v>
+        <v>11034021304.62094</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>344.98</v>
+        <v>346.02</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.09465336087968867</v>
+        <v>0.09795337680906102</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1557230611096155</v>
+        <v>-0.1531778468466264</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4174986351444</v>
+        <v>4187572547182</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.95283018867924</v>
+        <v>17.01042701092353</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.63136393946234</v>
+        <v>20.71212650332069</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.293288060058403</v>
+        <v>9.324861776926252</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.477510507744192</v>
+        <v>6.499517689857607</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1507625048674289</v>
+        <v>0.1512747167575564</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.95366175149261</v>
+        <v>12.99707590429712</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.420781522219681</v>
+        <v>9.452355239087529</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01285681513087965</v>
+        <v>0.01281328232036988</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1782981368355891</v>
+        <v>-0.178721363632251</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2899057486593579</v>
+        <v>0.2911016373680599</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002492898139022552</v>
+        <v>0.002485405467892029</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.772002268076359</v>
+        <v>0.7633398457606374</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3675627713635436</v>
+        <v>0.3637372338581698</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8473543582.787918</v>
+        <v>8096334386.816304</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>248.42</v>
+        <v>247.92</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.09677704194260484</v>
+        <v>0.09456953642384103</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1350278551532034</v>
+        <v>-0.1367688022284123</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2672278782000</v>
+        <v>2666900232000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.71587301587302</v>
+        <v>19.67619047619047</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.05656601495863</v>
+        <v>22.02367326563975</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.445078875309406</v>
+        <v>3.43814489480198</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.843924295710814</v>
+        <v>4.834174830499256</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2231796793167352</v>
+        <v>0.2227304810248973</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.09185455733729</v>
+        <v>11.07067891353048</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.632036125721947</v>
+        <v>3.625102145214522</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004350219774337901</v>
+        <v>-0.004358993208861815</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1061222765818656</v>
+        <v>-0.1065890671885193</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1785740462863659</v>
+        <v>0.1790016137663992</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8356151450503818</v>
+        <v>0.8318213742314999</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4607508117976845</v>
+        <v>0.4600177075852392</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8923821402.908955</v>
+        <v>8378234518.323593</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>212.17</v>
+        <v>216.66229</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1234842104463678</v>
+        <v>0.1472718188912288</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.1030269721822947</v>
+        <v>-0.0840353005834108</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5138969570000</v>
+        <v>5247777386169</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>26.6880503144654</v>
+        <v>27.25311823899371</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>15.86809355463913</v>
+        <v>16.18266927000292</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>16.96203099987127</v>
+        <v>17.32116944693682</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>22.41375947664465</v>
+        <v>22.88832754733955</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.214230607966457</v>
+        <v>0.2187665273606298</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>22.06296383314717</v>
+        <v>22.52861716104114</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>17.01621806191392</v>
+        <v>17.37535650897947</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02471429306400816</v>
+        <v>0.02420186502856161</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6818687274920301</v>
+        <v>0.6840928887740156</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9361767872730502</v>
+        <v>0.9386961152552931</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002450864872507895</v>
+        <v>0.002400048480979316</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.326698277194909</v>
+        <v>1.330883068060406</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4129865725171606</v>
+        <v>0.4118331113816031</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27161914412.29845</v>
+        <v>26479586834.7751</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>670.24</v>
+        <v>679</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.03048850367345501</v>
+        <v>0.04395693183676874</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.1524532119372787</v>
+        <v>-0.1413758219524531</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1707427398677</v>
+        <v>1729743381030</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>24.90672612411743</v>
+        <v>25.23225566703828</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>20.26970589738644</v>
+        <v>20.53056884773238</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7.48057988975588</v>
+        <v>7.578350658187586</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>6.524821205033287</v>
+        <v>6.61010025993316</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.105878855444069</v>
+        <v>-5.172612411742842</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>16.8511225967293</v>
+        <v>17.05954293400702</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.904925338565946</v>
+        <v>8.002696106997652</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02399867779546601</v>
+        <v>0.02368906304217234</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2287660339131452</v>
+        <v>0.229009086605275</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.271779256228301</v>
+        <v>0.2723933984855693</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.00313320601575555</v>
+        <v>0.003092783505154639</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7737419082192315</v>
+        <v>0.7739591816512366</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4141160903999248</v>
+        <v>0.4089750218803272</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10085256584.06548</v>
+        <v>9895654934.539257</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>356.58</v>
+        <v>362.4</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.186020512616166</v>
+        <v>-0.1727349648665056</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2851672914620211</v>
+        <v>-0.2734999899765451</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1408329609753</v>
+        <v>1431315975586</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>302.1864406779661</v>
+        <v>307.1186440677966</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>169.5194756773143</v>
+        <v>172.3743528501283</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.59142251665235</v>
+        <v>13.81325795062682</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.2889251421861</v>
+        <v>13.5058232977964</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.044117927906418</v>
+        <v>-8.175411792790637</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>116.5989865108913</v>
+        <v>118.510057830562</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.53470511926384</v>
+        <v>13.75654055323831</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004091371764178535</v>
+        <v>0.00402566595935671</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7826060366844672</v>
+        <v>0.7816957046668216</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.122312558453592</v>
+        <v>0.1224683805249129</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.539929601112977</v>
+        <v>1.535828499738731</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.575054620584088</v>
+        <v>0.5734854086589536</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12770236754.12082</v>
+        <v>12585173296.70041</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>339.27</v>
+        <v>342.85</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-0.02402046842665828</v>
+        <v>-0.01372186636036121</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.3146060606060607</v>
+        <v>-0.3073737373737373</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1614104166600</v>
+        <v>1631136303000</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>42.09305210918114</v>
+        <v>42.53722084367246</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>18.56984765925968</v>
+        <v>18.74384510101777</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.11483397602801</v>
+        <v>18.30598293005925</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.21988985856154</v>
+        <v>16.39104323402548</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4188467066309606</v>
+        <v>0.4232664054246614</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>31.56244698161223</v>
+        <v>31.89289137630828</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>18.51261634270066</v>
+        <v>18.70643497486084</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02441168346835987</v>
+        <v>0.02415325707293803</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.266741918488052</v>
+        <v>1.269396733403582</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8525743408863151</v>
+        <v>0.8547782329035543</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007486662540159755</v>
+        <v>0.0074084876768266</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.605083990203484</v>
+        <v>1.604331866251678</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3892366707697041</v>
+        <v>0.3900621800999269</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8765279017.475498</v>
+        <v>8448720235.190298</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>901.35</v>
+        <v>901.08</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.05482738443534241</v>
+        <v>0.05451141018139261</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1779753761969904</v>
+        <v>-0.1782216142270862</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>399729796650</v>
+        <v>399610057320</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>45.27122049221497</v>
+        <v>45.25765946760422</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.7678389432304</v>
+        <v>39.75143661554289</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.361537795099919</v>
+        <v>1.361129945535736</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.94097096451699</v>
+        <v>11.93739403861649</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.571171723649282</v>
+        <v>3.570101976752533</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>26.88429831720802</v>
+        <v>26.87602331167934</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.325044353632824</v>
+        <v>1.324636504068641</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02202988136936526</v>
+        <v>0.02203648241252428</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1383877448518331</v>
+        <v>0.13851632345555</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1136368918037924</v>
+        <v>0.1137619578080773</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006146336051478338</v>
+        <v>0.006148177742264838</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.187307937102089</v>
+        <v>-0.1857028973985057</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.176444822708197</v>
+        <v>0.1761879455002504</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1730378059.199019</v>
+        <v>1670251785.627592</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>77.90000000000001</v>
+        <v>77.27500000000001</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1438619427529596</v>
+        <v>-0.15073082960507</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3761012333813871</v>
+        <v>-0.3811068396604196</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>324370925922</v>
+        <v>321768463423</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>24.11764705882353</v>
+        <v>23.92507739938081</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.77359786945086</v>
+        <v>20.60368904786809</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.705929348604045</v>
+        <v>6.652385214403478</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.82336630687689</v>
+        <v>10.73694610350234</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.708823529411765</v>
+        <v>0.7031638601525336</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10.77166358135712</v>
+        <v>10.68701582300221</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.813640568546736</v>
+        <v>6.760096434346169</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03389517099520758</v>
+        <v>0.03416798856755578</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1609759277323042</v>
+        <v>0.1612035759128481</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1434269861448505</v>
+        <v>0.1437995609359888</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1010625785780117</v>
+        <v>0.09691944164778994</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3818256902419801</v>
+        <v>0.3311391987215864</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2197050104.863083</v>
+        <v>2109589813.140972</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>516.76</v>
+        <v>520.3099999999999</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.04007244369910756</v>
+        <v>0.04721745719692438</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.03901513742700935</v>
+        <v>-0.03241343400156216</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1114575663752</v>
+        <v>1122232494014</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.97140516110474</v>
+        <v>13.08306342574169</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.2953406022426</v>
+        <v>23.45534582253936</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.893036591696626</v>
+        <v>2.917939941900818</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.481267354237733</v>
+        <v>1.494018150329856</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3573291791599261</v>
+        <v>0.3604050800013231</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.70529010834619</v>
+        <v>15.83049588872625</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.123772228721012</v>
+        <v>3.148675578925204</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02175820361113868</v>
+        <v>0.02157250679244771</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4431759817301831</v>
+        <v>-0.44221400423056</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05906971911748538</v>
+        <v>0.06094355877574542</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.05340833797176848</v>
+        <v>0.05623404467829123</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1395663401249826</v>
+        <v>0.1395117083446725</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2101104811.616488</v>
+        <v>2040535266.620744</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>352.49</v>
+        <v>351.37</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.08298509309933144</v>
+        <v>0.07954402156745477</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.03822646657571616</v>
+        <v>-0.04128240109140513</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>944500479900</v>
+        <v>941499428700</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.15434221840069</v>
+        <v>15.10619088564059</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.07451446459346</v>
+        <v>14.02917206195688</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.173372844745038</v>
+        <v>3.16328978540686</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.624116687755941</v>
+        <v>2.615778832241496</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.793469982641731</v>
+        <v>0.7909488150041846</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.10047745706312</v>
+        <v>20.06826351116359</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.291508266556463</v>
+        <v>6.281425207218286</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1720846134638369</v>
+        <v>-0.1726331371484984</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07672220285280162</v>
+        <v>0.07676994899822165</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.289427374123294</v>
+        <v>-0.2893751396518991</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01702175948253851</v>
+        <v>0.0170760167344964</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7694580071536945</v>
+        <v>0.7670347220969244</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1701887373192562</v>
+        <v>0.169646219936739</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2109494571.052096</v>
+        <v>2044868972.712569</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>375.62</v>
+        <v>371.775</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.08410294415172404</v>
+        <v>0.0730056228688758</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.02580594963301086</v>
+        <v>-0.03577819851129505</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>701300273396</v>
+        <v>694121476870</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.91333899745115</v>
+        <v>31.58666100254885</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.10661718726129</v>
+        <v>24.8621010308201</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.76380761994246</v>
+        <v>15.60244283559612</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.43124863892205</v>
+        <v>20.22210601867645</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.152050820551805</v>
+        <v>2.130021547869249</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.49650400013747</v>
+        <v>24.24979300536119</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>16.02228181523108</v>
+        <v>15.86091703088473</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.02996291431378736</v>
+        <v>0.03027279907078205</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2711126616310331</v>
+        <v>0.2704743240884069</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1378301271625042</v>
+        <v>0.1381361933238576</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007134870347691817</v>
+        <v>0.007208661152578845</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3037793366634721</v>
+        <v>0.3014679487895589</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1804353882007724</v>
+        <v>0.176358785651124</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2272636613.31724</v>
+        <v>2201177220.262569</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>573.27</v>
+        <v>570.76</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.01800649056037718</v>
+        <v>0.01354926047454219</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.04712276852498254</v>
+        <v>-0.05129483727269712</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>502778427720</v>
+        <v>500577067360</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.48105436573311</v>
+        <v>31.34321801208127</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.85925181506215</v>
+        <v>25.73607075446453</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.33111272468147</v>
+        <v>14.26836551492176</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>90.11301728747104</v>
+        <v>89.7184672963821</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.391350170628382</v>
+        <v>1.385258296069663</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.33742212515826</v>
+        <v>23.23788512208356</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.71169591312031</v>
+        <v>14.6489487033606</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03271421185389437</v>
+        <v>0.0328580773520955</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2174000466400365</v>
+        <v>0.2178711471192254</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1568220736126735</v>
+        <v>0.1571890126686657</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.00587855635215518</v>
+        <v>0.005904408157544327</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.292833232438592</v>
+        <v>0.29062514884985</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1965507417402079</v>
+        <v>0.1932066487787013</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1532145762.413241</v>
+        <v>1480861028.262964</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>375.93</v>
+        <v>379.60999</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1175089382304795</v>
+        <v>0.1284482666096955</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1856288722325722</v>
+        <v>-0.1776569689354881</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>341398725796</v>
+        <v>344740683900</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.17400810237284</v>
+        <v>24.41064818982702</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.34874484258084</v>
+        <v>17.51259204373629</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7584464137969337</v>
+        <v>0.7658708590204141</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.459642774386218</v>
+        <v>3.493509320853149</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7324787572533598</v>
+        <v>-0.739649013689145</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.98822830400186</v>
+        <v>15.11794759538874</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.857846807906178</v>
+        <v>0.8652712531296584</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06917717675991604</v>
+        <v>0.06850656479770359</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3934153923942698</v>
+        <v>0.3938912143252915</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01032894715891031</v>
+        <v>0.01040690486613927</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,26 +2549,26 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02410023142606336</v>
+        <v>0.02386660056022235</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.429900752815327</v>
+        <v>0.435637936826805</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2290281710049149</v>
+        <v>0.2300048304031516</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1805017710.513059</v>
+        <v>1751533147.843852</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
-          <t>2026-10-27 (E)</t>
+          <t>2026-10-13 (C)</t>
         </is>
       </c>
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>169.28</v>
+        <v>164.09</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3801875083082022</v>
+        <v>0.3378719768330156</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.04041720990873532</v>
+        <v>-0.06983731081004474</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>701574188800</v>
+        <v>680064441400</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.78635778635779</v>
+        <v>21.11196911196911</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.31735582137103</v>
+        <v>14.8510519789708</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.943095853320778</v>
+        <v>1.8829480374453</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.723993743850721</v>
+        <v>2.639673521628498</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.133247533247534</v>
+        <v>2.067213642213643</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>10.21029152523495</v>
+        <v>9.909086078663419</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>2.031114465185841</v>
+        <v>1.971196221126682</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04354920760733665</v>
+        <v>0.04493484008149426</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.422331506849315</v>
+        <v>0.4215807164276184</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08215438117185392</v>
+        <v>0.08166324800680869</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02433837429111531</v>
+        <v>0.02510817234444512</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5501222862545879</v>
+        <v>-0.5583743515301339</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2367982598190592</v>
+        <v>0.2513330320572517</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2242445686.619956</v>
+        <v>2195296767.427505</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>267.2</v>
+        <v>267.85999</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2886423541584338</v>
+        <v>0.2918253297097848</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.0493471377236987</v>
+        <v>-0.04699900380688093</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>643924856755</v>
+        <v>645515354409</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>30.89017341040462</v>
+        <v>30.95954913294797</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.58852845169736</v>
+        <v>21.61749441164768</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.57542563239694</v>
+        <v>6.59019327058379</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.673144013840015</v>
+        <v>7.690376999329182</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.824691207788263</v>
+        <v>-3.833281017645275</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.93771068288272</v>
+        <v>19.98058332725602</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.867616913835534</v>
+        <v>6.882384552022383</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02905307941407518</v>
+        <v>0.02898797580521503</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.430860536859609</v>
+        <v>0.4321525216292743</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08875387185717587</v>
+        <v>0.08933884426234107</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01976047904191617</v>
+        <v>0.01971179047680843</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1742644611003474</v>
+        <v>-0.1727717519192965</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2096265966257698</v>
+        <v>0.207938150586052</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1659349928.772552</v>
+        <v>1608307061.057868</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>108.09</v>
+        <v>108.3701</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.04141541369064916</v>
+        <v>-0.0389313768451941</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2002811482687185</v>
+        <v>-0.1982087895827168</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>860188867200</v>
+        <v>862417925408</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>39.02166064981949</v>
+        <v>39.1227797833935</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.85644000821016</v>
+        <v>34.93631460727707</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.168989001956947</v>
+        <v>1.172018272189606</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.751683259024002</v>
+        <v>8.774362012663124</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.436147029865449</v>
+        <v>9.460599474893344</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.53212883587385</v>
+        <v>21.58416222152711</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.253553581213307</v>
+        <v>1.256582851445966</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01570469058030608</v>
+        <v>0.01566409927484873</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.119496444290589</v>
+        <v>0.1198313337619308</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05094654776722218</v>
+        <v>0.05107088152361516</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009043389767786104</v>
+        <v>0.009020015668528497</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.0564845450081595</v>
+        <v>-0.05629082922172535</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3071438071916167</v>
+        <v>0.3070729759507302</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2764095681.859236</v>
+        <v>2669157998.060524</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>146.66</v>
+        <v>147.96</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.03434661784657456</v>
+        <v>0.04351510689062588</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1231091180866966</v>
+        <v>-0.1153363228699551</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>348641462700</v>
+        <v>351731834319</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.72740740740741</v>
+        <v>21.92</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.76270500940494</v>
+        <v>20.94335688581644</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.005899700110304</v>
+        <v>4.041408152392224</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.541655465743587</v>
+        <v>6.599640956712268</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.73415449735472</v>
+        <v>20.91794285714308</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.5837707113955</v>
+        <v>17.72917259428813</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.294115528771027</v>
+        <v>4.329623981052946</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04564287872350072</v>
+        <v>0.04524185316012042</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04646323287671228</v>
+        <v>0.04663259665144603</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02535486436829393</v>
+        <v>0.02543466982807141</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02925542070094096</v>
+        <v>0.02899837793998378</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.04817637593459839</v>
+        <v>-0.0442625259997273</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1501291257052752</v>
+        <v>0.1500394124977721</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1296691230.419818</v>
+        <v>1268543724.111756</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>305.48</v>
+        <v>308.04</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1166502992014529</v>
+        <v>-0.1092476043145723</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2841710603397773</v>
+        <v>-0.2781722319859402</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,37 +3110,37 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>304599301160</v>
+        <v>307151920680</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>21.33240223463687</v>
+        <v>21.51117318435754</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>20.35687844315328</v>
+        <v>20.52747425569247</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.800487664680569</v>
+        <v>1.815576208682083</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>18.27328157910573</v>
+        <v>18.42641632063549</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.317510068858028</v>
+        <v>-7.378832662076166</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.26578721137362</v>
+        <v>15.37252438553209</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.157997004066771</v>
+        <v>2.173085548068284</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.0495766075053066</v>
+        <v>0.0491645957041977</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04792108938547468</v>
+        <v>0.0479210893854749</v>
       </c>
       <c r="V21" s="4" t="n">
         <v>0.01423568777486173</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03041115621317271</v>
+        <v>0.03015842098428775</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.709807233714538</v>
+        <v>0.7118905014936657</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2470891658608973</v>
+        <v>0.2413912795913898</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1240432383.593238</v>
+        <v>1200616632.192054</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>504.2</v>
+        <v>526.3273</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.256231249142218</v>
+        <v>1.355248118874754</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.1377216835120484</v>
+        <v>-0.09987977357070776</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.85</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>822148520000</v>
+        <v>858229295380</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>127.9695431472081</v>
+        <v>133.5856091370558</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>37.29149383605141</v>
+        <v>38.77943549487809</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>19.9043340999879</v>
+        <v>20.77785486938627</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>12.23298524336547</v>
+        <v>12.76984151939784</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.033148605225166</v>
+        <v>1.078489321473478</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>76.63169621197984</v>
+        <v>80.02129949617466</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>19.88472388330711</v>
+        <v>20.76427279990316</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01022078103357773</v>
+        <v>0.009788249880584051</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.431601418538349</v>
+        <v>2.444753834921077</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8934119722057594</v>
+        <v>0.8988302387766913</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.538601164745802</v>
+        <v>2.543980070502435</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6646592840893162</v>
+        <v>0.6723667388671691</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10183663363.32363</v>
+        <v>9526354595.547436</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1591.48</v>
+        <v>1609.3425</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.3675092886423992</v>
+        <v>0.3828579795894262</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.2042440848816977</v>
+        <v>-0.1953126562531251</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>861.1799999999999</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>613385024317</v>
+        <v>620269553181</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>50.02902757619739</v>
+        <v>50.66037735849056</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>32.76190382771456</v>
+        <v>33.02961111517773</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.04251152759182</v>
+        <v>15.23234304816361</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>24.34729810221118</v>
+        <v>24.65455295206502</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.40565873273661</v>
+        <v>3.448637019616227</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>38.15616835024811</v>
+        <v>38.64197175080589</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>14.90982452737952</v>
+        <v>15.09965604795131</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01882128409193356</v>
+        <v>0.01858672575990359</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5270488503746813</v>
+        <v>0.5337866734740684</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2826890123849841</v>
+        <v>0.2856935401255383</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004888531429864026</v>
+        <v>0.004834272381422849</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.697316872671875</v>
+        <v>1.685865454439055</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4375157394443653</v>
+        <v>0.4362877663565686</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2072147632.963916</v>
+        <v>2024414593.658516</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>209.69</v>
+        <v>211.34</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.07937833750414935</v>
+        <v>-0.07213418783979642</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.1755848240613328</v>
+        <v>-0.169097700019658</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>165732685300</v>
+        <v>167036795800</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>78.53558052434454</v>
+        <v>79.15355805243443</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>82.93066134929298</v>
+        <v>83.13396862336106</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.763207461035161</v>
+        <v>1.777081714984839</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>27.19248837367869</v>
+        <v>27.40645950161312</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4203282135993536</v>
+        <v>0.4236356748633096</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>29.40772450359712</v>
+        <v>29.59536630215827</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.174410184584286</v>
+        <v>2.188284438533965</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001267100690608312</v>
+        <v>-0.001257208024101717</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.05299705505104957</v>
+        <v>-0.04787947257708691</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1533729156417385</v>
+        <v>0.1537975177777891</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.239882327225976</v>
+        <v>1.241962403843824</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3346242894193652</v>
+        <v>0.3351803178530742</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1079004709.662687</v>
+        <v>1023742467.130764</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>976.67</v>
+        <v>978.925</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.0681693585688159</v>
+        <v>0.07063561831220166</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1536581772805657</v>
+        <v>-0.1517040875570846</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>288124486690</v>
+        <v>288789727475</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>14.87918951858623</v>
+        <v>14.9135435709933</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.48483516185687</v>
+        <v>13.51438611179333</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.443037271509365</v>
+        <v>2.448677916811518</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.387924809763569</v>
+        <v>2.393438207785436</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3487475852012999</v>
+        <v>0.3495527965875705</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.8445986904724</v>
+        <v>26.86578942678304</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.145615766807702</v>
+        <v>7.151256412109855</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1440870245945704</v>
+        <v>-0.1437551133240841</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1034016611989015</v>
+        <v>0.1035309667509787</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.382285490439393</v>
+        <v>-0.3822426848979621</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01842997122876714</v>
+        <v>0.01838751691906939</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.570100090379177</v>
+        <v>1.568520056957277</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3090673866755244</v>
+        <v>0.3026975806733175</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1862475948.847695</v>
+        <v>1793973811.470195</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>248.37</v>
+        <v>240.94</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.1479588336192109</v>
+        <v>-0.1734476843910806</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.2529326836311134</v>
+        <v>-0.2752812368405221</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>233997821580</v>
+        <v>226997765960</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>21.69170305676856</v>
+        <v>21.04279475982533</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>19.25049067595444</v>
+        <v>18.67129747777815</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.386512027729135</v>
+        <v>3.285204364299463</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.775890020898642</v>
+        <v>6.573188958551028</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2644201787346401</v>
+        <v>0.2565100368978709</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>18.00738681832193</v>
+        <v>17.57584402687874</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.22735895306598</v>
+        <v>4.126051289636308</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.05825267905470558</v>
+        <v>0.06004904912765512</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1268129951546333</v>
+        <v>0.1270129879763118</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04600047137561836</v>
+        <v>0.04610799352298289</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02713693280186818</v>
+        <v>0.02797376940317092</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8958469001438731</v>
+        <v>0.8855233417986426</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3171415193881565</v>
+        <v>0.3176603538400597</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1199632443.267902</v>
+        <v>1161328547.549453</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1136.98</v>
+        <v>1145.75</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.05240847070989285</v>
+        <v>0.06052613530216844</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1204270297450973</v>
+        <v>-0.1136425173094032</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1070740682180</v>
+        <v>1078999750750</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.03880896620944</v>
+        <v>38.3322181331549</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.0617277011639</v>
+        <v>26.21265617928169</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.4404058225738</v>
+        <v>13.54407726715855</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>29.94896401900882</v>
+        <v>30.17997284453496</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4021170720722484</v>
+        <v>0.40521876842757</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>25.78833483078088</v>
+        <v>25.97905430229443</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.01804390566592</v>
+        <v>14.12171535025067</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.018728997911213</v>
+        <v>0.0185856391403805</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4595658968730096</v>
+        <v>0.4623553550232133</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.228246464557607</v>
+        <v>0.2290918506683588</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005884008513782125</v>
+        <v>0.005838970106916867</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3411813514063061</v>
+        <v>0.3457100598959101</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.324628723651813</v>
+        <v>0.3246364649911769</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3123924853.497945</v>
+        <v>2988368156.592773</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>206.27</v>
+        <v>207.415</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.133974749429536</v>
+        <v>0.1402694170404188</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1118622174381054</v>
+        <v>-0.1069321851453175</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>325345545600</v>
+        <v>327151531200</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>16.58118971061093</v>
+        <v>16.67323151125402</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.31735301105928</v>
+        <v>15.39986893249027</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.571312075492575</v>
+        <v>2.585585369361965</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.934785132724128</v>
+        <v>2.951076057128884</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4218519205577083</v>
+        <v>0.4241936108133857</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.5045335332402</v>
+        <v>23.56607255256074</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.451616195496685</v>
+        <v>5.465889489366075</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04820720680553863</v>
+        <v>-0.04794108694057062</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08251012421265891</v>
+        <v>0.08268658547328567</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3272876063513729</v>
+        <v>-0.3271879519250608</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02011926116255393</v>
+        <v>0.02000819612853458</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.376706477173516</v>
+        <v>1.377667327960806</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2623913333312874</v>
+        <v>0.2611880847700112</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>922096790.9233246</v>
+        <v>866532109.8652943</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>927.6</v>
+        <v>929.47</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>1.940840658522518</v>
+        <v>1.946769261402464</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2608764940239043</v>
+        <v>-0.2593864541832669</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,40 +4120,40 @@
         <v>154.65</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1047622164000</v>
+        <v>1049734123300</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>20.70073644275831</v>
+        <v>20.74246819906271</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.958988590810979</v>
+        <v>5.95494329743573</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.60491574539735</v>
+        <v>11.62831073509538</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.38811802549541</v>
+        <v>10.40906000555975</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.02950461925421188</v>
+        <v>0.02956409924343717</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.05579205805753</v>
+        <v>15.08670792366781</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.39866588386468</v>
+        <v>11.42207213318342</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02498228932086626</v>
+        <v>0.02493200333010484</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.473867440303503</v>
+        <v>2.483235215353715</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.765110056317434</v>
+        <v>1.772514181536212</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005713669685209142</v>
+        <v>0.0005702174357429503</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.880005584881958</v>
+        <v>2.877844639466991</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8124061229988889</v>
+        <v>0.8122173015895694</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>26371464494.61606</v>
+        <v>25488204420.92985</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>141.9</v>
+        <v>140.83</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.03763985800684921</v>
+        <v>-0.0448965553425269</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2712837525548719</v>
+        <v>-0.2767786530817661</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>146705017800</v>
+        <v>145598785460</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>88.13664596273293</v>
+        <v>87.47204968944101</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>29.93846993704728</v>
+        <v>29.69648027762235</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.958255348900353</v>
+        <v>9.883164910399131</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.7116251198466</v>
+        <v>11.62331335890061</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>141.0186335403757</v>
+        <v>139.9552795031086</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>43.75322952135282</v>
+        <v>43.43616665520207</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.36213805321749</v>
+        <v>10.28704761471626</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03121910939845167</v>
+        <v>0.03145630635262581</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.943926197566579</v>
+        <v>1.945535931251596</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2456309996565116</v>
+        <v>0.2461938219817823</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.7103996960341029</v>
+        <v>0.703517495086097</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6278912580281349</v>
+        <v>0.6279114251488768</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2235182723.005687</v>
+        <v>2176582239.990946</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.55</v>
+        <v>27.605</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.09412230604052318</v>
+        <v>0.09630657924677455</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.05682985279014041</v>
+        <v>-0.05494693598082845</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>157019572000</v>
+        <v>157333041200</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.40327695560254</v>
+        <v>36.47595137420719</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.436249022534287</v>
+        <v>9.455778672075736</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.465140228585782</v>
+        <v>2.470061561165536</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.84302676370466</v>
+        <v>1.846706127479751</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6088689685494584</v>
+        <v>-0.6100844964358547</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.36672782002535</v>
+        <v>17.39155903041825</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.441936259733735</v>
+        <v>3.446857592313489</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06996580018699834</v>
+        <v>0.06982640083868155</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.85781223753946</v>
+        <v>2.857530155811058</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05031934638406599</v>
+        <v>-0.05042615492450442</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06243194192377495</v>
+        <v>0.06230755297953269</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3485226448608757</v>
+        <v>0.3479709659284707</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2082879551631476</v>
+        <v>0.2077863857129715</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>990061057.8431157</v>
+        <v>945056547.4672413</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>174.83</v>
+        <v>179.3187</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.04059285587850292</v>
+        <v>0.06730971884356518</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.1252814329314054</v>
+        <v>-0.1028233351678591</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1241039305935</v>
+        <v>1272902562428</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.38409031764871</v>
+        <v>7.685570928250936</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003632702452335887</v>
+        <v>0.003723068627362769</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.341654943554526</v>
+        <v>6.600574583261782</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.595548771687055</v>
+        <v>4.78317768603404</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01652467209504274</v>
+        <v>0.01719934805631963</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.457154914126215</v>
+        <v>7.763078014576559</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.311402639305264</v>
+        <v>6.57032227901252</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07600842642420826</v>
+        <v>0.07302685654173505</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2031.671382953652</v>
+        <v>2063.310840731131</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2628.263433149657</v>
+        <v>2670.248850300211</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.715952639707144</v>
+        <v>1.672998967759637</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.9140153423105198</v>
+        <v>0.9154040808242494</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3276414380.73785</v>
+        <v>3140685843.304704</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>542.11</v>
+        <v>552.1356</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.4522100662394151</v>
+        <v>0.4790667507501045</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1930845600821637</v>
+        <v>-0.1781617373442688</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>301.37</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>68327949898</v>
+        <v>69591584021</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.826660385047441</v>
+        <v>1.827958376954615</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.4040658528778202</v>
+        <v>0.4033292719119316</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3866996224.813599</v>
+        <v>3720531518.062378</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>143.49</v>
+        <v>152.2995</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.1084808777837809</v>
+        <v>-0.05374648718399166</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3640755185250841</v>
+        <v>-0.3250332387874491</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1876255932273</v>
+        <v>1991447762499</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-93.17532467532467</v>
+        <v>-98.89577922077922</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>129.4811985463176</v>
+        <v>136.8285069042755</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>113.1979446318552</v>
+        <v>120.1476779788235</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.613731371439352</v>
+        <v>7.019778249386908</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9317532467532468</v>
+        <v>-0.9889577922077922</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>437.2685222637389</v>
+        <v>464.9123500117591</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>109.9304936514631</v>
+        <v>116.8802269984314</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.0151487862135987</v>
+        <v>-0.01427253103758692</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.204788528688608</v>
+        <v>4.214836670179136</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.482105313712486</v>
+        <v>3.539215959670987</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7857677087761391</v>
+        <v>0.7842372976340035</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>14385635156.2712</v>
+        <v>14075368301.73266</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>757.39</v>
+        <v>760.87</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1086406296331734</v>
+        <v>0.1137345302538886</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.02820226593274056</v>
+        <v>-0.02373712100799363</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>806800779990</v>
+        <v>810507809017</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9952239310757131</v>
+        <v>0.995029222259491</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1152127708860105</v>
+        <v>0.1128091657703609</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>30114175362.7381</v>
+        <v>28658069989.11263</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>413.75</v>
+        <v>418.95001</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.2945465378526455</v>
+        <v>0.3108163987403776</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1362212943632568</v>
+        <v>-0.1253653235908142</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>257.98</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2145906100000</v>
+        <v>2172875859312</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.64576330126348</v>
+        <v>27.58780572620842</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6312544601519919</v>
+        <v>0.6385199650913073</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.92836064111815</v>
+        <v>13.89916072363153</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.614041390167893</v>
+        <v>9.59388616712771</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5193381627831609</v>
+        <v>0.5182494035320432</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.31455399061033</v>
+        <v>18.27477474575392</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.44378122964753</v>
+        <v>13.41458131216091</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01808392229407813</v>
+        <v>0.01812191372746905</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.7949591589531</v>
+        <v>42.20586236056598</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.77793072328573</v>
+        <v>42.17267580496152</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2658610271903323</v>
+        <v>0.286430354781469</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.18286906950038</v>
+        <v>2.184027822511649</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3624691173247276</v>
+        <v>0.3565425843995432</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4136072980.466634</v>
+        <v>4015868130.797678</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.03</v>
+        <v>28.045</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.01683620571828592</v>
+        <v>-0.0163100745404684</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.06566666666666665</v>
+        <v>-0.0651666666666666</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>70275041757</v>
+        <v>70312648808</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.07086614173228</v>
+        <v>-22.08267716535433</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-82.12552064591577</v>
+        <v>-82.92737924132929</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.945868524352762</v>
+        <v>1.946909838238959</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.143350082221816</v>
+        <v>2.144497076557647</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.164248306171031</v>
+        <v>0.1643362021607765</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.35190772842975</v>
+        <v>16.35812376991736</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.739278464820712</v>
+        <v>2.740319778706909</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.0310209705394142</v>
+        <v>0.0310043788273834</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02058038420274655</v>
+        <v>0.02065405918635133</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2391619887635157</v>
+        <v>0.2328888598444398</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.1893262260542644</v>
+        <v>0.1849474654543697</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>517302914.2458267</v>
+        <v>491962398.8552333</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>324.43</v>
+        <v>317.42</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1295844433307513</v>
+        <v>-0.1483916222360665</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1627396836047382</v>
+        <v>-0.1808304730444656</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>219090823300</v>
+        <v>214356900200</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>19.67434808975137</v>
+        <v>19.24924196482717</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.69644268586448</v>
+        <v>16.3298736552132</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.605959384106669</v>
+        <v>2.549652090445208</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.416672695449241</v>
+        <v>6.278026837806301</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.219981409932183</v>
+        <v>1.193621117469635</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.419868277786767</v>
+        <v>9.228397516583078</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.770173816802065</v>
+        <v>2.713866523140604</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06870210159094327</v>
+        <v>0.07021933973646816</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1783556809024982</v>
+        <v>0.1787747028086761</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.005891366142209531</v>
+        <v>0.006124458394295207</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01091144468760595</v>
+        <v>0.01115241635687732</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9594673178377636</v>
+        <v>0.9525098451541913</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2215095071081895</v>
+        <v>0.2235971589181255</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>770275394.8168274</v>
+        <v>750498659.687384</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>140.37</v>
+        <v>143.85</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2827653406336837</v>
+        <v>-0.2649839299718987</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5739908952959029</v>
+        <v>-0.5634294385432473</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>329.5</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>404331573900</v>
+        <v>414355609500</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>21.66203703703704</v>
+        <v>22.19907407407407</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.64795504241688</v>
+        <v>16.01392939571599</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.633163463226382</v>
+        <v>5.7728187232679</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.235209668723416</v>
+        <v>6.38979063080333</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4714678649237475</v>
+        <v>0.4831563180827889</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>13.88901309384942</v>
+        <v>14.15476165164369</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.298905971272135</v>
+        <v>7.438561231313653</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.0710308119719166</v>
+        <v>-0.0693124440493426</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3843366100118384</v>
+        <v>0.3862352908844917</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4232963938119607</v>
+        <v>0.42786578758453</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01424805870200185</v>
+        <v>0.01390337156760514</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.076681238992412</v>
+        <v>2.074360657889285</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5630995647140897</v>
+        <v>0.5644469665851484</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4198679391.222831</v>
+        <v>4070435031.170095</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15 17:41 ET</t>
+          <t>2026-09-16 11:49 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-17)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN39"/>
+  <dimension ref="A1:AN41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>332.41</v>
+        <v>333.25</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2265598613404538</v>
+        <v>0.2296593778517679</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.03529036190033941</v>
+        <v>-0.03285254084801348</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>236.65</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4882224007960</v>
+        <v>4894561387000</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>37.94634703196348</v>
+        <v>38.04223744292238</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.73668116848796</v>
+        <v>34.79607211064622</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.45840502280307</v>
+        <v>10.48483341009333</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.42353898018974</v>
+        <v>45.53832425362724</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.159471714865549</v>
+        <v>1.162401699644849</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.24270864024311</v>
+        <v>29.3159335909215</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.5542936144106</v>
+        <v>10.58072200170086</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02799605257299776</v>
+        <v>0.0279254848785902</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09239989991868391</v>
+        <v>0.0932911428035279</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.118190305206118</v>
+        <v>0.1193167545241032</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003188833067597245</v>
+        <v>0.0031807951987997</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3070200193013617</v>
+        <v>0.3059345400831398</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2949067799982662</v>
+        <v>0.2899507877068625</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13207349211.33701</v>
+        <v>12766832784.5418</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>490.3</v>
+        <v>496.065</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.03670655361986341</v>
+        <v>0.04889626049650708</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.114534421729394</v>
+        <v>-0.1041230224662285</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3640747165000</v>
+        <v>3683555460750</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.23888888888889</v>
+        <v>27.55916666666667</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>23.87896674381447</v>
+        <v>24.14760878035563</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>10.97142639954918</v>
+        <v>11.10042960818349</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.233602479277193</v>
+        <v>8.330414060539752</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8651981180716664</v>
+        <v>0.8753712103634942</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.06398674338254</v>
+        <v>18.2702728942892</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.29650362073174</v>
+        <v>11.42550682936605</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01839924525492283</v>
+        <v>0.01818541914565362</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1407063455098934</v>
+        <v>0.1412793257229832</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2261231413426967</v>
+        <v>0.2267520769688407</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.00742402610646543</v>
+        <v>0.007337748077368893</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5568418062448269</v>
+        <v>0.5577324893737594</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4356886680199505</v>
+        <v>0.434154881478208</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>11219174471.19954</v>
+        <v>10740454964.50076</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>342.87</v>
+        <v>345.55</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.08795813625375049</v>
+        <v>0.09646202345636401</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1608869092777955</v>
+        <v>-0.154328087907785</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4149450896631</v>
+        <v>4181884554877</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.85004965243297</v>
+        <v>16.97715988083416</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.52357324488055</v>
+        <v>20.72668875166784</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.236945306686314</v>
+        <v>9.306625233563446</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.438239070696978</v>
+        <v>6.486806645016238</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.149848471580736</v>
+        <v>0.1509788702348104</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.87618994433856</v>
+        <v>12.97200048845385</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.364438768847592</v>
+        <v>9.434118695724724</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01293523806617031</v>
+        <v>0.01283839023787929</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1789904491102158</v>
+        <v>-0.1809034195359334</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2906786180835044</v>
+        <v>0.2907051226099779</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002508239274360545</v>
+        <v>0.002488785993343944</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7646756005936947</v>
+        <v>0.762699498306213</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3639582618317491</v>
+        <v>0.3625398837283717</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8244449990.676066</v>
+        <v>7721348481.462392</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>245.96</v>
+        <v>250.51</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.08591611479028693</v>
+        <v>0.1060044150110375</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1435933147632311</v>
+        <v>-0.1277506963788301</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2645816316000</v>
+        <v>2694761121000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.52063492063492</v>
+        <v>19.89444444444444</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>21.84955903685363</v>
+        <v>22.29743425320788</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.410963691212872</v>
+        <v>3.476281787592822</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.795956926869946</v>
+        <v>4.887796889162829</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2209696237208928</v>
+        <v>0.2252010716300056</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>10.98767038980775</v>
+        <v>11.18714495446797</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.597920941625413</v>
+        <v>3.663239038005363</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004393729046759722</v>
+        <v>-0.004311172443216265</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1065890671885193</v>
+        <v>-0.1077697900787722</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1790016137663994</v>
+        <v>0.1803222819468244</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8342653851018501</v>
+        <v>0.8371813960180776</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4606488180473121</v>
+        <v>0.4622122391380389</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8552608470.084135</v>
+        <v>8206834687.93328</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>213.9</v>
+        <v>219.3</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1326449197081496</v>
+        <v>0.1612390411033062</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.09571319861334227</v>
+        <v>-0.07288407880273939</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5180871900000</v>
+        <v>5311665300000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>26.90566037735849</v>
+        <v>27.58490566037736</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>15.97635175393754</v>
+        <v>16.35811684068175</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.10033666810796</v>
+        <v>17.53204222214154</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>22.59651766062257</v>
+        <v>23.16697673199874</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2159774098318573</v>
+        <v>0.2214298549608523</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>22.2422888127121</v>
+        <v>22.80203152349283</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>17.15452373015061</v>
+        <v>17.58622928418419</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.0245144065422656</v>
+        <v>0.02391076862467219</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6840928887740156</v>
+        <v>0.6863130352373565</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9386961152552931</v>
+        <v>0.9412154432375359</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002431042543244507</v>
+        <v>0.002371181030551756</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.328855676123753</v>
+        <v>1.329916978183309</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.409323484252594</v>
+        <v>0.4133781954716744</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26912650248.31583</v>
+        <v>25936219477.06731</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>673.3099999999999</v>
+        <v>671.9299999999999</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.03520860349781252</v>
+        <v>0.03308686481455081</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.148571067273647</v>
+        <v>-0.1503161355589276</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1715248182447</v>
+        <v>1711732650980</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>25.02081010776663</v>
+        <v>24.96952805648458</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>20.35852328551795</v>
+        <v>20.32732684915943</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7.514844302894221</v>
+        <v>7.499442058550349</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>6.554707814455958</v>
+        <v>6.541273442793649</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.129266072092154</v>
+        <v>-5.118753251579334</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>16.92416488388187</v>
+        <v>16.89133154307382</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.939189751704287</v>
+        <v>7.923787507360416</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.0238892542894539</v>
+        <v>0.0239383176902891</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2290090866052747</v>
+        <v>0.2283724388244934</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2723933984855695</v>
+        <v>0.273007539505155</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003118919962572961</v>
+        <v>0.003125325554745286</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7724072583281306</v>
+        <v>0.7681630389364189</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4080010568011128</v>
+        <v>0.4080591679147746</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10138078593.51151</v>
+        <v>9923380411.759483</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>358.08</v>
+        <v>371.9586</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1825964023714082</v>
+        <v>-0.1509151647428107</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2821602549966923</v>
+        <v>-0.2543379508048834</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1414253930844</v>
+        <v>1469068119306</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>303.4576271186441</v>
+        <v>315.2191525423729</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>170.3195592399943</v>
+        <v>176.787074434236</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.64859659757381</v>
+        <v>14.1775940638879</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.3448267286836</v>
+        <v>13.86205056759308</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.077956552876579</v>
+        <v>-8.391045046550486</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>117.0915306654473</v>
+        <v>121.6464476616229</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.59187920018529</v>
+        <v>14.12060985411942</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004074232974951922</v>
+        <v>0.003922288124775936</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7816957046668216</v>
+        <v>0.7830441142326445</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1224683805249132</v>
+        <v>0.1228443872713618</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.535109374454157</v>
+        <v>1.542491792865234</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5719937960643585</v>
+        <v>0.5752781187290299</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12789598512.76878</v>
+        <v>12645955770.24886</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>339.51</v>
+        <v>349.15</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-0.02333005934958809</v>
+        <v>0.004401371912730934</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.3141212121212121</v>
+        <v>-0.2946464646464647</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1615245985800</v>
+        <v>1661109057000</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>42.1228287841191</v>
+        <v>43.31885856079404</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>18.56124500582337</v>
+        <v>19.08416468427096</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.12764843104686</v>
+        <v>18.64236237430418</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.23136382786639</v>
+        <v>16.69223492827766</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4191429992875215</v>
+        <v>0.431044087659386</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>31.58429454489792</v>
+        <v>32.46183833687312</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>18.52543079771952</v>
+        <v>19.04014474097684</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02439442682192116</v>
+        <v>0.02372089889821123</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.269396733403582</v>
+        <v>1.269884968897651</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8547782329035543</v>
+        <v>0.855594416107851</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007481370210008542</v>
+        <v>0.00727481025347272</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.605185479351388</v>
+        <v>1.606646864702752</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3888614920512946</v>
+        <v>0.3924352387694716</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8628716383.128927</v>
+        <v>8452103139.321651</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>893.74</v>
+        <v>890.34</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.04592159157401987</v>
+        <v>0.04194265652428331</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1849156406748745</v>
+        <v>-0.188016415868673</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>396354921460</v>
+        <v>394847092860</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>44.88900050226017</v>
+        <v>44.7182320441989</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.42763013359002</v>
+        <v>39.27749941106249</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.350042479605705</v>
+        <v>1.344906596204873</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.8401546456176</v>
+        <v>11.79511187501865</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.541020709263116</v>
+        <v>3.527549822415158</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>26.65106575397374</v>
+        <v>26.54686198064962</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.31354903813861</v>
+        <v>1.308413154737778</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02221746097553805</v>
+        <v>0.02230230425711232</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.13851632345555</v>
+        <v>0.1385203415369163</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1137619578080773</v>
+        <v>0.1141243314792548</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006198670754358091</v>
+        <v>0.006222342026641507</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1859168656137269</v>
+        <v>-0.1866324341762206</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1771192357234746</v>
+        <v>0.176938987211484</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1715705441.000846</v>
+        <v>1673972933.153744</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>76.41</v>
+        <v>75.88</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1602373690083909</v>
+        <v>-0.1660621850589805</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3880345987506006</v>
+        <v>-0.3922793528752203</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>318166655324</v>
+        <v>315959767124</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>23.65634674922601</v>
+        <v>23.49226006191951</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.37305571203624</v>
+        <v>20.22856225925758</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.577664461202226</v>
+        <v>6.532040038151972</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.61634684863239</v>
+        <v>10.54270905476019</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.695265800800423</v>
+        <v>0.6904432530393417</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10.56889001229465</v>
+        <v>10.49676250112838</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.685375681144917</v>
+        <v>6.639751258094662</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03455612904753898</v>
+        <v>0.03479749368116578</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1611584969676407</v>
+        <v>0.1613410662029773</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1437551576299556</v>
+        <v>0.1440833291150601</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.0988661944525397</v>
+        <v>0.09619721903937392</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3345329005052507</v>
+        <v>0.3307769568007074</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2157532253.854227</v>
+        <v>2098409556.235269</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>520.67</v>
+        <v>511.2</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.04794202194599873</v>
+        <v>0.02888194368562536</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.03174396548517877</v>
+        <v>-0.04935470673559716</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1123008961309</v>
+        <v>1102583557764</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>13.07989678192819</v>
+        <v>12.87376236710941</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.47157446411095</v>
+        <v>23.04464410713981</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.917233679448487</v>
+        <v>2.871259137948514</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.49365653599084</v>
+        <v>1.470117052375639</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3603178470284479</v>
+        <v>0.3546393688428563</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.82694503549677</v>
+        <v>15.59580029798468</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.147969316472873</v>
+        <v>3.1019947749729</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02157772949766241</v>
+        <v>0.02192323165285077</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4427345808468063</v>
+        <v>-0.4413555571847257</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05995338976402564</v>
+        <v>0.06262062115746447</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.05282987392123903</v>
+        <v>0.04345626494962505</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1393146521303358</v>
+        <v>0.1458735753051842</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2110350198.758909</v>
+        <v>2062158632.583562</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>348.92</v>
+        <v>346.4</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.07201667759147434</v>
+        <v>0.06427426664475133</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.04796725784447475</v>
+        <v>-0.05484311050477497</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>934934629200</v>
+        <v>928182264000</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.00085984522786</v>
+        <v>14.89251934651763</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.9313507580556</v>
+        <v>13.83162337433422</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.141233093104595</v>
+        <v>3.118546209593694</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.597539773303648</v>
+        <v>2.578779598396147</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7854337607970518</v>
+        <v>0.7797611336125723</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.99779550450837</v>
+        <v>19.92531412623444</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.25936851491602</v>
+        <v>6.236681631405119</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1738453095261604</v>
+        <v>-0.175110004041189</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07676994899822165</v>
+        <v>0.07670075619265249</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2893751396518991</v>
+        <v>-0.2892987416862425</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.0171959188352631</v>
+        <v>0.01732101616628176</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7708858064475166</v>
+        <v>0.7629048937547521</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1714957115652187</v>
+        <v>0.171736261843984</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2116091765.374923</v>
+        <v>2067967030.863235</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>370.93</v>
+        <v>370.105</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.07056680973909524</v>
+        <v>0.06818571999700174</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.03796975905801792</v>
+        <v>-0.04010944834919727</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>692543821976</v>
+        <v>691003508027</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.51486830926083</v>
+        <v>31.44477485131691</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.80559245608796</v>
+        <v>24.72162350065607</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.56698035371336</v>
+        <v>15.53235722053138</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.17614359628177</v>
+        <v>20.13126904187276</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.125180264275814</v>
+        <v>2.120453567276306</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.19557433418104</v>
+        <v>24.14263894518524</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.82545454900198</v>
+        <v>15.79083141582</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03034176225851626</v>
+        <v>0.03040939699423197</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2704743240884069</v>
+        <v>0.2719542812583653</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1381361933238576</v>
+        <v>0.1384422594852113</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007225082899738495</v>
+        <v>0.007241188311425137</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3080010447724384</v>
+        <v>0.305358848336019</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1773232932326329</v>
+        <v>0.1770610234061577</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2269386064.094275</v>
+        <v>2201657438.223872</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>567.75</v>
+        <v>565.52</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.008204135949298141</v>
+        <v>0.00424412674953234</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05629799541238656</v>
+        <v>-0.06000465410059508</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>497937189000</v>
+        <v>495981398720</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.17792421746293</v>
+        <v>31.05546403075233</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.60034720521277</v>
+        <v>25.48993445147995</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.1931188609868</v>
+        <v>14.13737133996523</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>89.24532168953841</v>
+        <v>88.89478524327214</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.377952900682513</v>
+        <v>1.372540597787714</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.11852003074697</v>
+        <v>23.03008675709893</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.57370204942565</v>
+        <v>14.51795452840407</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.0330322786956971</v>
+        <v>0.0331625340031865</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2178711471192254</v>
+        <v>0.218342247598414</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1571890126686657</v>
+        <v>0.1575559517246576</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005935711140466755</v>
+        <v>0.005959117272598671</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2945476222545185</v>
+        <v>0.291689229362848</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1945693605476321</v>
+        <v>0.1943447227578078</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1516304142.725171</v>
+        <v>1475026974.375448</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>375.26</v>
+        <v>379.5</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1155172616188378</v>
+        <v>0.128121304653704</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.187080282483428</v>
+        <v>-0.1778952385078636</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>340790269045</v>
+        <v>344640801318</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.13092405633078</v>
+        <v>24.40357533277603</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.31191344656784</v>
+        <v>17.45369538426162</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7570946751820034</v>
+        <v>0.7656489613377498</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.45347683748616</v>
+        <v>3.492497094883541</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7311732994091873</v>
+        <v>-0.7394347042738011</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.96461083899391</v>
+        <v>15.11407061747467</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8564950692912475</v>
+        <v>0.865049355446994</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06930068768155311</v>
+        <v>0.06852641912879201</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3938912143252915</v>
+        <v>0.3981895979908796</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01040690486613927</v>
+        <v>0.01048486257114667</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02414326067260033</v>
+        <v>0.02387351778656127</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4338100090495249</v>
+        <v>0.435169589702524</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2278803417529079</v>
+        <v>0.2298487125057489</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1782957324.889425</v>
+        <v>1722683059.549052</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>163.345</v>
+        <v>162.11</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3317977820451516</v>
+        <v>0.3217284792760082</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.0740604274134119</v>
+        <v>-0.08106116433308763</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>676976818700</v>
+        <v>671858410600</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.02252252252252</v>
+        <v>20.86486486486487</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.78362536111271</v>
+        <v>14.675127491552</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.874970416828228</v>
+        <v>1.860909143078713</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.62848982803223</v>
+        <v>2.608777562340967</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.058455330330331</v>
+        <v>2.04301801801802</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.867829010790116</v>
+        <v>9.797143824573617</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.962989028693292</v>
+        <v>1.948927754943777</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04513153058722304</v>
+        <v>0.04547255035634067</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.422014019498951</v>
+        <v>0.4217842316447407</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08199294297389192</v>
+        <v>0.08189823918495898</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02522268817533442</v>
+        <v>0.025414841774104</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5384489964726794</v>
+        <v>-0.538773887662406</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2553168456323008</v>
+        <v>0.256266719295899</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2241902169.930573</v>
+        <v>2190166836.893951</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>267.28</v>
+        <v>268.1</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.289028175222553</v>
+        <v>0.2929828411297759</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.0490625111182269</v>
+        <v>-0.04614508841213927</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>644117648628</v>
+        <v>646093765330</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>30.89942196531792</v>
+        <v>31.00520231213873</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.57068663500358</v>
+        <v>21.63110372538485</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.577394322703183</v>
+        <v>6.599911218117207</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.675441362347152</v>
+        <v>7.701717285897541</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.825836324916343</v>
+        <v>-3.838933602068762</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.94342608288865</v>
+        <v>20.00879597056208</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.869585604141776</v>
+        <v>6.892102499555801</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02904438349088694</v>
+        <v>0.02894529286317761</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4324728038641219</v>
+        <v>0.433362009898415</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08958244178047914</v>
+        <v>0.09018004880011765</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01975456450164622</v>
+        <v>0.01969414397612831</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1723926613704065</v>
+        <v>-0.1714348386445364</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2079413320510723</v>
+        <v>0.2029502185939068</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1640539099.46374</v>
+        <v>1590417696.347237</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>107.5</v>
+        <v>106.97</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.04664776548935878</v>
+        <v>-0.05134801371531816</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2046463450725067</v>
+        <v>-0.2085676235572654</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>855493600000</v>
+        <v>851275817600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.8086642599278</v>
+        <v>38.6173285198556</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.6558120762303</v>
+        <v>34.47464110138019</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.162608175690367</v>
+        <v>1.15687624701022</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.703912946110465</v>
+        <v>8.66100063112034</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.384640630128002</v>
+        <v>9.338372169346906</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.42252620275917</v>
+        <v>21.32406960013072</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.247172754946728</v>
+        <v>1.24144082626658</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.0157908837658166</v>
+        <v>0.01586912222889861</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1198313337619308</v>
+        <v>0.1201662232332723</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05107088152361516</v>
+        <v>0.05119521528000814</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009093023255813954</v>
+        <v>0.009138076096101712</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.05510360733280622</v>
+        <v>-0.05802065046066822</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.307080509567927</v>
+        <v>0.3044032628724372</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2709248419.584712</v>
+        <v>2637779378.25264</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>147.04</v>
+        <v>147.09</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.03702663772098957</v>
+        <v>0.03737927191499169</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1208370702541106</v>
+        <v>-0.1205381165919283</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>349544802096</v>
+        <v>349663662543</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.7837037037037</v>
+        <v>21.79111111111111</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.81313325554507</v>
+        <v>20.81684209135355</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.016279093850538</v>
+        <v>4.017644803555014</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.558605070795971</v>
+        <v>6.560835281987075</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.78787724867747</v>
+        <v>20.79494603174625</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.62627280022584</v>
+        <v>17.63186518034252</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.30449492251126</v>
+        <v>4.305860632215737</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04552492242648085</v>
+        <v>0.04550944723357719</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04663259665144581</v>
+        <v>0.04680196042617957</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02543466982807141</v>
+        <v>0.02551447528784867</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02917981501632209</v>
+        <v>0.02916989598205181</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.04729346856656391</v>
+        <v>-0.04587182024652679</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1484728506341582</v>
+        <v>0.1479062117411055</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1293885600.720227</v>
+        <v>1250660853.280223</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -3095,52 +3095,52 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>302.47</v>
+        <v>306.755</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1253542490489179</v>
+        <v>-0.1129634101464636</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2912243702401874</v>
+        <v>-0.2720401528275469</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>426.75</v>
+        <v>421.39</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>301597978990</v>
+        <v>305870630204</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>21.12220670391061</v>
+        <v>21.42143854748603</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>20.15629508544118</v>
+        <v>20.4418431544765</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.78274683755379</v>
+        <v>1.808002495649501</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>18.09322862129145</v>
+        <v>18.34954985857856</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.245408113550766</v>
+        <v>-7.348051594777218</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.14028764332009</v>
+        <v>15.31790543027389</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.140256176939991</v>
+        <v>2.165364521947557</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05006996416411895</v>
+        <v>0.04937456889857118</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04792108938547468</v>
+        <v>0.0479210893854749</v>
       </c>
       <c r="V21" s="4" t="n">
         <v>0.01423568777486173</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03071378979733527</v>
+        <v>0.03028475493471989</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7117966030708344</v>
+        <v>0.7165636912018102</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2406043143442007</v>
+        <v>0.2411228897150816</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1228364276.919541</v>
+        <v>1199237626.261287</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>512.5</v>
+        <v>534.59003</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.293372699693349</v>
+        <v>1.39222279088829</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.123527097976844</v>
+        <v>-0.0857489268551298</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.85</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>835682500000</v>
+        <v>871702497791</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>130.0761421319797</v>
+        <v>135.6827487309644</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>37.76064948773325</v>
+        <v>39.32269655737718</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>20.23199370536255</v>
+        <v>21.1040430405762</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>12.43436124003332</v>
+        <v>12.97031326505415</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.050156009872863</v>
+        <v>1.095420356727052</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>77.89442993095727</v>
+        <v>81.25513134829259</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>20.21238348868176</v>
+        <v>21.08443282389541</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01005525423830223</v>
+        <v>0.00963975670747098</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.444753834921077</v>
+        <v>2.450494513594325</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8988302387766913</v>
+        <v>0.9013639506361797</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.540113897603888</v>
+        <v>2.539787156299862</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6652753068779969</v>
+        <v>0.6720455582023733</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>9727006093.451742</v>
+        <v>9056204706.384535</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -3347,55 +3347,55 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1602.22</v>
+        <v>1628.76</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.3767378367611436</v>
+        <v>0.3995428336951732</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1988739774795496</v>
+        <v>-0.1856037120742415</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>861.1799999999999</v>
+        <v>916.03</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>617524413540</v>
+        <v>627753407021</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>50.66037735849056</v>
+        <v>51.5166908563135</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>32.88343129008279</v>
+        <v>33.40077303828817</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.23234304816361</v>
+        <v>15.48981568528766</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>24.65455295206502</v>
+        <v>25.07128941508517</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.448637019616227</v>
+        <v>3.506929408717318</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>38.64197175080589</v>
+        <v>39.30087751255025</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.09965604795131</v>
+        <v>15.35712868507537</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01858672575990359</v>
+        <v>0.01827777609942123</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5406049603396792</v>
+        <v>0.5423801957295591</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2914089551371388</v>
+        <v>0.2926613335233557</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004855762629351774</v>
+        <v>0.004776639897836391</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.687391075987521</v>
+        <v>1.683761660048894</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4356364583820855</v>
+        <v>0.4380186529883067</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2056543960.434692</v>
+        <v>2011817038.896167</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>201.96</v>
+        <v>200.47</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1133160810832085</v>
+        <v>-0.1198577677498059</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2059760172989974</v>
+        <v>-0.2118340868881462</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>159623125200</v>
+        <v>158445473900</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>75.64044943820222</v>
+        <v>75.11235955056178</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>79.44419562398977</v>
+        <v>78.43648954995538</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.698208683440608</v>
+        <v>1.686352502792702</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>26.19006605917377</v>
+        <v>26.00721800439344</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4048332587082143</v>
+        <v>0.4020068827190155</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>28.52865110791367</v>
+        <v>28.37569461151079</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.109411406989734</v>
+        <v>2.098101787861056</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001315598850335001</v>
+        <v>-0.001324419130242788</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.04787947257708691</v>
+        <v>-0.04237989255340768</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1537975177777893</v>
+        <v>0.1546827263367114</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.250796279330109</v>
+        <v>1.240887169138777</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3467118317299859</v>
+        <v>0.3433122505972865</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1102622816.760091</v>
+        <v>1068844576.232046</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>937.98</v>
+        <v>937.5</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.02585468474549035</v>
+        <v>0.02532971593093358</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.187185330895415</v>
+        <v>-0.1876012790405462</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>276710665860</v>
+        <v>276569062500</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>14.28976234003656</v>
+        <v>14.28244972577697</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.94912673099564</v>
+        <v>12.94098381920838</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.346258306214335</v>
+        <v>2.345057636704342</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.293329080510339</v>
+        <v>2.292155496895928</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3349322288665724</v>
+        <v>0.3347608313209361</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.48102015927118</v>
+        <v>26.47650949256204</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.048836801512672</v>
+        <v>7.047636132002679</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.150030357055352</v>
+        <v>-0.1501071725981643</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1035309667509787</v>
+        <v>0.1036602723030562</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3822426848979621</v>
+        <v>-0.3821998793565314</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01919017463058914</v>
+        <v>0.0192</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.579849670566597</v>
+        <v>1.571253186595629</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3167145219979272</v>
+        <v>0.3163314308983209</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1880047207.127384</v>
+        <v>1849787123.847054</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>237.49</v>
+        <v>239.24</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.1852830188679245</v>
+        <v>-0.1792795883361921</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.285658425073693</v>
+        <v>-0.2803946339409251</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>223747403660</v>
+        <v>225396138160</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.74148471615721</v>
+        <v>20.89432314410481</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.40394470821588</v>
+        <v>18.5381623043999</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.238163793797126</v>
+        <v>3.262024952747587</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.479068007662836</v>
+        <v>6.526810518982934</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2528370908229242</v>
+        <v>0.2547001794116652</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.37546413044818</v>
+        <v>17.47710610689846</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.079010719133971</v>
+        <v>4.102871878084432</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06092137730774864</v>
+        <v>0.0604757477713477</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1270129879763118</v>
+        <v>0.1270978644493628</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04610799352298289</v>
+        <v>0.04621551567034698</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02838014232178197</v>
+        <v>0.02817254639692359</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.906225736184853</v>
+        <v>0.9065330631436457</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3287362947330283</v>
+        <v>0.3289476276953931</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1191779268.202718</v>
+        <v>1154475069.088229</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1138.21</v>
+        <v>1142</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.05354698011108994</v>
+        <v>0.05705507005461619</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1194754960739567</v>
+        <v>-0.1165435345994663</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1071899023610</v>
+        <v>1075468222000</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.07995985279358</v>
+        <v>38.2067581130813</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.04015482419395</v>
+        <v>26.11002880644067</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.4549458313354</v>
+        <v>13.49974797215367</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>29.98136320434487</v>
+        <v>30.08119484046164</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4025520876386162</v>
+        <v>0.4038925014569365</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>25.81508339976169</v>
+        <v>25.89750378710905</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.03258391442752</v>
+        <v>14.07738605524579</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01870875852882241</v>
+        <v>0.01864666904123551</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4623553550232131</v>
+        <v>0.4632981984170268</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2290918506683588</v>
+        <v>0.2295582709788979</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005877649994289279</v>
+        <v>0.005858143607705779</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3439939232763189</v>
+        <v>0.3459308472144155</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3238698314038505</v>
+        <v>0.3169698287472685</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3028410172.677368</v>
+        <v>2789503758.887024</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>202.51</v>
+        <v>201.36</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1133040505501302</v>
+        <v>0.1069818953077588</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1280516684607105</v>
+        <v>-0.1330032292787944</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>319414972800</v>
+        <v>317601100800</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>16.27893890675241</v>
+        <v>16.18649517684888</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.0356891137025</v>
+        <v>14.95626223681858</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.52444082226209</v>
+        <v>2.510105199598511</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.881288297997591</v>
+        <v>2.864926234184954</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4141621778840429</v>
+        <v>0.411810261906725</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.30244906804784</v>
+        <v>23.24064131938529</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.4047449422662</v>
+        <v>5.390409319602621</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04910226925968324</v>
+        <v>-0.0493827003763332</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08268658547328567</v>
+        <v>0.08225537373915337</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3271879519250608</v>
+        <v>-0.3271714729502154</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02049281516962126</v>
+        <v>0.0206098529996027</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.382020009427655</v>
+        <v>1.371311450104973</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2643246497965434</v>
+        <v>0.2597608951352844</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>904693082.6014979</v>
+        <v>878899504.3350958</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>926.55</v>
+        <v>976.29</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>1.937511763857309</v>
+        <v>2.095206259712106</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2617131474103586</v>
+        <v>-0.2220796812749004</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,40 +4120,40 @@
         <v>154.65</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1046436304500</v>
+        <v>1102612163100</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>20.67730417317563</v>
+        <v>21.78732425797813</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.936235394621748</v>
+        <v>6.245951893330358</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.59177952123535</v>
+        <v>12.2140612258236</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.37635915968389</v>
+        <v>10.93339343155554</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.02947122139929928</v>
+        <v>0.03105332549773018</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.03844123284464</v>
+        <v>15.85830903564217</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.38552965970268</v>
+        <v>12.00624752808117</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02501060015545361</v>
+        <v>0.02373940017726055</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.483235215353715</v>
+        <v>2.488231198393215</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.772514181536212</v>
+        <v>1.775779220960631</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005720144622524419</v>
+        <v>0.0005428714828585769</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.885412599554037</v>
+        <v>2.886543086267324</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8122571376334372</v>
+        <v>0.820553352657822</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25876878867.02397</v>
+        <v>25126493470.53228</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>139.82</v>
+        <v>139.65</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.05174633507059667</v>
+        <v>-0.05289926829215286</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2819654283454701</v>
+        <v>-0.2828384499245092</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>144554584840</v>
+        <v>144378828300</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>86.84472049689441</v>
+        <v>86.73913043478262</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>29.48350402909293</v>
+        <v>29.43157220450732</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.81228515069237</v>
+        <v>9.800354894108064</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.53995365931607</v>
+        <v>11.52592281879195</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>138.951552795034</v>
+        <v>138.7826086956551</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>43.1368830151906</v>
+        <v>43.08650854112926</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.2161678550095</v>
+        <v>10.2042375984252</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03168353328308034</v>
+        <v>0.03172210256813671</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.945535931251596</v>
+        <v>1.947145664936612</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2461938219817823</v>
+        <v>0.2467566443070532</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.7092741804550352</v>
+        <v>0.7036776976367544</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6292117067564663</v>
+        <v>0.6293165069886928</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2205532578.031082</v>
+        <v>2158145546.582966</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.46</v>
+        <v>27.67</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.09054804079392964</v>
+        <v>0.09888799303598095</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.05991098938719619</v>
+        <v>-0.05272167066073263</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>156506622400</v>
+        <v>157703504800</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.28435517970402</v>
+        <v>36.56183932346723</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.406110571823934</v>
+        <v>9.478736814759447</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.457087138909821</v>
+        <v>2.475877681487063</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.837005986618148</v>
+        <v>1.851054466486677</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6068799229171734</v>
+        <v>-0.611521029392505</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.32609493029151</v>
+        <v>17.42090500633714</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.433883170057774</v>
+        <v>3.452673712635016</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.07019511271492368</v>
+        <v>0.06966237062348407</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.857530155811058</v>
+        <v>2.857248074082654</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05042615492450442</v>
+        <v>-0.05053296346494318</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06263656227239621</v>
+        <v>0.06216118539934947</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3486650696099421</v>
+        <v>0.350326043615645</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2082359037915937</v>
+        <v>0.205500723789221</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>962789277.6907185</v>
+        <v>926092622.4251246</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>174.87</v>
+        <v>183.0973</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.04083093695289031</v>
+        <v>0.08980004753556603</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.1250813028468505</v>
+        <v>-0.08391804673037484</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1241323247892</v>
+        <v>1299725139339</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.685570928250936</v>
+        <v>7.624400949288165</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003630703383790578</v>
+        <v>0.003799028885083867</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.600574583261782</v>
+        <v>6.548040163611034</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.78317768603404</v>
+        <v>4.745108051239</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01719934805631963</v>
+        <v>0.0170624572815678</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.763078014576559</v>
+        <v>7.701006660861996</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.57032227901252</v>
+        <v>6.517787859361772</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07302685654173505</v>
+        <v>0.0736127453621272</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2115.826993514116</v>
+        <v>2005.934187635125</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2738.205531036524</v>
+        <v>2597.278524310316</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.71556013038257</v>
+        <v>1.638473095998685</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.9138247017200472</v>
+        <v>0.9179793845077476</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3192177153.981171</v>
+        <v>3129659147.48306</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -4611,22 +4611,22 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>545.5599999999999</v>
+        <v>560.53</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.4614519631395386</v>
+        <v>0.5015537592539878</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1879493324204041</v>
+        <v>-0.1656669097837251</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>301.37</v>
+        <v>312.6</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>68762790479</v>
+        <v>70649620476</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.827995764366803</v>
+        <v>1.827084824638465</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.4010232887662645</v>
+        <v>0.4064685706510061</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3790851939.296896</v>
+        <v>3707929935.446554</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>150.88</v>
+        <v>155.23</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.06256599651555428</v>
+        <v>-0.03553896897607034</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3313242332919695</v>
+        <v>-0.3120457365715299</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1972886577889</v>
+        <v>2029766592562</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-97.97402597402596</v>
+        <v>-100.7987012987013</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>135.5532035345952</v>
+        <v>124.8406962652859</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>119.0278478364404</v>
+        <v>122.4595229298341</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.954350751430548</v>
+        <v>7.154850657108721</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9797402597402596</v>
+        <v>-1.007987012987013</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>460.4580220515959</v>
+        <v>474.1081335641949</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>115.7603968560483</v>
+        <v>119.1920719494419</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01440680894611426</v>
+        <v>-0.01400308789402435</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.214836670179135</v>
+        <v>4.22540548358437</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.389296132328293</v>
+        <v>3.379435704680966</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7805915312933192</v>
+        <v>0.7765044942046671</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>14333385617.08179</v>
+        <v>13747121358.51425</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>754.05</v>
+        <v>761.4299999999999</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1037516560489238</v>
+        <v>0.1145542383997509</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.03248777859039997</v>
+        <v>-0.02301859193964362</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>803242884315</v>
+        <v>811104342423</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9950518300915309</v>
+        <v>0.9951548821037018</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1129920049986955</v>
+        <v>0.1151848510987127</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>29850488196.7432</v>
+        <v>28945458724.08904</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>417.72</v>
+        <v>425.89</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.306967926989262</v>
+        <v>0.3325303323409383</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1279331941544884</v>
+        <v>-0.1108768267223382</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>257.98</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2166496425600</v>
+        <v>2208869967200</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.58780572620842</v>
+        <v>28.10942390170396</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6366453119739534</v>
+        <v>0.6487089672437216</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.89916072363153</v>
+        <v>14.16195998101111</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.59388616712771</v>
+        <v>9.775283174489369</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5182494035320432</v>
+        <v>0.5280482367921029</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.27477474575392</v>
+        <v>18.63278794946157</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.41458131216091</v>
+        <v>13.67738056954049</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01812191372746905</v>
+        <v>0.01778563079232014</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.3330854831412</v>
+        <v>42.3313324172736</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.29980143517859</v>
+        <v>42.30502496853178</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2872737719046251</v>
+        <v>0.2817628965225762</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.178038787717862</v>
+        <v>2.177289933983538</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3560357257084865</v>
+        <v>0.3582524327454802</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4087324559.874907</v>
+        <v>3941303051.731517</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.07</v>
+        <v>28.205</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.01543318924410586</v>
+        <v>-0.01069800864374804</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.06433333333333335</v>
+        <v>-0.0598333333333334</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>70375327225</v>
+        <v>70713790680</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.10236220472441</v>
+        <v>-22.20866141732283</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-83.0013027386027</v>
+        <v>-84.17691565632209</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.948645361345701</v>
+        <v>1.958017186210716</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.146408733784031</v>
+        <v>2.156731682806505</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1644826954770189</v>
+        <v>0.1652737593847281</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.36848383884297</v>
+        <v>16.42442821157025</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.742055301813651</v>
+        <v>2.751427126678665</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03097676538014847</v>
+        <v>0.03082849864272048</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02065405918635133</v>
+        <v>0.02072773416995544</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.233659034991004</v>
+        <v>0.2308629111581491</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.1849426260663523</v>
+        <v>0.1565242418943464</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>507601729.8974198</v>
+        <v>492363203.8141126</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>312.43</v>
+        <v>314.505</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1617793287606775</v>
+        <v>-0.1562122964884195</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1937082247283801</v>
+        <v>-0.1883532478257504</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>210987103300</v>
+        <v>212388371550</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.94663432383263</v>
+        <v>19.07246816252274</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.07315993352108</v>
+        <v>16.17416015942142</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.509570293673355</v>
+        <v>2.526237573894116</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.179333138856476</v>
+        <v>6.220373103850642</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.17485680086648</v>
+        <v>1.182659597850758</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.09210092622553</v>
+        <v>9.148777364099661</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.673784726368751</v>
+        <v>2.690452006589512</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07134085337243454</v>
+        <v>0.0708701700104918</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1787747028086761</v>
+        <v>0.1791937247148543</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.006124458394295207</v>
+        <v>0.006357550646380439</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01133053804052108</v>
+        <v>0.01125578289693328</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9688452790398139</v>
+        <v>0.9678293910321804</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2350337985736363</v>
+        <v>0.2356061711049984</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>786557594.6112345</v>
+        <v>768638995.0475057</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>143.235</v>
+        <v>150.05</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2681263344423002</v>
+        <v>-0.2333044052296377</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5652959028831562</v>
+        <v>-0.5446130500758726</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>329.5</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>412584120450</v>
+        <v>432214523500</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>22.10416666666667</v>
+        <v>23.15586419753086</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.94546525544234</v>
+        <v>16.68949480784257</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.748138267829527</v>
+        <v>6.021629818744167</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.362472443539208</v>
+        <v>6.665193494279039</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4810906862745101</v>
+        <v>0.5039805737109662</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>14.10779746686108</v>
+        <v>14.62822172587487</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.413880775875281</v>
+        <v>7.687372326789919</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.06961004696127296</v>
+        <v>-0.0664484843485367</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3862352908844917</v>
+        <v>0.3874514755623204</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.42786578758453</v>
+        <v>0.4294717829481378</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01396306768597061</v>
+        <v>0.01332889036987671</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.059635807325663</v>
+        <v>2.079370502183088</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5634892069469046</v>
+        <v>0.5627040552432833</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4150823064.088405</v>
+        <v>4077758386.893623</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,259 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16 17:37 ET</t>
+          <t>2026-09-17 10:19 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Cisco</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="3" t="n">
+        <v>111.0801</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>0.4608113974564338</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>-0.1479627214850042</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>130.37</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>66.81</v>
+      </c>
+      <c r="K40" s="5" t="n">
+        <v>437814956732</v>
+      </c>
+      <c r="L40" s="6" t="n">
+        <v>33.05955357142857</v>
+      </c>
+      <c r="M40" s="6" t="n">
+        <v>21.41135533812198</v>
+      </c>
+      <c r="N40" s="6" t="n">
+        <v>6.913777445432294</v>
+      </c>
+      <c r="O40" s="6" t="n">
+        <v>8.732219057372975</v>
+      </c>
+      <c r="P40" s="6" t="n">
+        <v>1.057905714285714</v>
+      </c>
+      <c r="Q40" s="6" t="n">
+        <v>22.98466240731305</v>
+      </c>
+      <c r="R40" s="6" t="n">
+        <v>7.266165917599685</v>
+      </c>
+      <c r="S40" s="4" t="n">
+        <v>0.03105193139466434</v>
+      </c>
+      <c r="T40" s="4" t="n">
+        <v>0.1177498499664631</v>
+      </c>
+      <c r="U40" s="4" t="n">
+        <v>0.5440196591650359</v>
+      </c>
+      <c r="V40" s="4" t="n">
+        <v>0.1662824832486469</v>
+      </c>
+      <c r="W40" s="4" t="n">
+        <v>0.1023396098336123</v>
+      </c>
+      <c r="X40" s="4" t="n">
+        <v>0.2739106646984134</v>
+      </c>
+      <c r="Y40" s="4" t="n">
+        <v>0.645242795104619</v>
+      </c>
+      <c r="Z40" s="4" t="n">
+        <v>0.2426845637583893</v>
+      </c>
+      <c r="AA40" s="5" t="n">
+        <v>12767000000</v>
+      </c>
+      <c r="AB40" s="6" t="n">
+        <v>0.9311258278145695</v>
+      </c>
+      <c r="AC40" s="6" t="n">
+        <v>0.794003612281758</v>
+      </c>
+      <c r="AD40" s="6" t="n">
+        <v>0.5873123197772696</v>
+      </c>
+      <c r="AE40" s="6" t="n">
+        <v>0.2278130472010306</v>
+      </c>
+      <c r="AF40" s="6" t="n">
+        <v>1.114691043508667</v>
+      </c>
+      <c r="AG40" s="6" t="n">
+        <v>11.89047619047619</v>
+      </c>
+      <c r="AH40" s="4" t="n">
+        <v>0.01494417091810324</v>
+      </c>
+      <c r="AI40" s="6" t="n">
+        <v>0.7135542224607341</v>
+      </c>
+      <c r="AJ40" s="4" t="n">
+        <v>0.3389550718206246</v>
+      </c>
+      <c r="AK40" s="5" t="n">
+        <v>1956947392.126263</v>
+      </c>
+      <c r="AL40" s="7" t="inlineStr">
+        <is>
+          <t>2026-11-12 (C)</t>
+        </is>
+      </c>
+      <c r="AM40" s="2" t="inlineStr"/>
+      <c r="AN40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:19 ET</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>WFC</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Wells Fargo</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="3" t="n">
+        <v>86.405</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>-0.09238442468673402</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>-0.1161518003273323</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>97.76000000000001</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>72.78</v>
+      </c>
+      <c r="K41" s="5" t="n">
+        <v>261288720000</v>
+      </c>
+      <c r="L41" s="6" t="n">
+        <v>12.32596291012839</v>
+      </c>
+      <c r="M41" s="6" t="n">
+        <v>11.1088018035119</v>
+      </c>
+      <c r="N41" s="6" t="n">
+        <v>2.023846636458696</v>
+      </c>
+      <c r="O41" s="6" t="n">
+        <v>1.462303565819413</v>
+      </c>
+      <c r="P41" s="6" t="n">
+        <v>0.655163794322141</v>
+      </c>
+      <c r="Q41" s="6" t="n">
+        <v>15.60631191331381</v>
+      </c>
+      <c r="R41" s="6" t="n">
+        <v>4.004900817164324</v>
+      </c>
+      <c r="S41" s="4" t="n">
+        <v>0.0733671166516488</v>
+      </c>
+      <c r="T41" s="4" t="n">
+        <v>-0.01489668811853551</v>
+      </c>
+      <c r="U41" s="4" t="n">
+        <v>0.1095672718034899</v>
+      </c>
+      <c r="V41" s="4" t="n">
+        <v>-0.2903031514796548</v>
+      </c>
+      <c r="W41" s="4" t="n">
+        <v>0.009923315255755299</v>
+      </c>
+      <c r="X41" s="4" t="n">
+        <v>0.1256670879245121</v>
+      </c>
+      <c r="Y41" s="4" t="n">
+        <v>0.6450486038495798</v>
+      </c>
+      <c r="Z41" s="4" t="n">
+        <v>0.2117113976995469</v>
+      </c>
+      <c r="AA41" s="5" t="n">
+        <v>-19001000000</v>
+      </c>
+      <c r="AB41" s="6" t="n">
+        <v>0.5121191082899736</v>
+      </c>
+      <c r="AC41" s="6" t="n">
+        <v>0.5121191082899736</v>
+      </c>
+      <c r="AD41" s="6" t="n">
+        <v>2.548082579499417</v>
+      </c>
+      <c r="AE41" s="6" t="n">
+        <v>0.2011825426419496</v>
+      </c>
+      <c r="AF41" s="6" t="n">
+        <v>7.719779058887447</v>
+      </c>
+      <c r="AG41" s="6" t="n">
+        <v>0.6326638212402712</v>
+      </c>
+      <c r="AH41" s="4" t="n">
+        <v>0.02141079798622765</v>
+      </c>
+      <c r="AI41" s="6" t="n">
+        <v>0.7265825765145346</v>
+      </c>
+      <c r="AJ41" s="4" t="n">
+        <v>0.2275485790211614</v>
+      </c>
+      <c r="AK41" s="5" t="n">
+        <v>1069516490.984844</v>
+      </c>
+      <c r="AL41" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-13 (C)</t>
+        </is>
+      </c>
+      <c r="AM41" s="2" t="inlineStr"/>
+      <c r="AN41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:19 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-18)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,55 +699,55 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>337</v>
+        <v>334.95001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2434965051344211</v>
+        <v>0.2359322457855768</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.02196941115012918</v>
+        <v>-0.02791882636329335</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>236.65</v>
+        <v>240.21</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4949638972000</v>
+        <v>4919530071489</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.4703196347032</v>
+        <v>38.23630251141553</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.18762581031591</v>
+        <v>34.96592892165118</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.60281728192484</v>
+        <v>10.53831981605234</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>46.05075851004465</v>
+        <v>45.77062914969449</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.175481988838152</v>
+        <v>1.168331465626584</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.64283069216433</v>
+        <v>29.464128007603</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.69870587353237</v>
+        <v>10.63420840765986</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02761474135249313</v>
+        <v>0.02778375129611313</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09329114280352813</v>
+        <v>0.09353029336335772</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1193167545241032</v>
+        <v>0.1195887273062486</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.00314540059347181</v>
+        <v>0.003164651346032203</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3103413413725857</v>
+        <v>0.3106259292367567</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2917215924056524</v>
+        <v>0.2921115474887587</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13105224218.6762</v>
+        <v>12853530533.36324</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>497.75</v>
+        <v>493.99</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.05245908028612467</v>
+        <v>0.04450881179415922</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.1010799682149823</v>
+        <v>-0.1078704038142021</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3696067512500</v>
+        <v>3668147444500</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.65277777777778</v>
+        <v>27.44388888888889</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.22963174265876</v>
+        <v>24.03453471715925</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.13813479578953</v>
+        <v>11.05399740386151</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.35871024691051</v>
+        <v>8.29556860848081</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8783446120134039</v>
+        <v>0.8717096029904599</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.33056641801474</v>
+        <v>18.19602419296546</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.46321201697209</v>
+        <v>11.37907462504407</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01812385725462313</v>
+        <v>0.01826180681489233</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.141279325722983</v>
+        <v>0.141852305936073</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2267520769688407</v>
+        <v>0.2273810125949838</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007312908086388749</v>
+        <v>0.007368570213971943</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5589055542321191</v>
+        <v>0.5592294162324398</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4345471733432665</v>
+        <v>0.4337751090459382</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10974084804.75201</v>
+        <v>10519018361.31958</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>347.33</v>
+        <v>350.89</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.1021101276431742</v>
+        <v>0.113406336016795</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1499718558038228</v>
+        <v>-0.1412593915958984</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4203426312966</v>
+        <v>4246509829145</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>17.06454816285998</v>
+        <v>17.21896722939424</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.83345624111356</v>
+        <v>21.06602106299623</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.354530183290496</v>
+        <v>9.439180406958592</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.52019685236073</v>
+        <v>6.579198866475145</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1517560193094865</v>
+        <v>0.1531292770493972</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>13.03787023753176</v>
+        <v>13.15426507823563</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.482023645451774</v>
+        <v>9.566673869119869</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01277264429159752</v>
+        <v>0.01265809968608074</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1809065204848667</v>
+        <v>-0.1826189113785507</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2907002362377471</v>
+        <v>0.2898682348804311</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002476031439841073</v>
+        <v>0.002450910541765226</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7641258961441091</v>
+        <v>0.76361573303143</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3634733575263296</v>
+        <v>0.3627388231963615</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>7900376292.188757</v>
+        <v>7828933134.829708</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>251.19</v>
+        <v>253.1237</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1090066225165562</v>
+        <v>0.1175439293598235</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1253830083565459</v>
+        <v>-0.1186500696378829</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2702075949000</v>
+        <v>2722876953270</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.93571428571428</v>
+        <v>20.08918253968254</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.35795980225655</v>
+        <v>22.54192257048372</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.483493127320545</v>
+        <v>3.510309603534963</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.89793633298285</v>
+        <v>4.935641414742032</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.225668237853517</v>
+        <v>0.2274054673273709</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.20916762402706</v>
+        <v>11.2900585833691</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.670450377733086</v>
+        <v>3.696938183271453</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004302247686376931</v>
+        <v>-0.004269781099727464</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1083392911502502</v>
+        <v>-0.1088079343335507</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1795688947640286</v>
+        <v>0.179997197688706</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8377679948319768</v>
+        <v>0.8370649725470469</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4627757144334783</v>
+        <v>0.4624436850486459</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8395580226.45627</v>
+        <v>8302822149.937873</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>219.34</v>
+        <v>219.838</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1614508494099369</v>
+        <v>0.1640878628274902</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.07271497421154982</v>
+        <v>-0.07060962205123866</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5312634140000</v>
+        <v>5324696198000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>27.58993710691823</v>
+        <v>27.65157232704402</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.36110053732391</v>
+        <v>16.37668653244966</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.53524004106031</v>
+        <v>17.57441332281521</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>23.17120235474967</v>
+        <v>23.22296623344862</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2214702434432892</v>
+        <v>0.2219650023531425</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>22.80617776579491</v>
+        <v>22.85696923399539</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>17.58942710310296</v>
+        <v>17.62860038485786</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.0239064081307131</v>
+        <v>0.02385312086335173</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6863130352373563</v>
+        <v>0.6884717352471565</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9412154432375359</v>
+        <v>0.9436640378699037</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002370748609464758</v>
+        <v>0.002365378142086445</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.329235799282248</v>
+        <v>1.327430813333441</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4134708612908174</v>
+        <v>0.411076577822255</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26440839904.5858</v>
+        <v>25969098564.80347</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>682.3099999999999</v>
+        <v>673.4400000000001</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.04904602969299798</v>
+        <v>0.03540847743174313</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.137190187152251</v>
+        <v>-0.1484066767830045</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1738175561577</v>
+        <v>1715579355701</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>25.35525826830175</v>
+        <v>25.02564102564103</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>20.64134416151976</v>
+        <v>20.3688613331893</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7.615293722516737</v>
+        <v>7.516295238954997</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>6.642323281818843</v>
+        <v>6.555973371206757</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.197827945001853</v>
+        <v>-5.130256410256407</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>17.1382953673883</v>
+        <v>16.92904264896518</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.039639171326803</v>
+        <v>7.94147792975185</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02357414343279777</v>
+        <v>0.02388198251828632</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2283724388244937</v>
+        <v>0.2286224848938367</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.273007539505155</v>
+        <v>0.2736216805247405</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.00307777989476924</v>
+        <v>0.00311831789023521</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7735940337248534</v>
+        <v>0.7735635086953959</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4090935415337825</v>
+        <v>0.4104482514708787</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10205541163.94253</v>
+        <v>10189928339.75648</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>366.2</v>
+        <v>363.0901</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1640605522464523</v>
+        <v>-0.1711596458799006</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2658821642643786</v>
+        <v>-0.2721165527333961</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1446324255683</v>
+        <v>1434041558242</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>310.3389830508475</v>
+        <v>307.6737288135594</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>174.050086912407</v>
+        <v>172.4382954336029</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.9580989556259</v>
+        <v>13.83822396596184</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.64744065025674</v>
+        <v>13.53023365723365</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.261136309381712</v>
+        <v>-8.190187992360942</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>119.7578363554207</v>
+        <v>118.7251354447123</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.90138155823739</v>
+        <v>13.78150656857333</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.00398389225469983</v>
+        <v>0.004018403117078524</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7830441142326448</v>
+        <v>0.7842540605026374</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1228443872713618</v>
+        <v>0.1231118120551531</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.535289737654368</v>
+        <v>1.536474236973029</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5703197237714112</v>
+        <v>0.5671256769133135</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12967035666.74941</v>
+        <v>12961748241.16383</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>347.3</v>
+        <v>357.54</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-0.0009205313896849532</v>
+        <v>0.02853692256530982</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2983838383838383</v>
+        <v>-0.2776969696969697</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1652307534000</v>
+        <v>1701025153200</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>43.0893300248139</v>
+        <v>44.35980148883375</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>18.98304566761365</v>
+        <v>19.52060367684623</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.54358428353385</v>
+        <v>19.0903343643383</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.60378974821948</v>
+        <v>17.09334577189287</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4287601650983955</v>
+        <v>0.4414019851116623</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>32.29343003654593</v>
+        <v>33.22559273673536</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>18.9413666502065</v>
+        <v>19.48811673101095</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02384725554365232</v>
+        <v>0.02316426651650291</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.269884968897651</v>
+        <v>1.272460535708215</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8555944161078508</v>
+        <v>0.857683211380821</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007313561762165275</v>
+        <v>0.007104100240532527</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.603180456370468</v>
+        <v>1.600346910029839</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3900005977275804</v>
+        <v>0.393113595417772</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8661789348.470654</v>
+        <v>8637120849.128256</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>893.9299999999999</v>
+        <v>895.3049999999999</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.04614394382679921</v>
+        <v>0.04775307197191325</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1847423620611035</v>
+        <v>-0.1834883720930233</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,31 +1724,31 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>396439182470</v>
+        <v>397048966095</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>44.89854344550477</v>
+        <v>44.96760421898543</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.43587286714187</v>
+        <v>39.49653122427534</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.350329484854575</v>
+        <v>1.352406496524029</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.84267174162165</v>
+        <v>11.86088756796681</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.541773494116385</v>
+        <v>3.547221279238721</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>26.65688890601244</v>
+        <v>26.70176088970284</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.31383604338748</v>
+        <v>1.316047645413455</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02221273877403978</v>
+        <v>0.02217641770508916</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006197353260322397</v>
+        <v>0.006187835430384059</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1847808843101222</v>
+        <v>-0.1839456753916672</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1768386631306476</v>
+        <v>0.1763109668287718</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1731346165.996574</v>
+        <v>1695283023.777081</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>75.31</v>
+        <v>71.845</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1723266098681051</v>
+        <v>-0.2104077185762052</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3968444658016979</v>
+        <v>-0.4245955470126542</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>313586321325</v>
+        <v>299158274311</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>23.31578947368421</v>
+        <v>22.24303405572756</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.07660811471651</v>
+        <v>19.14987640120978</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.482972262439353</v>
+        <v>6.18469194141734</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.46351369153914</v>
+        <v>9.982089246695383</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6852567394094996</v>
+        <v>0.6537281960280905</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10.41919140424638</v>
+        <v>9.948321237107983</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.590683482382044</v>
+        <v>6.292833475361275</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03506086602739671</v>
+        <v>0.03674925289529826</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1613410662029773</v>
+        <v>0.1615236354383141</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1440833291150601</v>
+        <v>0.1444115006001652</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.0926744441018264</v>
+        <v>0.09495447893104303</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3326241973936346</v>
+        <v>0.3523153787817147</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2155970177.13188</v>
+        <v>2171170761.703859</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>509.2</v>
+        <v>507.81</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.02485658396854551</v>
+        <v>0.02205895896517496</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.05307397627106036</v>
+        <v>-0.05565886859820735</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1098269850574</v>
+        <v>1095271824077</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.80563770215411</v>
+        <v>12.76808939621049</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.95448509263613</v>
+        <v>22.89179783164884</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.856065167359437</v>
+        <v>2.84769069892666</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.46233756812059</v>
+        <v>1.458049745859977</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3527627078098621</v>
+        <v>0.3517283476017706</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.51941005614659</v>
+        <v>15.47730600802468</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.086800804383824</v>
+        <v>3.078426335951046</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02203986097236272</v>
+        <v>0.02210467563781969</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4421291677650311</v>
+        <v>-0.44224173697017</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06114910458549239</v>
+        <v>0.06097915463345482</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.03887823087399517</v>
+        <v>0.03939255501932271</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1493477437764856</v>
+        <v>0.1492536220272904</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2144255896.806022</v>
+        <v>2108237113.600871</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>349.31</v>
+        <v>347</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.07321490785703855</v>
+        <v>0.06611769782254262</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.04690313778990451</v>
+        <v>-0.05320600272851295</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>935979638100</v>
+        <v>929789970000</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.01762682717111</v>
+        <v>14.9183147033534</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.94781859378952</v>
+        <v>13.85497449975836</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.144744158409853</v>
+        <v>3.123947848524861</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.600443133705999</v>
+        <v>2.583246306707457</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7863116673851259</v>
+        <v>0.7811117591326865</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.00901286066982</v>
+        <v>19.94257159725204</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.262879580221279</v>
+        <v>6.242083270336287</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.173651213534877</v>
+        <v>-0.1748072201725299</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07670075619265249</v>
+        <v>0.07674790044641289</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2892987416862425</v>
+        <v>-0.2892465869116644</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01717671981907188</v>
+        <v>0.01729106628242075</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7660134893613323</v>
+        <v>0.7674338664160787</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1705710040290456</v>
+        <v>0.1654414159399357</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2128423294.955566</v>
+        <v>2096482695.002885</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>369.93</v>
+        <v>369.98999</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.06768064035473964</v>
+        <v>0.06785378165610689</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.04056332183520495</v>
+        <v>-0.04040773400420161</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>690676774765</v>
+        <v>690788779365</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.42990654205607</v>
+        <v>31.43500339847068</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.7099341581381</v>
+        <v>24.70576767734846</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.52501291955134</v>
+        <v>15.52753055576785</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.12175019699812</v>
+        <v>20.12501325702115</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.119450934579441</v>
+        <v>2.119794637067926</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.13141022630421</v>
+        <v>24.13525944618187</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.78348711483996</v>
+        <v>15.78600475105647</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03042378253872745</v>
+        <v>0.0304188496219003</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2719542812583653</v>
+        <v>0.2723750910720311</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1384422594852113</v>
+        <v>0.1387483256465651</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007244613845862731</v>
+        <v>0.007243439207639105</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3041296675936401</v>
+        <v>0.3058432740746191</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1771115692814877</v>
+        <v>0.1736684649057387</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2252382337.061794</v>
+        <v>2215551708.526697</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -2339,55 +2339,55 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>565.73</v>
+        <v>567.24</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.004617042414084338</v>
+        <v>0.007298483621100527</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05965559655596553</v>
+        <v>-0.05653410508457668</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>601.62</v>
+        <v>601.23</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>496165576280</v>
+        <v>497489900640</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.06699615595826</v>
+        <v>31.1499176276771</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.49939987486871</v>
+        <v>25.55757834192488</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.14262110651883</v>
+        <v>14.18036942792806</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>88.92779540188916</v>
+        <v>89.16515416146855</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.373050276535655</v>
+        <v>1.376715109437514</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.03841455416893</v>
+        <v>23.09829538071984</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.52320429495767</v>
+        <v>14.5609526163669</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03315022401053865</v>
+        <v>0.03306197769812078</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.218342247598414</v>
+        <v>0.2188133480776031</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1575559517246576</v>
+        <v>0.1579228907806498</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005956905237480777</v>
+        <v>0.005941047880967492</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2909059922383178</v>
+        <v>0.2926366823843486</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1942915591974401</v>
+        <v>0.1892272728790046</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1508107121.504842</v>
+        <v>1466547292.951424</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>375.21</v>
+        <v>374.76999</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1153686290358795</v>
+        <v>0.1140606325793296</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.187188596681253</v>
+        <v>-0.188141783284953</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>340744861825</v>
+        <v>340345268310</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.12770882901421</v>
+        <v>24.09941418558293</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.25639274078736</v>
+        <v>17.23026590034443</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7569937991664611</v>
+        <v>0.7561060680604893</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.453016692941379</v>
+        <v>3.448967328918403</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7310758771820103</v>
+        <v>-0.7302185420984069</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.96284834161394</v>
+        <v>14.94733797733183</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8563941932757053</v>
+        <v>0.8555064621697335</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06930992260164802</v>
+        <v>0.06939129818748853</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3981895979908794</v>
+        <v>0.3986675728028772</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01048486257114667</v>
+        <v>0.01056282027615407</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.0241464779723355</v>
+        <v>0.02417482787242383</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4276747997915096</v>
+        <v>0.4282999180245435</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2271589811774222</v>
+        <v>0.2070963720507303</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1773592635.472208</v>
+        <v>1731751011.940075</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>163.3</v>
+        <v>163.265</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3314308843734017</v>
+        <v>0.3311455195175956</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.07431551499348099</v>
+        <v>-0.074513916444646</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>676790318000</v>
+        <v>676645261900</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.01673101673102</v>
+        <v>21.01222651222651</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.78285312053816</v>
+        <v>14.78298599456936</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.874453880241511</v>
+        <v>1.874052129562954</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.627765703986429</v>
+        <v>2.62720249639525</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.057888245388247</v>
+        <v>2.05744717932218</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.865232412112775</v>
+        <v>9.862924324399582</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.962472492106575</v>
+        <v>1.962013348473938</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04514396732253489</v>
+        <v>0.04515502795399944</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.421696532148587</v>
+        <v>0.4213790447982231</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08183150477592971</v>
+        <v>0.08167006657796794</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02522963870177587</v>
+        <v>0.02523504731571372</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5338359743767092</v>
+        <v>-0.5333224483281266</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2551697232515629</v>
+        <v>0.2502025527989721</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2239596334.706132</v>
+        <v>2208923240.115904</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>270.22</v>
+        <v>269.195</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.3032070993289373</v>
+        <v>0.2982637669449086</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.03860248336713257</v>
+        <v>-0.04224926174974208</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>651202749972</v>
+        <v>648732604095</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.2393063583815</v>
+        <v>31.12080924855491</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.80215161758111</v>
+        <v>21.7136705641696</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.649743691572466</v>
+        <v>6.624519846980976</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.759868919984465</v>
+        <v>7.730434142236763</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.867919379373295</v>
+        <v>-3.853247566169766</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.15346703344006</v>
+        <v>20.08023847073995</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.941934973011059</v>
+        <v>6.916711128419569</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02872837991056456</v>
+        <v>0.02883776748988619</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4328542845831023</v>
+        <v>0.4332357653020824</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08979388535784305</v>
+        <v>0.09000526221088045</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01953963437199319</v>
+        <v>0.01961403443600364</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1659690344752618</v>
+        <v>-0.1651940988356478</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2041548623999825</v>
+        <v>0.2042261709506598</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1642467131.754413</v>
+        <v>1607087263.489426</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>106.79</v>
+        <v>107.22</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.05294432443356845</v>
+        <v>-0.04913091549552595</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2098993785143533</v>
+        <v>-0.2067179638946434</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>849843363200</v>
+        <v>853265337600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.55234657039712</v>
+        <v>38.70938628158845</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.41663011326906</v>
+        <v>34.54795667197718</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.154929554250924</v>
+        <v>1.159634061752555</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.646426637350109</v>
+        <v>8.681647122294834</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.322658352477855</v>
+        <v>9.360633409911395</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.290631508672</v>
+        <v>21.37144022969724</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.239494133507284</v>
+        <v>1.244198641008915</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01589587044503497</v>
+        <v>0.01583138265166971</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1201662232332725</v>
+        <v>0.1204537116079782</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05119521528000814</v>
+        <v>0.05132784400687207</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.00915347879014889</v>
+        <v>0.009116769259466518</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.05953211276586588</v>
+        <v>-0.05913344462291252</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3045596561609127</v>
+        <v>0.3024289948247972</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2697221653.592152</v>
+        <v>2648813132.931631</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>147.51</v>
+        <v>146.34</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.04034139914460799</v>
+        <v>0.03208975900496203</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1180269058295965</v>
+        <v>-0.1250224215246637</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>350662090297</v>
+        <v>347880755841</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.85333333333333</v>
+        <v>21.68</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.87628239102293</v>
+        <v>20.70734842384243</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.029116765063425</v>
+        <v>3.997159158022337</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.57956905599234</v>
+        <v>6.527382114120527</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.85432380952403</v>
+        <v>20.68891428571451</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.67884117328503</v>
+        <v>17.54686100268185</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.317332593724148</v>
+        <v>4.28510184473527</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04537986979579737</v>
+        <v>0.0457458114780605</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04680196042617957</v>
+        <v>0.04697132420091332</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02551447528784867</v>
+        <v>0.02559428074762593</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02908684157006305</v>
+        <v>0.02931939319393194</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.04359774690612261</v>
+        <v>-0.04143308998853398</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1482119462395578</v>
+        <v>0.1486293926706055</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1278594925.52955</v>
+        <v>1250507529.617664</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -3095,46 +3095,46 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>302.51</v>
+        <v>301.09</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1252385819413104</v>
+        <v>-0.1293447642613771</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2821139561926007</v>
+        <v>-0.2806870849061112</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>421.39</v>
+        <v>418.58</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>301637863670</v>
+        <v>300221953878</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>21.125</v>
+        <v>21.02583798882681</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>20.1589606450121</v>
+        <v>20.06433328024427</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.782982596053814</v>
+        <v>1.774613147715988</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>18.09562135162785</v>
+        <v>18.01067942468556</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.246366279069798</v>
+        <v>-7.212351403144112</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.14195541166632</v>
+        <v>15.08274948266778</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.140491935440015</v>
+        <v>2.13212248710219</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.0500633435612742</v>
+        <v>0.05029945280462911</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03070972860401309</v>
+        <v>0.03085456175894251</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7075997509067974</v>
+        <v>0.7070411579141297</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.237857828174506</v>
+        <v>0.2378792183223306</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1233270114.127983</v>
+        <v>1227428075.027888</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -3221,55 +3221,55 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>545.09</v>
+        <v>543.03</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.439208829026045</v>
+        <v>1.429990589491667</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.06779197236331291</v>
+        <v>-0.07131496588168906</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>149.85</v>
+        <v>154.78</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>888823754000</v>
+        <v>885464718000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>138.3477157360406</v>
+        <v>137.8248730964467</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>40.0950400561356</v>
+        <v>39.87724253966871</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>21.51855111971916</v>
+        <v>21.43722837428883</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>13.22506530405808</v>
+        <v>13.17508523741521</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.116935686676291</v>
+        <v>1.112714571787826</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>82.85256148535174</v>
+        <v>82.53916010449711</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>21.49894090303837</v>
+        <v>21.41761815760804</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.009454067763359979</v>
+        <v>0.009489932042667791</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.450494513594326</v>
+        <v>2.456228774076907</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9013639506361797</v>
+        <v>0.9038976624956678</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.546665325354219</v>
+        <v>2.546240113360414</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6809501234510832</v>
+        <v>0.653668679826144</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>9447557508.112457</v>
+        <v>9227197779.396566</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -3347,55 +3347,55 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1629.67</v>
+        <v>1656.07</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4003247684054205</v>
+        <v>0.4230094676917195</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1851487029740595</v>
+        <v>-0.1719484389687794</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>916.03</v>
+        <v>925.87</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>628104137393</v>
+        <v>638279172355</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>51.45137880986938</v>
+        <v>52.16255370101596</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>33.41943429191968</v>
+        <v>33.93304611035687</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.47017794177341</v>
+        <v>15.68401088251362</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>25.03950443061753</v>
+        <v>25.38560724165421</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.502483379040117</v>
+        <v>3.55089565279154</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>39.25062198833714</v>
+        <v>39.79784812575609</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.33749094156111</v>
+        <v>15.55132388230132</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01830097778982211</v>
+        <v>0.01805146560008102</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5395646245965797</v>
+        <v>0.5372198986018875</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2903016170625285</v>
+        <v>0.2881019734108514</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004773972644768572</v>
+        <v>0.004697869051428986</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.682070708349278</v>
+        <v>1.681579670631043</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4380536520947686</v>
+        <v>0.4305795533260287</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2063913814.663717</v>
+        <v>2030263382.988037</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>197</v>
+        <v>196.385</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1350924340136269</v>
+        <v>-0.1377925261612494</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2254767053273049</v>
+        <v>-0.2278946333792019</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>155702890000</v>
+        <v>155216812450</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>73.78277153558049</v>
+        <v>73.55243445692881</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>77.078807010232</v>
+        <v>76.42957280766605</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.656501835204</v>
+        <v>1.651330522368211</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>25.54685588065574</v>
+        <v>25.46710300569836</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3948908296965647</v>
+        <v>0.3936580486799993</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>27.96458848920863</v>
+        <v>27.89464927338129</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.067704558753125</v>
+        <v>2.062533245917336</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001348722557429731</v>
+        <v>-0.001352946222031504</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.04276189010312492</v>
+        <v>-0.03764430762916227</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1542221199138396</v>
+        <v>0.1546467220498906</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.225929111018157</v>
+        <v>1.226012386886879</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3480121506438135</v>
+        <v>0.3439755139730449</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1127466386.077801</v>
+        <v>1092878111.053377</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>951.47</v>
+        <v>941.29</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.04060849580459247</v>
+        <v>0.0294747821958703</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1754954548999558</v>
+        <v>-0.1843170218112808</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>280690310290</v>
+        <v>277687139030</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>14.49527726995734</v>
+        <v>14.34018890920171</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.13382173275968</v>
+        <v>12.99177777803206</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.380002122234752</v>
+        <v>2.354537923043659</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.326311670007006</v>
+        <v>2.301421917518046</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3397492140553931</v>
+        <v>0.3361141577750228</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.6077886882426</v>
+        <v>26.51212496511961</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.08258061753309</v>
+        <v>7.057116418341995</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1479032174538126</v>
+        <v>-0.1495027826820417</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1036602723030562</v>
+        <v>0.1037895778551334</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3821998793565314</v>
+        <v>-0.3821570738151003</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01891809515801864</v>
+        <v>0.01912269332511766</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.577549927393038</v>
+        <v>1.57960728667643</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3190602947673415</v>
+        <v>0.3099646591195975</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1924642858.382861</v>
+        <v>1901801597.025374</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>237.75</v>
+        <v>229.87</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.1843910806174958</v>
+        <v>-0.2114236706689536</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.2848763761053961</v>
+        <v>-0.3085784756060879</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>223992358500</v>
+        <v>216568342580</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.76419213973799</v>
+        <v>20.07598253275109</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.42270560053117</v>
+        <v>17.80894327846084</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.241708880269766</v>
+        <v>3.134265490252833</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.486161180773251</v>
+        <v>6.271183472657611</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2531138925561086</v>
+        <v>0.2447246707965202</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.39056522409223</v>
+        <v>16.93288592441896</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.082555805606611</v>
+        <v>3.975112415589678</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06085475456074543</v>
+        <v>0.06294087047817125</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1270978644493628</v>
+        <v>0.127297797451696</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04621551567034698</v>
+        <v>0.04632303781771174</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02834910620399579</v>
+        <v>0.02932092052029408</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.9011723088955274</v>
+        <v>0.9049354814923495</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3287473900314055</v>
+        <v>0.3390150801183113</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1191876703.17749</v>
+        <v>1184209801.843376</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1152.13</v>
+        <v>1146.73</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.06643157431000435</v>
+        <v>0.06143324035352893</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1087069198932425</v>
+        <v>-0.1128843847909334</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1085008058330</v>
+        <v>1079922656930</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.5456674473068</v>
+        <v>38.36500501840081</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.34163527912828</v>
+        <v>26.20129058188018</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.61949617439353</v>
+        <v>13.5556619895865</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.34802715546504</v>
+        <v>30.20578682959945</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.407475190633608</v>
+        <v>0.4055653661958957</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.11779891212983</v>
+        <v>26.00036617026288</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.19713425748565</v>
+        <v>14.13330007267862</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01848271987110044</v>
+        <v>0.01856975577955661</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4632981984170268</v>
+        <v>0.4642410418108409</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2295582709788979</v>
+        <v>0.230024722751039</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005806636403878035</v>
+        <v>0.005833980099936341</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3510644524708125</v>
+        <v>0.3509779977696696</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3183724314684314</v>
+        <v>0.312613469175804</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2849968516.693994</v>
+        <v>2748902137.458256</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>203.46</v>
+        <v>202.25</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1185267005329589</v>
+        <v>0.1118746937127244</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1239612486544671</v>
+        <v>-0.1291711517761034</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>320913388800</v>
+        <v>319004880000</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>16.35530546623794</v>
+        <v>16.258038585209</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.11224232570077</v>
+        <v>15.01994671915705</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.53628329315809</v>
+        <v>2.521199724964238</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.894804785494987</v>
+        <v>2.877589048787777</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4161050649957403</v>
+        <v>0.4136304403587362</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.35350764302995</v>
+        <v>23.28847514226327</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.4165874131622</v>
+        <v>5.401503844968348</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04887299984163204</v>
+        <v>-0.0491653920780146</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08225537373915337</v>
+        <v>0.08242984407347054</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3271714729502155</v>
+        <v>-0.3270721467871623</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02039712965693502</v>
+        <v>0.02051915945611867</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.374613089101811</v>
+        <v>1.376177867515408</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2600437713250752</v>
+        <v>0.2517194542518957</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>905752149.6856415</v>
+        <v>891502602.344251</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>977.5</v>
+        <v>991.1</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.099042414516776</v>
+        <v>2.142159526370923</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2211155378486056</v>
+        <v>-0.2102788844621514</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,40 +4120,40 @@
         <v>154.65</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1103978725000</v>
+        <v>1119338429000</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>21.81432715911627</v>
+        <v>22.11604597188128</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.253693037653182</v>
+        <v>6.340700940785748</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>12.22919916033409</v>
+        <v>12.39834392912688</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.94694412453834</v>
+        <v>11.09835374448989</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03109181254958183</v>
+        <v>0.03152185032708219</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.8803693705557</v>
+        <v>16.1037822236561</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>12.02294929880143</v>
+        <v>12.19209406759421</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02370697859236372</v>
+        <v>0.02338355544523191</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.488231198393215</v>
+        <v>2.487949704365118</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.775779220960631</v>
+        <v>1.775555219220929</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005421994884910487</v>
+        <v>0.0005347593582887701</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.885038377702729</v>
+        <v>2.885542369802312</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8210021951492738</v>
+        <v>0.7721368978843398</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25563845399.48759</v>
+        <v>24945013988.89314</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>138.47</v>
+        <v>136.73</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.06090198124177881</v>
+        <v>-0.07270259186241368</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2888982467672524</v>
+        <v>-0.297833879399772</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>143158871140</v>
+        <v>141359951260</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>86.00621118012423</v>
+        <v>84.92546583850933</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>29.18288437635609</v>
+        <v>28.80044437670449</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.717544877816998</v>
+        <v>9.595435192777627</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.42853227868329</v>
+        <v>11.28492249920102</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>137.6099378882017</v>
+        <v>135.8807453416178</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>42.73685042705646</v>
+        <v>42.22125286901691</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.12142758213413</v>
+        <v>9.999317897094761</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03199242885563871</v>
+        <v>0.03239955842638991</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.947145664936612</v>
+        <v>1.948755398621629</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2467566443070532</v>
+        <v>0.2473194666323242</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6967141468686718</v>
+        <v>0.6997775735484316</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6303167794631368</v>
+        <v>0.6270241528624115</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2189840012.617457</v>
+        <v>2144377934.183103</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.635</v>
+        <v>27.45</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.09749800099563899</v>
+        <v>0.09015090021097483</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.05391989044847656</v>
+        <v>-0.06025333789798015</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>157504024400</v>
+        <v>156449628000</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.51559196617337</v>
+        <v>36.27629492600423</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.466747086226141</v>
+        <v>9.404060528651197</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.472745924390856</v>
+        <v>2.45654126323474</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.848713053175255</v>
+        <v>1.836597911726729</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6107475116466164</v>
+        <v>-0.6067451098243185</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.4051033269962</v>
+        <v>17.32334064504119</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.449541955538809</v>
+        <v>3.433337294382693</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06975059870279733</v>
+        <v>0.0702107109892593</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.857248074082655</v>
+        <v>2.857513976593605</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05053296346494307</v>
+        <v>-0.05050491154177539</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06223991315360955</v>
+        <v>0.06265938069216757</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3497169902670222</v>
+        <v>0.3509371480600263</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.205383182098487</v>
+        <v>0.2061895175678352</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>948904358.3716139</v>
+        <v>912778413.2761378</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>182.99</v>
+        <v>183.41499</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.08916139505352216</v>
+        <v>0.0916909469486189</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.08445489568219344</v>
+        <v>-0.08232856356631824</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1298963465041</v>
+        <v>1301980300669</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.624400949288165</v>
+        <v>8.113760780990328</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003796802550783091</v>
+        <v>0.003802660961113973</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.548040163611034</v>
+        <v>6.968315520817014</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.745108051239</v>
+        <v>5.049665129599325</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.0170624572815678</v>
+        <v>0.01815758347958247</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.701006660861996</v>
+        <v>8.197577490578496</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.517787859361772</v>
+        <v>6.938063216567753</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.0736127453621272</v>
+        <v>0.06917298904518683</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2007.110995320426</v>
+        <v>2132.706071606614</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2598.802079070919</v>
+        <v>2762.495665002442</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.639433848844199</v>
+        <v>1.635635124479193</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.9179194720631826</v>
+        <v>0.8633465846030076</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3195371538.874002</v>
+        <v>3136792281.322672</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -4611,22 +4611,22 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>560.61</v>
+        <v>565.575</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.5017680641096429</v>
+        <v>0.515068359213734</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1655478320408437</v>
+        <v>-0.1581575696232678</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>312.6</v>
+        <v>313.43</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>70659703736</v>
+        <v>71285496050</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.825747298502964</v>
+        <v>1.82540761846922</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.4065995578440564</v>
+        <v>0.3919771357421525</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3788770992.865133</v>
+        <v>3700231626.092234</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>154.81</v>
+        <v>151.06</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.03814847508333075</v>
+        <v>-0.06144763675529974</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3139071086686757</v>
+        <v>-0.3305265023931927</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>2040671353285</v>
+        <v>1991239646310</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-100.525974025974</v>
+        <v>-98.09090909090909</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>124.5029194667842</v>
+        <v>120.9805814591333</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>123.1174270458522</v>
+        <v>120.1351219493213</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>7.135492045526002</v>
+        <v>6.962647299251714</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-1.00525974025974</v>
+        <v>-0.980909090909091</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>476.7250667830574</v>
+        <v>465.2356919906408</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>119.84997606546</v>
+        <v>116.9615160497737</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.0139282594202372</v>
+        <v>-0.01426288111263989</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.225405483584371</v>
+        <v>4.235448666294758</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.352311236959702</v>
+        <v>3.360207879037847</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7761116655888158</v>
+        <v>0.777214118082028</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>14014369031.58549</v>
+        <v>13243498224.01919</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>762.6</v>
+        <v>759.59</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1162668429187845</v>
+        <v>0.1118609116347751</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.02151737942184073</v>
+        <v>-0.0253794731642224</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>812350671148</v>
+        <v>809144304087</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9950494992563612</v>
+        <v>0.9953050681130762</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1159911935350224</v>
+        <v>0.1148931228142449</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>29967795305.13551</v>
+        <v>29752244927.56256</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -4899,55 +4899,55 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>430.26</v>
+        <v>431.545</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3462032468313698</v>
+        <v>0.3502237720305015</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1017536534446765</v>
+        <v>-0.09907098121085589</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>257.98</v>
+        <v>262.81</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2231534884800</v>
+        <v>2238199511600</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.10942390170396</v>
+        <v>28.51512692708937</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6553652826933801</v>
+        <v>0.6568678259280953</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.16195998101111</v>
+        <v>14.36635940341746</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.775283174489369</v>
+        <v>9.916369735770658</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5280482367921029</v>
+        <v>0.535669551549927</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.63278794946157</v>
+        <v>18.9112426634564</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.67738056954049</v>
+        <v>13.88177999194684</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01778563079232014</v>
+        <v>0.01753258319974648</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.89123126294021</v>
+        <v>42.41075297271571</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.86519100973364</v>
+        <v>42.38729125771043</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2789011295495747</v>
+        <v>0.2780706531184465</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.181320079760245</v>
+        <v>2.181299131737951</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3622360240570155</v>
+        <v>0.3376196867388273</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4090305043.943522</v>
+        <v>3987349271.78236</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.24</v>
+        <v>27.945</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.009470369228840481</v>
+        <v>-0.01981761572591878</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.05866666666666676</v>
+        <v>-0.06850000000000001</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>70801540464</v>
+        <v>70061934372</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.23622047244094</v>
+        <v>-22.00393700787401</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-84.28137203100643</v>
+        <v>-84.18468056003628</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.960446918565693</v>
+        <v>1.939967724546587</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.159408002923442</v>
+        <v>2.13685044765211</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1654788500274675</v>
+        <v>0.1637502288958067</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.43893230809917</v>
+        <v>16.31668336727273</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.753856859033643</v>
+        <v>2.733377665014537</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03079029051788005</v>
+        <v>0.03111532702515889</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02072773416995544</v>
+        <v>0.02080140915356021</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2312026372878777</v>
+        <v>0.2301265938031586</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.1566866355788266</v>
+        <v>0.1595246601947214</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>512930202.3334476</v>
+        <v>500518907.9641965</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>311.481</v>
+        <v>310.065</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1643254076167608</v>
+        <v>-0.1681244040974922</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1961573201889081</v>
+        <v>-0.1998116080414979</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>210346234110</v>
+        <v>209389996799</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.88908429351122</v>
+        <v>18.80321406913281</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.0186438391019</v>
+        <v>15.94015843164978</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.501947523104921</v>
+        <v>2.490573630047697</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.160563535589265</v>
+        <v>6.132557467911319</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.171288196366201</v>
+        <v>1.165963492496447</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.06617999150623</v>
+        <v>9.027503510718331</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.666161955800316</v>
+        <v>2.654788062743092</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07155821003255326</v>
+        <v>0.07188500038255832</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1791937247148543</v>
+        <v>0.1796127466210324</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.006357550646380439</v>
+        <v>0.006590642898466115</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01136505918499042</v>
+        <v>0.01141696095979875</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9595618726755274</v>
+        <v>0.9625112973030167</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2344650763840535</v>
+        <v>0.2344689035074583</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>809555341.3908346</v>
+        <v>792471917.9137064</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>150.58</v>
+        <v>145.53</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2305963168242509</v>
+        <v>-0.2563998006868988</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5430045523520486</v>
+        <v>-0.5583308042488619</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>329.5</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>433741172600</v>
+        <v>419194799100</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>23.23765432098766</v>
+        <v>22.45833333333333</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.7484447061975</v>
+        <v>16.1725760427441</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.042899154325202</v>
+        <v>5.840238503977598</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.688735997124543</v>
+        <v>6.464415922841909</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.5057607116920845</v>
+        <v>0.4887990196078434</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>14.66869492576882</v>
+        <v>14.28305405885472</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.708641662370955</v>
+        <v>7.505981012023351</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.06621460404102758</v>
+        <v>-0.06851230039509333</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3874514755623204</v>
+        <v>0.3886676602401486</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4294717829481378</v>
+        <v>0.4310425747096076</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01328197635808208</v>
+        <v>0.01374287088572803</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.082813057538501</v>
+        <v>2.084383119342286</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5644318004989367</v>
+        <v>0.5630369937724207</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4173676568.913514</v>
+        <v>4128313146.163589</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>110.24</v>
+        <v>108.61</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4497632650276444</v>
+        <v>0.4283271790153527</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1544066886553656</v>
+        <v>-0.1669095650839918</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>434503757470</v>
+        <v>428079218966</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>32.80952380952381</v>
+        <v>32.32440476190476</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>21.24942102567937</v>
+        <v>20.93001124173748</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.861488471693645</v>
+        <v>6.760035040915911</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.666177190016905</v>
+        <v>8.538039773292235</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.049904761904762</v>
+        <v>1.034380952380952</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>22.81925957690194</v>
+        <v>22.49833752764873</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>7.213876943861035</v>
+        <v>7.112423513083301</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.03128856716719799</v>
+        <v>0.03175814054426168</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5440196591650359</v>
+        <v>0.544404558056099</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1662824832486469</v>
+        <v>0.166508857283745</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01505805515239477</v>
+        <v>0.01528404382653531</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.7104760944116318</v>
+        <v>0.7115021341152543</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3352034490599405</v>
+        <v>0.3353961628243654</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>2004914121.130584</v>
+        <v>1975705326.379649</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>86.88500000000001</v>
+        <v>86.25</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.08734240771838298</v>
+        <v>-0.09401257599943069</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1112418166939444</v>
+        <v>-0.1177373158756138</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>262740240000</v>
+        <v>260820000000</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>12.3944365192582</v>
+        <v>12.30385164051355</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>11.170513797791</v>
+        <v>11.08621319741697</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>2.035089578250261</v>
+        <v>2.020216103171837</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.47042700441201</v>
+        <v>1.45968037210722</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6588033825551672</v>
+        <v>0.653988510621893</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.65012344933748</v>
+        <v>15.59216443813951</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>4.016143758955889</v>
+        <v>4.001270283877464</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.07296179679214726</v>
+        <v>0.07349896480331262</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1095672718034899</v>
+        <v>0.109833576300002</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2903031514796548</v>
+        <v>-0.2902196875898506</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.02129251309201818</v>
+        <v>0.02144927536231884</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.7275824742256217</v>
+        <v>0.7295619626306802</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.226931730102077</v>
+        <v>0.2240177252206077</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1098841160.247248</v>
+        <v>1069867249.031316</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17 17:39 ET</t>
+          <t>2026-09-18 11:30 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-19)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -711,7 +711,7 @@
         <v>344.57</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>240.21</v>
+        <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
         <v>4936860972280</v>
@@ -720,7 +720,7 @@
         <v>38.37100456621005</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.08910982995525</v>
+        <v>35.08143766439387</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.57544502365993</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09353029336335772</v>
+        <v>0.09376944392318731</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1195887273062486</v>
+        <v>0.119860700088394</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003153541784428644</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3096765658979816</v>
+        <v>0.3096765527226455</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.291748504721329</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13594114828.82618</v>
+        <v>13596266632.27844</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.43222222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.02431740043097</v>
+        <v>24.01226807110472</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.04929824101447</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.141852305936073</v>
+        <v>0.1424252861491628</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.227381012594984</v>
+        <v>0.2280099482211277</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007371703997731784</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5574561254179546</v>
+        <v>0.5574561004202877</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4338476357762108</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>11015710913.17164</v>
+        <v>11018804543.62</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.10079443892751</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.98497250522871</v>
+        <v>21.0039634442356</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.374399849939218</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1850933121467472</v>
+        <v>-0.1858301179999097</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2859635067242161</v>
+        <v>0.2866631499931194</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002460376494821765</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7637474871723581</v>
+        <v>0.7637474801987068</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.3622167366566593</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8153408895.182483</v>
+        <v>8154185526.476135</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.13571428571429</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.59413549721904</v>
+        <v>22.60602312396835</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.51844038907797</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1088079343335506</v>
+        <v>-0.1092765775168516</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.179997197688706</v>
+        <v>0.1804255006133832</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8378168744020118</v>
+        <v>0.8378168738742139</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4627066709514093</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8563813948.280845</v>
+        <v>8564928276.458333</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>27.95849056603773</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.55785676528892</v>
+        <v>16.5361144646673</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>17.76948027686001</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6885331817006977</v>
+        <v>0.6907533281640386</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9437347712197781</v>
+        <v>0.9462540992020205</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1292,13 +1292,13 @@
         <v>0.002339497008143249</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.328091171552411</v>
+        <v>1.328091165640004</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.4121028150628047</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27017728029.57898</v>
+        <v>27024314319.52759</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -1337,10 +1337,10 @@
         <v>0.02358516549385681</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.1581310065756196</v>
+        <v>-0.1526987642065341</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>790.8</v>
+        <v>785.73</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>520.26</v>
@@ -1352,7 +1352,7 @@
         <v>24.73987365291713</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>20.13626964922009</v>
+        <v>20.13216724768483</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>7.430466790412184</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.228622484893837</v>
+        <v>0.2288728455582536</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2736216805247405</v>
+        <v>0.2742358205935815</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003154337213668795</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.769151071197354</v>
+        <v>0.7691510145943935</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.4138640308670974</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10585494580.24203</v>
+        <v>10588895009.32536</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>308.7033898305085</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>172.998652063492</v>
+        <v>170.5690820590555</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.88453497150137</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7844265614116559</v>
+        <v>0.8098437659623872</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1232203940178107</v>
+        <v>0.1235964007642594</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.53428605529164</v>
+        <v>1.534286015864648</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.5669001191480243</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13320249859.17986</v>
+        <v>13320828659.90774</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>44.36848635235732</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.52442546533809</v>
+        <v>19.50232187666616</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>19.0940719137188</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.272460535708215</v>
+        <v>1.27503610251878</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.857683211380821</v>
+        <v>0.8597720066537917</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1670,13 +1670,13 @@
         <v>0.007102709655770252</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.603588744680662</v>
+        <v>1.60358876268177</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.3932084614129385</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9006536579.43968</v>
+        <v>9007092889.453226</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -1796,13 +1796,13 @@
         <v>0.006187800873440485</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1835038483254343</v>
+        <v>-0.1835038416372886</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.1763090659402758</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1789294524.128361</v>
+        <v>1789685237.411296</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>22.22600619195047</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.13521646381585</v>
+        <v>19.13220924751302</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.179957226394026</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1615236354383138</v>
+        <v>0.1617062046736504</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1444115006001652</v>
+        <v>0.1447396720852696</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.08771628690465143</v>
+        <v>0.08771620800657744</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3530217611262856</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2357773889.265933</v>
+        <v>2359371527.876307</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.80000643688118</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.98015356263096</v>
+        <v>22.98012671355498</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.854809215804017</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4429973497785569</v>
+        <v>-0.4429966989985737</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05954181252370994</v>
+        <v>0.05958716313017343</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2054,7 +2054,7 @@
         <v>0.14899060627112</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2282909512.691259</v>
+        <v>2283300251.387838</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.03310404127257</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.96158194043373</v>
+        <v>13.96097067428319</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.147985141768554</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07674790044641289</v>
+        <v>0.07679504470017307</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2892465869116644</v>
+        <v>-0.2891944321370867</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.1645804732340038</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2272143514.789128</v>
+        <v>2272708907.889506</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.29056924384027</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.59225228739476</v>
+        <v>24.58412163495041</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.45618632752652</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2723750910720313</v>
+        <v>0.2727959008856973</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1387483256465651</v>
+        <v>0.1390543918079188</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2306,7 +2306,7 @@
         <v>0.1741592411990704</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2431162237.331487</v>
+        <v>2431231782.761434</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.04008786381109</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.4674662964347</v>
+        <v>25.4576263156245</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.13037165122709</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2188133480776031</v>
+        <v>0.2192844485567917</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1579228907806498</v>
+        <v>0.1582898298366417</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.1892630957122217</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1553689433.673885</v>
+        <v>1553690111.961873</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>24.23638351231432</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.32819433551714</v>
+        <v>17.32227469374443</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.760403408507339</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.398667572802877</v>
+        <v>0.3991455476148742</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01056282027615407</v>
+        <v>0.01064077798116125</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.2079717007585567</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1819232989.747476</v>
+        <v>1819773200.508728</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.001287001287</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.77528958805518</v>
+        <v>14.77859061855424</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.873076449343599</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4213790447982231</v>
+        <v>0.4210615574478587</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08167006657796794</v>
+        <v>0.08150862838000572</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.250161637469347</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2383481130.017454</v>
+        <v>2383692668.998769</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>173.33</v>
+        <v>174.12</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>650648473336</v>
@@ -2738,7 +2738,7 @@
         <v>31.21271676300578</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.77779645097476</v>
+        <v>21.77200145271355</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.644083706930531</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4332357653020824</v>
+        <v>0.4336172460210626</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09000526221088045</v>
+        <v>0.09021663906391786</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2810,7 +2810,7 @@
         <v>0.2038433219200969</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1729617379.845727</v>
+        <v>1732490820.314128</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>38.53068592057762</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.39007102779449</v>
+        <v>34.37980093004954</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.154280656664492</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1204014638247368</v>
+        <v>0.1207361554819246</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05127881962617709</v>
+        <v>0.05140285797353572</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2936,7 +2936,7 @@
         <v>0.3021983656671209</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2766554545.643186</v>
+        <v>2771984633.79331</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.67925925925926</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.7066409156962</v>
+        <v>20.70329183862584</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.997022587048442</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.0469713242009131</v>
+        <v>0.04714068797564686</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02559428074762593</v>
+        <v>0.02567408620740341</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.1484968291390396</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1299735702.618421</v>
+        <v>1300175287.388255</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -3101,10 +3101,10 @@
         <v>-0.1325545264974853</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2833389077356777</v>
+        <v>-0.276947551099113</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>418.58</v>
+        <v>414.88</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>289.1</v>
@@ -3188,7 +3188,7 @@
         <v>0.2382806161863175</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1284599331.473999</v>
+        <v>1284660327.409566</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>142.0862944162436</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>41.1102110722379</v>
+        <v>41.0421177227628</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>22.10004822660695</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.456228774076907</v>
+        <v>2.461963034559488</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9038976624956678</v>
+        <v>0.9064313743551562</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.547107438065864</v>
+        <v>2.54710742323953</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.6568543593127123</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>9638713874.855129</v>
+        <v>9640699873.652445</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3359,7 @@
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>925.87</v>
+        <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
         <v>647471391441</v>
@@ -3368,7 +3368,7 @@
         <v>52.46734397677794</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>34.42173508469492</v>
+        <v>34.39361158387129</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>15.77565395190715</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5242504146778677</v>
+        <v>0.5254967873563541</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2772342948012847</v>
+        <v>0.2780463161960551</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004631172912995857</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.684420144898762</v>
+        <v>1.684420158995621</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.4356624008892414</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2144072722.60616</v>
+        <v>2144411058.503011</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>74.23220973782769</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>77.13593874521685</v>
+        <v>76.72791762618546</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.666592201712857</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.03764430762916227</v>
+        <v>-0.03252672515520005</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1546467220498906</v>
+        <v>0.1550713241859412</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,7 +3568,7 @@
         <v>0.3443784423467804</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1137354153.473872</v>
+        <v>1137444493.032481</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>14.35100548446069</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.00157726832984</v>
+        <v>13.00005435197084</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.356313913360523</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1037895778551334</v>
+        <v>0.1039188834072107</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3821570738151003</v>
+        <v>-0.3821142682736697</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.3098876404351355</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1990542610.318058</v>
+        <v>1991869448.718058</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.04803493449782</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.78415160556265</v>
+        <v>17.78099803928185</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.129902306901892</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1272977974516962</v>
+        <v>0.127497730454029</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04632303781771174</v>
+        <v>0.04643055996507583</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.3397939648974554</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1262584088.404345</v>
+        <v>1263032973.435313</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>38.54867848778856</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.32672994885804</v>
+        <v>26.29556379699387</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.62056007747365</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4642410418108409</v>
+        <v>0.4659764964687874</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.230024722751039</v>
+        <v>0.2311671946536107</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3946,7 +3946,7 @@
         <v>0.3124183205632644</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2888317711.147994</v>
+        <v>2888595298.273926</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>16.27974276527331</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.03999806953615</v>
+        <v>15.03757425369097</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.524565479850469</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08242984407347032</v>
+        <v>0.08260431440778748</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3270721467871623</v>
+        <v>-0.3269728206241095</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.2515769412288019</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>930258124.2022237</v>
+        <v>930398066.4674886</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -4192,13 +4192,13 @@
         <v>0.0005217562512305573</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.887672519638909</v>
+        <v>2.887672514345583</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>0.7770948884887525</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25714651977.77043</v>
+        <v>25726528135.60771</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>84.14285714285715</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.53504132020887</v>
+        <v>28.51947246172641</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.507010938093945</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.948755398621629</v>
+        <v>1.950365132306645</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2473194666323242</v>
+        <v>0.2478822889575949</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.6292376666408013</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2212118088.143447</v>
+        <v>2213456242.752838</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.4693446088795</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.45544883755093</v>
+        <v>9.456140418560089</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.46961416729465</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.856965992354253</v>
+        <v>2.85668391062585</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05063977200538161</v>
+        <v>-0.05074658054582049</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.2050434135637993</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>973988281.7226467</v>
+        <v>974085769.3921089</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>8.113760780990328</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003887353646552389</v>
+        <v>0.003884332858249072</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.968315520817014</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2086.219614862221</v>
+        <v>2087.842814734405</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2702.288207161095</v>
+        <v>2705.457791183441</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4574,7 +4574,7 @@
         <v>0.8651532945538819</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3530852861.059164</v>
+        <v>3534679079.809164</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
         <v>671.83</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>313.43</v>
+        <v>313.6</v>
       </c>
       <c r="K33" s="5" t="n">
         <v>72221348604</v>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.826773975279009</v>
+        <v>1.826773971888191</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.3952270456297697</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3788902302.625822</v>
+        <v>3790890765.425822</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-99.16233766233766</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>122.302029621503</v>
+        <v>121.7942751010598</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>121.447337279095</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.235448666294758</v>
+        <v>4.245491849005145</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4782,7 +4782,7 @@
         <v>0.7751488656668594</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>14746294264.62609</v>
+        <v>14747168834.83454</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -4866,7 +4866,7 @@
         <v>0.1144605303882855</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>30644354666.64014</v>
+        <v>30651027451.90654</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
         <v>479</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>262.81</v>
+        <v>265.45</v>
       </c>
       <c r="K36" s="5" t="n">
         <v>2254407261600</v>
@@ -4920,7 +4920,7 @@
         <v>28.51512692708937</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6616244838803953</v>
+        <v>0.6609707103451463</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.36635940341746</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.0986573529588</v>
+        <v>42.1412867178325</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.07536431271689</v>
+        <v>42.12152275071068</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4990,7 +4990,7 @@
         <v>0.3384223806071351</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4128968528.000573</v>
+        <v>4129131543.744608</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
         <v>-21.88976377952756</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-83.74786615025975</v>
+        <v>-84.54231820018896</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.929901711643361</v>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02080140915356021</v>
+        <v>0.02087508413716432</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2271828744710579</v>
+        <v>0.2271828399419369</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.1624865549921377</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>527905689.5206326</v>
+        <v>528269668.4239769</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
         <v>18.89387507580352</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.01701501609278</v>
+        <v>16.01132747416185</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.50258208461694</v>
@@ -5200,10 +5200,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1796127466210324</v>
+        <v>0.1800317685272104</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.006590642898466115</v>
+        <v>0.006823735150551569</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5248,7 +5248,7 @@
         <v>0.2346867436799534</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>837896450.1384989</v>
+        <v>838049893.4372965</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
         <v>22.77777777777778</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.40261268404473</v>
+        <v>16.38825996939477</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>5.92330930520919</v>
@@ -5326,10 +5326,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3886676602401486</v>
+        <v>0.3898838449179773</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4310425747096076</v>
+        <v>0.4326133664710774</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5374,7 +5374,7 @@
         <v>0.5583366535191318</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4260293875.820374</v>
+        <v>4260749803.749593</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
         <v>32.59226190476191</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>21.10344840330238</v>
+        <v>21.09819027971051</v>
       </c>
       <c r="N40" s="6" t="n">
         <v>6.816052272625346</v>
@@ -5452,10 +5452,10 @@
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.544404558056099</v>
+        <v>0.5447894569471623</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.166508857283745</v>
+        <v>0.1667352313188437</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5494,13 +5494,13 @@
         <v>0.01515843301981554</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.7094121871053773</v>
+        <v>0.7094121578490867</v>
       </c>
       <c r="AJ40" s="4" t="n">
         <v>0.3338654993278114</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>2099773678.943522</v>
+        <v>2099847167.455622</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
         <v>12.28530670470756</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>11.0695035427426</v>
+        <v>11.06684805325145</v>
       </c>
       <c r="N41" s="6" t="n">
         <v>2.017171139769955</v>
@@ -5578,10 +5578,10 @@
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.109833576300002</v>
+        <v>0.1100998807965139</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2902196875898506</v>
+        <v>-0.2901362237000468</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5626,7 +5626,7 @@
         <v>0.2243370392460025</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1132664655.30247</v>
+        <v>1132677059.453532</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18 18:46 ET</t>
+          <t>2026-09-19 11:04 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-20)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>38.37100456621005</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.08143766439387</v>
+        <v>35.04041588562982</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.57544502365993</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09376944392318731</v>
+        <v>0.09504991868393065</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.119860700088394</v>
+        <v>0.1201326728705394</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.43222222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.01226807110472</v>
+        <v>23.99611740230289</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.04929824101447</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1424252861491628</v>
+        <v>0.1431941993911721</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2280099482211277</v>
+        <v>0.228638883847271</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.10079443892751</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>21.0039634442356</v>
+        <v>20.98435250321343</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.374399849939218</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1858301179999097</v>
+        <v>-0.1850692349783587</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2866631499931194</v>
+        <v>0.2865650075664814</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.13571428571429</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.60602312396835</v>
+        <v>22.60671328362403</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.51844038907797</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1092765775168516</v>
+        <v>-0.1093037703848662</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1804255006133832</v>
+        <v>0.1808538035380607</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>27.95849056603773</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.5361144646673</v>
+        <v>16.50246367594439</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>17.76948027686001</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6907533281640386</v>
+        <v>0.6942010062893076</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9462540992020205</v>
+        <v>0.9491140480986955</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>24.73987365291713</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>20.13216724768483</v>
+        <v>20.12807171920323</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>7.430466790412184</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2288728455582536</v>
+        <v>0.2291228885732759</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2742358205935815</v>
+        <v>0.2748499616223978</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>308.7033898305085</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>170.5690820590555</v>
+        <v>170.4397970293183</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.88453497150137</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8098437659623872</v>
+        <v>0.8112166008822852</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1235964007642594</v>
+        <v>0.1239724075107083</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>44.36848635235732</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.50232187666616</v>
+        <v>19.48032505772298</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>19.0940719137188</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.27503610251878</v>
+        <v>1.277605030762432</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8597720066537917</v>
+        <v>0.8596106943360324</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>44.96785534907082</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.49675180011946</v>
+        <v>39.5141661094671</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.352414049293736</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1385203415369163</v>
+        <v>0.1380185836263184</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1141243314792548</v>
+        <v>0.114432509886337</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>22.22600619195047</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.13220924751302</v>
+        <v>19.13709820116455</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.179957226394026</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1617062046736504</v>
+        <v>0.1614094236396795</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1447396720852696</v>
+        <v>0.1450676707331524</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.80000643688118</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.98012671355498</v>
+        <v>22.98009986454174</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.854809215804017</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4429966989985737</v>
+        <v>-0.4429960482185905</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05958716313017343</v>
+        <v>0.05963251373663692</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.03310404127257</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.96097067428319</v>
+        <v>13.96035946165523</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.147985141768554</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07679504470017307</v>
+        <v>0.07684218895393347</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2891944321370867</v>
+        <v>-0.2891422773625089</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.29056924384027</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.58412163495041</v>
+        <v>24.57599635701665</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.45618632752652</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2727959008856973</v>
+        <v>0.2732167106993633</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1390543918079188</v>
+        <v>0.1393604579692722</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.04008786381109</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.4576263156245</v>
+        <v>25.44779393571381</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.13037165122709</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2192844485567917</v>
+        <v>0.2197555490359804</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1582898298366417</v>
+        <v>0.1586567688926339</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>24.23638351231432</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.32227469374443</v>
+        <v>17.31678331622206</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.760403408507339</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3991455476148742</v>
+        <v>0.399589234890414</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01064077798116125</v>
+        <v>0.01071873568616866</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.001287001287</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.77859061855424</v>
+        <v>14.78189312438647</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.873076449343599</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4210615574478587</v>
+        <v>0.4207440700974949</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08150862838000572</v>
+        <v>0.08134719018204395</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.21271676300578</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.77200145271355</v>
+        <v>21.78939291273559</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.644083706930531</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4336172460210626</v>
+        <v>0.4324729875682951</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09021663906391786</v>
+        <v>0.09040105275409904</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>38.53068592057762</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.37980093004954</v>
+        <v>34.36953696450584</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.154280656664492</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1207361554819246</v>
+        <v>0.1210708471391129</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05140285797353572</v>
+        <v>0.05152689632089458</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,7 +2927,7 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009158624566663543</v>
+        <v>0.009163309285111965</v>
       </c>
       <c r="AI19" s="6" t="n">
         <v>-0.05882571029802023</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.67925925925926</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.70329183862584</v>
+        <v>20.69994384473488</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.997022587048442</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04714068797564686</v>
+        <v>0.04731005175038039</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02567408620740341</v>
+        <v>0.02575389166718089</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>142.0862944162436</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>41.0421177227628</v>
+        <v>40.9741537717905</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>22.10004822660695</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.461963034559488</v>
+        <v>2.467705402962242</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9064313743551562</v>
+        <v>0.9135852965836171</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>52.46734397677794</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>34.39361158387129</v>
+        <v>34.26854356414675</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>15.77565395190715</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5254967873563541</v>
+        <v>0.5310643091255145</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2780463161960551</v>
+        <v>0.2810928551907987</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>74.23220973782769</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>76.72791762618546</v>
+        <v>76.3241903614753</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.666592201712857</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.03252672515520005</v>
+        <v>-0.02740914268123762</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1550713241859412</v>
+        <v>0.1554959263219917</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>14.35100548446069</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.00005435197084</v>
+        <v>13.01185074089099</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.356313913360523</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1039188834072107</v>
+        <v>0.1029180836943728</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3821142682736697</v>
+        <v>-0.3820415698249855</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.04803493449782</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.78099803928185</v>
+        <v>17.77784559121205</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.129902306901892</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.127497730454029</v>
+        <v>0.1276976634563622</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04643055996507583</v>
+        <v>0.04653808211244037</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>38.54867848778856</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.29556379699387</v>
+        <v>26.27867849323994</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.62056007747365</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4659764964687874</v>
+        <v>0.4669184562574189</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2311671946536107</v>
+        <v>0.2316358049677185</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>16.27974276527331</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.03757425369097</v>
+        <v>15.03565888435984</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.524565479850469</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08260431440778748</v>
+        <v>0.08274222569704426</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3269728206241095</v>
+        <v>-0.3268734944610564</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>22.66904708770364</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.498722647210335</v>
+        <v>6.474647909946941</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.70835857500498</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.488231198393215</v>
+        <v>2.501201517518411</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.775779220960631</v>
+        <v>1.784318972372998</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>84.14285714285715</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.51947246172641</v>
+        <v>28.50428043394301</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.507010938093945</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.950365132306645</v>
+        <v>1.951937598910916</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2478822889575949</v>
+        <v>0.2489068021146772</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.4693446088795</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.456140418560089</v>
+        <v>9.456832100742504</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.46961416729465</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.85668391062585</v>
+        <v>2.856401828897448</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05074658054582049</v>
+        <v>-0.05085331782783276</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>8.113760780990328</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003884332858249072</v>
+        <v>0.003878990629858609</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.968315520817014</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2087.842814734405</v>
+        <v>2090.719613482562</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2705.457791183441</v>
+        <v>2709.926668716981</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-99.16233766233766</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>121.7942751010598</v>
+        <v>134.8342969109074</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>121.447337279095</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.245491849005145</v>
+        <v>4.295094526746421</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
         <v>28.51512692708937</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6609707103451463</v>
+        <v>0.6605140703029319</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.36635940341746</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.1412867178325</v>
+        <v>42.17111203098439</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.12152275071068</v>
+        <v>42.15420560240253</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
         <v>-21.88976377952756</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-84.54231820018896</v>
+        <v>-87.36095804432952</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.929901711643361</v>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02087508413716432</v>
+        <v>0.02094875164040277</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
         <v>18.89387507580352</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.01132747416185</v>
+        <v>16.00561869427619</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.50258208461694</v>
@@ -5200,10 +5200,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1800317685272104</v>
+        <v>0.1804526545768712</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.006823735150551569</v>
+        <v>0.007056827402637245</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
         <v>22.77777777777778</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.38825996939477</v>
+        <v>16.36102450346003</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>5.92330930520919</v>
@@ -5326,10 +5326,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3898838449179773</v>
+        <v>0.3921975224082528</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4326133664710774</v>
+        <v>0.43520912853463</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
         <v>32.59226190476191</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>21.09819027971051</v>
+        <v>21.08743235214967</v>
       </c>
       <c r="N40" s="6" t="n">
         <v>6.816052272625346</v>
@@ -5452,10 +5452,10 @@
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5447894569471623</v>
+        <v>0.5455775440313109</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1667352313188437</v>
+        <v>0.1669616053539418</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
         <v>12.28530670470756</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>11.06684805325145</v>
+        <v>11.06339943310153</v>
       </c>
       <c r="N41" s="6" t="n">
         <v>2.017171139769955</v>
@@ -5578,10 +5578,10 @@
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1100998807965139</v>
+        <v>0.1104459148379029</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2901362237000468</v>
+        <v>-0.2900527598102426</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19 11:04 ET</t>
+          <t>2026-09-20 11:09 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-21)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -446,7 +446,7 @@
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -454,7 +454,7 @@
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>336.13</v>
+        <v>338.73001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2402862916048456</v>
+        <v>0.2498800700864909</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.02449429724003827</v>
+        <v>-0.01694863162782601</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4936860972280</v>
+        <v>4975048259240</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.37100456621005</v>
+        <v>38.66780936073059</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.04041588562982</v>
+        <v>35.30365975903797</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.57544502365993</v>
+        <v>10.65724752045208</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.93187376255581</v>
+        <v>46.28716288016323</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.172447361745306</v>
+        <v>1.181516397133433</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.56699056467599</v>
+        <v>29.79364017924338</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.67133361526746</v>
+        <v>10.7531361120596</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02768621615383984</v>
+        <v>0.02747370334471489</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09504991868393065</v>
+        <v>0.09529180896978762</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1201326728705394</v>
+        <v>0.1204046456526846</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003153541784428644</v>
+        <v>0.003129335956976472</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3096765527226455</v>
+        <v>0.3109023404336923</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.291748504721329</v>
+        <v>0.2918276013444279</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13596266632.27844</v>
+        <v>13426178369.28659</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>493.78</v>
+        <v>497.21</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.04406478084115051</v>
+        <v>0.05131728640695932</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.1082496568662863</v>
+        <v>-0.1020551903489129</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3666588079000</v>
+        <v>3692057715500</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.43222222222222</v>
+        <v>27.62277777777777</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>23.99611740230289</v>
+        <v>24.15071427882669</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.04929824101447</v>
+        <v>11.12605123418284</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.292042080802554</v>
+        <v>8.349642032880713</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8713390306780081</v>
+        <v>0.8773917117813853</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.18850986656644</v>
+        <v>18.31213842708379</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.37437546219703</v>
+        <v>11.45168787951386</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01826957338994829</v>
+        <v>0.01814262863331959</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1431941993911721</v>
+        <v>0.1437664931506848</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.228638883847271</v>
+        <v>0.2292678194734146</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007371703997731784</v>
+        <v>0.00732085034492468</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5574561004202877</v>
+        <v>0.5552190936757947</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4338476357762108</v>
+        <v>0.4296743117557364</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>11018804543.62</v>
+        <v>10717377452.03641</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>349.54</v>
+        <v>355.99</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.1091226614930907</v>
+        <v>0.1295891064396788</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1445632754949707</v>
+        <v>-0.1287780524216245</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4230171978908</v>
+        <v>4308230596703</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>17.10079443892751</v>
+        <v>17.48108738828202</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.98435250321343</v>
+        <v>21.39083141810268</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.374399849939218</v>
+        <v>9.582870759293151</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.534046199725207</v>
+        <v>6.679352413970772</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1520783595506874</v>
+        <v>0.1554603268676488</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>13.06519121300237</v>
+        <v>13.35184064207868</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.501893312100496</v>
+        <v>9.710364221454428</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01274557181886761</v>
+        <v>0.01246829781465144</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1850692349783587</v>
+        <v>-0.1827766276775904</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2865650075664814</v>
+        <v>0.2920481943604654</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002460376494821765</v>
+        <v>0.002415798196578555</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7637474801987068</v>
+        <v>0.7624166777559729</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3622167366566593</v>
+        <v>0.3629042708997856</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8154185526.476135</v>
+        <v>8089666871.93655</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>253.71</v>
+        <v>257.575</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1201324503311259</v>
+        <v>0.1371964679911699</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.116608635097493</v>
+        <v>-0.1031511142061281</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2729183841000</v>
+        <v>2770760032500</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.13571428571429</v>
+        <v>20.44319841269841</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.60671328362403</v>
+        <v>22.96315303847702</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.51844038907797</v>
+        <v>3.57216903043781</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.947073637649106</v>
+        <v>5.022618343787389</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.22793219724438</v>
+        <v>0.231412855128515</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.31589286881341</v>
+        <v>11.47997446241491</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.705397639490512</v>
+        <v>3.759126280850351</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004259515180091527</v>
+        <v>-0.004195448233223147</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1093037703848662</v>
+        <v>-0.1097390511466859</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1808538035380607</v>
+        <v>0.1813247578209447</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8378168738742139</v>
+        <v>0.8364343821079248</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4627066709514093</v>
+        <v>0.4630905271732186</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8564928276.458333</v>
+        <v>8437203402.756631</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>222.27</v>
+        <v>227.27</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1769658078706424</v>
+        <v>0.2034418461994911</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.06032806290690784</v>
+        <v>-0.03918998900820148</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5383601670000</v>
+        <v>5504706670000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>27.95849056603773</v>
+        <v>28.58742138364779</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.50246367594439</v>
+        <v>16.85156152217641</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.76948027686001</v>
+        <v>18.16920764170592</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>23.48072922125563</v>
+        <v>24.00893206512245</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2244286997817995</v>
+        <v>0.2294772600864245</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.10989001442223</v>
+        <v>23.62817030218216</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>17.82366733890266</v>
+        <v>18.22339470374857</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02359126989423049</v>
+        <v>0.02307225572838743</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6942010062893076</v>
+        <v>0.6964256603773582</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9491140480986955</v>
+        <v>0.9516327173898933</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002339497008143249</v>
+        <v>0.002288027456329476</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.328091165640004</v>
+        <v>1.316562868039854</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4121028150628047</v>
+        <v>0.4119391543254972</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27024314319.52759</v>
+        <v>26685025267.72803</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>665.75</v>
+        <v>737.5309999999999</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.02358516549385681</v>
+        <v>0.1339478643512575</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.1526987642065341</v>
+        <v>-0.06134295495908271</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>785.73</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1695989183978</v>
+        <v>1878850317459</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>24.73987365291713</v>
+        <v>27.40732069862505</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>20.12807171920323</v>
+        <v>22.29374016167409</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7.430466790412184</v>
+        <v>8.231617878180751</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>6.481110821871137</v>
+        <v>7.179902584401713</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.071674098848008</v>
+        <v>-5.61850074321813</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>16.74429527773834</v>
+        <v>18.45212863735617</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.85481223922225</v>
+        <v>8.655963326990818</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02416053143917428</v>
+        <v>0.02180908165979761</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2291228885732759</v>
+        <v>0.2293729315882977</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2748499616223978</v>
+        <v>0.2754641026512139</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003154337213668795</v>
+        <v>0.002847337942405133</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7691510145943935</v>
+        <v>0.8244058033176008</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4138640308670974</v>
+        <v>0.4774682281582845</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10588895009.32536</v>
+        <v>11033935205.32499</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>364.27</v>
+        <v>373.1022</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1684662407613742</v>
+        <v>-0.1483046230922074</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2697512178497685</v>
+        <v>-0.2520453862037167</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1438701629212</v>
+        <v>1473584821706</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>308.7033898305085</v>
+        <v>316.1883050847458</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>170.4397970293183</v>
+        <v>174.4401124928839</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.88453497150137</v>
+        <v>14.22118358318455</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.57551394229662</v>
+        <v>13.90466993713878</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.217597278586773</v>
+        <v>-8.416843614227735</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>119.1240962098437</v>
+        <v>122.024262970735</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.82781757411286</v>
+        <v>14.16446631420878</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.00400499998262735</v>
+        <v>0.0039101922489268</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8112166008822852</v>
+        <v>0.8125894358021826</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1239724075107083</v>
+        <v>0.1243484142571567</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.534286015864648</v>
+        <v>1.534176558605315</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5669001191480243</v>
+        <v>0.5692931213186111</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13320828659.90774</v>
+        <v>13184996020.47722</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>357.61</v>
+        <v>359.223</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.0287382918794552</v>
+        <v>0.03337841621826443</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2775555555555556</v>
+        <v>-0.2742969696969697</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1701358183800</v>
+        <v>1709032160340</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>44.36848635235732</v>
+        <v>44.5854094292804</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.48032505772298</v>
+        <v>19.54608832275813</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>19.0940719137188</v>
+        <v>19.18742521853115</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>17.09669234627345</v>
+        <v>17.18028021265924</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4414884038031592</v>
+        <v>0.4436468958062057</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>33.23196494269368</v>
+        <v>33.39112444122993</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.49185428039145</v>
+        <v>19.58520758520381</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02315973225108485</v>
+        <v>0.02304705233079414</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.277605030762432</v>
+        <v>1.28104000621793</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8596106943360324</v>
+        <v>0.8623942193149883</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007102709655770252</v>
+        <v>0.007237843901977323</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.60358876268177</v>
+        <v>1.586250399704904</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3932084614129385</v>
+        <v>0.3872302666399897</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9007092889.453226</v>
+        <v>8946248609.782087</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>895.3099999999999</v>
+        <v>897.3899</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.04775892334698639</v>
+        <v>0.05019297834991221</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.183483812129503</v>
+        <v>-0.1815869585043319</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>397051183490</v>
+        <v>397973575462</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>44.96785534907082</v>
+        <v>45.07081868407835</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.5141661094671</v>
+        <v>39.60596170439074</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.352414049293736</v>
+        <v>1.355510684873649</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.86095380733534</v>
+        <v>11.88811194843176</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.547241089366438</v>
+        <v>3.555363241730649</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>26.69918337871458</v>
+        <v>26.7620121243953</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.315920607826641</v>
+        <v>1.319017243406554</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02217850082348838</v>
+        <v>0.02212783450597016</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1380185836263184</v>
+        <v>0.1379806661551608</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.114432509886337</v>
+        <v>0.1143953782763263</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006187800873440485</v>
+        <v>0.006173459273388301</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1835038416372886</v>
+        <v>-0.1773280087527101</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1763090659402758</v>
+        <v>0.1764326601584382</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1789685237.411296</v>
+        <v>1770592802.520325</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>71.79000000000001</v>
+        <v>73.62</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2110121806191908</v>
+        <v>-0.1909000799162116</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.425036040365209</v>
+        <v>-0.4103796251802018</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>298929252528</v>
+        <v>306549262726</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>22.22600619195047</v>
+        <v>22.79256965944273</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.13709820116455</v>
+        <v>19.62186658715291</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.179957226394026</v>
+        <v>6.33749061160167</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.974447588840722</v>
+        <v>10.22870638655041</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6532277429585444</v>
+        <v>0.6698791814543534</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.940155858485387</v>
+        <v>10.18919990640924</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.287668446336717</v>
+        <v>6.44520183154436</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03677996685510115</v>
+        <v>0.03586571340028701</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1614094236396795</v>
+        <v>0.1615902879681073</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1450676707331524</v>
+        <v>0.1453958417687611</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.08771620800657744</v>
+        <v>0.1067428780225328</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3530217611262856</v>
+        <v>0.3578414218266984</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2359371527.876307</v>
+        <v>2342091763.981251</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>509.77</v>
+        <v>507.64499</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.02600381148791331</v>
+        <v>0.02172684666171731</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.0520139844534534</v>
+        <v>-0.0559657269312307</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1099499257123</v>
+        <v>1094915919538</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.80000643688118</v>
+        <v>12.77318609861637</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.98009986454174</v>
+        <v>22.8842790595741</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.854809215804017</v>
+        <v>2.848827425933291</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.461694506763071</v>
+        <v>1.458631762903955</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3526075807921941</v>
+        <v>0.3518687487737715</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.51309554852707</v>
+        <v>15.48302109417884</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.085544852828403</v>
+        <v>3.079563062957677</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02204955724121188</v>
+        <v>0.02209585552413306</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4429960482185905</v>
+        <v>-0.4418357657077925</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05963251373663692</v>
+        <v>0.06188401707386548</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.03918452948205382</v>
+        <v>0.03626418744575198</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.14899060627112</v>
+        <v>0.1494815903370572</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2283300251.387838</v>
+        <v>2251531071.274144</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>349.67</v>
+        <v>352.255</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.07432096656371323</v>
+        <v>0.08226308255469661</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.04592087312414728</v>
+        <v>-0.03886766712141887</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>936944261700</v>
+        <v>943870808134</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.03310404127257</v>
+        <v>15.14423903697335</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.96035946165523</v>
+        <v>14.06294831787748</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.147985141768554</v>
+        <v>3.17125724679051</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.603123158692786</v>
+        <v>2.622367227000678</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7871220426971945</v>
+        <v>0.7929409876463529</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.01936734328038</v>
+        <v>20.0937184213611</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.266120563579979</v>
+        <v>6.289392668601936</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1734724322929273</v>
+        <v>-0.1721994139445038</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07684218895393347</v>
+        <v>0.07688933320769409</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2891422773625089</v>
+        <v>-0.2890901225879311</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01715903566219578</v>
+        <v>0.01703311521483017</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7668452127602949</v>
+        <v>0.763789019754343</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1645804732340038</v>
+        <v>0.1642307875462587</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2272708907.889506</v>
+        <v>2246023087.747815</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>368.29</v>
+        <v>368.25</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.06294732256439617</v>
+        <v>0.06283187578902183</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.04481676478979169</v>
+        <v>-0.04492050730087915</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>687614817339</v>
+        <v>687540135451</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.29056924384027</v>
+        <v>31.28632115548004</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.57599635701665</v>
+        <v>24.56520812966425</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.45618632752652</v>
+        <v>15.45408795583079</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.03254502217295</v>
+        <v>20.02982535220877</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.110054833877388</v>
+        <v>2.109768367392569</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.02618108938758</v>
+        <v>24.02297288401265</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.71466052281514</v>
+        <v>15.7125621511194</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03055926002484675</v>
+        <v>0.03056340939208615</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2732167106993633</v>
+        <v>0.2736029342938711</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1393604579692722</v>
+        <v>0.1396355759563579</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007276874202394852</v>
+        <v>0.007277664630006789</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3055468132238942</v>
+        <v>0.3079912209734742</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1741592411990704</v>
+        <v>0.1731368413704722</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2431231782.761434</v>
+        <v>2393201495.369767</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>565.24</v>
+        <v>565.23</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.003746905863463379</v>
+        <v>0.003729147974675051</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05986061906425166</v>
+        <v>-0.05987725163415003</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>495735828640</v>
+        <v>495727058280</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.04008786381109</v>
+        <v>31.03953871499176</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.44779393571381</v>
+        <v>25.43751910952335</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.13037165122709</v>
+        <v>14.13012166234359</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>88.85077169844948</v>
+        <v>88.84919978613438</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.371861026123793</v>
+        <v>1.371836755707224</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.01898302767227</v>
+        <v>23.01858646590703</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.51095483966593</v>
+        <v>14.51070485078243</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03317896155523677</v>
+        <v>0.03317954855453891</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2197555490359804</v>
+        <v>0.2202266495151692</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1586567688926339</v>
+        <v>0.1590237079486261</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005962069209539311</v>
+        <v>0.005962174689949224</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2928800069420453</v>
+        <v>0.2950387562166457</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1892630957122217</v>
+        <v>0.1864926849625038</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1553690111.961873</v>
+        <v>1512409281.778219</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>376.9</v>
+        <v>377.315</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1203924103398708</v>
+        <v>0.121626060778425</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1835275767947663</v>
+        <v>-0.1826285689528183</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>342279625868</v>
+        <v>342656508012</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.23638351231432</v>
+        <v>24.26306989904187</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.31678331622206</v>
+        <v>17.32993387047288</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.760403408507339</v>
+        <v>0.7612406843638156</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.468569578554958</v>
+        <v>3.472388778276636</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7343687484605945</v>
+        <v>-0.735177352946164</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.02242075332842</v>
+        <v>15.03704956767457</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8598038026165832</v>
+        <v>0.8606410784730599</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06899914051299065</v>
+        <v>0.06892324951602238</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.399589234890414</v>
+        <v>0.4000670793315502</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01071873568616866</v>
+        <v>0.01079669339117584</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02403820642080128</v>
+        <v>0.0240117673561878</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4284111499557166</v>
+        <v>0.4297623421872889</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2079717007585567</v>
+        <v>0.2072665871450886</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1819773200.508728</v>
+        <v>1787935432.073832</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>163.18</v>
+        <v>158.325</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3304524905820678</v>
+        <v>0.2908683084410213</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.07499574854033209</v>
+        <v>-0.102516864123349</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>676292982800</v>
+        <v>656171616852</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.001287001287</v>
+        <v>20.37644787644788</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.78189312438647</v>
+        <v>14.34530170298521</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.873076449343599</v>
+        <v>1.817347855902066</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.625834706530958</v>
+        <v>2.547709767811705</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.056376018876021</v>
+        <v>1.995193854568856</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.858308148973199</v>
+        <v>9.578163826689872</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.961095061208663</v>
+        <v>1.90536646776713</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04517716548455662</v>
+        <v>0.04656251385358421</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4207440700974949</v>
+        <v>0.4204265827471307</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08134719018204395</v>
+        <v>0.08118575198408196</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02524819218041427</v>
+        <v>0.02602242223274909</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5335105066356072</v>
+        <v>-0.551854144028243</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.250161637469347</v>
+        <v>0.2603882970005258</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2383692668.998769</v>
+        <v>2318966523.51605</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>269.99</v>
+        <v>270.88</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.3020978637695941</v>
+        <v>0.3063901231079211</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.03942078485786449</v>
+        <v>-0.03625431387198919</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>174.12</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>650648473336</v>
+        <v>652793282926</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.21271676300578</v>
+        <v>31.31560693641618</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.78939291273559</v>
+        <v>21.85550363721279</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.644083706930531</v>
+        <v>6.665985386616835</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.753264043026444</v>
+        <v>7.778822045168351</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.864627167630064</v>
+        <v>-3.877366595679957</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.13703525838966</v>
+        <v>20.20061908354085</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.936274988369124</v>
+        <v>6.958176668055428</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02875285314062213</v>
+        <v>0.02865838311960805</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4324729875682951</v>
+        <v>0.43284764589437</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09040105275409904</v>
+        <v>0.09061244409666647</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01955627986221712</v>
+        <v>0.01949202598936799</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1659156819489056</v>
+        <v>-0.1582184663195926</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2038433219200969</v>
+        <v>0.1988117512032154</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1732490820.314128</v>
+        <v>1690795642.735026</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>106.73</v>
+        <v>107.7035</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.05347642800631869</v>
+        <v>-0.04484304753844781</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2103432968333826</v>
+        <v>-0.2031407221071322</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>849365878400</v>
+        <v>857113069280</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.53068592057762</v>
+        <v>38.88212996389892</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.36953696450584</v>
+        <v>34.6726751551757</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.154280656664492</v>
+        <v>1.164809020004349</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.641568639426698</v>
+        <v>8.720389655734033</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.317420413521504</v>
+        <v>9.402405973088291</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.27948547818577</v>
+        <v>21.460329822825</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.238845235920852</v>
+        <v>1.249373599260709</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01590480656633828</v>
+        <v>0.01576104773591652</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1210708471391129</v>
+        <v>0.1214055387963009</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05152689632089458</v>
+        <v>0.05165093466825343</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009163309285111965</v>
+        <v>0.009075842474942782</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.05882571029802023</v>
+        <v>-0.04943727187952437</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3021983656671209</v>
+        <v>0.3023135323099588</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2771984633.79331</v>
+        <v>2729666069.604243</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>146.335</v>
+        <v>146.67</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.03205449558556195</v>
+        <v>0.03441714468537493</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1250523168908819</v>
+        <v>-0.1230493273542602</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>347868869796</v>
+        <v>348665230437</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.67925925925926</v>
+        <v>21.72888888888889</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.69994384473488</v>
+        <v>20.74397698593049</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.997022587048442</v>
+        <v>4.006172792042007</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.527159093001417</v>
+        <v>6.542101507981807</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.68820740740763</v>
+        <v>20.73556825396847</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.54742024070763</v>
+        <v>17.58488898263856</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.285238415709165</v>
+        <v>4.29438862070273</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04574424842709216</v>
+        <v>0.04563976734948713</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04731005175038039</v>
+        <v>0.04747941552511414</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02575389166718089</v>
+        <v>0.02583369712695816</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.0293203949841118</v>
+        <v>0.02925342605849868</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.04268400994052118</v>
+        <v>-0.03592844684359042</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1484968291390396</v>
+        <v>0.1475051370718759</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1300175287.388255</v>
+        <v>1273994170.671572</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>299.98</v>
+        <v>299.0801</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1325545264974853</v>
+        <v>-0.1351567472508853</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.276947551099113</v>
+        <v>-0.2791166120323949</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>414.88</v>
@@ -3110,31 +3110,31 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>299115157660</v>
+        <v>298217852072</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20.94832402234637</v>
+        <v>20.88548184357542</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>19.99036400215111</v>
+        <v>19.93039557570422</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.768070870927318</v>
+        <v>1.76276689407481</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17.94428115785039</v>
+        <v>17.89045070710718</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.185762309990937</v>
+        <v>-7.164205981226483</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.03646906376751</v>
+        <v>14.99894844541083</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.12558021031352</v>
+        <v>2.120276233461011</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05048557257390845</v>
+        <v>0.0506374782565133</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03096873124874991</v>
+        <v>0.03106191284542167</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7063059258783332</v>
+        <v>0.6973263151319282</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2382806161863175</v>
+        <v>0.2382353227908371</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1284660327.409566</v>
+        <v>1262761881.639897</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -3221,55 +3221,55 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>559.8200000000001</v>
+        <v>606.64001</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.505123716570402</v>
+        <v>1.714637341416001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.04260085851589612</v>
+        <v>-0.01517880160392227</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>584.73</v>
+        <v>615.99</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>154.78</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>912842492000</v>
+        <v>989187207886</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>142.0862944162436</v>
+        <v>153.9695456852792</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>40.9741537717905</v>
+        <v>44.32768658139424</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>22.10004822660695</v>
+        <v>23.94836479569059</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>13.58244704272284</v>
+        <v>14.71840200389742</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.14711870721371</v>
+        <v>1.243056882596749</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>85.09353349505504</v>
+        <v>92.21230893823474</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>22.08043800992616</v>
+        <v>23.92764864302143</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.009205312059465348</v>
+        <v>0.008495245391007581</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.467705402962242</v>
+        <v>2.473439684305681</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9135852965836171</v>
+        <v>0.9161344104613689</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.54710742323953</v>
+        <v>2.564944611511842</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6568543593127123</v>
+        <v>0.6845070365174124</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>9640699873.652445</v>
+        <v>9816473311.898008</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1679.92</v>
+        <v>1710.1299</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4435030312515014</v>
+        <v>0.4694614591669999</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1600232004640093</v>
+        <v>-0.1449179483589672</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>647471391441</v>
+        <v>659114830407</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>52.46734397677794</v>
+        <v>53.75181422351234</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>34.26854356414675</v>
+        <v>34.9922796659698</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.77565395190715</v>
+        <v>16.16186290756493</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>25.53393752233636</v>
+        <v>26.15904221686658</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.571643840685479</v>
+        <v>3.659082424337115</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>40.03237458698251</v>
+        <v>41.0207332295266</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.64296695169486</v>
+        <v>16.02917590735263</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01794660200965958</v>
+        <v>0.01751774436748071</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5310643091255145</v>
+        <v>0.5361049561965605</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2810928551907987</v>
+        <v>0.2850763763526722</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004631172912995857</v>
+        <v>0.004549362010453125</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.684420158995621</v>
+        <v>1.658503110145121</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4356624008892414</v>
+        <v>0.4382365466804631</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2144411058.503011</v>
+        <v>2126492654.149658</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>198.2</v>
+        <v>200.71</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1298239615304612</v>
+        <v>-0.1188040732531728</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2207587969333595</v>
+        <v>-0.2108905052093571</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>156651334000</v>
+        <v>158635162700</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>74.23220973782769</v>
+        <v>75.17228464419473</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>76.3241903614753</v>
+        <v>76.88619795501751</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.666592201712857</v>
+        <v>1.687697884993883</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>25.70247124642623</v>
+        <v>26.02796671982951</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3972962560703509</v>
+        <v>0.4023276062355203</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>28.10105525179856</v>
+        <v>28.38649823021583</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.077794925261982</v>
+        <v>2.098900608543008</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001340556729634999</v>
+        <v>-0.001323792256557505</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.02740914268123762</v>
+        <v>-0.02229156020727541</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1554959263219917</v>
+        <v>0.1559205284580425</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.22626418528472</v>
+        <v>1.223270381950688</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3443784423467804</v>
+        <v>0.3425999429553007</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1137444493.032481</v>
+        <v>1131035388.394091</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>942</v>
+        <v>953.635</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.03025129856740216</v>
+        <v>0.04297632389524897</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1837017651799409</v>
+        <v>-0.1736193554536868</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>277896594000</v>
+        <v>281329000445</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>14.35100548446069</v>
+        <v>14.52780316879951</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.01185074089099</v>
+        <v>13.17505273292933</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.356313913360523</v>
+        <v>2.385342600159407</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.303157843281028</v>
+        <v>2.331531672125271</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3363676833112766</v>
+        <v>0.3405115760552547</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.51879699296022</v>
+        <v>26.62785175787596</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.05889240865886</v>
+        <v>7.087921095457744</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1493901001175998</v>
+        <v>-0.1475720810092009</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1029180836943728</v>
+        <v>0.1026751439475575</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3820415698249855</v>
+        <v>-0.3821630148620359</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01910828025477707</v>
+        <v>0.01887514615130527</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.577960615288972</v>
+        <v>1.568739059563203</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3098876404351355</v>
+        <v>0.3100899717742037</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1991869448.718058</v>
+        <v>1969286600.109009</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>229.55</v>
+        <v>228.765</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2125214408233276</v>
+        <v>-0.2152144082332762</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3095409974132226</v>
+        <v>-0.3119021837213499</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>216266859700</v>
+        <v>215527284510</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.04803493449782</v>
+        <v>19.97947598253275</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.77784559121205</v>
+        <v>17.71390952978631</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.129902306901892</v>
+        <v>3.119198872744113</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.262453413444794</v>
+        <v>6.24103748693835</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2443839917402933</v>
+        <v>0.2435482634304865</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>16.91429996301091</v>
+        <v>16.86870627643179</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.970749232238737</v>
+        <v>3.960045798080959</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06302861205322251</v>
+        <v>0.0632448927800023</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1276976634563622</v>
+        <v>0.1278975964586948</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04653808211244037</v>
+        <v>0.04664560425980491</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02936179481594424</v>
+        <v>0.02946254890389701</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8996161912189466</v>
+        <v>0.8823698743961197</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3397939648974554</v>
+        <v>0.3343853572537092</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1263032973.435313</v>
+        <v>1256225166.119612</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1152.22</v>
+        <v>1167.33</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.06651487987594562</v>
+        <v>0.08050095878008312</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.108637295478281</v>
+        <v>-0.09694812981085377</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1085092815020</v>
+        <v>1099322521530</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.54867848778856</v>
+        <v>39.0541987286718</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.27867849323994</v>
+        <v>26.60614431054024</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.62056007747365</v>
+        <v>13.79917758347999</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.35039782756279</v>
+        <v>30.74840733197556</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4075070210409032</v>
+        <v>0.4128509927545759</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.11975612449428</v>
+        <v>26.44835033368125</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.19819816056576</v>
+        <v>14.3768156665721</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01848127618431459</v>
+        <v>0.01824205327121804</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4669184562574189</v>
+        <v>0.4678638991370185</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2316358049677185</v>
+        <v>0.2321044287935796</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005806182847025742</v>
+        <v>0.005731027215954358</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.350247177976581</v>
+        <v>0.3548820357182461</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3124183205632644</v>
+        <v>0.3129111703445646</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2888595298.273926</v>
+        <v>2811762385.221431</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>202.52</v>
+        <v>205.62</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1133590258131074</v>
+        <v>0.1304013573360217</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1280086114101183</v>
+        <v>-0.1146609257265877</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>319430745600</v>
+        <v>324320313600</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>16.27974276527331</v>
+        <v>16.52893890675241</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.03565888435984</v>
+        <v>15.26334534500181</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.524565479850469</v>
+        <v>2.563209332247943</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.881430576813353</v>
+        <v>2.925537009699593</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4141826293273239</v>
+        <v>0.4205225767444417</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.30298652673186</v>
+        <v>23.46959871877875</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.404869599854579</v>
+        <v>5.443513452252053</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04909984469572612</v>
+        <v>-0.04835959803413313</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08274222569704426</v>
+        <v>0.08291718054882602</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3268734944610564</v>
+        <v>-0.3267741682980033</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02049180327868853</v>
+        <v>0.02018286158933956</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.375227679397425</v>
+        <v>1.370230159780131</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2515769412288019</v>
+        <v>0.2533154516306673</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>930398066.4674886</v>
+        <v>904113498.0990347</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1015.8</v>
+        <v>1040.34</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.220467810400145</v>
+        <v>2.298268834289906</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.190597609561753</v>
+        <v>-0.1710438247011953</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,31 +4120,31 @@
         <v>154.65</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1147234362000</v>
+        <v>1174949592600</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>22.66904708770364</v>
+        <v>23.21669270252175</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.474647909946941</v>
+        <v>6.63106438928352</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>12.70835857500498</v>
+        <v>13.01537089970534</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>11.37586275366348</v>
+        <v>11.65068424605854</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03231003906686979</v>
+        <v>0.03309059464739843</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>16.51326137594007</v>
+        <v>16.91877494805841</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>12.50210871347232</v>
+        <v>12.80912103817267</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02281312421149394</v>
+        <v>0.02227499814871632</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
@@ -4153,7 +4153,7 @@
         <v>2.501201517518411</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.784318972372998</v>
+        <v>1.784318972372997</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005217562512305573</v>
+        <v>0.000509448834035027</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.887672514345583</v>
+        <v>2.849763739789576</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.7770948884887525</v>
+        <v>0.7784115439297378</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25726528135.60771</v>
+        <v>25346216338.7304</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>135.47</v>
+        <v>137.405</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.08124786162218367</v>
+        <v>-0.0681247687768225</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.3043045099267689</v>
+        <v>-0.2943674701888808</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>140057285140</v>
+        <v>142057806848</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>84.14285714285715</v>
+        <v>85.34472049689442</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.50428043394301</v>
+        <v>28.89566710342278</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.507010938093945</v>
+        <v>9.642805243551452</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.18092921061042</v>
+        <v>11.34063318951742</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>134.6285714285743</v>
+        <v>136.551552795034</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>41.84788912009171</v>
+        <v>42.42126880137575</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>9.910893642411079</v>
+        <v>10.04668794786859</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03270090517192214</v>
+        <v>0.03224039636836391</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.951937598910916</v>
+        <v>1.953547332595934</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2489068021146772</v>
+        <v>0.2494717167744058</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6973746617483811</v>
+        <v>0.703082710186232</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6292376666408013</v>
+        <v>0.6016878335038168</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2213456242.752838</v>
+        <v>2132357723.640202</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.6</v>
+        <v>27.7137</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.09610800895529725</v>
+        <v>0.1006234973834934</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.05511811023622049</v>
+        <v>-0.05122560766860673</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>157304544000</v>
+        <v>157952566571</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.4693446088795</v>
+        <v>36.61958245243129</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.456832100742504</v>
+        <v>9.49648477055605</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.46961416729465</v>
+        <v>2.479787844935318</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.846371639863834</v>
+        <v>1.853977888249795</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6099739939007278</v>
+        <v>-0.6124868215495144</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.38930164765526</v>
+        <v>17.44063423407795</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.446410198442602</v>
+        <v>3.456583876083271</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06983905054897842</v>
+        <v>0.06955252604307491</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.856401828897448</v>
+        <v>2.856119747169046</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05085331782783276</v>
+        <v>-0.05096012505918535</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06231884057971014</v>
+        <v>0.06206316731436077</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3502851110013918</v>
+        <v>0.3470077692005</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2050434135637993</v>
+        <v>0.2042335836475987</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>974085769.3921089</v>
+        <v>949503793.4137268</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>187.5</v>
+        <v>187.42</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.1160050361906955</v>
+        <v>0.1155288740419207</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.06189022864862159</v>
+        <v>-0.06229048881773158</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1330977920625</v>
+        <v>1330410023714</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>8.113760780990328</v>
+        <v>8.16182290731822</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003878990629858609</v>
+        <v>0.004325440585223388</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.968315520817014</v>
+        <v>7.009592564828316</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>5.049665129599325</v>
+        <v>5.079576985509715</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01815758347958247</v>
+        <v>0.01826514051688748</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>8.197577490578496</v>
+        <v>8.246347839925653</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.938063216567753</v>
+        <v>6.979340260579054</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.06917298904518683</v>
+        <v>0.06876565345659098</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2090.719613482562</v>
+        <v>1885.934462861591</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2709.926668716981</v>
+        <v>2499.96749011031</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.6</v>
+        <v>1.600682958062107</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.8651532945538819</v>
+        <v>0.8588674710572904</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3534679079.809164</v>
+        <v>3456528975.402265</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>573</v>
+        <v>592.87</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.5349585286292171</v>
+        <v>0.5881864971525375</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1471056666120895</v>
+        <v>-0.1175297322239257</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>313.6</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>72221348604</v>
+        <v>74725778267</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.826773971888191</v>
+        <v>1.814977300506886</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.3952270456297697</v>
+        <v>0.4040323760577721</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3790890765.425822</v>
+        <v>3780078705.484049</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>152.71</v>
+        <v>154.25</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.05119600561963333</v>
+        <v>-0.04162781655967818</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3232139691544051</v>
+        <v>-0.3163889381315369</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>2012989615401</v>
+        <v>2033289556516</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-99.16233766233766</v>
+        <v>-100.1623376623377</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>134.8342969109074</v>
+        <v>135.6101115205819</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>121.447337279095</v>
+        <v>122.672069774721</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>7.038698987612401</v>
+        <v>7.109680563415708</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9916233766233766</v>
+        <v>-1.001623376623377</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>470.081981137749</v>
+        <v>474.9535772776578</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>118.1798862987029</v>
+        <v>119.4046187943288</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.0141197946489843</v>
+        <v>-0.01397882554843897</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.295094526746421</v>
+        <v>4.305288125787722</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.346077245157795</v>
+        <v>3.218096694234215</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7751488656668594</v>
+        <v>0.7523639494381489</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>14747168834.83454</v>
+        <v>13939309755.23863</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>761.6900000000001</v>
+        <v>772.62</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1149348171817584</v>
+        <v>0.1309337636715331</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.02268498915790951</v>
+        <v>-0.008660841448862588</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>811381304362</v>
+        <v>823024352971</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9948420724730013</v>
+        <v>0.995118982523625</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1144605303882855</v>
+        <v>0.1192715547493287</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>30651027451.90654</v>
+        <v>30155278187.22266</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>434.67</v>
+        <v>442.2113</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3600013138571829</v>
+        <v>0.3835966342340003</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.09254697286012525</v>
+        <v>-0.07680313152400842</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>265.45</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2254407261600</v>
+        <v>2293520082471</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.51512692708937</v>
+        <v>28.74695722730961</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6605140703029319</v>
+        <v>0.6777653749865373</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.36635940341746</v>
+        <v>14.48315907336394</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.916369735770658</v>
+        <v>9.996990627931394</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.535669551549927</v>
+        <v>0.5400245885543979</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.9112426634564</v>
+        <v>19.07035964288201</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.88177999194684</v>
+        <v>13.99857966189332</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01753258319974648</v>
+        <v>0.01739119139974853</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.17111203098439</v>
+        <v>41.41431959825422</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.15420560240253</v>
+        <v>41.40052630287702</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2760715025191525</v>
+        <v>0.2713634861886162</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.182055485317523</v>
+        <v>2.16778013413212</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3384223806071351</v>
+        <v>0.3401245430090488</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4129131543.744608</v>
+        <v>4080379986.731384</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -5027,53 +5027,53 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>27.8</v>
+        <v>30.9</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.02490355044482162</v>
+        <v>0.08383022630413706</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.07333333333333336</v>
+        <v>-0.0005724876041879323</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>30</v>
+        <v>30.9177</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>69698400316</v>
+        <v>77470524092</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-21.88976377952756</v>
+        <v>-24.3267716535433</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-87.36095804432952</v>
+        <v>-98.07278392725289</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.929901711643361</v>
+        <v>2.144759474124325</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.125762835739083</v>
+        <v>2.36242600036543</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1629005676616005</v>
+        <v>0.1810364402124154</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.25659509355372</v>
+        <v>17.53917163768595</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.723311652111311</v>
+        <v>2.938169414592275</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03127761885662041</v>
+        <v>0.02814428885652349</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02094875164040277</v>
+        <v>0.02085721239547977</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2271828399419369</v>
+        <v>0.2833535847437162</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.1624865549921377</v>
+        <v>0.3020347553594716</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>528269668.4239769</v>
+        <v>690960971.7207906</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>311.56</v>
+        <v>313.46</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1641134579543472</v>
+        <v>-0.1590159344279423</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1959534439598442</v>
+        <v>-0.1910500916152675</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>210399583600</v>
+        <v>211682672600</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.89387507580352</v>
+        <v>19.00909642207398</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.00561869427619</v>
+        <v>16.09751262125699</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.50258208461694</v>
+        <v>2.517843690602215</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.162126021003501</v>
+        <v>6.199704784130688</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.171585266709216</v>
+        <v>1.178729996477953</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.06833779323734</v>
+        <v>9.12023429056787</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.666796517312336</v>
+        <v>2.68205812329761</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07154006553841868</v>
+        <v>0.07110643405585952</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1804526545768712</v>
+        <v>0.1808716582071328</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.007056827402637245</v>
+        <v>0.007289919654722699</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01136217742970856</v>
+        <v>0.01129330696101576</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9623591680626296</v>
+        <v>0.953805729113185</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2346867436799534</v>
+        <v>0.2355795532036712</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>838049893.4372965</v>
+        <v>825938388.2113851</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>147.6</v>
+        <v>148.49</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2458229271035957</v>
+        <v>-0.2412753824228517</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5520485584218513</v>
+        <v>-0.5493474962063732</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>329.5</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>425157372000</v>
+        <v>427720990300</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>22.77777777777778</v>
+        <v>22.91512345679012</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.36102450346003</v>
+        <v>16.44530522845881</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.92330930520919</v>
+        <v>5.95902573665659</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.556364943389444</v>
+        <v>6.595898580243216</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4957516339869283</v>
+        <v>0.4987409222948441</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>14.44112863202545</v>
+        <v>14.50909306203605</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.589051813254943</v>
+        <v>7.624768244702342</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.06755145715784507</v>
+        <v>-0.0671465760421438</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3921975224082528</v>
+        <v>0.3934142990021985</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.43520912853463</v>
+        <v>0.4367736814882319</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01355013550135501</v>
+        <v>0.01346892046602465</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.080442925700819</v>
+        <v>2.069945695208964</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5583366535191318</v>
+        <v>0.5573848342617406</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4260749803.749593</v>
+        <v>4215373940.411263</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>109.51</v>
+        <v>109.8502</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4401630547276612</v>
+        <v>0.4446370157469137</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1600061363810693</v>
+        <v>-0.1573966403313646</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>431626510164</v>
+        <v>432967386237</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>32.59226190476191</v>
+        <v>32.69351190476191</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>21.08743235214967</v>
+        <v>21.14767862253797</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.816052272625346</v>
+        <v>6.837226786213976</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.608790494183157</v>
+        <v>8.635534266679924</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.042952380952381</v>
+        <v>1.046192380952381</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>22.67553375113642</v>
+        <v>22.74251392362256</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>7.168440744792736</v>
+        <v>7.189615258381367</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.0314971385674028</v>
+        <v>0.03139959366952941</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5455775440313109</v>
+        <v>0.5459622064579257</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1669616053539418</v>
+        <v>0.1671879793890401</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01515843301981554</v>
+        <v>0.01511148819028094</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.7094121578490867</v>
+        <v>0.6981848286848316</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3338654993278114</v>
+        <v>0.3339784224757248</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>2099847167.455622</v>
+        <v>2055917983.750985</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>86.12</v>
+        <v>86.81999999999999</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.0953781222616924</v>
+        <v>-0.08802518084951394</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1190671031096563</v>
+        <v>-0.1119067103109658</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>260426880000</v>
+        <v>262543680000</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>12.28530670470756</v>
+        <v>12.38516405135521</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>11.06339943310153</v>
+        <v>11.15065860608368</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>2.017171139769955</v>
+        <v>2.03356709654932</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.457480274155059</v>
+        <v>1.469326955435929</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6530027888087817</v>
+        <v>0.6583105216486115</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.58029881379976</v>
+        <v>15.64419063716761</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>3.998225320475582</v>
+        <v>4.014621277254947</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.07360991307809701</v>
+        <v>0.07301642149603449</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1104459148379029</v>
+        <v>0.1107114376722098</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2900527598102426</v>
+        <v>-0.2899692959204386</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.02148165350673479</v>
+        <v>0.02130845427320894</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.728303923042646</v>
+        <v>0.7244587304160582</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.2243370392460025</v>
+        <v>0.2221829194790843</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1132677059.453532</v>
+        <v>1121901762.751183</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20 11:09 ET</t>
+          <t>2026-09-21 13:30 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-22)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -446,7 +446,7 @@
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,55 +699,55 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>338.98</v>
+        <v>342.035</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2508025083396619</v>
+        <v>0.2620751546992632</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.01622311866964621</v>
+        <v>-0.009570278566050749</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>344.57</v>
+        <v>345.34</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4978719936880</v>
+        <v>5023589809460</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.69634703196348</v>
+        <v>39.04509132420092</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.32971461583428</v>
+        <v>35.64024671329591</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.66511276625188</v>
+        <v>10.76123029383728</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>46.32132379743305</v>
+        <v>46.73878690499443</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.182388381532216</v>
+        <v>1.19304445712836</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.81543236162055</v>
+        <v>30.08174453343304</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.7610013578594</v>
+        <v>10.8571188854448</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02745344219656082</v>
+        <v>0.02720823259546592</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09529180896978762</v>
+        <v>0.09553369925564503</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1204046456526848</v>
+        <v>0.12067661843483</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003127028143253289</v>
+        <v>0.003099098045521657</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3105715180243301</v>
+        <v>0.3066953314996754</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2919331128025581</v>
+        <v>0.2904370008317946</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13631088621.46381</v>
+        <v>13377787210.86424</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>501.61</v>
+        <v>494.31</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.06062079208904669</v>
+        <v>0.04518543038922007</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.09410893592429392</v>
+        <v>-0.1072924944015026</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3724730135500</v>
+        <v>3670523620500</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.86722222222222</v>
+        <v>27.44088333333333</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.3644331155895</v>
+        <v>23.99784659996998</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.22450988431137</v>
+        <v>11.05278681000425</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.423531184234617</v>
+        <v>8.294660107778935</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8851560840422773</v>
+        <v>0.8716141365042521</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.46868689373022</v>
+        <v>18.19408835935505</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.54958710549393</v>
+        <v>11.37786403118681</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01798439016066</v>
+        <v>0.01826380700104743</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.143766493150685</v>
+        <v>0.1434727369816449</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2292678194734146</v>
+        <v>0.2289659538289326</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.00725663363968023</v>
+        <v>0.007363800044506484</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5595574674859327</v>
+        <v>0.5558263108504464</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4303611555697466</v>
+        <v>0.4275414227053552</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10978589959.94085</v>
+        <v>10635196552.72783</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>354.97</v>
+        <v>355.3</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.1263525523551021</v>
+        <v>0.1273996727942299</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1312743202564792</v>
+        <v>-0.1304667041922616</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4295886443191</v>
+        <v>4299880139916</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>17.42154915590864</v>
+        <v>17.41906653426018</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>21.32954135926265</v>
+        <v>21.36862619792303</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.550232790419093</v>
+        <v>9.548871854348617</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.656603438046465</v>
+        <v>6.655654852610542</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1549308499043283</v>
+        <v>0.1549087718056159</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>13.30696313291947</v>
+        <v>13.30509183323157</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.677726252580371</v>
+        <v>9.676365316509894</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01251090828550775</v>
+        <v>0.01251269138058117</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1832197016114886</v>
+        <v>-0.1848298354363436</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2913476846888949</v>
+        <v>0.2906644510841097</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002422739949854917</v>
+        <v>0.002420489726991275</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7585210482680368</v>
+        <v>0.7575506963266133</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3621372614873961</v>
+        <v>0.3096187195513636</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8253448509.16108</v>
+        <v>8203004777.064982</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>258.45</v>
+        <v>255.06</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1410596026490065</v>
+        <v>0.1260927152317881</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1001044568245125</v>
+        <v>-0.1119080779944289</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2780172495000</v>
+        <v>2743705926000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.51190476190476</v>
+        <v>20.24285714285714</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.041160449556</v>
+        <v>22.75088302514024</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.584174524288366</v>
+        <v>3.53716213644802</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>5.039498567854682</v>
+        <v>4.973397193720315</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2321905970510031</v>
+        <v>0.2291450326323423</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.51663797210203</v>
+        <v>11.37306710709182</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.771131774700908</v>
+        <v>3.724119386860561</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004181395226701572</v>
+        <v>-0.004236970110330986</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1097711937377691</v>
+        <v>-0.110238617090672</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1812821064627377</v>
+        <v>0.1817104093874151</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.836520583502414</v>
+        <v>0.835858925969679</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4638156688227242</v>
+        <v>0.4494876839122866</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8606352112.473917</v>
+        <v>8435044943.857761</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>227.38</v>
+        <v>228.4872</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.2040243190427258</v>
+        <v>0.209887172970266</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.03872495138243004</v>
+        <v>-0.0340441362983005</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5507370980000</v>
+        <v>5534188471200</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.60125786163521</v>
+        <v>28.74052830188679</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.85971777582818</v>
+        <v>16.90008346609313</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18.17800164373253</v>
+        <v>18.26651727140401</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>24.02055252768752</v>
+        <v>24.13751776543339</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2295883284131262</v>
+        <v>0.2307062816069824</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.63957246851288</v>
+        <v>23.75434045543444</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.23218870577518</v>
+        <v>18.32070433344666</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02306109402493892</v>
+        <v>0.02294934490593176</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6964256603773582</v>
+        <v>0.7006145774101828</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9516327173898933</v>
+        <v>0.9556370711452142</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002286920573489313</v>
+        <v>0.00227583864654125</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.312998078869084</v>
+        <v>1.313988303737439</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4120962992058929</v>
+        <v>0.4098475614106242</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27063682401.42276</v>
+        <v>26519949001.64756</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -1331,55 +1331,55 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>741.245</v>
+        <v>753.4450000000001</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.1396581088944708</v>
+        <v>0.1584155088479444</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.05661614040446461</v>
+        <v>-0.02226187386452116</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>785.73</v>
+        <v>770.6</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1888311682580</v>
+        <v>1919391018734</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>27.54533630620587</v>
+        <v>27.99869936826459</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>22.40600520675078</v>
+        <v>22.78286272941931</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.273070005345064</v>
+        <v>8.409234774166697</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.216058567266797</v>
+        <v>7.334826200803152</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.646793942772199</v>
+        <v>-5.739733370494235</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>18.54049315021668</v>
+        <v>18.83075891674761</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.697415454155131</v>
+        <v>8.833580222976762</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02169980749365195</v>
+        <v>0.02134843791601522</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2293729315882977</v>
+        <v>0.2289368417301711</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2754641026512139</v>
+        <v>0.27607824368003</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.002833071386653536</v>
+        <v>0.002787197472940958</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8337369446796072</v>
+        <v>0.8360591572265491</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4838029410403111</v>
+        <v>0.4750792422406967</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>11563975508.17238</v>
+        <v>11655568881.85717</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>375.3</v>
+        <v>376.955</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1432876167615881</v>
+        <v>-0.1395096817915387</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2476394763747168</v>
+        <v>-0.2443217128079707</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1482265136968</v>
+        <v>1488801637905</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>318.0508474576271</v>
+        <v>319.4533898305085</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>175.4676713741686</v>
+        <v>176.1235996227109</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14.30495504654552</v>
+        <v>14.36803711582818</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.98657694167492</v>
+        <v>14.04825502544383</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.466423967534014</v>
+        <v>-8.503759250417758</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>122.745937559694</v>
+        <v>123.2953541459927</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>14.24823764915701</v>
+        <v>14.31201343062566</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.003887293748125436</v>
+        <v>0.00387003994891712</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8125894358021826</v>
+        <v>0.8138022985837015</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1243484142571569</v>
+        <v>0.1246066548924558</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.533736783990318</v>
+        <v>1.53169713719462</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5709828204719943</v>
+        <v>0.4132807444310989</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13342347926.85518</v>
+        <v>13243018876.38941</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>362.66</v>
+        <v>363.08</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.04326564954280698</v>
+        <v>0.04447386542767973</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2673535353535353</v>
+        <v>-0.2665050505050506</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1725383962800</v>
+        <v>1727382146400</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>44.99503722084367</v>
+        <v>45.04714640198511</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.73310281115481</v>
+        <v>19.73366625091677</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>19.36370940474053</v>
+        <v>19.38613470102352</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>17.33812378372956</v>
+        <v>17.35820323001304</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4477228951182957</v>
+        <v>0.4482414072672773</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>33.69167408683007</v>
+        <v>33.72990732258003</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.76149177141318</v>
+        <v>19.78391706769617</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02283723556584805</v>
+        <v>0.02281081814010811</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.280180549984704</v>
+        <v>1.282756069206975</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8616925015388202</v>
+        <v>0.863774308741609</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007169249434732256</v>
+        <v>0.007160956263082517</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.586133867910815</v>
+        <v>1.587507400653102</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3889214972981607</v>
+        <v>0.3883598063218221</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9109853972.231266</v>
+        <v>9020501050.464323</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>898.48</v>
+        <v>901.73</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.05146869514335872</v>
+        <v>0.05527208894090108</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1805927952576379</v>
+        <v>-0.1776288189694483</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,31 +1724,31 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>398457011920</v>
+        <v>399898318670</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>45.12707182320442</v>
+        <v>45.29030637870417</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.65407285301627</v>
+        <v>39.79751036611874</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.357202505288041</v>
+        <v>1.362111805597659</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.902949566982</v>
+        <v>11.94600515652511</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.559800710339388</v>
+        <v>3.572677293355819</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>26.79633807325501</v>
+        <v>26.89594462128542</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.320709063820946</v>
+        <v>1.325618364130564</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02210025105987599</v>
+        <v>0.02202059770915615</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006165969192413854</v>
+        <v>0.00614374591063844</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1753623077384928</v>
+        <v>-0.1749913588006265</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1766123257139956</v>
+        <v>0.1769260237719299</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1804523230.726188</v>
+        <v>1779144757.75872</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>73.36</v>
+        <v>72.06999999999999</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1937575368466896</v>
+        <v>-0.2079349193094455</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.4124619573922793</v>
+        <v>-0.4227935287522026</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>305466638327</v>
+        <v>300095155728</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>22.71207430340558</v>
+        <v>22.3153560371517</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.55256904147701</v>
+        <v>19.20575618902683</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.315108819182596</v>
+        <v>6.204801016002146</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.19258218578291</v>
+        <v>10.01454545169264</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6675134033074079</v>
+        <v>0.6558537567016538</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10.15381659907733</v>
+        <v>9.979431329660079</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.422820039125287</v>
+        <v>6.312512235944837</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03599282743351614</v>
+        <v>0.03663270125287068</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1615902879681075</v>
+        <v>0.1619097846249624</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1453958417687611</v>
+        <v>0.1458607302528572</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1060156206289896</v>
+        <v>0.1020327625487605</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.356490446342517</v>
+        <v>0.3594881217782371</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2388117769.965398</v>
+        <v>2355267701.787415</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>502.01</v>
+        <v>504.19501</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01038541578564312</v>
+        <v>0.01478314140335169</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.06644475025105068</v>
+        <v>-0.06238142968720939</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1082762073226</v>
+        <v>1087474814128</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.60857627251609</v>
+        <v>12.67847677911876</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.63025767416082</v>
+        <v>22.72872983271185</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.81211419060171</v>
+        <v>2.82770423045229</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.439834172468631</v>
+        <v>1.447816448651452</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3473341672607027</v>
+        <v>0.3492597482087166</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.29843913061662</v>
+        <v>15.37682067726168</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.042849827626096</v>
+        <v>3.058439867476676</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02238432543990719</v>
+        <v>0.02226091347840205</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4428443346046148</v>
+        <v>-0.4421827848526968</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05996525504052541</v>
+        <v>0.06126800812246214</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02658849397143491</v>
+        <v>0.02514360964938905</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1542243684565831</v>
+        <v>0.1543894780154173</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2299833880.106328</v>
+        <v>2219071042.253333</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>352.04</v>
+        <v>339.165</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.0816025197159882</v>
+        <v>0.04204555902588658</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.03945429740791262</v>
+        <v>-0.07458390177353336</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>943294700400</v>
+        <v>908796009150</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.13499570077386</v>
+        <v>14.58147033533964</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.05436495103147</v>
+        <v>13.53976825978721</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.169321615546663</v>
+        <v>3.053411446815373</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.620766656522459</v>
+        <v>2.524918540675604</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7924570135016454</v>
+        <v>0.7634748408825293</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.08753435379991</v>
+        <v>19.71721778821383</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.287457037358088</v>
+        <v>6.171546868626798</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1723045830015563</v>
+        <v>-0.1788454156527586</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07688933320769409</v>
+        <v>0.07693647746145427</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2890901225879311</v>
+        <v>-0.2890379678133532</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01704351778207022</v>
+        <v>0.01769050462164433</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7625563978645357</v>
+        <v>0.7647540521108812</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1640717347099889</v>
+        <v>0.1877126667115692</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2292921037.383805</v>
+        <v>2281129938.724064</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>369.95</v>
+        <v>360.65</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.0677383637424267</v>
+        <v>0.04089698846791778</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.04051145057966132</v>
+        <v>-0.06463158440750061</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>690714115709</v>
+        <v>673350576647</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.43160577740017</v>
+        <v>30.64146134239592</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.67861167024925</v>
+        <v>24.05028138275176</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.52585226822963</v>
+        <v>15.13555513052958</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.1228380649838</v>
+        <v>19.61697945164591</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.119565521173368</v>
+        <v>2.066282754997094</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.13269350845419</v>
+        <v>23.53660894628497</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.78432646351825</v>
+        <v>15.39444900015735</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03042213778768761</v>
+        <v>0.03120576131135153</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2736375205130295</v>
+        <v>0.2740583303266952</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1396665241306259</v>
+        <v>0.1399725902919797</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007244222192188134</v>
+        <v>0.007431027311798143</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3114815638989182</v>
+        <v>0.3110932334412584</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1733265299386152</v>
+        <v>0.1846868710109555</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2453149791.321373</v>
+        <v>2389781632.623775</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>567.65</v>
+        <v>554.79498</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.008026557061416195</v>
+        <v>-0.01480124449157527</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05585216971874329</v>
+        <v>-0.07723337158824406</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>497849485400</v>
+        <v>486575172632</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.17243272926963</v>
+        <v>30.46650082372323</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.54642839644202</v>
+        <v>24.95826737115231</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.19061897215175</v>
+        <v>13.86925783519083</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>89.22960256638746</v>
+        <v>87.20890614150775</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.377710196516827</v>
+        <v>1.346510527477053</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.11455441309459</v>
+        <v>22.60477358618195</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.5712021605906</v>
+        <v>14.24984102362968</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03303809782345112</v>
+        <v>0.0338036154023825</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2202266495151692</v>
+        <v>0.2206977499943581</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1590237079486261</v>
+        <v>0.159390647004618</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.00593675680436889</v>
+        <v>0.00607431595722081</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2985024035678206</v>
+        <v>0.3011427114135778</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1865666401680327</v>
+        <v>0.1954628576038141</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1543984005.893982</v>
+        <v>1516658553.014166</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>377.56</v>
+        <v>374</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1223543604349209</v>
+        <v>0.111771720528288</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1820978293834756</v>
+        <v>-0.1898098002686193</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>342879001174</v>
+        <v>339646007096</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.27882451289307</v>
+        <v>24.04990032795319</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.34118662691846</v>
+        <v>17.1718164264016</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7617349719169393</v>
+        <v>0.7545525995792317</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.47464348654606</v>
+        <v>3.441881194957693</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7356547218593317</v>
+        <v>-0.7287182592843257</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.04568571882157</v>
+        <v>14.92019590482475</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8611353660261836</v>
+        <v>0.8539529936884759</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06887852542481929</v>
+        <v>0.06953416058656836</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4000670793315502</v>
+        <v>0.4005449237726861</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01079669339117584</v>
+        <v>0.01087465109618346</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02399618603665643</v>
+        <v>0.02422459893048129</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.429638174493114</v>
+        <v>0.4295224668361777</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2073363274630195</v>
+        <v>0.2045515501352251</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1826761950.108105</v>
+        <v>1809760801.46766</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>158.4</v>
+        <v>159.655</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.2914798045606051</v>
+        <v>0.3017121729616377</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.102091718156567</v>
+        <v>-0.09497760897908281</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>656482464000</v>
+        <v>661683756241</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.38610038610039</v>
+        <v>20.54761904761905</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.35209720355508</v>
+        <v>14.46541864839635</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.81820878524345</v>
+        <v>1.832614402705921</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.548916641221374</v>
+        <v>2.569111656276506</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>1.996138996138998</v>
+        <v>2.011954365079367</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.582491667246781</v>
+        <v>9.654330897319875</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.906227397108514</v>
+        <v>1.920518242674348</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04654046631167897</v>
+        <v>0.04617751801666165</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4204265827471307</v>
+        <v>0.4204648719169268</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08118575198408196</v>
+        <v>0.08326165345216396</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02601010101010101</v>
+        <v>0.0258056434186214</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5528607939779836</v>
+        <v>-0.5510548260295102</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2605115245499678</v>
+        <v>0.2585352904061354</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2369884024.641066</v>
+        <v>2291035534.40596</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -2717,55 +2717,55 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>269.47</v>
+        <v>268.31</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2995900268528189</v>
+        <v>0.293995621423089</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.04127085779343209</v>
+        <v>-0.04539794357277538</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>174.12</v>
+        <v>174.83</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>649395326160</v>
+        <v>646599843997</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.15260115606937</v>
+        <v>31.01849710982659</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.74174012522051</v>
+        <v>21.64248841124343</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.631287219924639</v>
+        <v>6.602741210438174</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.738331277730049</v>
+        <v>7.705019724376552</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.857183906297542</v>
+        <v>-3.840579707940377</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.09988515830665</v>
+        <v>20.01701185808728</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.923478501363233</v>
+        <v>6.894932491876768</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02880833792048369</v>
+        <v>0.02893288665885728</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.43284764589437</v>
+        <v>0.4332223042204451</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09061244409666647</v>
+        <v>0.09082376367910938</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.0195940178869633</v>
+        <v>0.01967872982743841</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.162530796680678</v>
+        <v>-0.1647735065411344</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1989029094187049</v>
+        <v>0.1966799321772688</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1713957958.583543</v>
+        <v>1652674329.867609</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>107.44</v>
+        <v>108.8272</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.04717986906210891</v>
+        <v>-0.03487763446012593</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2050902633915359</v>
+        <v>-0.1948268718555786</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>855016115200</v>
+        <v>866055563776</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.78700361010831</v>
+        <v>39.28779783393502</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.58784736496099</v>
+        <v>35.02397147515342</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.161959278103936</v>
+        <v>1.17696179030224</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.699054948187054</v>
+        <v>8.811371860176306</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.379402691171652</v>
+        <v>9.500503839842477</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.41138017227293</v>
+        <v>21.66907639711478</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.246523857360296</v>
+        <v>1.2615263695586</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01579970220425618</v>
+        <v>0.01559830635011545</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1214055387963011</v>
+        <v>0.1217402304534891</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05165093466825343</v>
+        <v>0.05177497301561229</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009098101265822785</v>
+        <v>0.008982129467633092</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.05105538844014994</v>
+        <v>-0.04878910481217182</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3019001602563294</v>
+        <v>0.3028956401913951</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2783208273.47593</v>
+        <v>2734571320.046837</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>146.11</v>
+        <v>147.39</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.03046764171255312</v>
+        <v>0.03949507707900324</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1263976083707025</v>
+        <v>-0.1187443946188341</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>347333997785</v>
+        <v>350376823773</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.64592592592593</v>
+        <v>21.83555555555555</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.66477451022229</v>
+        <v>20.84243878959935</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.990876893384043</v>
+        <v>4.025839045098355</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.517123142641454</v>
+        <v>6.574216549133692</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.6563978835981</v>
+        <v>20.83735873015895</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.52225453020608</v>
+        <v>17.66541939272608</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.279092722044766</v>
+        <v>4.314054873759077</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.0458146916267326</v>
+        <v>0.04541681675358076</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04747941552511414</v>
+        <v>0.04764877929984768</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02583369712695816</v>
+        <v>0.02591350258673564</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02936554650605708</v>
+        <v>0.02911052310197436</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.03921007522841973</v>
+        <v>-0.03786949574715978</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1474481024279957</v>
+        <v>0.1448577766112893</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1291182410.505503</v>
+        <v>1263948096.16414</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -3095,46 +3095,46 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>297.2</v>
+        <v>301.435</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1405933904762073</v>
+        <v>-0.1283471354582623</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2836482838411107</v>
+        <v>-0.2714209750320258</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>414.88</v>
+        <v>413.73</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>296343172400</v>
+        <v>300565960461</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20.75418994413408</v>
+        <v>21.04993016759776</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>19.80510761197183</v>
+        <v>20.0873237315435</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.751685655175675</v>
+        <v>1.776646571978295</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17.77798639947042</v>
+        <v>18.03131672383703</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.119169806418115</v>
+        <v>-7.220615580745776</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14.92055916370479</v>
+        <v>15.09713403558436</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.109194994561876</v>
+        <v>2.134155911364496</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05095781312490262</v>
+        <v>0.0502418836013183</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03125841184387618</v>
+        <v>0.03081924793073133</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.6909603171589628</v>
+        <v>0.6913635909177618</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2388260751544433</v>
+        <v>0.2379191415327999</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1295256769.800313</v>
+        <v>1271811403.085502</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -3221,55 +3221,55 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>615.52</v>
+        <v>616.74</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.754374173883415</v>
+        <v>1.759833519627076</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.001881040409937085</v>
+        <v>-0.008456591639871336</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>616.6799999999999</v>
+        <v>622</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>154.78</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>1003666912000</v>
+        <v>1005656244000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>156.2233502538071</v>
+        <v>156.5329949238579</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>44.97655478506896</v>
+        <v>44.99142511106167</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>24.29892051809708</v>
+        <v>24.34708253238107</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>14.93384981554207</v>
+        <v>14.96344966083542</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.261252735994039</v>
+        <v>1.263752619568761</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>93.56754170554208</v>
+        <v>93.75314834857249</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>24.2793103014163</v>
+        <v>24.32747231570028</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.008372299514442896</v>
+        <v>0.008355737907594595</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.473439684305681</v>
+        <v>2.479173965649121</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9161344104613689</v>
+        <v>0.9186835243391209</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.571460069794117</v>
+        <v>2.574312322560814</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6956125599575856</v>
+        <v>0.6926150801345953</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10117800446.24058</v>
+        <v>10096968671.57735</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1711.32</v>
+        <v>1715.475</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4704840750995993</v>
+        <v>0.4740543374304544</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1443228864577292</v>
+        <v>-0.1422453449068982</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>659573516358</v>
+        <v>661174928111</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>53.75181422351234</v>
+        <v>54.69521117561683</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.01663121495475</v>
+        <v>35.05310298567643</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.16186290756493</v>
+        <v>16.44551946905385</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.15904221686658</v>
+        <v>26.61815901234341</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.659082424337115</v>
+        <v>3.723302902408138</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.0207332295266</v>
+        <v>41.74664703850193</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.02917590735263</v>
+        <v>16.31283246884155</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01751774436748071</v>
+        <v>0.01721559379439168</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5350367056599163</v>
+        <v>0.5603529079284835</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2841826981421678</v>
+        <v>0.3052661781915773</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3410,7 +3410,7 @@
         <v>0.3542113084707381</v>
       </c>
       <c r="AA23" s="5" t="n">
-        <v>10647408853</v>
+        <v>11084900000</v>
       </c>
       <c r="AB23" s="6" t="n">
         <v>1.333772670235527</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004546198256316762</v>
+        <v>0.004535187047319256</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.653122399365981</v>
+        <v>1.653896279462934</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.438446111564085</v>
+        <v>0.4385148305466236</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2157284592.566</v>
+        <v>2123347428.091606</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>201.15</v>
+        <v>198.89</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1168723000093453</v>
+        <v>-0.1267945898526409</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2091606054649106</v>
+        <v>-0.218045999606841</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>158982925500</v>
+        <v>157196688818</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>75.33707865168537</v>
+        <v>74.49063670411982</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>77.05474923348</v>
+        <v>76.61485035166442</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.69139768604713</v>
+        <v>1.672394157327517</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>26.08502568727869</v>
+        <v>25.79195008174426</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4032095959059086</v>
+        <v>0.3986793762352779</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>28.43653604316547</v>
+        <v>28.17952357093525</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.102600409596255</v>
+        <v>2.083596880876642</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001320896563826283</v>
+        <v>-0.001335906001449782</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.02229156020727541</v>
+        <v>-0.02772587348006805</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1559205284580425</v>
+        <v>0.1565026205340272</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.224131186530198</v>
+        <v>1.226111366957066</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3431721222120872</v>
+        <v>0.3439834760145967</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1147000040.889345</v>
+        <v>1139738020.7513</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>959.39</v>
+        <v>949</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.04927048124477706</v>
+        <v>0.03790709377968637</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1686323105052904</v>
+        <v>-0.1776358547301103</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>283026765730</v>
+        <v>279961643000</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>14.61593540524071</v>
+        <v>14.4576477757465</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.25456158954429</v>
+        <v>13.1093469100376</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.399813169149631</v>
+        <v>2.373823677047915</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.345675799644783</v>
+        <v>2.320272604324518</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3425772735583924</v>
+        <v>0.3388672308518062</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.6822146889434</v>
+        <v>26.58457754913516</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.102391664447968</v>
+        <v>7.076402172346253</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.146682240080446</v>
+        <v>-0.1482881710334869</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1027098336296779</v>
+        <v>0.1028503460135399</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3821435779782588</v>
+        <v>-0.3821015920407239</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01876192163770729</v>
+        <v>0.01896733403582719</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.5724118754812</v>
+        <v>1.574806304943169</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3123067749938691</v>
+        <v>0.3095589636000783</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2000075362.964942</v>
+        <v>1963933472.066854</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>231.93</v>
+        <v>231.26</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2043567753001715</v>
+        <v>-0.2066552315608919</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3023822414726584</v>
+        <v>-0.3043975215063466</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>218509138620</v>
+        <v>217877908840</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.25589519650655</v>
+        <v>20.19737991266376</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.9589842731333</v>
+        <v>17.90393063116934</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.162353483074519</v>
+        <v>3.153218067933485</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.327383228840127</v>
+        <v>6.309104667363289</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2469177922209811</v>
+        <v>0.2462044954470059</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.05253305098329</v>
+        <v>17.01361869428519</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.003200408411364</v>
+        <v>3.99406499327033</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06238183027990008</v>
+        <v>0.06256256117278053</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.127897596458695</v>
+        <v>0.1280975294610278</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04664560425980491</v>
+        <v>0.04675312640716922</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02906049238994524</v>
+        <v>0.02914468563521578</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8927625755996577</v>
+        <v>0.8924933898332964</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3345769130356219</v>
+        <v>0.3348455959904766</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1288105420.322951</v>
+        <v>1242531746.807552</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1164.41</v>
+        <v>1165.36</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.07779815597398931</v>
+        <v>0.07867749250336908</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.09920705527404938</v>
+        <v>-0.09847213089390028</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1096572637810</v>
+        <v>1097467291760</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.95650719304115</v>
+        <v>38.98829039812647</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.53959077264884</v>
+        <v>26.54414652932222</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.76465983910285</v>
+        <v>13.77588992717076</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.6714921928038</v>
+        <v>30.6965159538357</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4118182728734426</v>
+        <v>0.4121542605060031</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.3848496658569</v>
+        <v>26.40550912970387</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.34229792219497</v>
+        <v>14.35352801026287</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01828779900987706</v>
+        <v>0.01827289081922406</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4678638991370183</v>
+        <v>0.4688093420166182</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2321044287935796</v>
+        <v>0.2325730526194412</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005745398957411908</v>
+        <v>0.005740715315439007</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3531140269710956</v>
+        <v>0.3577064461286681</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3124462814953532</v>
+        <v>0.3086254921096016</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2860567556.832145</v>
+        <v>2784184443.682739</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>206.13</v>
+        <v>200.11</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1332050957478559</v>
+        <v>0.1001099874356157</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.112465016146394</v>
+        <v>-0.1383853606027986</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>325124726400</v>
+        <v>315629500800</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>16.56993569131833</v>
+        <v>16.08601286173634</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.30120307346184</v>
+        <v>14.85193395461831</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.56956686925527</v>
+        <v>2.494523001051143</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.932793229303459</v>
+        <v>2.847141382214696</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.421565600351774</v>
+        <v>0.4092538314965968</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.49700911166389</v>
+        <v>23.17345898388251</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.44987098925938</v>
+        <v>5.374827121055253</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04823994832279849</v>
+        <v>-0.04969117259396559</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08291718054882602</v>
+        <v>0.083092135400608</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3267741682980034</v>
+        <v>-0.3266748421349503</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02013292582350944</v>
+        <v>0.02073859377342462</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.371197823858876</v>
+        <v>1.373858562814496</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2543653725170145</v>
+        <v>0.2613446422191189</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>920475083.9029135</v>
+        <v>911503965.6598917</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1043.96</v>
+        <v>1077.54</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.309745594945201</v>
+        <v>2.416206816714483</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1681593625498008</v>
+        <v>-0.1414023904382471</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,40 +4120,40 @@
         <v>154.65</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1179037984400</v>
+        <v>1216962900600</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>23.29747824146396</v>
+        <v>24.04686453916536</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.65413805086455</v>
+        <v>6.831499505709432</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>13.06065959634003</v>
+        <v>13.48076855573033</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>11.69122433580874</v>
+        <v>12.06728406338112</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03320573772814471</v>
+        <v>0.03427383293573034</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>16.97859398355427</v>
+        <v>17.53348989845784</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>12.85440973480736</v>
+        <v>13.27451869419766</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.0221977581267822</v>
+        <v>0.0215059965978391</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.501201517518411</v>
+        <v>2.51999799151975</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.784318972372998</v>
+        <v>1.791598046203779</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005076822866776504</v>
+        <v>0.0004918610910035823</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.841072474561936</v>
+        <v>2.851897963747316</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.7790262254450785</v>
+        <v>0.7790694217447429</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25664233069.36735</v>
+        <v>25423266368.3484</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>137.68</v>
+        <v>135.61501</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.06625972974195204</v>
+        <v>-0.08026440958419612</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2929552293992584</v>
+        <v>-0.3035598225198484</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>142342120160</v>
+        <v>140207200809</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>85.51552795031057</v>
+        <v>84.23292546583852</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.95349839379389</v>
+        <v>28.50370507441258</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.662104273689927</v>
+        <v>9.517187130667933</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.3633301374241</v>
+        <v>11.1928975175775</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>136.8248447204998</v>
+        <v>134.7726807453445</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>42.50275728288908</v>
+        <v>41.8908572109487</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.06598697800706</v>
+        <v>9.921069834985067</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.0321759995906471</v>
+        <v>0.0326659399344203</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.953547332595933</v>
+        <v>1.95515706628095</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.249471716774406</v>
+        <v>0.2500363865009168</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.7045888413355811</v>
+        <v>0.7025367485113688</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6018202937953619</v>
+        <v>0.5936989237375224</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2151589588.927145</v>
+        <v>2106974334.16539</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.74</v>
+        <v>27.765</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1016679771166644</v>
+        <v>0.1026608285740516</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.05032523108524489</v>
+        <v>-0.04946935980828482</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>158102465600</v>
+        <v>158244951600</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.65433403805497</v>
+        <v>36.68736786469345</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.50549683135867</v>
+        <v>9.514759449941941</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.482141195679477</v>
+        <v>2.484378165033911</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.85573729310952</v>
+        <v>1.857409731189107</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6130680648842822</v>
+        <v>-0.6136205775599169</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.45250836501901</v>
+        <v>17.46379527883397</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.45893722682743</v>
+        <v>3.461174196181864</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06948658237749836</v>
+        <v>0.06942401567267439</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.856119747169047</v>
+        <v>2.855837665440645</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05096012505918535</v>
+        <v>-0.05106693229053749</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06200432588320116</v>
+        <v>0.06194849630830181</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.347412484551476</v>
+        <v>0.349157228923028</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2042272140221108</v>
+        <v>0.2038758278150289</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>962328650.2470809</v>
+        <v>927171406.7117437</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>188.86</v>
+        <v>193.03</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.1240997927198655</v>
+        <v>0.1489197447247466</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.05508580577375288</v>
+        <v>-0.03422224445889832</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1340631947143</v>
+        <v>1370232896097</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>8.16182290731822</v>
+        <v>8.039482949392678</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004358674148571599</v>
+        <v>0.004484655584626593</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>7.009592564828316</v>
+        <v>6.904523725526821</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>5.079576985509715</v>
+        <v>5.003437715919633</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01826514051688748</v>
+        <v>0.01799135896738381</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>8.246347839925653</v>
+        <v>8.122205132496529</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.979340260579054</v>
+        <v>6.874271421277559</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.06876565345659098</v>
+        <v>0.06981208731353911</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1871.547162075185</v>
+        <v>1791.664519646066</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2480.898350189539</v>
+        <v>2377.274386534076</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.588478237848141</v>
+        <v>1.554162565404341</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.8588846982043815</v>
+        <v>0.8583457734322725</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3503480905.519937</v>
+        <v>3494245124.660982</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>596.03</v>
+        <v>602.29</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.5966515389509113</v>
+        <v>0.613420893905918</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1128261613801111</v>
+        <v>-0.1035083279996428</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>313.6</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>75124067030</v>
+        <v>75913082113</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.813631666234359</v>
+        <v>1.81652060401248</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.406968829295984</v>
+        <v>0.4065669844724565</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3858424448.601904</v>
+        <v>3797348724.132422</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>151.85</v>
+        <v>152.86</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.05653928002973829</v>
+        <v>-0.05026403915275457</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3270253501152278</v>
+        <v>-0.3225491934054244</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>2001653284648</v>
+        <v>2014966882393</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-98.6038961038961</v>
+        <v>-99.25974025974027</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>133.5001324758533</v>
+        <v>133.814366230963</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>120.7633957555354</v>
+        <v>121.5666294053092</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.999059925800164</v>
+        <v>7.045612777463372</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.986038961038961</v>
+        <v>-0.9925974025974027</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>467.3614793971682</v>
+        <v>470.5564872553396</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>117.4959447751433</v>
+        <v>118.299178424917</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01419976187584271</v>
+        <v>-0.01410593903471232</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.305288125787722</v>
+        <v>4.315481724829025</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.141874476645022</v>
+        <v>3.138954943739724</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7529425494206111</v>
+        <v>0.7514386129038967</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>14084807270.65069</v>
+        <v>13466771452.53553</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>773.5</v>
+        <v>773.12</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1322218764721739</v>
+        <v>0.1316656459446244</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.007531724341455326</v>
+        <v>-0.008019297637835709</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>823961767811</v>
+        <v>823556977285</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9954280715019884</v>
+        <v>0.9961081730098671</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1200907886367417</v>
+        <v>0.1154719943238862</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>30798997417.08495</v>
+        <v>30158689268.10339</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -4899,55 +4899,55 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>445.14</v>
+        <v>447.01</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.392759989993297</v>
+        <v>0.3986108710223832</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.07068893528183717</v>
+        <v>-0.06678496868475992</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>265.45</v>
+        <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2308709707200</v>
+        <v>2318408424800</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.74695722730961</v>
+        <v>28.51512692708937</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6822541147670971</v>
+        <v>0.6867115167424048</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.48315907336394</v>
+        <v>14.36635940341746</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.996990627931394</v>
+        <v>9.916369735770658</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5400245885543979</v>
+        <v>0.535669551549927</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>19.07035964288201</v>
+        <v>18.9112426634564</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.99857966189332</v>
+        <v>13.88177999194684</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01739119139974853</v>
+        <v>0.01753258319974648</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.13526398022977</v>
+        <v>40.52417169637451</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.1215617882634</v>
+        <v>40.51342183057069</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2695781102574471</v>
+        <v>0.2684503702378023</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.171328976876655</v>
+        <v>2.177508912040121</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.342414782443128</v>
+        <v>0.3404584394472164</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4147834624.161417</v>
+        <v>4038438288.264493</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>30.8</v>
+        <v>30.7952</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.0803226851186869</v>
+        <v>0.08015432314178517</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.003880983182406261</v>
+        <v>-0.004036222509702481</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30.92</v>
@@ -5042,16 +5042,16 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>77219810422</v>
+        <v>77207776165</v>
       </c>
       <c r="L37" s="6" t="n">
         <v>-24.25196850393701</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-97.75539627700289</v>
+        <v>-98.72652184256341</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.138164486279939</v>
+        <v>2.138164433310259</v>
       </c>
       <c r="O37" s="6" t="n">
         <v>2.355161702905171</v>
@@ -5060,20 +5060,20 @@
         <v>0.1804797656106941</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>17.49980337553719</v>
+        <v>17.49980305933884</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.931574426747888</v>
+        <v>2.931574373778208</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.02823109753943291</v>
+        <v>0.0282310982388142</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02102242638678953</v>
+        <v>0.02125523250771089</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2888685722098194</v>
+        <v>0.2840008849070663</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.295372177229257</v>
+        <v>0.2955484820158784</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>757424217.0106068</v>
+        <v>793516295.9472675</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>313.59</v>
+        <v>306.71</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1586671565024513</v>
+        <v>-0.1771255574822758</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1907145990864281</v>
+        <v>-0.2084698959973161</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>211770462900</v>
+        <v>207124330100</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>19.01697998787144</v>
+        <v>18.5997574287447</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.10418867766215</v>
+        <v>15.74913384909243</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.518887905748576</v>
+        <v>2.463624827233476</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.202275962660443</v>
+        <v>6.066201283547258</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.179218846409498</v>
+        <v>1.153347403878494</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.123785103543117</v>
+        <v>8.935865155314675</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.683102338443971</v>
+        <v>2.627839259928871</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07107695659666993</v>
+        <v>0.07267132737488091</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1808716582071328</v>
+        <v>0.1810019272784669</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.007289919654722699</v>
+        <v>0.007624244083216158</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01128862527504066</v>
+        <v>0.0115418473476574</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9531044347040731</v>
+        <v>0.9558681720109012</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2356533411484481</v>
+        <v>0.2350316354700897</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>841547167.1961569</v>
+        <v>831457999.4335175</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -5281,55 +5281,55 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>148.57</v>
+        <v>149.5812</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2408666143616613</v>
+        <v>-0.2356997860682138</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5491047040971169</v>
+        <v>-0.5397501538461539</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>329.5</v>
+        <v>325</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>427951427900</v>
+        <v>430864159164</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>22.92746913580247</v>
+        <v>23.08351851851852</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.45416524878527</v>
+        <v>16.55168242726109</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.962236202404671</v>
+        <v>6.002816489460413</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.599452165578385</v>
+        <v>6.644369484214939</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4990096223674658</v>
+        <v>0.5024059912854033</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>14.5152022242842</v>
+        <v>14.59242203510074</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.627978710450424</v>
+        <v>7.668558997506166</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.06711041984584999</v>
+        <v>-0.06665673945989156</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3934142990021987</v>
+        <v>0.3946327583291052</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4367736814882321</v>
+        <v>0.4383382396000859</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01346166790065289</v>
+        <v>0.01337066422785751</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.067951702590242</v>
+        <v>2.058566880990198</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5573964398591271</v>
+        <v>0.542437047283972</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4256263103.73419</v>
+        <v>4216230372.700067</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>111.46</v>
+        <v>105.27</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4658074521043292</v>
+        <v>0.3844029291496747</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1450487075247374</v>
+        <v>-0.1925289560481707</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>439312307761</v>
+        <v>414914827185</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>33.17261904761904</v>
+        <v>31.32738095238095</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>21.45758732590457</v>
+        <v>20.25886881596112</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.937422941350178</v>
+        <v>6.551526456186341</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.762083722780153</v>
+        <v>8.274689867753803</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.061523809523809</v>
+        <v>1.002476190476191</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>23.05945890209301</v>
+        <v>21.83877380678356</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>7.289811413517569</v>
+        <v>6.903914928353731</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.03094609406526374</v>
+        <v>0.03276887368909605</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5459622064579255</v>
+        <v>0.5463539073662103</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1671879793890401</v>
+        <v>0.1673054104256659</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01489323524134219</v>
+        <v>0.01576897501662392</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.7054999351091104</v>
+        <v>0.7025116552981655</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3368364100527863</v>
+        <v>0.3643592750576282</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>2114568641.540187</v>
+        <v>2067218277.429659</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>86.545</v>
+        <v>83.59</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.09091383640429829</v>
+        <v>-0.1219537533657091</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1147197217675942</v>
+        <v>-0.1449468085106383</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>261712080000</v>
+        <v>252776148926</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>12.34593437945792</v>
+        <v>11.9243937232525</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>11.11533919676932</v>
+        <v>10.73325023573479</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>2.02712582781457</v>
+        <v>1.957911381635103</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.464672902075587</v>
+        <v>1.414662983239914</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6562253408901071</v>
+        <v>0.6338191258305396</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.61909027798738</v>
+        <v>15.35028824967553</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>4.008180008520196</v>
+        <v>3.939199876069865</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.07324843392784926</v>
+        <v>0.07582877648667122</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.11071143767221</v>
+        <v>0.1109769605065172</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2899692959204386</v>
+        <v>-0.2898858320306344</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.0213761626899301</v>
+        <v>0.0221318339514296</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.7210938220749589</v>
+        <v>0.7207686626217215</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.2216094995299331</v>
+        <v>0.2372732327721036</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1139014104.219312</v>
+        <v>1122565546.335122</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 18:46 ET</t>
+          <t>2026-09-22 11:59 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-23)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -454,7 +454,7 @@
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>339.75</v>
+        <v>336.84</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2536437318083666</v>
+        <v>0.2429061210370278</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.0161869461979498</v>
+        <v>-0.02461342445126546</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>345.34</v>
@@ -714,40 +714,40 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4990029201000</v>
+        <v>4947288995040</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.78424657534246</v>
+        <v>38.45205479452055</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.40214837909069</v>
+        <v>35.09117666201139</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.68933878793461</v>
+        <v>10.59778330339336</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>46.42654363141742</v>
+        <v>46.0288946484375</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.185074200913241</v>
+        <v>1.174923896499238</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.88255523307574</v>
+        <v>29.6288830825113</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.78522737954214</v>
+        <v>10.69367189500089</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02739122247473197</v>
+        <v>0.02762785843661734</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09553369925564503</v>
+        <v>0.09577558954150245</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1206766184348302</v>
+        <v>0.1209485912169754</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003119941133186166</v>
+        <v>0.003146894668091676</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.305883251416088</v>
+        <v>0.3064999910368851</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2898211767858162</v>
+        <v>0.2904102583543329</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13633123038.90549</v>
+        <v>13306450825.16526</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>498</v>
+        <v>498.6373</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.0529876885635161</v>
+        <v>0.05433521678424191</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.1006284764863108</v>
+        <v>-0.09947753377158142</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3697923900000</v>
+        <v>3702656203015</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.66666666666666</v>
+        <v>27.70207222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.17698935240042</v>
+        <v>24.19582855816018</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.1437290372741</v>
+        <v>11.15798987766658</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.362908494146527</v>
+        <v>8.373610666000582</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8787857695282273</v>
+        <v>0.8799103682650151</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.33951204468025</v>
+        <v>18.36231623617597</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.46880625845666</v>
+        <v>11.48306709884914</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01811475893270816</v>
+        <v>0.01809160676204661</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.144338786910198</v>
+        <v>0.1449110806697109</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2298967550995579</v>
+        <v>0.2305256907257016</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007309236947791165</v>
+        <v>0.007299895134198746</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5551258780098055</v>
+        <v>0.5574671628106231</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4256687513058974</v>
+        <v>0.425430681631548</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10826827816.26078</v>
+        <v>10628201819.56524</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>351.16</v>
+        <v>340.7333</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.114263070921536</v>
+        <v>0.08117819006501015</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1405986148160837</v>
+        <v>-0.1661161009275349</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4249777399192</v>
+        <v>4123592315446</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>17.24975173783515</v>
+        <v>16.74776067527308</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>21.11963629513834</v>
+        <v>20.51104820072775</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.456056014248674</v>
+        <v>9.180872018653584</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.59096132588059</v>
+        <v>6.399155453566076</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1534030454734308</v>
+        <v>0.1489388097575881</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>13.17746919438791</v>
+        <v>12.79908865451915</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.583549476409951</v>
+        <v>9.308365480814862</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01263550960000055</v>
+        <v>0.01301424159964541</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1832363258165587</v>
+        <v>-0.183476119241977</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2931874656741222</v>
+        <v>0.2946766836599939</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.00244902608497551</v>
+        <v>0.002523968159261217</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7545417882669316</v>
+        <v>0.7599190601892666</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3113445623864178</v>
+        <v>0.3281658756889414</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8400258774.429591</v>
+        <v>8216564058.020625</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>254.98</v>
+        <v>249.8263</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1257395143487858</v>
+        <v>0.1029858719646799</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1121866295264624</v>
+        <v>-0.1301312674094707</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2742845358000</v>
+        <v>2687406491730</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.23650793650793</v>
+        <v>19.82748412698412</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.743747172235</v>
+        <v>22.2957593649618</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.536052699566832</v>
+        <v>3.464581388884592</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.971837279286465</v>
+        <v>4.871345641564845</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2290731609056482</v>
+        <v>0.2244430944323584</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.36967900408273</v>
+        <v>11.15141317310835</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.723009949979373</v>
+        <v>3.651538639297133</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004238299460118524</v>
+        <v>-0.004325731903890908</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.110238617090672</v>
+        <v>-0.1107060404435748</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1817104093874151</v>
+        <v>0.1821387053820989</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8335175037192174</v>
+        <v>0.8389052743684878</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4495666057793393</v>
+        <v>0.4566589543582185</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8645900000.19035</v>
+        <v>8438313438.459865</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>228.87</v>
+        <v>225.02</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.2119141784647227</v>
+        <v>0.1915276289515091</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.03242580536061546</v>
+        <v>-0.04870212226261939</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5543460270000</v>
+        <v>5450209420000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.78867924528301</v>
+        <v>28.30440251572326</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.92839731453112</v>
+        <v>16.62181499486396</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18.29712039845661</v>
+        <v>17.98933032752526</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>24.17795697515983</v>
+        <v>23.77124078538239</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2310927993839045</v>
+        <v>0.2272054079493432</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.79401999426534</v>
+        <v>23.3949441726902</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.35130746049926</v>
+        <v>18.04351738956791</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02291096063001097</v>
+        <v>0.02330295777882238</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7006145774101828</v>
+        <v>0.7028466821745494</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9556370711452142</v>
+        <v>0.9581614945672863</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002272032157993621</v>
+        <v>0.002310905697271354</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.313260114087219</v>
+        <v>1.314516122584504</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4099364246706426</v>
+        <v>0.4109370533215882</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26943866743.53516</v>
+        <v>26488705033.30817</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1331,55 +1331,55 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>736.595</v>
+        <v>755.39001</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.1325087720269584</v>
+        <v>0.1614059457728219</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.04412795224500388</v>
+        <v>-0.0110107227022781</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>770.6</v>
+        <v>763.8</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1876465870029</v>
+        <v>1924345917429</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>27.3725380899294</v>
+        <v>28.07097770345596</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>22.27334811721707</v>
+        <v>22.8369274688528</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.221171138537906</v>
+        <v>8.430943173342154</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.170790575795974</v>
+        <v>7.353760974155983</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.611370308435522</v>
+        <v>-5.754550429208467</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>18.42985906706702</v>
+        <v>18.87691593207374</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.645516587347974</v>
+        <v>8.855232653425222</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02183679471844949</v>
+        <v>0.02129361028566728</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2289368417301711</v>
+        <v>0.2291924008491011</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2760782436800298</v>
+        <v>0.2766923847088458</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.002850956088488247</v>
+        <v>0.002780020879545389</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8326109235690381</v>
+        <v>0.8338451668171675</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4750402490545419</v>
+        <v>0.4755196196717496</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>11960319102.00639</v>
+        <v>11679694346.40072</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>378.9</v>
+        <v>380.31799</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1350697521741694</v>
+        <v>-0.1318328494501931</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2404225888579276</v>
+        <v>-0.2375799570996131</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1496483507587</v>
+        <v>1502083938792</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>321.1016949152543</v>
+        <v>322.3033813559322</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>177.0323563742228</v>
+        <v>177.5605464148964</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14.4421728407628</v>
+        <v>14.49622114469354</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>14.12074074926892</v>
+        <v>14.17358600969398</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.547636667462397</v>
+        <v>-8.579625222010023</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>123.9280435306784</v>
+        <v>124.3936596933821</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>14.38545544337429</v>
+        <v>14.43950374730503</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.003850359840778278</v>
+        <v>0.003836004001636482</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8138022985837012</v>
+        <v>0.8151745298351523</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.124606654892456</v>
+        <v>0.1249822127972511</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.531477630366722</v>
+        <v>1.530892612158433</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.4135098112030287</v>
+        <v>0.41393497447659</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13426396096.73609</v>
+        <v>13312005539.78218</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>364.54</v>
+        <v>355.685</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.0486738539798568</v>
+        <v>0.02320063574045461</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2635555555555555</v>
+        <v>-0.2814444444444444</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1734328213200</v>
+        <v>1692199842300</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>45.22828784119107</v>
+        <v>44.12965260545906</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.81301832959458</v>
+        <v>19.31001093988323</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>19.46408930238822</v>
+        <v>18.99128930575507</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>17.42800320995085</v>
+        <v>17.0046615508075</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4500438542613565</v>
+        <v>0.4391118897869933</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>33.86281333256797</v>
+        <v>33.05672927883971</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.86187166906087</v>
+        <v>19.38907167242773</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.0227194597309224</v>
+        <v>0.02328507485643323</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.282756069206975</v>
+        <v>1.285325096026378</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.863774308741609</v>
+        <v>0.8658561159443974</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007132276293410874</v>
+        <v>0.007309838761825773</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.586612050074967</v>
+        <v>1.588752008543647</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.388675290699761</v>
+        <v>0.3906097935396015</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9172166657.698132</v>
+        <v>9019575445.422403</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>899.41</v>
+        <v>896.11</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.05255705090696305</v>
+        <v>0.0486951433586893</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1797446420428637</v>
+        <v>-0.1827542179662562</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,37 +1724,37 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>398869447390</v>
+        <v>397405966690</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>45.17378201908588</v>
+        <v>45.0080361627323</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.69511804907328</v>
+        <v>39.54238834066352</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.358607320453562</v>
+        <v>1.353622492446873</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.91527008952819</v>
+        <v>11.8715521062998</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.563485394094859</v>
+        <v>3.550410709801252</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>26.82484087007602</v>
+        <v>26.72370191361438</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.322113878986467</v>
+        <v>1.317129050979778</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02207739915308633</v>
+        <v>0.02215870102138954</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1380185836263184</v>
+        <v>0.1382225012556504</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>0.114432509886337</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006159593511301854</v>
+        <v>0.00618227672941938</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1749015345156363</v>
+        <v>-0.1752091936288123</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.17665930336363</v>
+        <v>0.1766675348426628</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1818578372.225741</v>
+        <v>1776116219.170398</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>72.16</v>
+        <v>71.48999999999999</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2069457996027416</v>
+        <v>-0.2143092463082039</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.4220727214480218</v>
+        <v>-0.4274387313791447</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>300469910328</v>
+        <v>297680070529</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>22.3405572755418</v>
+        <v>22.13312693498452</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.22974006660436</v>
+        <v>19.07029044415169</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.211808238712128</v>
+        <v>6.154132081291914</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.02585510531754</v>
+        <v>9.932765818724377</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6565944272445823</v>
+        <v>0.6504979989428379</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.990509026658069</v>
+        <v>9.899328965405081</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.31951945865482</v>
+        <v>6.261843301234606</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03659137777888651</v>
+        <v>0.03693430998071772</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1617711522965353</v>
+        <v>0.1606077526612666</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1457240128043698</v>
+        <v>0.1457385824409956</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1005588924704437</v>
+        <v>0.1045972132901628</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3590998569138451</v>
+        <v>0.36265088544876</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2402459178.304428</v>
+        <v>2350129265.243847</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>503.55</v>
+        <v>509.1798</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01348494276779477</v>
+        <v>0.02481592783540298</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.063580912708744</v>
+        <v>-0.05311154089336856</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1086083627762</v>
+        <v>1098226282131</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.66672611841649</v>
+        <v>12.80671152144739</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.6996532695991</v>
+        <v>22.95341357920923</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.825083458765178</v>
+        <v>2.856304663271699</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.446474583998177</v>
+        <v>1.46246019272785</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3489360474306452</v>
+        <v>0.3527922887967998</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.36364430695036</v>
+        <v>15.52061416211412</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.055819095789564</v>
+        <v>3.087040300296085</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02228156446893913</v>
+        <v>0.02203801297040496</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4419859207549829</v>
+        <v>-0.4420563426327374</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06164254375943301</v>
+        <v>0.06155275025681428</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02532596612377708</v>
+        <v>0.01949593598259655</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1542210757671408</v>
+        <v>0.157685874843172</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2271938896.882467</v>
+        <v>2220766260.649499</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>340</v>
+        <v>337.52</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.0446110007483127</v>
+        <v>0.03699148521344253</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.07230559345156895</v>
+        <v>-0.07907230559345158</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>911033400000</v>
+        <v>904388215200</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>14.61736887360275</v>
+        <v>14.51074806534824</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.57310220195967</v>
+        <v>13.47350857781688</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.060928727661247</v>
+        <v>3.038601953412424</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.531134709742177</v>
+        <v>2.512672315388763</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7653544613980213</v>
+        <v>0.7597718759148828</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.74123443537999</v>
+        <v>19.6699035551739</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.179064149472673</v>
+        <v>6.156737375223849</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1784061923525526</v>
+        <v>-0.1797170698028795</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07693647746145427</v>
+        <v>0.07698362171521467</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2890379678133532</v>
+        <v>-0.2889858130387755</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01764705882352941</v>
+        <v>0.0177767243422612</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7635860744810713</v>
+        <v>0.7773876354604339</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1847039223507914</v>
+        <v>0.1937456284642861</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2359171398.514547</v>
+        <v>2258044569.59788</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>362.04</v>
+        <v>363.04</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.04490876391217236</v>
+        <v>0.04779493329652817</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.06102653214721054</v>
+        <v>-0.05843296937002351</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>675945772270</v>
+        <v>677812819481</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>30.75955819881054</v>
+        <v>30.84451996601529</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.14297482825856</v>
+        <v>24.22212222917169</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.19388986400827</v>
+        <v>15.23585729817029</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>19.69258627665018</v>
+        <v>19.74697967593382</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.074246523275054</v>
+        <v>2.079975852971427</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.62515541514881</v>
+        <v>23.68931952302563</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.45236405929689</v>
+        <v>15.49433149345891</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03108681326526081</v>
+        <v>0.03100118409694525</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2740583303266955</v>
+        <v>0.2734028700783278</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1399725902919797</v>
+        <v>0.1402786564533332</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007402496961661694</v>
+        <v>0.007382106654914059</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.310193311260266</v>
+        <v>0.3162803446393336</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1814658674006106</v>
+        <v>0.1793494196148869</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2472105623.610636</v>
+        <v>2385889648.834672</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>555.89</v>
+        <v>559.9528800000001</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-0.01285672015349126</v>
+        <v>-0.005641903033516416</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.07541207191923227</v>
+        <v>-0.06865445836036121</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>487535542040</v>
+        <v>491098834817</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>30.5266337177375</v>
+        <v>30.74974629324547</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.00752845483544</v>
+        <v>25.18055219974834</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>13.89663204515007</v>
+        <v>13.99819955012399</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>87.38103368383533</v>
+        <v>88.01968279451079</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.349168186632148</v>
+        <v>1.359028965638973</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>22.64819777717489</v>
+        <v>22.80931609771206</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.27721523358892</v>
+        <v>14.37878273856284</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03373702752249911</v>
+        <v>0.0334922399197487</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2206977499943581</v>
+        <v>0.2211704512799679</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.159390647004618</v>
+        <v>0.15975758606061</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.006062350465020058</v>
+        <v>0.006018363545161157</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3004264513376782</v>
+        <v>0.3043762495695085</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1942412372936649</v>
+        <v>0.1899298228300389</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1566088507.779964</v>
+        <v>1513056099.937492</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>372.95</v>
+        <v>370.87</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1086504362861631</v>
+        <v>0.1024673208350966</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1920843984229453</v>
+        <v>-0.1965902690524673</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>338692455472</v>
+        <v>336803515111</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>23.98238055430519</v>
+        <v>23.84862709793583</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.12360678135422</v>
+        <v>17.02229802327957</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7524342032439589</v>
+        <v>0.7482377609774087</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.432218159517304</v>
+        <v>3.413076146454437</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7266723925136076</v>
+        <v>-0.7226196278630425</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.88318345969025</v>
+        <v>14.80986356833443</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8518345973532031</v>
+        <v>0.8476381550866529</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06972992642274088</v>
+        <v>0.07012100212854538</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4005449237726861</v>
+        <v>0.4010227682138225</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01087465109618346</v>
+        <v>0.01095260880119087</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.0242928006435179</v>
+        <v>0.02442904521800092</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4293539902906266</v>
+        <v>0.4352545259631662</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2052267863289102</v>
+        <v>0.2072245642091893</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1848488639.768079</v>
+        <v>1813327092.142834</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>158.69</v>
+        <v>161.28</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.293844256222995</v>
+        <v>0.314961255552616</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.1004478204183437</v>
+        <v>-0.08576611303214099</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>657684357400</v>
+        <v>668418508800</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.42342342342342</v>
+        <v>20.75933075933076</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.37798556458625</v>
+        <v>14.54212612503437</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.82153757658007</v>
+        <v>1.851496698609649</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.553583218405428</v>
+        <v>2.595582413061917</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>1.999793543543545</v>
+        <v>2.032684470184472</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.599225303167421</v>
+        <v>9.749828026453185</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.909556188445134</v>
+        <v>1.939515310474713</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04645541536183722</v>
+        <v>0.04570371893223774</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4204648719169268</v>
+        <v>0.4275306499778893</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08326165345216396</v>
+        <v>0.08867701733167643</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02596256852983805</v>
+        <v>0.02554563492063492</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5506463485509412</v>
+        <v>-0.556155110884903</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2578110344256239</v>
+        <v>0.2616178680814166</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2342594486.681976</v>
+        <v>2288952033.018799</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2717,55 +2717,55 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>269.19</v>
+        <v>269.25</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2982396531284013</v>
+        <v>0.2985290189264906</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.04226705091258409</v>
+        <v>-0.04205358095848011</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>174.83</v>
+        <v>175.74</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>648720554603</v>
+        <v>648865148508</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.12023121387283</v>
+        <v>31.1271676300578</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.71347119161648</v>
+        <v>21.71263503151273</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.624396803837474</v>
+        <v>6.625873321569709</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.730290557955066</v>
+        <v>7.73201356933542</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.853175996349261</v>
+        <v>-3.854034834195321</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.07988125824143</v>
+        <v>20.08416780825329</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.916588085276067</v>
+        <v>6.918064603008302</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02883830312953288</v>
+        <v>0.02883187676671672</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4332223042204451</v>
+        <v>0.4335969625465197</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09082376367910938</v>
+        <v>0.09103515418237729</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01961439875181099</v>
+        <v>0.0196100278551532</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1650902407366153</v>
+        <v>-0.1639020728353169</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1963181941908759</v>
+        <v>0.1962789336404106</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1688794559.070471</v>
+        <v>1658114940.475466</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>110.12</v>
+        <v>109.91</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.0234125761459365</v>
+        <v>-0.02527493865056207</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.1852619118082273</v>
+        <v>-0.1868156259248298</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>876343769600</v>
+        <v>874672572800</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>39.75451263537906</v>
+        <v>39.67870036101083</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>35.44003464982922</v>
+        <v>35.36189926281685</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.190943370297891</v>
+        <v>1.188672228745379</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.916045522099392</v>
+        <v>8.899042529367454</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.613363964555308</v>
+        <v>9.595031178208082</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.90923620065828</v>
+        <v>21.87208276570415</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.275507949554251</v>
+        <v>1.273344957599478</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01541518348006978</v>
+        <v>0.01544323148494618</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1217402304534889</v>
+        <v>0.1220749221106774</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05177497301561229</v>
+        <v>0.05189901136297137</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.008876679985470396</v>
+        <v>0.008893640251114549</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.04888254484173982</v>
+        <v>-0.05710075392862948</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3073018862382155</v>
+        <v>0.3063283552002343</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2786925596.681353</v>
+        <v>2738985613.667252</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>148.22</v>
+        <v>147.37</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.04534880469943614</v>
+        <v>0.0393540234014027</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1137817638266069</v>
+        <v>-0.118863976083707</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>352349908642</v>
+        <v>350329281046</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.95851851851852</v>
+        <v>21.83259259259259</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.9598091959727</v>
+        <v>20.83624218276071</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.048509842839415</v>
+        <v>4.025292777897785</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.611238054906003</v>
+        <v>6.573324464657252</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.95470052910075</v>
+        <v>20.83453121693144</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.75825297082902</v>
+        <v>17.66597869902136</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.336725671500138</v>
+        <v>4.314191461405001</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04516249219797066</v>
+        <v>0.04541527591561959</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04764877929984768</v>
+        <v>0.04781814307458143</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02591350258673564</v>
+        <v>0.0259933080465129</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02894751045742815</v>
+        <v>0.02911447377349529</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.0378176858877666</v>
+        <v>-0.04087171479025685</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1475959676423625</v>
+        <v>0.1448071245478448</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1283541093.667109</v>
+        <v>1266047183.628479</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3095,46 +3095,46 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>305.35</v>
+        <v>299.34</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1170262173011772</v>
+        <v>-0.1344052002192057</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.261958281971334</v>
+        <v>-0.2724046571546633</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>413.73</v>
+        <v>411.41</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>304469675950</v>
+        <v>298477002780</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>21.32332402234637</v>
+        <v>20.9036312849162</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>20.34821537454777</v>
+        <v>19.94771504901631</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.799721449555493</v>
+        <v>1.76429873492694</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>18.26550520551243</v>
+        <v>17.90599747246795</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.31439603092117</v>
+        <v>-7.170431661686401</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.26036696424838</v>
+        <v>15.00978477022789</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.157230788941694</v>
+        <v>2.121808074313142</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04959771429743265</v>
+        <v>0.05059351259678312</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03042410348780088</v>
+        <v>0.03103494354246008</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.6913532470641138</v>
+        <v>0.6869951638396742</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2452141816800173</v>
+        <v>0.2356533343502523</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1314925233.931646</v>
+        <v>1271171353.354848</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3221,55 +3221,55 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>623.77</v>
+        <v>612.52</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.791291880756528</v>
+        <v>1.740949553202284</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.001200922308332797</v>
+        <v>-0.01948150594398912</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>624.52</v>
+        <v>624.6899</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>154.78</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>1017119362000</v>
+        <v>998775112000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>158.3172588832487</v>
+        <v>155.4416243654822</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.50426637079959</v>
+        <v>44.60995768295669</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>24.62460627042731</v>
+        <v>24.17733117056046</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>15.13401270379626</v>
+        <v>14.85912233726051</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.27815768639687</v>
+        <v>1.254941554510315</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>94.82266859488711</v>
+        <v>93.09896100018661</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>24.60499605374652</v>
+        <v>24.15772095387968</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.008261567239735625</v>
+        <v>0.008414404345127508</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.47917396564912</v>
+        <v>2.484460251457915</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9186835243391209</v>
+        <v>0.9209817103025144</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.573212847457155</v>
+        <v>2.575704489460866</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6930523222105468</v>
+        <v>0.6928912683402073</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10401702868.40332</v>
+        <v>9983450900.512308</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1747.9</v>
+        <v>1729.3123</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.5019161319137215</v>
+        <v>0.4859442991514511</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1260325206504129</v>
+        <v>-0.1353265565311306</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>673672106469</v>
+        <v>666508072478</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.69521044992743</v>
+        <v>55.00000181422351</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.71565817552797</v>
+        <v>35.30696364391776</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.44551920268912</v>
+        <v>16.53716253844739</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.61815865917692</v>
+        <v>26.7664894696088</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.723302853007808</v>
+        <v>3.744051115002241</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.74664635684016</v>
+        <v>41.98117349972835</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.31283220247682</v>
+        <v>16.40447553823509</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01721559407322915</v>
+        <v>0.01712019110042394</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5314070422872417</v>
+        <v>0.5577664046366735</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.28105238329808</v>
+        <v>0.302866930446487</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004451055552377139</v>
+        <v>0.004498898203638521</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.655587699436945</v>
+        <v>1.653831460337632</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4418483297116296</v>
+        <v>0.4393392668226614</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2161989618.558667</v>
+        <v>2130086997.517497</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>197.72</v>
+        <v>201.585</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1319313505237274</v>
+        <v>-0.1149624787341977</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2226459602909376</v>
+        <v>-0.2074503636721053</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>156271956400</v>
+        <v>159326736450</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>74.05243445692881</v>
+        <v>75.49999999999997</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>76.16415210182055</v>
+        <v>77.24978876620249</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.662556055109314</v>
+        <v>1.695055443906591</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>25.64022510011803</v>
+        <v>26.14143625737049</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3963340855208364</v>
+        <v>0.4040815629664061</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>28.04646854676259</v>
+        <v>28.48600524460432</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.073758778658439</v>
+        <v>2.106258167455715</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001343811166364844</v>
+        <v>-0.001318046202910221</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.02772587348006816</v>
+        <v>-0.02265104920219618</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.156502620534027</v>
+        <v>0.1569278172805462</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.226068212316861</v>
+        <v>1.220982437914445</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3453483057059483</v>
+        <v>0.3431352149978705</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1170781957.972447</v>
+        <v>1151175601.650696</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>949.49</v>
+        <v>938.22498</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.03844299944454632</v>
+        <v>0.02612261570421959</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1772112409986222</v>
+        <v>-0.1869730413608437</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>280106196430</v>
+        <v>276782935373</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>14.4651127361365</v>
+        <v>14.2934945155393</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.11611569822086</v>
+        <v>12.95885129665275</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.375049360506033</v>
+        <v>2.346871086876892</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.321470637597562</v>
+        <v>2.293928048247543</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3390421991796433</v>
+        <v>0.3350197058889265</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.5891821880674</v>
+        <v>26.4833222493231</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.07762785580437</v>
+        <v>7.049449582175229</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1482116444731162</v>
+        <v>-0.1499911833222423</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1028503460135399</v>
+        <v>0.1029908583974022</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3821015920407239</v>
+        <v>-0.3820596061031889</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01895754562975913</v>
+        <v>0.01918516388254766</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.574502784024422</v>
+        <v>1.579073730509181</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3094381403092941</v>
+        <v>0.3125671244056419</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2003544419.166903</v>
+        <v>1966614315.556508</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>231.38</v>
+        <v>236.53999</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2062435677530017</v>
+        <v>-0.1885420583190395</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3040365758286711</v>
+        <v>-0.2885159417674307</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>217990964920</v>
+        <v>222852370035</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.20786026200874</v>
+        <v>20.65851441048035</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.91322091775475</v>
+        <v>18.30945747708902</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.154854261690088</v>
+        <v>3.225210501686036</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.312378439568096</v>
+        <v>6.453150371560432</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2463322500930911</v>
+        <v>0.2518256892285299</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.02058842981321</v>
+        <v>17.32028666759139</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.995701187026933</v>
+        <v>4.066057427022881</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06253011451645443</v>
+        <v>0.06116605355311765</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.128097529461028</v>
+        <v>0.1282974624633608</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04675312640716922</v>
+        <v>0.04686064855453376</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02912957040366497</v>
+        <v>0.02849412482007799</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8924395690563937</v>
+        <v>0.8815409608474524</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3347993523668889</v>
+        <v>0.3370993903126021</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1267952572.554952</v>
+        <v>1246474828.921168</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1170.48</v>
+        <v>1155.88</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.08341665358802719</v>
+        <v>0.06990263955755682</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.09451127528720071</v>
+        <v>-0.1058059026031795</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1102289005680</v>
+        <v>1088539587080</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>39.15958514553363</v>
+        <v>38.6711274673804</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.66076802845565</v>
+        <v>26.20198643029194</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.83641419128409</v>
+        <v>13.66382546939841</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.83138085539715</v>
+        <v>30.44680515953836</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4139650570099081</v>
+        <v>0.4088014576042415</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.51685276643698</v>
+        <v>26.19934942731522</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.41405227437621</v>
+        <v>14.24146355249053</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01819296019162306</v>
+        <v>0.01842275672655548</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4688093420166182</v>
+        <v>0.4758853329789137</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2325730526194412</v>
+        <v>0.2362005159552316</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005715603854828788</v>
+        <v>0.005787798041319168</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3575119817227</v>
+        <v>0.3605930583649538</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3088566626110504</v>
+        <v>0.3091346884879779</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2841294139.703023</v>
+        <v>2771667935.98112</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>200.21</v>
+        <v>198.725</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1006597400653872</v>
+        <v>0.09249591351328124</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1379547900968783</v>
+        <v>-0.1443487621097955</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>315787228800</v>
+        <v>313444968000</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>16.09405144694534</v>
+        <v>15.97467845659164</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.8593558395589</v>
+        <v>14.74675876368561</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.495769576934932</v>
+        <v>2.477257925060658</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.848564170372316</v>
+        <v>2.827435766231649</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4094583459294071</v>
+        <v>0.4064213066021748</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.17883357072273</v>
+        <v>23.09902095614543</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.376073696939042</v>
+        <v>5.357562045064768</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04966635306817069</v>
+        <v>-0.05003749174879081</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.083092135400608</v>
+        <v>0.08326709025238954</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3266748421349505</v>
+        <v>-0.3265755159718975</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02072823535287948</v>
+        <v>0.02088312995345327</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.37302606731343</v>
+        <v>1.38333878052623</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2612473633000939</v>
+        <v>0.2666492970132273</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>944993728.1738445</v>
+        <v>902277030.530247</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1096.16</v>
+        <v>1073.6</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.475239215444204</v>
+        <v>2.403715535780267</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1265657370517927</v>
+        <v>-0.1445418326693227</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,31 +4120,31 @@
         <v>154.65</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1237992142400</v>
+        <v>1212513104000</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>24.4623967864316</v>
+        <v>23.95893773711225</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.949548506949581</v>
+        <v>6.806520286327788</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>13.71371759753639</v>
+        <v>13.43147643839865</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>12.27580795043882</v>
+        <v>12.02316031928835</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03486608822951368</v>
+        <v>0.03414851146110594</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>17.84117786556638</v>
+        <v>17.46516118043484</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>13.50746773600372</v>
+        <v>13.22278735890733</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02114068345317795</v>
+        <v>0.02158884199490616</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0004835060575098525</v>
+        <v>0.0004936661698956782</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.854506809666866</v>
+        <v>2.849432249096472</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.7841782537302334</v>
+        <v>0.778168165728248</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25953687819.252</v>
+        <v>25305391536.10796</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>137</v>
+        <v>140.13</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.07087146262817723</v>
+        <v>-0.04964392743128809</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2964473157154155</v>
+        <v>-0.2803734478189867</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>141639094000</v>
+        <v>144875087108</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>85.09316770186336</v>
+        <v>87.03726708074535</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.79480372559441</v>
+        <v>29.43663567980646</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.614383247352702</v>
+        <v>9.834040667119197</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.30720677532758</v>
+        <v>11.5655393096836</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>136.1490683229843</v>
+        <v>139.2596273291955</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>42.30125938664374</v>
+        <v>43.22874379707653</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.01826595166983</v>
+        <v>10.23792337143633</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03233570528204593</v>
+        <v>0.03161344087120892</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.95515706628095</v>
+        <v>1.956766799965967</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2500363865009168</v>
+        <v>0.2506013002363694</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.7017471529900561</v>
+        <v>0.6919234449279938</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5916164933224918</v>
+        <v>0.590812956017886</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2136378199.038193</v>
+        <v>2102725457.704269</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.93</v>
+        <v>28.05</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1092136481928061</v>
+        <v>0.1139793351882639</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.04382060938034926</v>
+        <v>-0.03971242725094148</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>159185359200</v>
+        <v>159869292000</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.9053911205074</v>
+        <v>37.0639534883721</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.57130313116796</v>
+        <v>9.613129076636429</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.499142162773173</v>
+        <v>2.509879615674453</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.86844782251438</v>
+        <v>1.876475525296396</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6172671612191061</v>
+        <v>-0.6199192220621528</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.53828891001267</v>
+        <v>17.59472361684094</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.475938193921125</v>
+        <v>3.487123067994851</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06901388453819565</v>
+        <v>0.0687063900976036</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.855837665440645</v>
+        <v>2.855555583712242</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05106693229053749</v>
+        <v>-0.05117373952189008</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06158252774794128</v>
+        <v>0.06131907308377896</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3489645535537724</v>
+        <v>0.3437825465866791</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2041167382567851</v>
+        <v>0.2049723415846015</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>942532162.6451607</v>
+        <v>928629981.7680613</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>195.37</v>
+        <v>188.95</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.1628474875764063</v>
+        <v>0.1246354751372369</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.02251463451243307</v>
+        <v>-0.05463551308350434</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1386843500547</v>
+        <v>1341270816545</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>8.039482949392678</v>
+        <v>8.13560720204846</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004539020678487786</v>
+        <v>0.004388923230096176</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.904523725526821</v>
+        <v>6.987077813549424</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>5.003437715919633</v>
+        <v>5.063261427740412</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01799135896738381</v>
+        <v>0.01820647304199383</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>8.122205132496529</v>
+        <v>8.21974583119084</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.874271421277559</v>
+        <v>6.956825509300162</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.06981208731353911</v>
+        <v>0.06898723988018901</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1770.193285700364</v>
+        <v>1852.66814945865</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2348.789142818615</v>
+        <v>2458.819074967014</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.535547934688028</v>
+        <v>1.587721619476052</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.8605049993100677</v>
+        <v>0.8571096938474391</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3547476346.818091</v>
+        <v>3480459417.234889</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>607.46</v>
+        <v>597.3200000000001</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6272703452026251</v>
+        <v>0.6001072047483491</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.0958129288659334</v>
+        <v>-0.1109060327761487</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>313.6</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>76564712780</v>
+        <v>75286659595</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.816962014580145</v>
+        <v>1.816222202408001</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.4083466501149629</v>
+        <v>0.4058909311008616</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3870846313.815714</v>
+        <v>3797538778.818359</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>154.72</v>
+        <v>151.92999</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.03870765496345807</v>
+        <v>-0.05604229337850075</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3143059741180642</v>
+        <v>-0.326670847367488</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>2039484993090</v>
+        <v>2002707730498</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-100.4675324675325</v>
+        <v>-98.65583766233766</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>135.4426190190671</v>
+        <v>132.4348538437657</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>123.0458517701357</v>
+        <v>120.8270123980694</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>7.131343771615419</v>
+        <v>7.002746819468025</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-1.004675324675325</v>
+        <v>-0.9865583766233766</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>476.440363112551</v>
+        <v>467.6145261574275</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>119.7784007897436</v>
+        <v>117.5595614176772</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01393636143256766</v>
+        <v>-0.01419228555777944</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.315481724829025</v>
+        <v>4.325675323870327</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.138311467073145</v>
+        <v>3.102981461540415</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7520735255522328</v>
+        <v>0.751561846976351</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>13603545310.74046</v>
+        <v>13404990684.26321</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>773.38</v>
+        <v>768.37</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1320462247266319</v>
+        <v>0.1247127643502575</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.00768569485610171</v>
+        <v>-0.01411396384259078</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>823833939224</v>
+        <v>818497090510</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9961140293327568</v>
+        <v>0.9962322025278201</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1154453238565853</v>
+        <v>0.1169599391013322</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>30709032091.06693</v>
+        <v>30175789521.90928</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>452</v>
+        <v>447.02</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.4142236498112286</v>
+        <v>0.3986421591562286</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.05636743215031315</v>
+        <v>-0.06676409185803767</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2344288960000</v>
+        <v>2318460289600</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.51512692708937</v>
+        <v>28.97878752752985</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6943773194504977</v>
+        <v>0.6854230119213095</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.36635940341746</v>
+        <v>14.59995874331043</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.916369735770658</v>
+        <v>10.07761152009213</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.535669551549927</v>
+        <v>0.5443796255588689</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.9112426634564</v>
+        <v>19.22947662230763</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.88177999194684</v>
+        <v>14.11537933183981</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01753258319974648</v>
+        <v>0.01725206186855054</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.06575219025745</v>
+        <v>41.27869071144752</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.05512100106947</v>
+        <v>41.3417521685823</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2654867256637168</v>
+        <v>0.2684443649053734</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.177246518186198</v>
+        <v>2.170754243235838</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3420329683202739</v>
+        <v>0.3404594246810089</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4153585236.954175</v>
+        <v>4064897734.611869</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>30.83</v>
+        <v>30.785</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.08137494747432172</v>
+        <v>0.07979655394086915</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.002910737386804807</v>
+        <v>-0.004366106080207044</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30.92</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>77295024523</v>
+        <v>77182203371</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-24.2755905511811</v>
+        <v>-24.24015748031496</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-98.83808737745589</v>
+        <v>-99.69995937833502</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.140247114024644</v>
+        <v>2.137123172393742</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.357455691576832</v>
+        <v>2.35401470856934</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.180655557590185</v>
+        <v>0.1803918696209486</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>17.51223545834711</v>
+        <v>17.49358733404959</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.933657054492593</v>
+        <v>2.930533112861692</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.02820362647470688</v>
+        <v>0.02824485314990503</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02109610113317628</v>
+        <v>0.02116970985440347</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2836759812629915</v>
+        <v>0.2843463774445587</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2954754953552399</v>
+        <v>0.2955922142851594</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>856826336.5067493</v>
+        <v>781638580.9003466</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>305.07</v>
+        <v>302.85999</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.181525525157699</v>
+        <v>-0.187454776720115</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.2127022632842138</v>
+        <v>-0.2184056620816022</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>206016821700</v>
+        <v>204524376708</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.50030321406913</v>
+        <v>18.36628259551243</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.66492211973078</v>
+        <v>15.5459458593702</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.450451651540923</v>
+        <v>2.432699994052788</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.03376487747958</v>
+        <v>5.990054842473747</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.147180373972848</v>
+        <v>1.138869925136581</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>8.891070283934638</v>
+        <v>8.830706463355444</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.614666084236319</v>
+        <v>2.596914426748183</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.0730619950147498</v>
+        <v>0.07359513576949654</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1810019272784669</v>
+        <v>0.1814194364019543</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.007624244083216158</v>
+        <v>0.007857868957289016</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.0116038941882191</v>
+        <v>0.01168856936170407</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9555036158598439</v>
+        <v>0.9655124589928612</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2383731754171033</v>
+        <v>0.2430425576545484</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>870623454.013031</v>
+        <v>828993996.776709</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -5281,55 +5281,55 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>149.12</v>
+        <v>147.28</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2380563339409768</v>
+        <v>-0.2474579993483574</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5411692307692307</v>
+        <v>-0.543374465182613</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>325</v>
+        <v>322.54</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>429535686400</v>
+        <v>424235621600</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>23.01234567901234</v>
+        <v>22.7283950617284</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.50064903579577</v>
+        <v>16.28275137765052</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.984308154422727</v>
+        <v>5.910467442216866</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.623883064757683</v>
+        <v>6.542150602048762</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.5008569353667395</v>
+        <v>0.4946768336964418</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>14.55720271474019</v>
+        <v>14.41669198303287</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.650050662468479</v>
+        <v>7.576209950262619</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.06686289616750223</v>
+        <v>-0.06769822838469536</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3946327583291052</v>
+        <v>0.395857157957044</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4383382396000857</v>
+        <v>0.4399027756407259</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01341201716738197</v>
+        <v>0.0135795763172189</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.059036083663228</v>
+        <v>2.056019652364687</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5424300178647384</v>
+        <v>0.5434857951109339</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4291276798.193616</v>
+        <v>4182115630.834729</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>106.44</v>
+        <v>106.13</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.3997895675756755</v>
+        <v>0.3957127659414361</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1835544987343715</v>
+        <v>-0.1859323463987114</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>419526305743</v>
+        <v>418304460996</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>31.67857142857143</v>
+        <v>31.58630952380952</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.4840315072756</v>
+        <v>20.41925966560972</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.624971271109357</v>
+        <v>6.605676446837743</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.367451924033013</v>
+        <v>8.343082231281695</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.013714285714286</v>
+        <v>1.010761904761905</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>22.07109774429292</v>
+        <v>22.01006348948499</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>6.977359743276748</v>
+        <v>6.958064919005133</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.03240559605892327</v>
+        <v>0.0325002510554866</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5465008153946509</v>
+        <v>0.5468880870841486</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1674163077675612</v>
+        <v>0.1676426683787162</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.0155956407365652</v>
+        <v>0.015641194761142</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.6978927180820386</v>
+        <v>0.7100524440934105</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3548026165483314</v>
+        <v>0.3571160115468119</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>2143866296.367806</v>
+        <v>2042579114.333982</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>83.15000000000001</v>
+        <v>82.52</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.1265756022533642</v>
+        <v>-0.1331932495243249</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1494476268412438</v>
+        <v>-0.1558919803600656</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>251445600000</v>
+        <v>249540480000</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>11.86162624821683</v>
+        <v>11.77175463623395</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.6767526869404</v>
+        <v>10.59332667056024</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>1.947605437434646</v>
+        <v>1.932849076333217</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.407216497863367</v>
+        <v>1.396554484710583</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6304828366169323</v>
+        <v>0.6257058770610853</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.30921493465334</v>
+        <v>15.25171229362229</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>3.928659618140273</v>
+        <v>3.913903257038844</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.07623915471179452</v>
+        <v>0.07682120351776192</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1109769605065172</v>
+        <v>0.1112424833408243</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2898858320306346</v>
+        <v>-0.2898023681408305</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.0222489476849068</v>
+        <v>0.0224188075618032</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.7199822914619393</v>
+        <v>0.7357314902504097</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.2422673233344571</v>
+        <v>0.2503929300275876</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1145266970.262696</v>
+        <v>1113465821.394708</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 17:37 ET</t>
+          <t>2026-09-23 11:49 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-24)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,7 +442,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="23" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>337.02</v>
+        <v>337.32</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.243570303146595</v>
+        <v>0.2446772733292073</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.02409219899229742</v>
+        <v>-0.02322348989401746</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>345.34</v>
@@ -714,40 +714,40 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4949932719120</v>
+        <v>4954338925920</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.47260273972603</v>
+        <v>38.50684931506849</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.10992862673993</v>
+        <v>35.13342626719232</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.60344652924127</v>
+        <v>10.6128852389878</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>46.05349149274554</v>
+        <v>46.09448623325893</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.175551750380516</v>
+        <v>1.176598173515981</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.64457414337096</v>
+        <v>29.67072591147039</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.6993351208488</v>
+        <v>10.70877383059532</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02761310259269535</v>
+        <v>0.0275885445149715</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09577558954150245</v>
+        <v>0.09601747982735986</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1209485912169754</v>
+        <v>0.1212205639991208</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003145213933891164</v>
+        <v>0.003142416696312107</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3064389556497845</v>
+        <v>0.3011602141208892</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2782260036483737</v>
+        <v>0.276779543968116</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13607174897.13764</v>
+        <v>13291129727.48807</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>500.59</v>
+        <v>494.3156</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.05846407031729006</v>
+        <v>0.04519727121463379</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.0959510221772738</v>
+        <v>-0.1072823809867803</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3717156074500</v>
+        <v>3670565203580</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.81055555555555</v>
+        <v>27.46197777777778</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.29196079694656</v>
+        <v>23.97553907375278</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.2016853790543</v>
+        <v>11.06128334397102</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.406402335511666</v>
+        <v>8.301036405680998</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8833561613817977</v>
+        <v>0.8722841665377659</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.43218873693493</v>
+        <v>18.20767497713463</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.52676260023686</v>
+        <v>11.38636056515358</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01802103507558813</v>
+        <v>0.01824977797279443</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1448460578386606</v>
+        <v>0.1454164885844746</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2303892021350757</v>
+        <v>0.2310165320130941</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007271419724724826</v>
+        <v>0.007363716621526814</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.557019221954559</v>
+        <v>0.5598459912917769</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4254120649872489</v>
+        <v>0.4266729420588734</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10774760097.58871</v>
+        <v>10417268506.58995</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>337.83</v>
+        <v>339.71</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.07196575136525363</v>
+        <v>0.07793116477604212</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.173221409167666</v>
+        <v>-0.1686204449230319</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4088456255749</v>
+        <v>4111208224967</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.63257199602781</v>
+        <v>16.67428003972195</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.33627888337258</v>
+        <v>20.46792619725784</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.11772730679397</v>
+        <v>9.140591032801336</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.355142986510118</v>
+        <v>6.371079221833625</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1479144301335306</v>
+        <v>0.1482853421918988</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.71226409151494</v>
+        <v>12.74370192630388</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.245220768955248</v>
+        <v>9.268084494962613</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01310437157482779</v>
+        <v>0.01307159308598496</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1821231361246237</v>
+        <v>-0.1853458978195917</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2968219677562676</v>
+        <v>0.2935799454621923</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002545659059290176</v>
+        <v>0.002531571045892085</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.759113098625588</v>
+        <v>0.7581301931576007</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3269726604057122</v>
+        <v>0.3233771138823707</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8468097353.138259</v>
+        <v>8296412745.988222</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>249.27</v>
+        <v>245.955</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1005298013245033</v>
+        <v>0.08589403973509935</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1320682451253481</v>
+        <v>-0.1436107242339832</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2681422317000</v>
+        <v>2645762530500</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.78333333333333</v>
+        <v>19.5202380952381</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.24611234647444</v>
+        <v>21.96180840708875</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.45686664217203</v>
+        <v>3.410894351407797</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.860498386570465</v>
+        <v>4.795859432217831</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2239433164128596</v>
+        <v>0.2209651317379744</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.12785315180888</v>
+        <v>10.98753486568739</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.643823892584571</v>
+        <v>3.597876564150165</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.00433538571164208</v>
+        <v>-0.004393786210997302</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1107060404435748</v>
+        <v>-0.1111734637964775</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1821387053820989</v>
+        <v>0.1825670082809854</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8379803434397678</v>
+        <v>0.8418837611686922</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4531687601723201</v>
+        <v>0.454536500738729</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8725609002.277155</v>
+        <v>8572123563.062869</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>225.66</v>
+        <v>222.05499</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1949165618576016</v>
+        <v>0.1758272852704252</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.045996448803585</v>
+        <v>-0.06123704236070004</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5465710860000</v>
+        <v>5378393977600</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.38490566037735</v>
+        <v>27.93144528301886</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.66916402885316</v>
+        <v>16.38139461854582</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18.04049543022554</v>
+        <v>17.75229141463318</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>23.83885074939733</v>
+        <v>23.45801544256367</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2278516236683352</v>
+        <v>0.22421160159158</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.46128404952347</v>
+        <v>23.08760320284849</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.09468249226819</v>
+        <v>17.80647847667583</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02323686767433578</v>
+        <v>0.02361411241514774</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7028391832514858</v>
+        <v>0.7050712673386745</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9581615092747187</v>
+        <v>0.9606859327356021</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002304351679517859</v>
+        <v>0.002341762281496129</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.31453162530712</v>
+        <v>1.311795620582262</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4111112294054029</v>
+        <v>0.3914433634125585</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26881190778.00841</v>
+        <v>26303392774.7808</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -1331,55 +1331,55 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>744.1</v>
+        <v>762</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.1440476479819435</v>
+        <v>0.1715687511923678</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.02591962298730199</v>
+        <v>-0.01154494746400303</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>763.9</v>
+        <v>770.9</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1895584756737</v>
+        <v>1941184766340</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>27.65143069490896</v>
+        <v>28.3106651802304</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>22.49560823497437</v>
+        <v>23.02543926992252</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.304934793457118</v>
+        <v>8.502931760580598</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.24385214052469</v>
+        <v>7.416551961748865</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.668543292456331</v>
+        <v>-5.803686361947227</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>18.60842009803683</v>
+        <v>19.03049507330581</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.729280242267183</v>
+        <v>8.927277209390663</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02161654858975275</v>
+        <v>0.02111319149117053</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2291924008491011</v>
+        <v>0.2295385485744814</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2766923847088461</v>
+        <v>0.2771164538812441</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.002822201317027281</v>
+        <v>0.002755905511811024</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8345412728962319</v>
+        <v>0.8297606808522185</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4717341864750667</v>
+        <v>0.4734295322716932</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>12452945322.60721</v>
+        <v>12637308343.50331</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>380.12</v>
+        <v>375.9701</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1322848091750995</v>
+        <v>-0.1417579525782466</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2379768658661267</v>
+        <v>-0.2462961329511055</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1501301955407</v>
+        <v>1484911728677</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>322.135593220339</v>
+        <v>318.5593220338983</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>177.4681100497781</v>
+        <v>175.3980330365794</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14.48867442657235</v>
+        <v>14.32782467891989</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>14.16620737295356</v>
+        <v>14.00893757627392</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.575158749104794</v>
+        <v>-8.479959417522076</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>124.3286461096608</v>
+        <v>122.9429552215664</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>14.43195702918384</v>
+        <v>14.27110728153138</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.003838002061642511</v>
+        <v>0.003881088969595335</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8151745298351523</v>
+        <v>0.8162080641318397</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1249822127972511</v>
+        <v>0.1251479466239211</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.531570923089669</v>
+        <v>1.529481762995835</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.4087011610149382</v>
+        <v>0.4084605364167712</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13586230859.29692</v>
+        <v>13421048012.41842</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>354.99</v>
+        <v>347.6</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.02120132612143899</v>
+        <v>-5.752004334713678e-05</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2828484848484848</v>
+        <v>-0.2977777777777777</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1688893324200</v>
+        <v>1653734808000</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>44.04342431761786</v>
+        <v>43.12283002481389</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.27227963942575</v>
+        <v>18.84983597170593</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.95418077976297</v>
+        <v>18.55800093650117</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.97143484802889</v>
+        <v>16.61669844176949</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4382538756357023</v>
+        <v>0.4290935066825539</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>32.9934623768249</v>
+        <v>32.31800921198553</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.35196314643563</v>
+        <v>18.95578330317382</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02333066241390026</v>
+        <v>0.02382872997031217</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.285325096026378</v>
+        <v>1.28770319749956</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8658561159443972</v>
+        <v>0.8677767480714249</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007324149976055664</v>
+        <v>0.007479861910241657</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.588734214025897</v>
+        <v>1.593317953732967</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3883959382806088</v>
+        <v>0.3910203082052489</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9260596096.118763</v>
+        <v>9148344542.181614</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>904.7</v>
+        <v>900.1492</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.05874780573434757</v>
+        <v>0.05342211819777631</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1749202006383949</v>
+        <v>-0.1790704970360237</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,31 +1724,31 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>401215451300</v>
+        <v>399197267067</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>45.4394776494224</v>
+        <v>45.21090909090909</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.92143680106046</v>
+        <v>39.72062495780383</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.36659815080368</v>
+        <v>1.359723921927742</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.98535134143066</v>
+        <v>11.92506291777134</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.584444509220066</v>
+        <v>3.566414123376627</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>26.9869696821009</v>
+        <v>26.84188125183138</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.330104709336585</v>
+        <v>1.322953746977898</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02194830725353971</v>
+        <v>0.02206375971123063</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.00612357687631259</v>
+        <v>0.006154535270375178</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1755853038126965</v>
+        <v>-0.1731437977178419</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1775938040841742</v>
+        <v>0.1760929537030719</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1827977888.973511</v>
+        <v>1799315219.446566</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>71.36</v>
+        <v>71.55500000000001</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2157379747734429</v>
+        <v>-0.2135948820755843</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.4284798974851834</v>
+        <v>-0.4269181483261252</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>297138758329</v>
+        <v>297950726628</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>22.09287925696595</v>
+        <v>22.15325077399381</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.03561233871401</v>
+        <v>19.08472473249073</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.142941185072041</v>
+        <v>6.159727529381178</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.914703718340629</v>
+        <v>9.941796868916253</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6493151098693651</v>
+        <v>0.6510894434795743</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.881637311722788</v>
+        <v>9.908174792213545</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.250652405014732</v>
+        <v>6.267438749323869</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03700159501853499</v>
+        <v>0.03690075914373279</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1606077526612666</v>
+        <v>0.160784401374104</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1457385824409956</v>
+        <v>0.1460656843464203</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1036945023817875</v>
+        <v>0.1022253865965918</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3579821120048619</v>
+        <v>0.3578906148095443</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2410991953.706758</v>
+        <v>2378846882.317126</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>507.17</v>
+        <v>508.15</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.02077084385570949</v>
+        <v>0.02274327011707844</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.0568490348495555</v>
+        <v>-0.05502659277717858</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1093891437776</v>
+        <v>1096005154299</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.8238094870912</v>
+        <v>12.77151351527133</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.86281342065719</v>
+        <v>22.90696426463185</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.860118054314287</v>
+        <v>2.848454386563622</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.464412691938036</v>
+        <v>1.458440762540041</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3532632942085442</v>
+        <v>0.3518226733620226</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.53978662676112</v>
+        <v>15.4811455760253</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.090853691338673</v>
+        <v>3.079190023588008</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.0220086297213006</v>
+        <v>0.02209874924223362</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4390974876475817</v>
+        <v>-0.4424615427985612</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06718231626317284</v>
+        <v>0.06082596432424459</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02039506041952629</v>
+        <v>0.0194013092825211</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1559220345317615</v>
+        <v>0.1548190544562866</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2283642007.064282</v>
+        <v>2218258312.994431</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>337.53</v>
+        <v>336.65</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.03702220906640563</v>
+        <v>0.03431851000564534</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.07904502046384732</v>
+        <v>-0.08144611186903139</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>904415010300</v>
+        <v>902057041500</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>14.51117798796217</v>
+        <v>14.47334479793637</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.47390776923007</v>
+        <v>13.43819067686066</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.038691980727943</v>
+        <v>3.030769576962232</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.512746760527285</v>
+        <v>2.506195588337364</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.759794386340218</v>
+        <v>0.7578134689107172</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.67019117969085</v>
+        <v>19.64488022219837</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.156827402539369</v>
+        <v>6.148904998773657</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1797117453259499</v>
+        <v>-0.1801815101733786</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07698362171521467</v>
+        <v>0.07703076596897485</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2889858130387755</v>
+        <v>-0.2889336582641977</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01777619767131811</v>
+        <v>0.01782266448834101</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7630181374515607</v>
+        <v>0.7650828758999543</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1836198037193955</v>
+        <v>0.1820900970450709</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2384200423.968785</v>
+        <v>2354926966.288455</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>361.52</v>
+        <v>365.22</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.04340795583230728</v>
+        <v>0.05408678255442378</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.06237518479134796</v>
+        <v>-0.05277900251575585</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>674974907721</v>
+        <v>681882982401</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>30.71537807986406</v>
+        <v>31.02973661852167</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.12070743799622</v>
+        <v>24.35957179768219</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.17206679826021</v>
+        <v>15.32734630464395</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>19.66430170902268</v>
+        <v>19.86555728637217</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.071267271832939</v>
+        <v>2.092465791709521</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.5917900790776</v>
+        <v>23.82919727819781</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.43054099354882</v>
+        <v>15.58582049993257</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03113152764589243</v>
+        <v>0.03081613787458143</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2734028700783278</v>
+        <v>0.2738211031063418</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1402786564533332</v>
+        <v>0.1405847226146868</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007413144500995796</v>
+        <v>0.007338042823503641</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3194013232807419</v>
+        <v>0.3139823787196808</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1825827463666815</v>
+        <v>0.1820449637008069</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2428074922.061113</v>
+        <v>2390781295.305777</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>559.92</v>
+        <v>562.11</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-0.005700290971852096</v>
+        <v>-0.001811313327239161</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.0687091462501872</v>
+        <v>-0.06506661344244302</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>491069997120</v>
+        <v>492990705960</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>30.74794069192751</v>
+        <v>30.86820428336079</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.17907361719988</v>
+        <v>25.26780796449444</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>13.99737756520252</v>
+        <v>14.05212513069008</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>88.01451434681874</v>
+        <v>88.35876314382463</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.358949164509295</v>
+        <v>1.36426438573782</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>22.80801216856574</v>
+        <v>22.89485919515283</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.37796075364136</v>
+        <v>14.43270831912892</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03349420672503577</v>
+        <v>0.03336371213727211</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2211704512799679</v>
+        <v>0.2216415577772259</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.15975758606061</v>
+        <v>0.1601245251166021</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.006018716959565653</v>
+        <v>0.005995267830140008</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3050504589526443</v>
+        <v>0.3032289525866348</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1899582967237246</v>
+        <v>0.1856986030677175</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1549774767.393294</v>
+        <v>1515183978.337231</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>371.29</v>
+        <v>370.09</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1037158345319467</v>
+        <v>0.1001486525409467</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.195680429790737</v>
+        <v>-0.1982799705385383</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>337184935761</v>
+        <v>336095162476</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>23.87563500739503</v>
+        <v>23.79846955179731</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.04157530418603</v>
+        <v>16.98070577844004</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7490851195124064</v>
+        <v>0.7466640951282854</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.416941360630593</v>
+        <v>3.405897891555862</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7234379745713296</v>
+        <v>-0.7210998411190804</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.82466854640376</v>
+        <v>14.78236860909056</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8484855136216506</v>
+        <v>0.8460644892375296</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.07004168186428103</v>
+        <v>0.07026878883353893</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4010227682138225</v>
+        <v>0.4015006126549587</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01095260880119087</v>
+        <v>0.01103056650619805</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02440141129575265</v>
+        <v>0.02448053176254425</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4355690498041813</v>
+        <v>0.4333784081627124</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2067485605835965</v>
+        <v>0.2065572184852278</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1840488513.408824</v>
+        <v>1819722408.093465</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>161.28</v>
+        <v>164.4475</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.314961255552616</v>
+        <v>0.3407867750030309</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.08576611303214099</v>
+        <v>-0.06781078170171762</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>668418508800</v>
+        <v>681546085850</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.75675675675676</v>
+        <v>21.16441441441441</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.54212612503437</v>
+        <v>14.83138385608188</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.851267126793331</v>
+        <v>1.887625563202792</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.595260580152672</v>
+        <v>2.646230867154368</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.032432432432434</v>
+        <v>2.072348911411412</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.748673982596589</v>
+        <v>9.931445678384964</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.939285738658395</v>
+        <v>1.975644175067856</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04570938655611327</v>
+        <v>0.04482895674163456</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4273536467974826</v>
+        <v>0.4270019992595337</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08854202948079837</v>
+        <v>0.08838045201477529</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02554563492063492</v>
+        <v>0.02505358853129418</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5566980615617219</v>
+        <v>-0.5603273422666567</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2615401382250962</v>
+        <v>0.2656911735294235</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2335130550.560269</v>
+        <v>2283732425.213267</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -2717,55 +2717,55 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>269.17</v>
+        <v>270.82</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2981431978623714</v>
+        <v>0.3061007573098318</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.04233820756395201</v>
+        <v>-0.03646778382609317</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>175.74</v>
+        <v>175.91</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>648672356635</v>
+        <v>652648689021</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.11791907514451</v>
+        <v>31.30867052023121</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.70618373791005</v>
+        <v>21.83353566033572</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.623904631263466</v>
+        <v>6.6645088688846</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.729716220828283</v>
+        <v>7.777099033787998</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.852889717067241</v>
+        <v>-3.876507757833897</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.07845240824736</v>
+        <v>20.19633253352899</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.91609591270206</v>
+        <v>6.956700150323194</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02884044588711642</v>
+        <v>0.0286647323662946</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4335969625465197</v>
+        <v>0.4339716208725948</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09103515418237729</v>
+        <v>0.09124654468564519</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01961585615038823</v>
+        <v>0.01949634443541836</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1631451998473887</v>
+        <v>-0.1614737864197995</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1963227738372549</v>
+        <v>0.1932055552768392</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1695220512.04985</v>
+        <v>1662074471.978333</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>110.53</v>
+        <v>108.6</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.01977653506547739</v>
+        <v>-0.03689253332227316</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.1822284699615271</v>
+        <v>-0.1965078425569695</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>879606582400</v>
+        <v>864247488000</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>39.90252707581228</v>
+        <v>39.2057761732852</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>35.56137499335044</v>
+        <v>34.93000745215789</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.195377503805175</v>
+        <v>1.174504631441618</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.949241841242696</v>
+        <v>8.79297624137299</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.649156547423704</v>
+        <v>9.480669510994428</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.98540074231425</v>
+        <v>21.62779893088074</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.279942083061535</v>
+        <v>1.259123285496847</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01535800239595842</v>
+        <v>0.0156302196475787</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1220749221106774</v>
+        <v>0.1224096137678654</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05189901136297137</v>
+        <v>0.05202304971033023</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.008843752827286709</v>
+        <v>0.009000920810313076</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.04939068075476223</v>
+        <v>-0.04438837183583323</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3065110282067564</v>
+        <v>0.3052086006142241</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2797169171.422363</v>
+        <v>2764757735.077515</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>147.45</v>
+        <v>147.02</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.03991823811180573</v>
+        <v>0.03688558404338882</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1183856502242153</v>
+        <v>-0.1209566517189835</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>350519457761</v>
+        <v>349497257918</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.84444444444444</v>
+        <v>21.78074074074074</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.84755316447083</v>
+        <v>20.78339731951832</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.027477913422649</v>
+        <v>4.01573280997794</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.576892802563016</v>
+        <v>6.55771298631953</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.84584126984149</v>
+        <v>20.78504973544996</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.67213031716383</v>
+        <v>17.62403584821681</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.315693742083372</v>
+        <v>4.303948638638662</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04539833566343755</v>
+        <v>0.0455311154507929</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04781814307458143</v>
+        <v>0.04798750684931496</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.0259933080465129</v>
+        <v>0.02607311350629038</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02909867751780265</v>
+        <v>0.02918378451911305</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.04154617768109044</v>
+        <v>-0.03640122277189876</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1448577766112893</v>
+        <v>0.1448027785759338</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1288055106.204311</v>
+        <v>1259114916.011968</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>296.72</v>
+        <v>292.31</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1419813957674974</v>
+        <v>-0.1547336943812253</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2787730001701465</v>
+        <v>-0.2894922340244526</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>411.41</v>
@@ -3110,37 +3110,37 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>295864556240</v>
+        <v>291467270270</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20.72067039106145</v>
+        <v>20.4127094972067</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>19.77312089712073</v>
+        <v>19.47924295442626</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.748856553175391</v>
+        <v>1.722864178547785</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17.74927363543359</v>
+        <v>17.48547511584522</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.107671820189715</v>
+        <v>-7.002034071716283</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14.90054594355007</v>
+        <v>14.71667448337863</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.106365892561592</v>
+        <v>2.080373517933986</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05104024690186391</v>
+        <v>0.05181027696870124</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.0479210893854749</v>
+        <v>0.04792108938547468</v>
       </c>
       <c r="V21" s="4" t="n">
         <v>0.01423568777486173</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03130897816122943</v>
+        <v>0.03178132804214703</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.6899167913620299</v>
+        <v>0.6955332034509617</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.234545376187727</v>
+        <v>0.2262913295060802</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1305537784.062278</v>
+        <v>1297557240.770199</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -3221,55 +3221,55 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>614.61</v>
+        <v>609.505</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.750302038943472</v>
+        <v>1.727457809417746</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.01613584596133211</v>
+        <v>-0.02454228282440307</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>624.6899</v>
+        <v>624.84</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>154.78</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>1002183066000</v>
+        <v>993858853000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>155.992385786802</v>
+        <v>154.6967005076142</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>44.76217281316857</v>
+        <v>44.31355271088389</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>24.26299639268854</v>
+        <v>24.06146599685268</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>14.91177124241342</v>
+        <v>14.78791287337856</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.259388068737484</v>
+        <v>1.248927490336702</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>93.4290974062325</v>
+        <v>92.65244010076506</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>24.24338617600775</v>
+        <v>24.04185578017189</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.008384695655993054</v>
+        <v>0.008454922924553352</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.484915409220499</v>
+        <v>2.490956852791877</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9212326386168381</v>
+        <v>0.9237817525864558</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.575987651987926</v>
+        <v>2.574270686711461</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6884477981739907</v>
+        <v>0.6742459450556689</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10454553343.8809</v>
+        <v>10390220973.25723</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1744.61</v>
+        <v>1712.8651</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4990891371920576</v>
+        <v>0.4718117314960866</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1276775535510711</v>
+        <v>-0.1435503210064202</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>672404081279</v>
+        <v>660169025696</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.99999999999999</v>
+        <v>54.54281386066763</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.51810473192195</v>
+        <v>34.8433369915667</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.53716200574623</v>
+        <v>16.39969726847357</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.76648858669256</v>
+        <v>26.54399281250286</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.744050991501416</v>
+        <v>3.712928660260179</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.98117213647723</v>
+        <v>41.62938210380673</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.40447500553393</v>
+        <v>16.26701026826127</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01712019165190583</v>
+        <v>0.0172636956818254</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5485060482568109</v>
+        <v>0.5653728537501701</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.295121958778827</v>
+        <v>0.3089924824959174</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004459449389834978</v>
+        <v>0.004542097331541171</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.653757948600914</v>
+        <v>1.653127690401735</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4412984153154328</v>
+        <v>0.4390636045397933</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2166265553.84552</v>
+        <v>2108341126.61512</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>199.93</v>
+        <v>196.4825</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1222285803672305</v>
+        <v>-0.1373644627719921</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2139571456654216</v>
+        <v>-0.2275113033221938</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>158018674100</v>
+        <v>155293873525</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>74.88014981273406</v>
+        <v>73.58895131086139</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>76.61557292470602</v>
+        <v>74.90550735622503</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.681139146763126</v>
+        <v>1.652150364647056</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>25.92681673207869</v>
+        <v>25.47974675416721</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4007640790925593</v>
+        <v>0.3938534895728694</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>28.29779483453238</v>
+        <v>27.90573719784173</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.09234187031225</v>
+        <v>2.06335308819618</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001328956853967173</v>
+        <v>-0.001352274853046235</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.02265104920219607</v>
+        <v>-0.01757622492432453</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1569278172805462</v>
+        <v>0.1573530140270649</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.215098992748783</v>
+        <v>1.223386386454588</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3466415068033091</v>
+        <v>0.3478556248701327</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1216236055.704639</v>
+        <v>1219611039.363186</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>936.36</v>
+        <v>917.41</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.02408291499636173</v>
+        <v>0.003357583671677711</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.188589155885233</v>
+        <v>-0.20501044203156</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>276232754520</v>
+        <v>270642371870</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>14.26508226691042</v>
+        <v>13.97295856185253</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.93310379333294</v>
+        <v>12.6697505005181</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.342206046618109</v>
+        <v>2.294241801088717</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.289368235811702</v>
+        <v>2.242486015381858</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3343537621500498</v>
+        <v>0.327506787280099</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.46579665912783</v>
+        <v>26.28560492132004</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.044784541916447</v>
+        <v>6.996820296387054</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1502899251471433</v>
+        <v>-0.1534319404599716</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1029898541651015</v>
+        <v>0.1028598046410736</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3820596061031889</v>
+        <v>-0.3821691838454292</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01922337562475971</v>
+        <v>0.01962045323246967</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.57994188417232</v>
+        <v>1.585467429156629</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3133464788090379</v>
+        <v>0.3154394603289127</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2004410030.090462</v>
+        <v>1974711534.311544</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>232.76</v>
+        <v>226.71</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2015094339622642</v>
+        <v>-0.2222641509433962</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.2998857005354028</v>
+        <v>-0.318083378451543</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>219291109840</v>
+        <v>213591199140</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.32838427947598</v>
+        <v>19.8</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.01686607988459</v>
+        <v>17.54578653422896</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.173670489891023</v>
+        <v>3.091179054662287</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.350026819923372</v>
+        <v>6.184974137931035</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2478014285230697</v>
+        <v>0.2413604651162792</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.10074038838543</v>
+        <v>16.74934955551446</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.014517415227869</v>
+        <v>3.932025979999132</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06215938261220667</v>
+        <v>0.06381817254120782</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1282974624633608</v>
+        <v>0.12847605670874</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04686064855453353</v>
+        <v>0.04696817070189807</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02895686544079739</v>
+        <v>0.02972961051563672</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8870520635741144</v>
+        <v>0.8906313744089469</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3345631371560517</v>
+        <v>0.3315931241274303</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1266125540.235118</v>
+        <v>1246352048.934212</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1152.7</v>
+        <v>1189.285</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.06695917622763226</v>
+        <v>0.1008228887827534</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.108265965265153</v>
+        <v>-0.07996364058329786</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1085544850700</v>
+        <v>1119998445185</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.56473737035798</v>
+        <v>39.79558347273336</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.12990081859494</v>
+        <v>26.94190423685462</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.62623422723427</v>
+        <v>14.06113404865074</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.36304141208418</v>
+        <v>31.33211922063815</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4076767832131442</v>
+        <v>0.4206883428363279</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.13019459043801</v>
+        <v>26.93025929903844</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.20387231032639</v>
+        <v>14.63877213174286</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01847358032887217</v>
+        <v>0.01790220701302499</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4758853329789134</v>
+        <v>0.477088743352291</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2362005159552316</v>
+        <v>0.2368798333089523</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005803765073306151</v>
+        <v>0.005625228603740903</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3629629728605771</v>
+        <v>0.3515427939865667</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3099185658125004</v>
+        <v>0.3199718323340568</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2829107977.523844</v>
+        <v>2784835846.702197</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>198.44</v>
+        <v>195.425</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.09092911851843266</v>
+        <v>0.07435407673082417</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1455758880516684</v>
+        <v>-0.1585575888051668</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>312995443200</v>
+        <v>308239948813</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>15.95176848874598</v>
+        <v>15.70940514469454</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.72560980785394</v>
+        <v>14.49953434582105</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.473705183791858</v>
+        <v>2.436120958934316</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.82338081998243</v>
+        <v>2.780483757030168</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4058384404686655</v>
+        <v>0.3996723303194365</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.0837033836508</v>
+        <v>22.92165975442124</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.354009303795968</v>
+        <v>5.316425078938425</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.05010935571345724</v>
+        <v>-0.0508824377255364</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08326709025238954</v>
+        <v>0.0834420451041713</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3265755159718975</v>
+        <v>-0.3264761898088444</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02091312235436404</v>
+        <v>0.02123576819751823</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.38523064200259</v>
+        <v>1.388237975834995</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2679048215853526</v>
+        <v>0.2698155913620479</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>921712425.0246739</v>
+        <v>905800484.5884796</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1071.88</v>
+        <v>1054.70496</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.398262489281067</v>
+        <v>2.343811156870814</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1459123505976094</v>
+        <v>-0.1595976414342629</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,31 +4120,31 @@
         <v>154.65</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1210570553200</v>
+        <v>1191173230319</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>23.9205534478911</v>
+        <v>23.53726757420219</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.795615652486058</v>
+        <v>6.686727558057507</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>13.40995805215234</v>
+        <v>13.19508640714935</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>12.00389817719709</v>
+        <v>11.81155628132322</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03409380259401103</v>
+        <v>0.03354750783778435</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>17.43996068826266</v>
+        <v>17.15615003539344</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>13.20370819061967</v>
+        <v>12.98883654561668</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02161955776209607</v>
+        <v>0.02197161532331536</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0004944583348882337</v>
+        <v>0.000502510199629667</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.851628818957584</v>
+        <v>2.852468195759498</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.7640968951329951</v>
+        <v>0.7628602577614688</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25881420587.94703</v>
+        <v>25111578512.30424</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -4231,55 +4231,55 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>140.78</v>
+        <v>138.83</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.04523565334886703</v>
+        <v>-0.0584604755961301</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2770354241344247</v>
+        <v>-0.2805468320844087</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>194.726</v>
+        <v>192.966</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>145547092360</v>
+        <v>143531061460</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>87.44099378881988</v>
+        <v>86.22981366459629</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>29.57232136567659</v>
+        <v>29.1468675886921</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.879656011403748</v>
+        <v>9.742808950583763</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.61918664109939</v>
+        <v>11.45824464685203</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>139.9055900621148</v>
+        <v>137.967701863357</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>43.42135063341932</v>
+        <v>42.83463617082258</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.28353871572088</v>
+        <v>10.14458631550367</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03146747850291443</v>
+        <v>0.03191636616455542</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.956852548285545</v>
+        <v>1.958459031736578</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2505986168833849</v>
+        <v>0.2511635155641063</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6850647890717061</v>
+        <v>0.6919678600734946</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5725581336249215</v>
+        <v>0.5562378900211961</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2130004486.810483</v>
+        <v>2097900883.087415</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.17</v>
+        <v>28.505</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1187450221837218</v>
+        <v>0.1320492317127082</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.03560424512153371</v>
+        <v>-0.02413557001027056</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>160553224800</v>
+        <v>162462537200</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>37.22251585623679</v>
+        <v>37.66516913319239</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.654278874930252</v>
+        <v>9.769803243961643</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.520617068575735</v>
+        <v>2.550592457925144</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.884503228078413</v>
+        <v>1.906913898344876</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6225712829051994</v>
+        <v>-0.6299749527587046</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.64664328263625</v>
+        <v>17.79788792775665</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.497413099723687</v>
+        <v>3.527388489073097</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06842590682115031</v>
+        <v>0.06762174338368021</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.855545954125518</v>
+        <v>2.855263836195662</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05117381470757509</v>
+        <v>-0.05128062324801363</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06105786297479588</v>
+        <v>0.06034029117698649</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3404420025652962</v>
+        <v>0.3365357676587639</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2063972299930804</v>
+        <v>0.1999928889745161</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>948353582.7354653</v>
+        <v>930864928.797188</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>189.28</v>
+        <v>185.3</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.1265996440009325</v>
+        <v>0.1029105770993914</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.05298443988592583</v>
+        <v>-0.07289738329914441</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,13 +4498,13 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1343613337685</v>
+        <v>1315361113023</v>
       </c>
       <c r="L32" s="6" t="n">
         <v>8.13560720204846</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004396588457224685</v>
+        <v>0.004288360368827701</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.987077813549424</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1849.43637383882</v>
+        <v>1896.137017958328</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2454.530506208376</v>
+        <v>2514.633014046512</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.584953508030431</v>
+        <v>1.618996222342148</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.8314589351070319</v>
+        <v>0.8082188946502746</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3555778355.093623</v>
+        <v>3452167849.428405</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>601.41</v>
+        <v>592.17</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6110635404937128</v>
+        <v>0.5863113296655558</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1048181831713381</v>
+        <v>-0.1185716624741379</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>313.6</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>75802166255</v>
+        <v>74637549743</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.816737529327231</v>
+        <v>1.816001265761091</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.4002136262142075</v>
+        <v>0.3978724941558385</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3898051175.675472</v>
+        <v>3806976826.23607</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>148.36</v>
+        <v>148.03999</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.07822303315911727</v>
+        <v>-0.08021129041955655</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3424924658748448</v>
+        <v>-0.3439106984577203</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1955648872640</v>
+        <v>1951430614557</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-96.33766233766235</v>
+        <v>-96.12986363636362</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>129.3229527380412</v>
+        <v>128.4977678295403</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>117.9878656193062</v>
+        <v>117.7333704106787</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.838199081934227</v>
+        <v>6.823449202666163</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9633766233766236</v>
+        <v>-0.9612986363636362</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>456.3213037293017</v>
+        <v>455.2954215032398</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>114.720414638914</v>
+        <v>114.4625050620814</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01453379509872382</v>
+        <v>-0.01456563410614119</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.325675323870327</v>
+        <v>4.33586892291163</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.175117469837644</v>
+        <v>3.153134786362624</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7569923775847366</v>
+        <v>0.7556669113243399</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>13423271510.75383</v>
+        <v>12809243886.49917</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>767.8099999999999</v>
+        <v>763.73</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1238930562043952</v>
+        <v>0.1179208968559706</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01483249291094091</v>
+        <v>-0.02006749040891997</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>817900562305</v>
+        <v>813554390343</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.995952230372839</v>
+        <v>0.9959639088772877</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.11723848865973</v>
+        <v>0.1182234025657467</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>31174333009.01348</v>
+        <v>30646646358.23315</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>446.57</v>
+        <v>445.77</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3972341931331864</v>
+        <v>0.394731142425556</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.06770354906054277</v>
+        <v>-0.06937369519832992</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2316126373600</v>
+        <v>2311977189600</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.97878752752985</v>
+        <v>28.68899965225455</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6847330196270842</v>
+        <v>0.6831076112931137</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.59995874331043</v>
+        <v>14.45395915587732</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>10.07761152009213</v>
+        <v>9.97683540489121</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5443796255588689</v>
+        <v>0.5389358293032802</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>19.22947662230763</v>
+        <v>19.03058039802561</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>14.11537933183981</v>
+        <v>13.9693797444067</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01725206186855054</v>
+        <v>0.01742632511974802</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.3212941349201</v>
+        <v>40.99777484245367</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.38441913787236</v>
+        <v>41.08316642894987</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2687148711288264</v>
+        <v>0.2691971195908204</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.17612928201688</v>
+        <v>2.169160174934068</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3346276755698885</v>
+        <v>0.3331898478548083</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4168788602.038975</v>
+        <v>4075024178.729728</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>30.76</v>
+        <v>30.765</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.07891966864450684</v>
+        <v>0.07909504570377912</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.005174644243208237</v>
+        <v>-0.005012936610608087</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30.92</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>77119524954</v>
+        <v>77132059107</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-24.22047244094488</v>
+        <v>-24.2244094488189</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-99.61899465576046</v>
+        <v>-100.6613837635715</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.135387649287</v>
+        <v>2.135734711532604</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.352103051342957</v>
+        <v>2.352485382788233</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1802453763047062</v>
+        <v>0.1802746749679547</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>17.48322726512396</v>
+        <v>17.48529902595041</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.92879758975495</v>
+        <v>2.929144652000554</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.02826780897963673</v>
+        <v>0.02826321538980096</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02116970985440347</v>
+        <v>0.02124338466777553</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2843463004546885</v>
+        <v>0.2828555334802347</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2956758480903653</v>
+        <v>0.2945583915326369</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>857008807.1127169</v>
+        <v>858654928.3067347</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>301.96</v>
+        <v>301.67</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1898693662982883</v>
+        <v>-0.1906474093628447</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.2207282768587577</v>
+        <v>-0.2214766832692456</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>203916607600</v>
+        <v>203720767700</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.31170406306853</v>
+        <v>18.29411764705883</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.50018055187204</v>
+        <v>15.47981979616623</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.425470812270289</v>
+        <v>2.423141409251484</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>5.972254375729288</v>
+        <v>5.966518669778297</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.135485579456653</v>
+        <v>1.134395068070899</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>8.806123911988351</v>
+        <v>8.798202867658956</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.589685244965684</v>
+        <v>2.587355841946879</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07381448807507525</v>
+        <v>0.07388544707511428</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1813865007434974</v>
+        <v>0.1818043031476113</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.007616444851921811</v>
+        <v>0.007849575618025462</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01172340707378461</v>
+        <v>0.01173467696489541</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9686130904719528</v>
+        <v>0.9678884349617677</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2461479634608577</v>
+        <v>0.2234969826824966</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>854233538.9691925</v>
+        <v>840646086.9519857</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>144.55</v>
+        <v>137.505</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.261407209436482</v>
+        <v>-0.2974043468250672</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5518385316549885</v>
+        <v>-0.5736807837787561</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>322.54</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>416371938500</v>
+        <v>396079027350</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>22.3070987654321</v>
+        <v>21.2199074074074</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.98093231694312</v>
+        <v>15.188804232973</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.800910298563607</v>
+        <v>5.518188658623236</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.420884502486072</v>
+        <v>6.107946893907625</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4855074437182282</v>
+        <v>0.4618450435729849</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>14.20821682131495</v>
+        <v>13.67022872083775</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.46665280660936</v>
+        <v>7.183931166668989</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.06897679056726345</v>
+        <v>-0.07251078198245833</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3958571579570438</v>
+        <v>0.3970755750042281</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4399027756407259</v>
+        <v>0.441467333100293</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01383604289173296</v>
+        <v>0.01454492563906767</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.065148741010364</v>
+        <v>2.063610910091541</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5369054284492318</v>
+        <v>0.5456908124153007</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4261383753.780463</v>
+        <v>4212676144.384814</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>106.43</v>
+        <v>105.3998</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.3996580578455389</v>
+        <v>0.3861099254468499</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1836312034977372</v>
+        <v>-0.1915333282196825</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>419486891396</v>
+        <v>415426425404</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>31.67559523809524</v>
+        <v>31.36898809523809</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.57756408037407</v>
+        <v>20.37358179628372</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.624348857418082</v>
+        <v>6.560227799510463</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.366665804912003</v>
+        <v>8.285679813065528</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.013619047619048</v>
+        <v>1.003807619047619</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>22.06912889734752</v>
+        <v>21.86629828682752</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>6.976737329585473</v>
+        <v>6.912616271677853</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.03240864083918698</v>
+        <v>0.0327254097684781</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5393267694063928</v>
+        <v>0.5396894080234835</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1676426683787162</v>
+        <v>0.1678690289898708</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01559710607911303</v>
+        <v>0.01574955550200285</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.707602115509821</v>
+        <v>0.7102951773258285</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3531309544989673</v>
+        <v>0.3534393689669285</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>2142529909.228722</v>
+        <v>2009975091.75386</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>81.95</v>
+        <v>81.16500000000001</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.1391806446742416</v>
+        <v>-0.147426443257899</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1617225859247136</v>
+        <v>-0.1697524549918167</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>247816800000</v>
+        <v>245442960000</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>11.6904422253923</v>
+        <v>11.57845934379458</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.52015415235594</v>
+        <v>10.41689243754332</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>1.919498082955734</v>
+        <v>1.901111188567445</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.386907901381875</v>
+        <v>1.373622694516899</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6213838660343667</v>
+        <v>0.6154316227782719</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.19968609459418</v>
+        <v>15.12803597838882</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>3.900552263661361</v>
+        <v>3.882165369273072</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.0773555303756646</v>
+        <v>0.07810368649400251</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1112424833408243</v>
+        <v>0.1115080061751315</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2898023681408305</v>
+        <v>-0.2897189042510265</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.02257474069554606</v>
+        <v>0.02279307583317933</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.74178452894059</v>
+        <v>0.742631122508727</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.2595217485790621</v>
+        <v>0.2601303459956825</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1141207451.567644</v>
+        <v>1120542724.279895</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23 17:42 ET</t>
+          <t>2026-09-24 12:11 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-25)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -443,10 +443,10 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="23" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>335.92</v>
+        <v>339.99</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.239511412477017</v>
+        <v>0.2545293079544564</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.02727746568599054</v>
+        <v>-0.01549197891932574</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>345.34</v>
@@ -714,40 +714,40 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4933776627520</v>
+        <v>4993554166440</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.34703196347032</v>
+        <v>38.81164383561644</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.98760984132351</v>
+        <v>35.40415855897812</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.56883792683737</v>
+        <v>10.69688975573183</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.90317744419644</v>
+        <v>46.45933942382813</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.171714865550481</v>
+        <v>1.185911339421612</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.5486843270064</v>
+        <v>29.90347664755528</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.66472651844489</v>
+        <v>10.79277834733935</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02770352415988981</v>
+        <v>0.02737188692546894</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09601747982735986</v>
+        <v>0.09624533996372042</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1212205639991211</v>
+        <v>0.1214925120824446</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003155513217432722</v>
+        <v>0.003117738757022265</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3018053049402016</v>
+        <v>0.3020535490086385</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2768863291026283</v>
+        <v>0.2775281360300466</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13462266250.39326</v>
+        <v>13168374522.62007</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>497.93</v>
+        <v>515.4816</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.05283967824584646</v>
+        <v>0.08995136241169255</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.1007548941703388</v>
+        <v>-0.06905728527053401</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3697404111500</v>
+        <v>3827734394880</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.66277777777778</v>
+        <v>28.63786666666666</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.15084648551193</v>
+        <v>24.98969768642956</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.14216264965842</v>
+        <v>11.53491420502111</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.361732984920442</v>
+        <v>8.656476809671169</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8786622454240768</v>
+        <v>0.9096343263727747</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.33700726921391</v>
+        <v>18.96504751314338</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.46723987084098</v>
+        <v>11.85999142620367</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01811730554192088</v>
+        <v>0.0175004305652979</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1454164885844749</v>
+        <v>0.1459869193302892</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2310165320130941</v>
+        <v>0.2316438618911127</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007310264495009339</v>
+        <v>0.007061357767183155</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5581903417397892</v>
+        <v>0.5569968503462129</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4251381132511839</v>
+        <v>0.4307659935872188</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10576914083.37581</v>
+        <v>10511927662.91089</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>342.36</v>
+        <v>345.32999</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.08633985921146214</v>
+        <v>0.09576391143268981</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1621350431952229</v>
+        <v>-0.1548665230904774</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4143278819875</v>
+        <v>4179221927890</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.83267130089374</v>
+        <v>16.99006901688183</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.62759180740395</v>
+        <v>20.82535420837175</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.227418754183992</v>
+        <v>9.313701901779908</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.431598972645516</v>
+        <v>6.491739099565951</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1496939248897493</v>
+        <v>0.1510936719324951</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.86309084651087</v>
+        <v>12.98173097272285</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.354912216345268</v>
+        <v>9.441195363941185</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01294859263778456</v>
+        <v>0.01282863546699388</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1839730270960702</v>
+        <v>-0.1841642237205334</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2957599112058258</v>
+        <v>0.2973304029620385</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002511975698095572</v>
+        <v>0.002490371600798413</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7604790531962132</v>
+        <v>0.7626896947667331</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3246233237972339</v>
+        <v>0.3211116102533135</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8453360492.534921</v>
+        <v>8337964009.67334</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>249.38</v>
+        <v>250.625</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1010154525386313</v>
+        <v>0.1065121412803531</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1316852367688022</v>
+        <v>-0.127350278551532</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2682605598000</v>
+        <v>2695998187500</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.79206349206349</v>
+        <v>19.89087301587302</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.26763343115526</v>
+        <v>22.3866560050357</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.458392117883664</v>
+        <v>3.475657729347154</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.862643268917007</v>
+        <v>4.886919437293789</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2240421400370639</v>
+        <v>0.2251606437837403</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.13251179344638</v>
+        <v>11.18523914652535</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.645349368296205</v>
+        <v>3.662614979759695</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004333473399394583</v>
+        <v>-0.004311946519066419</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1111734637964775</v>
+        <v>-0.1114852968036529</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1825670082809852</v>
+        <v>0.1829953111798719</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8404262925368271</v>
+        <v>0.8345848255124496</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4530208456736868</v>
+        <v>0.4529689510118438</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8734993361.570723</v>
+        <v>8578400644.839294</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>224.58</v>
+        <v>225.66499</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1891977375785705</v>
+        <v>0.194942984943854</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.05056227276570546</v>
+        <v>-0.04597535300583411</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5439552180000</v>
+        <v>5465831802383</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.24905660377358</v>
+        <v>28.38553333333332</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.56766913201555</v>
+        <v>16.62042468032613</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.95415431941882</v>
+        <v>18.0408946208457</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>23.7247589351221</v>
+        <v>23.83937789583551</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2267611346425362</v>
+        <v>0.2278566621315192</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.34933550736732</v>
+        <v>23.46180163387641</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.00834138146147</v>
+        <v>18.09508168288835</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02334861323087813</v>
+        <v>0.02323635351249333</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7050712673386745</v>
+        <v>0.7078705195140857</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9606859327356021</v>
+        <v>0.963210356196486</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002315433253183721</v>
+        <v>0.002304300724715872</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.310862305973913</v>
+        <v>1.30579723908577</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.3891900465865184</v>
+        <v>0.3892065814874117</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26660962703.30736</v>
+        <v>26211022083.42736</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1331,55 +1331,55 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>777.59</v>
+        <v>749.9799</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.195538248346028</v>
+        <v>0.1530879460136181</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.002858611329395355</v>
+        <v>-0.03826536893129184</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>779.8192</v>
+        <v>779.8200000000001</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1980900081966</v>
+        <v>1910563723020</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>28.89594946116685</v>
+        <v>27.8699331103679</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>23.49652404448695</v>
+        <v>22.65617687497076</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.678718244917809</v>
+        <v>8.370560631506082</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.569879029633912</v>
+        <v>7.301093272363249</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.9236696395392</v>
+        <v>-5.713336287625413</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>19.40522341943739</v>
+        <v>18.7483163013673</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>9.103063693727876</v>
+        <v>8.794906080316148</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02068554611766799</v>
+        <v>0.02144707318907418</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2297967736188105</v>
+        <v>0.2301251558976394</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.277384671134894</v>
+        <v>0.2783344562737575</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.0027006520145578</v>
+        <v>0.002800075042011126</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8362670605897318</v>
+        <v>0.8247579868365913</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4807077381802287</v>
+        <v>0.4917069151137234</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>13053222140.50982</v>
+        <v>13182541196.04464</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>377.94</v>
+        <v>373.65</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1372611827308143</v>
+        <v>-0.1470541380308218</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.242347092195738</v>
+        <v>-0.2509472164865786</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1492691942088</v>
+        <v>1475748383768</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>320.2881355932204</v>
+        <v>316.6525423728814</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>176.3170332051533</v>
+        <v>174.0975952958937</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14.40558142896573</v>
+        <v>14.24206355753289</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>14.08496373391052</v>
+        <v>13.92508519652766</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.525979947481495</v>
+        <v>-8.429201480066839</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>123.6128152716994</v>
+        <v>122.2041389896907</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>14.34886403157722</v>
+        <v>14.18534616014438</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.003860140084859055</v>
+        <v>0.003904459637819827</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8165467610866035</v>
+        <v>0.8188220338983054</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1253577707020463</v>
+        <v>0.1273363645261019</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.530222740471378</v>
+        <v>1.526943589757414</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.4073609353916587</v>
+        <v>0.4084960779093921</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13607240531.06975</v>
+        <v>13584041917.33246</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>350.36</v>
+        <v>353.485</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.007882184342959953</v>
+        <v>0.01687188586731136</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2922020202020201</v>
+        <v>-0.2858888888888889</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1666865728800</v>
+        <v>1681733166300</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>43.46898263027295</v>
+        <v>43.85669975186104</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>18.99950670611879</v>
+        <v>19.14988013635172</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.70696858502424</v>
+        <v>18.87382346808224</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.75008285685626</v>
+        <v>16.89948349884643</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4325378964695475</v>
+        <v>0.4363958737685181</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>32.57198646843847</v>
+        <v>32.84963258519412</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.10475095169689</v>
+        <v>19.2676013175615</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02363897662492993</v>
+        <v>0.02343496746076923</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.287900591454502</v>
+        <v>1.290181423569801</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8679379231471858</v>
+        <v>0.8706498006139047</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007420938463294897</v>
+        <v>0.007355333323903419</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.591917106898439</v>
+        <v>1.59610562394907</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3891608060280554</v>
+        <v>0.3899200000768171</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9295561458.191223</v>
+        <v>9199697731.073896</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>896.48</v>
+        <v>920.9206</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.04912814511410191</v>
+        <v>0.07773036863662974</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1824167806657546</v>
+        <v>-0.1601271317829457</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>397570053920</v>
+        <v>408408946767</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>32.44589214621789</v>
+        <v>33.33045964531308</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.30070795291062</v>
+        <v>40.36118888919702</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.311445845741768</v>
+        <v>1.347199597455419</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.11612998538297</v>
+        <v>11.41918737263172</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>0.6312766862137273</v>
+        <v>0.6484870879818374</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>32.69362891912709</v>
+        <v>33.60563616782199</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.260168277245229</v>
+        <v>1.295321383260653</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02361847907661948</v>
+        <v>0.02300191621815292</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.174419652055786</v>
+        <v>-0.1741952959608127</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.08443444611195838</v>
+        <v>0.08464992278891481</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1793,26 +1793,26 @@
         <v>0</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006179725147242549</v>
+        <v>0.006015719487651812</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1745799194417197</v>
+        <v>-0.1715925773727313</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1769202108170901</v>
+        <v>0.1790017783437975</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1855945303.043123</v>
+        <v>1909160808.21167</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24 (C)</t>
+          <t>2026-12-10 (E)</t>
         </is>
       </c>
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>71.72</v>
+        <v>71.31</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2117814959466273</v>
+        <v>-0.2162874857216117</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.4255966682684607</v>
+        <v>-0.428880345987506</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>298637776728</v>
+        <v>296930561329</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>22.20433436532508</v>
+        <v>22.07739938080496</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.12873255278087</v>
+        <v>19.01648584950514</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.17393135919871</v>
+        <v>6.138636994218244</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.964721842480241</v>
+        <v>9.907756756654573</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6525908026882128</v>
+        <v>0.6488601525334141</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.93062958342569</v>
+        <v>9.87483282953729</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.2816425791414</v>
+        <v>6.246348214160935</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.0368158647591792</v>
+        <v>0.03702753920239938</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.160784401374104</v>
+        <v>0.1609610500869418</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1460656843464201</v>
+        <v>0.1463927862518446</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1033890277680657</v>
+        <v>0.09973703261896731</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3580276760827857</v>
+        <v>0.3516070434856325</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2427312844.202382</v>
+        <v>2340375995.62526</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>505.18</v>
+        <v>505.16949</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01676561093721496</v>
+        <v>0.01674445767190158</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.0605497080373415</v>
+        <v>-0.06056925279875036</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1089599299122</v>
+        <v>1089576640575</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.72625050665295</v>
+        <v>12.70262011237051</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.77307922307728</v>
+        <v>22.77257883493221</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.83835929365952</v>
+        <v>2.833088962920504</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.453271961150502</v>
+        <v>1.45057349238913</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3505757927415319</v>
+        <v>0.3499248355563004</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.43039079906945</v>
+        <v>15.40389332513004</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.069094930683907</v>
+        <v>3.06382459994489</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02217734708823681</v>
+        <v>0.02221860310087839</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4411712890474334</v>
+        <v>-0.4421966785384354</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06328092444720101</v>
+        <v>0.06137408607629702</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02025407086795528</v>
+        <v>0.02305414717536615</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1551792338755417</v>
+        <v>0.134744341271376</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2248568181.218565</v>
+        <v>2188271868.95728</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>338.56</v>
+        <v>342.825</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.04018676592161396</v>
+        <v>0.05329048921041246</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.07623465211459757</v>
+        <v>-0.06459754433833564</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>907174905600</v>
+        <v>918603015750</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>14.55546001719691</v>
+        <v>14.73882201203783</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.51443289932554</v>
+        <v>13.68751278619112</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.047964794226447</v>
+        <v>3.086361444295491</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.520414609795034</v>
+        <v>2.552165461374594</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7621129601497474</v>
+        <v>0.7717136565552255</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.69981650493774</v>
+        <v>19.82248836142121</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.166100216037872</v>
+        <v>6.204496866106917</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1791650088606684</v>
+        <v>-0.1769360618387454</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07703076596897507</v>
+        <v>0.0768079082203561</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2889336582641977</v>
+        <v>-0.2888815034896199</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01772211720226843</v>
+        <v>0.01750164077882302</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7653259037803147</v>
+        <v>0.7719066907625598</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1823753360191121</v>
+        <v>0.1851990525156858</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2409470705.965403</v>
+        <v>2373085164.889997</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>367.98</v>
+        <v>367</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.06205261005524587</v>
+        <v>0.05922416405857711</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.04562076925071967</v>
+        <v>-0.04816246077236297</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>687036032704</v>
+        <v>685206326437</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.2642310960068</v>
+        <v>31.18096856414613</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.54365924678575</v>
+        <v>24.47026055461406</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.44317642294551</v>
+        <v>15.40204833746179</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.01568306839502</v>
+        <v>19.96237753709705</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.108278741671513</v>
+        <v>2.102663998569066</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.00629021595986</v>
+        <v>23.943409390233</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.70165061823413</v>
+        <v>15.66052253275041</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03058500427888498</v>
+        <v>0.03066667540748692</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2738211031063418</v>
+        <v>0.274239336134356</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1405847226146868</v>
+        <v>0.1408907887760404</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007283004511114735</v>
+        <v>0.007302452316076295</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3170293196148956</v>
+        <v>0.3006967619846748</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1853863456078985</v>
+        <v>0.1767349458132721</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2428531327.194058</v>
+        <v>2409323931.971454</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>566.08</v>
+        <v>567.12</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.005238568521670928</v>
+        <v>0.007085388955642369</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05846348319278805</v>
+        <v>-0.05673369592335709</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>496472538880</v>
+        <v>497384656320</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.08621636463482</v>
+        <v>31.14332784184514</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.44626626913062</v>
+        <v>25.48318886813402</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.15137071744149</v>
+        <v>14.177369561326</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>88.98281233291749</v>
+        <v>89.14629121368741</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.373899741115556</v>
+        <v>1.376423864438691</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.05229421595225</v>
+        <v>23.09353663953699</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.53195390588034</v>
+        <v>14.55795274976484</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.0331297276524202</v>
+        <v>0.03306897346149321</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2216415577772259</v>
+        <v>0.222112664274484</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1601245251166021</v>
+        <v>0.1604914641725943</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005953222159412097</v>
+        <v>0.005942304979545775</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3046042048111296</v>
+        <v>0.2866628186135127</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1871701356820057</v>
+        <v>0.1784030869831516</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1544259520.245494</v>
+        <v>1532806721.019979</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>375.01</v>
+        <v>378.17</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1147740987040462</v>
+        <v>0.1241676779470124</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1876218534725532</v>
+        <v>-0.18077639617001</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>340563232944</v>
+        <v>343432969261</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.11484791974793</v>
+        <v>24.31805028615523</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.20644836113594</v>
+        <v>17.3455235086315</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7565902951020707</v>
+        <v>0.762965659313219</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.451176114762258</v>
+        <v>3.480257249992381</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7306861882733021</v>
+        <v>-0.7368432730308916</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.95579835205527</v>
+        <v>15.06718818697357</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8559906892113149</v>
+        <v>0.8623660534224633</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06934688690802811</v>
+        <v>0.06876742221580859</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4015006126549587</v>
+        <v>0.4019784570960951</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01103056650619805</v>
+        <v>0.0123935693274897</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02415935575051332</v>
+        <v>0.02395747944046328</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4324875849547393</v>
+        <v>0.4390237538661194</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2090043499433815</v>
+        <v>0.1961586276094192</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1852949489.783638</v>
+        <v>1827730616.419602</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>162.05</v>
+        <v>160.39</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3212392823803414</v>
+        <v>0.3077048349335569</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.08140128110651312</v>
+        <v>-0.09081117850461995</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>671609743000</v>
+        <v>664729939400</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.85585585585586</v>
+        <v>20.64221364221364</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.61515531630501</v>
+        <v>14.38513754422254</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.860105641721598</v>
+        <v>1.841051180967152</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.607651147158609</v>
+        <v>2.580939015691263</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.042135885885887</v>
+        <v>2.021216752466754</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.793104671075531</v>
+        <v>9.697319030978072</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.948124253586661</v>
+        <v>1.929069792832216</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04549219292668898</v>
+        <v>0.04596302677080833</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4270019992595337</v>
+        <v>0.4349681105763297</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08838045201477529</v>
+        <v>0.09998999948518406</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02542425177414378</v>
+        <v>0.02568738699420164</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5553934121772781</v>
+        <v>-0.5522253949501161</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2618220565417985</v>
+        <v>0.2581899615884734</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2328993637.387376</v>
+        <v>2296226157.903534</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2717,55 +2717,55 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>270.68</v>
+        <v>270.07</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.305425570447623</v>
+        <v>0.3024836848337134</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.03696588038566895</v>
+        <v>-0.03913615825239269</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>175.91</v>
+        <v>177.32</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>652311303243</v>
+        <v>650841265209</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.29248554913295</v>
+        <v>31.22196531791908</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.82224884624353</v>
+        <v>21.76738335136334</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.661063660846123</v>
+        <v>6.646052397236773</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.773078673900507</v>
+        <v>7.755561391533582</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.874503802859757</v>
+        <v>-3.865772284758144</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.1863305835112</v>
+        <v>20.13775622414918</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.953254942284716</v>
+        <v>6.936523327645539</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02867955822165305</v>
+        <v>0.02875177847085937</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4339716208725948</v>
+        <v>0.4343462791986696</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09124654468564519</v>
+        <v>0.09145793518891288</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01950642825476578</v>
+        <v>0.01955048691080091</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1605160830141961</v>
+        <v>-0.1584050580200415</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1931232326667517</v>
+        <v>0.1918339198243154</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1701652822.237221</v>
+        <v>1682440243.509306</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>107.59</v>
+        <v>107.85</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.04584961013023348</v>
+        <v>-0.04354382798164969</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2039804675939627</v>
+        <v>-0.2020568215448357</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>856209827200</v>
+        <v>858278928000</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.84115523465704</v>
+        <v>38.93501805054152</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.60515195007061</v>
+        <v>34.67803195644259</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.163581522070015</v>
+        <v>1.16639341161122</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.711199942995583</v>
+        <v>8.73225126733036</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.392497538562528</v>
+        <v>9.415195274040046</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.43924524848853</v>
+        <v>21.4875447139289</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.248146101326375</v>
+        <v>1.25095799086758</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01577767454991435</v>
+        <v>0.01573963843138882</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1224096137678654</v>
+        <v>0.1227574303941448</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05202304971033023</v>
+        <v>0.05214708805768908</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009085416860303001</v>
+        <v>0.009063514140009273</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.04909827468557183</v>
+        <v>-0.05023922604558911</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3092427320528622</v>
+        <v>0.3076419708481803</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2809815948.429217</v>
+        <v>2777406450.32153</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>145.71</v>
+        <v>145.955</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.02764656816053734</v>
+        <v>0.02937447571114693</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1287892376681614</v>
+        <v>-0.1273243647234678</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>346383114210</v>
+        <v>346965530400</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.58666666666667</v>
+        <v>21.62296296296296</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.59820992672435</v>
+        <v>20.62951030420584</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.979951215759721</v>
+        <v>3.986643193308208</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.499281453112629</v>
+        <v>6.510209487949035</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.59984761904784</v>
+        <v>20.63448465608488</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.47751548931966</v>
+        <v>17.50491815187729</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.268167044420443</v>
+        <v>4.274859021968931</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04594046114601448</v>
+        <v>0.04586334550770695</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04798750684931496</v>
+        <v>0.0481568706240485</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02607311350629016</v>
+        <v>0.02615291896606742</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.0294461601811818</v>
+        <v>0.02939673186941181</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.03671320429147355</v>
+        <v>-0.03092617907907086</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1474675339672246</v>
+        <v>0.1493573806387046</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1285206366.136294</v>
+        <v>1250089853.271231</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>292.18</v>
+        <v>296.215</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1551096124809497</v>
+        <v>-0.1434416930010423</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2898082205099536</v>
+        <v>-0.2800004861330547</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>411.41</v>
@@ -3110,40 +3110,40 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>291337645060</v>
+        <v>295361012155</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20.4036312849162</v>
+        <v>20.69553002793296</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>19.47057988582075</v>
+        <v>19.7394682075378</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.722097963422708</v>
+        <v>1.746734640339055</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17.47769874225191</v>
+        <v>17.72773846422339</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-6.998920033779426</v>
+        <v>-7.099048090977034</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14.7112542362534</v>
+        <v>14.88553541768764</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.079607302808909</v>
+        <v>2.104243979725256</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05183332897775706</v>
+        <v>0.05110224999756584</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.0479210893854749</v>
+        <v>0.0484340211369052</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01423568777486173</v>
+        <v>0.01473211543034436</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03179546854678622</v>
+        <v>0.03136235504616579</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.6929312628780876</v>
+        <v>0.7097058976024576</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2264373562986717</v>
+        <v>0.2387004247155522</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1344065075.865914</v>
+        <v>1350336960.088204</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3221,55 +3221,55 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>629.26</v>
+        <v>631.5401000000001</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.815858936602999</v>
+        <v>1.826062095808016</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.002425529891088907</v>
+        <v>-0.01159699507003675</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>630.79</v>
+        <v>638.95</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>154.78</v>
+        <v>157.05</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>1026071356000</v>
+        <v>1029789287060</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>159.7106598984771</v>
+        <v>160.2893654822335</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.74982351063699</v>
+        <v>45.84034202054882</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>24.84133533470524</v>
+        <v>24.93134698123714</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>15.26721200761633</v>
+        <v>15.32253217749613</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.289407162483118</v>
+        <v>1.294079280957481</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>95.65789848852398</v>
+        <v>96.00478513342041</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>24.82172511802445</v>
+        <v>24.91173676455635</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.008189488918936356</v>
+        <v>0.00815992174864255</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.490956852791877</v>
+        <v>2.496687817258883</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9237817525864558</v>
+        <v>0.9263308665560739</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.576018985711944</v>
+        <v>2.57542051915521</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6749100291172855</v>
+        <v>0.6354866964637982</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10684692728.66114</v>
+        <v>10603688172.86188</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1722.5</v>
+        <v>1744.325</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4800907015397822</v>
+        <v>0.4988442455520352</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1387327746554932</v>
+        <v>-0.127820056401128</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>663882489498</v>
+        <v>672294237151</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.54281567489114</v>
+        <v>55.24673367198839</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.03933144996278</v>
+        <v>35.38525566330379</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.39969780117472</v>
+        <v>16.61134877041965</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.5439936954191</v>
+        <v>26.88656484151493</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.712928783761004</v>
+        <v>3.760847054214961</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.62938346705784</v>
+        <v>42.17102565735811</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.26701080096242</v>
+        <v>16.47866177020735</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01726369512105955</v>
+        <v>0.01704373238018761</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5566169049994556</v>
+        <v>0.5612924828824084</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3016706021814304</v>
+        <v>0.3053450603513164</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004516690856313498</v>
+        <v>0.00446017800581887</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.651996506580348</v>
+        <v>1.65358269024515</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.437899388451972</v>
+        <v>0.3971516486250771</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2150216026.780436</v>
+        <v>2085731297.082227</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>196.8</v>
+        <v>200.935</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1359705127608211</v>
+        <v>-0.1178162346625793</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2262630233929623</v>
+        <v>-0.2100058973854924</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>155544816000</v>
+        <v>158812994020</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>73.7078651685393</v>
+        <v>75.25655430711608</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>75.02654866313839</v>
+        <v>76.20927701201983</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.654820107452524</v>
+        <v>1.689589808181286</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>25.52091998636066</v>
+        <v>26.05714460091148</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3944899253009337</v>
+        <v>0.4027786236806052</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>27.94184402877698</v>
+        <v>28.4120854705036</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.066022831001649</v>
+        <v>2.100792531730411</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001350093210435248</v>
+        <v>-0.00132230993626097</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.01757622492432453</v>
+        <v>-0.01250140064645278</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1573530140270649</v>
+        <v>0.1577782107735839</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.22063201693637</v>
+        <v>1.235555250187288</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3474316412516655</v>
+        <v>0.3308421728170492</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1253088267.691053</v>
+        <v>1244533216.344474</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>923.29</v>
+        <v>930.78998</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.009788451649996421</v>
+        <v>0.01799106750374335</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1999150772537024</v>
+        <v>-0.1934159048171995</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>272377013030</v>
+        <v>274589559048</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>14.06596587446679</v>
+        <v>14.18022516758074</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.75095534125784</v>
+        <v>12.94895017364616</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.309512816418935</v>
+        <v>2.328273222551023</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.257412531977644</v>
+        <v>2.275749727053494</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3296867498136609</v>
+        <v>0.332364829322664</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.3429749635269</v>
+        <v>26.41345392437805</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.012091311717272</v>
+        <v>7.03085171784936</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1524174141502443</v>
+        <v>-0.1511892882742235</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1031303536099775</v>
+        <v>0.09508685858105248</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3820176201656539</v>
+        <v>-0.3855660834560499</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01949549978879875</v>
+        <v>0.01933841187246128</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.582001578200555</v>
+        <v>1.578150848072844</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3136271706913739</v>
+        <v>0.3098960578833395</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2014615966.992969</v>
+        <v>1991840169.872546</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>227.06</v>
+        <v>227.17</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2210634648370498</v>
+        <v>-0.2206861063464838</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3170306202249894</v>
+        <v>-0.316699753353787</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>213920946040</v>
+        <v>214024580780</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>19.83056768558952</v>
+        <v>19.84017467248908</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.57287411434003</v>
+        <v>17.57826960599472</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.095951286452379</v>
+        <v>3.097451130729265</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.194522640195054</v>
+        <v>6.19752359804946</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2417330828340274</v>
+        <v>0.2418501912596054</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>16.76967795080451</v>
+        <v>16.77606687503853</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.936798211789224</v>
+        <v>3.93829805606611</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06371980047924436</v>
+        <v>0.06368894614965544</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1284760567087397</v>
+        <v>0.1286762074534906</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04696817070189807</v>
+        <v>0.04707569284926238</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02968378402184445</v>
+        <v>0.02966941057357926</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8847492074191293</v>
+        <v>0.882749406281232</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.330742388938541</v>
+        <v>0.3059815948123619</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1261569169.501882</v>
+        <v>1222679221.431328</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3853,55 +3853,55 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1183.86</v>
+        <v>1162.245</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.09580141439129397</v>
+        <v>0.07579419430440226</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.08416044559625591</v>
+        <v>-0.1008819092561793</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>712.05</v>
+        <v>716.08</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1114889500260</v>
+        <v>1094533768545</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>39.60722649715624</v>
+        <v>38.89528136500502</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.81900700828036</v>
+        <v>26.31371491257727</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.99458111586151</v>
+        <v>13.74302662365783</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>31.18382077393075</v>
+        <v>30.62328747318398</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4186971775611286</v>
+        <v>0.4111710404449257</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.80782500461843</v>
+        <v>26.3450520587787</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.57221919895363</v>
+        <v>14.32066470674995</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01798734313608953</v>
+        <v>0.01831658625644434</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4768341902042652</v>
+        <v>0.4781372183375783</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2366666761671541</v>
+        <v>0.2374937896030991</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005651006031118545</v>
+        <v>0.005756101338358092</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3615639490502712</v>
+        <v>0.3519843123169681</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3162684387679197</v>
+        <v>0.3162587251728303</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2838472646.784391</v>
+        <v>2803958568.568034</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>196.34</v>
+        <v>196.86501</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.07938431329323259</v>
+        <v>0.08227056957479584</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1546178686759957</v>
+        <v>-0.1523573304628633</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>309683155200</v>
+        <v>310511235864</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>15.78295819935691</v>
+        <v>15.8251615755627</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.56742266065501</v>
+        <v>14.62890900848772</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.447527090232279</v>
+        <v>2.454071682096595</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.793502268672396</v>
+        <v>2.800972048778721</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4015436373796503</v>
+        <v>0.4026173586033474</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>22.97083706000614</v>
+        <v>22.99905393614339</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.327831210236389</v>
+        <v>5.334375802100705</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.05064531194753211</v>
+        <v>-0.05051024951274032</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.0834420451041713</v>
+        <v>0.08177319076774014</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3264761898088444</v>
+        <v>-0.3272042798206312</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.0211368035041255</v>
+        <v>0.02108043476085466</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.386033743939316</v>
+        <v>1.371397666966507</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2687086733205608</v>
+        <v>0.2611419043364485</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>928573209.9117961</v>
+        <v>939847234.6253</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4105,55 +4105,55 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1080.53</v>
+        <v>1080.34</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.425686240570652</v>
+        <v>2.425083869155042</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1390199203187251</v>
+        <v>-0.1391713147410359</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>154.65</v>
+        <v>155.18</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1220339776700</v>
+        <v>1220125192600</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>24.11359071635795</v>
+        <v>24.10667194822584</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.850455816864536</v>
+        <v>6.8259139833998</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>13.51817551786782</v>
+        <v>13.51429683753905</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>12.10076883364441</v>
+        <v>12.09729683253247</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03436893730352907</v>
+        <v>0.03435907603023521</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>17.58289843882597</v>
+        <v>17.57777533011442</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>13.31192565633516</v>
+        <v>13.30804697600638</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02144648605224801</v>
+        <v>0.02145264131615646</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.51999799151975</v>
+        <v>2.531640159376719</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.791598046203779</v>
+        <v>1.800718448984278</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0004905000323915116</v>
+        <v>0.0004905862969065295</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.852771197448738</v>
+        <v>2.856482916504727</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.761275794500771</v>
+        <v>0.7215175127503144</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25559606799.82983</v>
+        <v>24819004906.63231</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4231,55 +4231,55 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>137.78</v>
+        <v>136.27</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.06558153372927189</v>
+        <v>-0.07582229352074232</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2859882051760414</v>
+        <v>-0.3556364668053715</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>192.966</v>
+        <v>211.48</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>142445506360</v>
+        <v>140884374740</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>85.57763975155281</v>
+        <v>84.63975155279505</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.92642380155584</v>
+        <v>28.59387777686755</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.669122071680695</v>
+        <v>9.563153322020092</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.37158357302653</v>
+        <v>11.24695669542985</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>136.9242236024874</v>
+        <v>135.423602484475</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>42.53238932645457</v>
+        <v>42.08494546861565</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.07300477599783</v>
+        <v>9.967036026337226</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03215264641922116</v>
+        <v>0.03250892803728108</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.958459031736579</v>
+        <v>1.960065515187612</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2511635155641063</v>
+        <v>0.2517284142448271</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6896999038513897</v>
+        <v>0.6814482751173407</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5581887768814184</v>
+        <v>0.5503333447217786</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2116630521.891403</v>
+        <v>2039077927.823326</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4357,55 +4357,55 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.43</v>
+        <v>28.285</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.129070677340547</v>
+        <v>0.1233121388877021</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.02670318384115034</v>
+        <v>-0.03166723724751797</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>23.58</v>
+        <v>23.61</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>162035079200</v>
+        <v>161208660400</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>37.56606765327696</v>
+        <v>37.37447145877379</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.744097745161534</v>
+        <v>9.695109909778507</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.543881549861844</v>
+        <v>2.530907127606129</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.901896584106116</v>
+        <v>1.892196443244512</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6283174147318005</v>
+        <v>-0.6251128412131192</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.76402718631179</v>
+        <v>17.69856308618504</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.520677581009796</v>
+        <v>3.507703158754082</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06780013349109407</v>
+        <v>0.06814770355848698</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.855263836195662</v>
+        <v>2.854981718265806</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05128062324801363</v>
+        <v>-0.05138743178845229</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06049947238832219</v>
+        <v>0.06080961640445465</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3404255456657939</v>
+        <v>0.343018398851778</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.1993484271494589</v>
+        <v>0.192025001341619</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>947418636.0117925</v>
+        <v>920907628.5617445</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>186.37</v>
+        <v>191.62</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.1092792458392531</v>
+        <v>0.1405273868525925</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.06754390353729922</v>
+        <v>-0.04127682993946069</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,13 +4498,13 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1322956560357</v>
+        <v>1360223942134</v>
       </c>
       <c r="L32" s="6" t="n">
         <v>8.13560720204846</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004313123162106954</v>
+        <v>0.0044406287409169</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.987077813549424</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1885.245047098128</v>
+        <v>1831.084526023363</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2500.190092304088</v>
+        <v>2429.751019160868</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.609701132156463</v>
+        <v>1.565598580523954</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.8071407005663245</v>
+        <v>0.7682407773246638</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3482514633.031157</v>
+        <v>3352281949.910736</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4611,22 +4611,22 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>600.52</v>
+        <v>608.54</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6086793989745505</v>
+        <v>0.6301634607539681</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1061429230608935</v>
+        <v>-0.09420537933703477</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>313.6</v>
+        <v>315.05</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>75689989989</v>
+        <v>76700836788</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.815691267313214</v>
+        <v>1.817606464034989</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.3955966239423021</v>
+        <v>0.3851697340638614</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3867187445.319987</v>
+        <v>3785548050.069753</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>148.03</v>
+        <v>149.25</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.08027335938625058</v>
+        <v>-0.07269336545563676</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3439549725226023</v>
+        <v>-0.3385481297642262</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1951298885258</v>
+        <v>1967380656791</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-96.12337662337663</v>
+        <v>-96.91344155844156</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>128.4890965732087</v>
+        <v>129.0019891543726</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>117.7254229416591</v>
+        <v>118.6930411412971</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.822988744262089</v>
+        <v>6.879068798339936</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9612337662337663</v>
+        <v>-0.9691344155844156</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>455.2773902706984</v>
+        <v>459.1262675586754</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>114.457971961267</v>
+        <v>115.425590160905</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01456619496620166</v>
+        <v>-0.01444744735291915</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.33586892291163</v>
+        <v>4.34594431755497</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.17507527356193</v>
+        <v>3.160454921684557</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7556669113243399</v>
+        <v>0.7541834967136585</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12969216400.05274</v>
+        <v>12541582768.92705</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>767.1799999999999</v>
+        <v>771.61902</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1229708845403001</v>
+        <v>0.1294685646360954</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01564083811283479</v>
+        <v>-0.009945186496785885</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>817229462223</v>
+        <v>821958074473</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9959052235771121</v>
+        <v>0.9958558868321901</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1173038786893492</v>
+        <v>0.1178604417442342</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>31416923259.33358</v>
+        <v>30906501351.84806</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>451.15</v>
+        <v>453.17</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.411564158434371</v>
+        <v>0.4178843614711381</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.05814196242171199</v>
+        <v>-0.05392484342379955</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,13 +4914,13 @@
         <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2339880452000</v>
+        <v>2350357141600</v>
       </c>
       <c r="L36" s="6" t="n">
         <v>28.68899965225455</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6913520399194388</v>
+        <v>0.6939774782506954</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.45395915587732</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.49694800292713</v>
+        <v>40.33995778158497</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.58132128789313</v>
+        <v>40.42758248836358</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2659869223096531</v>
+        <v>0.264801288699605</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.171388878656856</v>
+        <v>2.185311310836871</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3334890498278422</v>
+        <v>0.3296867461108848</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4148484555.274498</v>
+        <v>4075911765.463005</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>30.84</v>
+        <v>30.845</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.08172570159286696</v>
+        <v>0.08190107865213947</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.002587322121604174</v>
+        <v>-0.002425614489004024</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30.92</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>77320095890</v>
+        <v>77332631573</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-24.28346456692913</v>
+        <v>-24.28740157480315</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-100.9067796284266</v>
+        <v>-101.9734182054428</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.140941323272878</v>
+        <v>2.141288427883151</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.358220354467385</v>
+        <v>2.358602685912662</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.180714154916682</v>
+        <v>0.1807434535799305</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>17.51637948595041</v>
+        <v>17.51845149966942</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.934351263740828</v>
+        <v>2.934698368351101</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.0281944813299429</v>
+        <v>0.02818991098139647</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02124338466777553</v>
+        <v>0.02131705948114759</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2830275584281875</v>
+        <v>0.2831904392030636</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2944126767979008</v>
+        <v>0.2882104855849396</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>886916354.4684997</v>
+        <v>962123292.8515366</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>305.675</v>
+        <v>309.38</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1799023663506069</v>
+        <v>-0.1699621954741172</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.2111409326692302</v>
+        <v>-0.2015793955973058</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>206425384250</v>
+        <v>208927407800</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.53699211643421</v>
+        <v>18.76167374166161</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.68533137598406</v>
+        <v>15.86983837770977</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.455311268183602</v>
+        <v>2.485071399854888</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.045730746791132</v>
+        <v>6.119009334889149</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.149455406346578</v>
+        <v>1.163387629395613</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>8.907595221242518</v>
+        <v>9.008793391037049</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.619525700878998</v>
+        <v>2.649285832550284</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07291738879250748</v>
+        <v>0.07204416193402846</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1818043031476113</v>
+        <v>0.182222105551725</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.007849575618025462</v>
+        <v>0.008004944927378022</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01158092745563098</v>
+        <v>0.01144223931734437</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9687967220792345</v>
+        <v>0.9619056895541279</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2261276737926173</v>
+        <v>0.2080481476155209</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>870611751.3417327</v>
+        <v>890849513.9410889</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>139.53</v>
+        <v>138.25</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2870574052761836</v>
+        <v>-0.293597694255231</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5674024927140819</v>
+        <v>-0.5713709927450858</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>322.54</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>401911979100</v>
+        <v>398224977500</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>21.5324074074074</v>
+        <v>21.33487654320988</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.41248576143939</v>
+        <v>15.25779032484425</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.599453572871533</v>
+        <v>5.548086120902239</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.197897022704127</v>
+        <v>6.1410396573414</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4686465141612202</v>
+        <v>0.464347312999274</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>13.8248668902439</v>
+        <v>13.7271202942736</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.265196080917286</v>
+        <v>7.213828628947992</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.07145843242670345</v>
+        <v>-0.07212003671969572</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3970755750042281</v>
+        <v>0.3982939920514121</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.441467333100293</v>
+        <v>0.44303189055986</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01433383501755895</v>
+        <v>0.01446654611211573</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.053552869674012</v>
+        <v>2.035959977467106</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5380484765925413</v>
+        <v>0.5389614281883208</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4302756336.46116</v>
+        <v>4219305478.389789</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>106.97</v>
+        <v>107.695</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4067595832729238</v>
+        <v>0.4162940387078389</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1794891462759838</v>
+        <v>-0.173928050931963</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>421615266115</v>
+        <v>424472806247</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>31.83630952380952</v>
+        <v>32.05208333333333</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.67709848356894</v>
+        <v>20.81233774095547</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.657959196446901</v>
+        <v>6.703084188661666</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.409116237446556</v>
+        <v>8.466109873719796</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.018761904761905</v>
+        <v>1.025666666666667</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>22.17544663145012</v>
+        <v>22.31818803371797</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>7.010347668614292</v>
+        <v>7.055472660829057</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.0322450373423903</v>
+        <v>0.03202796457139611</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5396894080234833</v>
+        <v>0.540052046640574</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1678690289898708</v>
+        <v>0.1647734682617721</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01551836963634664</v>
+        <v>0.01541390036677654</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.708965770644159</v>
+        <v>0.6981618134185805</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3532923468035524</v>
+        <v>0.3529606354509493</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>2096051407.181834</v>
+        <v>1887371559.469777</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>82.19</v>
+        <v>82.995</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.1366596361900662</v>
+        <v>-0.1282037535660608</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1592675941080197</v>
+        <v>-0.1510331423895254</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>248542560000</v>
+        <v>250976880000</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>11.7246790299572</v>
+        <v>11.839514978602</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.54844316443893</v>
+        <v>10.63660916086357</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>1.925119553851516</v>
+        <v>1.943974904147787</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.390969620678173</v>
+        <v>1.404593304151174</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6232036601508798</v>
+        <v>0.6293075529166842</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.22159186260602</v>
+        <v>15.29506745947904</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>3.906173734557143</v>
+        <v>3.925029084853414</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.07712964733283507</v>
+        <v>0.07638153761414199</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1115080061751315</v>
+        <v>0.1130910988216443</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2897189042510264</v>
+        <v>-0.2891645749529771</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.02250882102445553</v>
+        <v>0.02229049942767636</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.740829605769277</v>
+        <v>0.7234626246998377</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.2596937577941547</v>
+        <v>0.2444670841790083</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1142531373.058048</v>
+        <v>1123044820.445852</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 17:43 ET</t>
+          <t>2026-09-25 12:12 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-26)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>38.93493150684932</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.51662213509418</v>
+        <v>35.52036130733035</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.7308691108193</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09624533996372042</v>
+        <v>0.09612993995121033</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1214925120824444</v>
+        <v>0.121704693985192</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003107866420382913</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3019846105116222</v>
+        <v>0.3019845712332221</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.2784776666105622</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13392913772.22273</v>
+        <v>13396328030.79305</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>28.67611111111111</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.02307018292088</v>
+        <v>25.01062080253352</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.55031850837304</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1459869193302892</v>
+        <v>0.1465573500761037</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2316438618911127</v>
+        <v>0.2322711917691311</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007051940252242479</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5559010507592201</v>
+        <v>0.5559009439283675</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4313552623124653</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10849661708.76946</v>
+        <v>10852564562.72502</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>16.93545183714002</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.74032382575059</v>
+        <v>20.75909794040633</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.283761507556081</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1834528727987628</v>
+        <v>-0.1841913417549715</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2984615599989464</v>
+        <v>0.2991646553014995</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002500581530588509</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7623052618179443</v>
+        <v>0.7623052681932441</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.3206523161285895</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8493374256.251143</v>
+        <v>8500131780.098979</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>19.81507936507936</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.30135223851277</v>
+        <v>22.31307595972942</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.462413826577971</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.111485296803653</v>
+        <v>-0.1119521395955644</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1829953111798719</v>
+        <v>0.183423614078758</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8343667788695565</v>
+        <v>0.8343667953128601</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4529088218280257</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8727941809.214376</v>
+        <v>8738257341.305389</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>28.31069182389937</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.576603144338</v>
+        <v>16.55501180290884</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>17.99332760117372</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.707870519514086</v>
+        <v>0.7100979546825186</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.963210356196486</v>
+        <v>0.9657347796573699</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1292,13 +1292,13 @@
         <v>0.00231039232238859</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.305861067803973</v>
+        <v>1.305861092676486</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.389194698065552</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26586020523.2412</v>
+        <v>26600098382.11532</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>27.93236714975846</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>22.7069310922073</v>
+        <v>22.61203173100634</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>8.389312305939155</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2301251558976396</v>
+        <v>0.2352878096954334</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2783344562737575</v>
+        <v>0.2795409325493587</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.002793816353138387</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8266592408905271</v>
+        <v>0.8266593683881774</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.4905097236598456</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>13478667019.444</v>
+        <v>13481261198.45398</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>315.3474576271187</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>173.3800513463268</v>
+        <v>173.2476662709221</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>14.18336483445121</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8188220338983052</v>
+        <v>0.8202118644067795</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1273363645261019</v>
+        <v>0.1277148676316173</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.52754997722397</v>
+        <v>1.527550059420665</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.409613927618917</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13772055498.52661</v>
+        <v>13786592185.9667</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>43.77295285359801</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.11331233547746</v>
+        <v>19.0918516570777</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>18.83778281334171</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.290181423569801</v>
+        <v>1.292755759883069</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8706498006139045</v>
+        <v>0.8727329956474132</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1670,13 +1670,13 @@
         <v>0.007369405629092146</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.596157963974802</v>
+        <v>1.596157977234559</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.3896621793452344</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9298018803.745872</v>
+        <v>9303515124.854837</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -1730,19 +1730,19 @@
         <v>33.39721317408615</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.44202341150788</v>
+        <v>40.2062941580495</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.349897739878082</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.44205747586329</v>
+        <v>11.44274476650001</v>
       </c>
       <c r="P10" s="6" t="n">
         <v>0.6497858639947462</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>33.69121946384253</v>
+        <v>27.41708332300299</v>
       </c>
       <c r="R10" s="6" t="n">
         <v>1.298620171381542</v>
@@ -1754,10 +1754,10 @@
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1741952959608127</v>
+        <v>-0.1693536080991972</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.08464992278891481</v>
+        <v>0.08879643901584977</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1787,22 +1787,22 @@
         <v>0.05235555056432141</v>
       </c>
       <c r="AF10" s="6" t="n">
-        <v>-1.330338040222508</v>
+        <v>-1.08259628107807</v>
       </c>
       <c r="AG10" s="6" t="n">
-        <v>0</v>
+        <v>80.58620689655173</v>
       </c>
       <c r="AH10" s="4" t="n">
         <v>0.006003695415409124</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1725163712655465</v>
+        <v>-0.1725160043142916</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1814059591717962</v>
+        <v>0.1814114731558173</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1974746146.924369</v>
+        <v>1975564704.342651</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>22.02631578947368</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>18.97248472532664</v>
+        <v>18.96959836222817</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.124433164400712</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1609610500869421</v>
+        <v>0.1611376987997795</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1463927862518444</v>
+        <v>0.1467198881572687</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.09973413764675718</v>
+        <v>0.09973998985696915</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3518704001679435</v>
+        <v>0.3518610586434247</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2374313889.873726</v>
+        <v>2374414112.674433</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.71461718493059</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.78657634189573</v>
+        <v>22.78654971920524</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.835764692303093</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4420128327240933</v>
+        <v>-0.442012180799171</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06172391298215096</v>
+        <v>0.06176934337546847</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2054,7 +2054,7 @@
         <v>0.1347616100089321</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2218904648.615773</v>
+        <v>2220159570.140381</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>14.74892519346518</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.69689531519208</v>
+        <v>13.69973006202843</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.088477086210198</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.0768079082203561</v>
+        <v>0.07658509523080359</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2888815034896199</v>
+        <v>-0.2884346927984077</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.1854938933482376</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2460538893.101328</v>
+        <v>2478789947.98411</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.21325403568394</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.49559760913927</v>
+        <v>24.48756025996492</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.41799596243931</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.274239336134356</v>
+        <v>0.2746575691623703</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1408907887760404</v>
+        <v>0.1411968549373943</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2306,7 +2306,7 @@
         <v>0.1766630962178798</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2445792406.227669</v>
+        <v>2445815294.001974</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.17243272926963</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.5070040926017</v>
+        <v>25.497175305699</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.19061897215175</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.222112664274484</v>
+        <v>0.222583770771742</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1604914641725943</v>
+        <v>0.1608584032285862</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.1784708934114141</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1564249896.078393</v>
+        <v>1564935163.187866</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>24.21644910295158</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.27305364813585</v>
+        <v>17.26707296067751</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7597779772065341</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4019784570960954</v>
+        <v>0.4024640515563904</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.0123935693274897</v>
+        <v>0.01247397052279386</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.1949010994954906</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1859764030.596038</v>
+        <v>1859810112.65859</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.66409266409266</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.4003845881936</v>
+        <v>14.17577945234648</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.84300254140586</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4349681105763297</v>
+        <v>0.457704158953474</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.09998999948518406</v>
+        <v>0.1135744714993598</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2578079794257925</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2334920119.138839</v>
+        <v>2337218226.222433</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>177.32</v>
+        <v>179.8</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>653612648388</v>
@@ -2738,7 +2738,7 @@
         <v>31.35491329479769</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.86007224999728</v>
+        <v>21.85425218979131</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.674352320436235</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4343462791986696</v>
+        <v>0.434728263520469</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09145793518891288</v>
+        <v>0.09166935202478976</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2810,7 +2810,7 @@
         <v>0.191741468346202</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1708166413.992211</v>
+        <v>1708404011.753947</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>38.98194945848376</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.71983208768355</v>
+        <v>34.70947884306728</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.167799356381822</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1227574303941448</v>
+        <v>0.1230923297561941</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05214708805768908</v>
+        <v>0.05227112640504772</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2936,7 +2936,7 @@
         <v>0.3077459276137968</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2817964186.638368</v>
+        <v>2821016151.449915</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.66222222222222</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.66696582289732</v>
+        <v>20.6636269430437</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.993881454729295</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.0481568706240485</v>
+        <v>0.04832623439878225</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02615291896606742</v>
+        <v>0.0262327244258449</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.1495866310155668</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1270649220.102621</v>
+        <v>1271269678.848826</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -3101,10 +3101,10 @@
         <v>-0.1521601012369582</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2873289419314067</v>
+        <v>-0.2865312081761772</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>411.41</v>
+        <v>410.95</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>289.1</v>
@@ -3188,7 +3188,7 @@
         <v>0.2352095735933773</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1384358548.704777</v>
+        <v>1385051008.94694</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -3227,13 +3227,13 @@
         <v>1.821989513380716</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.0130213631739573</v>
+        <v>-0.01309859154929582</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>638.95</v>
+        <v>639</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>157.05</v>
+        <v>159.33</v>
       </c>
       <c r="K22" s="5" t="n">
         <v>1028305278000</v>
@@ -3242,7 +3242,7 @@
         <v>160.0583756345177</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.77428240648329</v>
+        <v>45.64730520466372</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>24.8954189081225</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.496687817258883</v>
+        <v>2.506414560878937</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9263308665560739</v>
+        <v>0.9293741779367319</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.576337754824986</v>
+        <v>2.57633782396688</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.6355259972551116</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10753238007.96615</v>
+        <v>10754885318.6439</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>55.24673439767779</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.37744558007368</v>
+        <v>35.34375703947268</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.61134903678438</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5616371813117982</v>
+        <v>0.5631256840062882</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3056332551042853</v>
+        <v>0.3066425281046585</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004461162654678487</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.653708994698487</v>
+        <v>1.653708998784613</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.3971159842269665</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2105264462.521533</v>
+        <v>2105351252.599284</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>74.18352059925091</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>75.12265905775881</v>
+        <v>74.73857231422116</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.665499078674398</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.01250140064645255</v>
+        <v>-0.007426576368580684</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1577782107735839</v>
+        <v>0.1582034075201026</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,7 +3568,7 @@
         <v>0.3265156952935771</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1265873706.105656</v>
+        <v>1266194328.628845</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>14.25121876904327</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.01377937044112</v>
+        <v>13.01213384565608</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.339929777338749</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09508685858105248</v>
+        <v>0.09522534413529993</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3855660834560498</v>
+        <v>-0.3855268961990271</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.3111826575726561</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2030201186.23431</v>
+        <v>2031486619.277751</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>19.69519650655022</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.44981986550983</v>
+        <v>17.44672599750871</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.074817117096256</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1286762074534906</v>
+        <v>0.1288763581982413</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04707569284926238</v>
+        <v>0.0471832149966267</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.3064314291585977</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1242529633.914498</v>
+        <v>1242825112.1433</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.60254265640683</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.79991793151699</v>
+        <v>26.78272248176846</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.99292615551466</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4777113406692117</v>
+        <v>0.4786600833192023</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2371372497922744</v>
+        <v>0.2376078234173944</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3946,7 +3946,7 @@
         <v>0.3139587734725938</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2853154336.569304</v>
+        <v>2853729577.00765</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>15.78054662379421</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.58766658156381</v>
+        <v>14.58531957976789</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.447153117467142</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08177319076774014</v>
+        <v>0.08194726467867675</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3272042798206313</v>
+        <v>-0.3271051416963593</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.2609535691634336</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>956798539.7301921</v>
+        <v>956808924.5290629</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>155.18</v>
+        <v>159.97</v>
       </c>
       <c r="K29" s="5" t="n">
         <v>1222316209200</v>
@@ -4126,7 +4126,7 @@
         <v>24.15264449899576</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.8381714885628</v>
+        <v>6.831530326419744</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>13.54006922480448</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.532032582012943</v>
+        <v>2.535466190582459</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.801029652513459</v>
+        <v>1.804235300496267</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4192,13 +4192,13 @@
         <v>0.0004897069150312304</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.857958739358943</v>
+        <v>2.857958824207671</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>0.721414067327511</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25141540468.57701</v>
+        <v>25155134915.873</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>84.2360248447205</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.45748663754881</v>
+        <v>28.44205059960733</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.517537635080098</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.960065515187612</v>
+        <v>1.961671998638645</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2517284142448271</v>
+        <v>0.2522933129255482</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.5513107222422996</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2059704671.221231</v>
+        <v>2062078409.913101</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -4369,7 +4369,7 @@
         <v>29.21</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>23.61</v>
+        <v>23.62</v>
       </c>
       <c r="K31" s="5" t="n">
         <v>163402944800</v>
@@ -4378,7 +4378,7 @@
         <v>37.88319238900635</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.827074460433085</v>
+        <v>9.827228116235348</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.565356455664406</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.854981718265806</v>
+        <v>2.854921442845145</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.0513874317884524</v>
+        <v>-0.0514940475070369</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.1918027931372212</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>939376654.2967064</v>
+        <v>939924699.5058314</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>8.13560720204846</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004439238292506218</v>
+        <v>0.00443531895025063</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.987077813549424</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1831.658367491108</v>
+        <v>1833.277826082549</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2430.51237362393</v>
+        <v>2432.935291707406</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4574,7 +4574,7 @@
         <v>0.7681477162484222</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3390494952.520805</v>
+        <v>3391219023.770243</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.817502974092652</v>
+        <v>1.817502989459575</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.3847343199442911</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3827303276.204826</v>
+        <v>3828740338.151042</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-96.54545454545455</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>128.5093182410192</v>
+        <v>127.9699106279624</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>118.2423554885671</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.346062521952933</v>
+        <v>4.356256120994235</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4782,7 +4782,7 @@
         <v>0.7541715269041857</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12672801786.38165</v>
+        <v>12673550841.14075</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -4866,7 +4866,7 @@
         <v>0.1177761963223539</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>31431973023.48468</v>
+        <v>31467728797.33297</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
         <v>28.68899965225455</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.690057134131884</v>
+        <v>0.6898227636857688</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.45395915587732</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.5748178422158</v>
+        <v>40.58894307715698</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.66294036140282</v>
+        <v>40.679954423938</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4990,7 +4990,7 @@
         <v>0.3298638145831211</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4147558160.561589</v>
+        <v>4147654996.64744</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
         <v>-24.29921259842519</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-102.0230081316247</v>
+        <v>-103.5919722461546</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>2.142329741769348</v>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02131705948114759</v>
+        <v>0.02136127112348496</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2833935460219251</v>
+        <v>0.2833935561927062</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2881687054257782</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>977331519.8900317</v>
+        <v>977437636.1167971</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
         <v>18.7319587628866</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.84470352476169</v>
+        <v>15.83910591624148</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.481135511995528</v>
@@ -5200,10 +5200,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.182222105551725</v>
+        <v>0.1826399079558387</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.008004944927378022</v>
+        <v>0.008237808786623502</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5248,7 +5248,7 @@
         <v>0.2074093233923537</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>910437467.8181722</v>
+        <v>912131760.4375204</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
         <v>21.15432098765432</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.12866472137179</v>
+        <v>15.11533578334685</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>5.501133059336556</v>
@@ -5326,10 +5326,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3982939920514124</v>
+        <v>0.3995270294266873</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.44303189055986</v>
+        <v>0.4445965742942801</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5374,7 +5374,7 @@
         <v>0.5405225003117969</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4276647851.485573</v>
+        <v>4277747868.814545</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
         <v>31.75595238095238</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.62005141334276</v>
+        <v>20.61519711858666</v>
       </c>
       <c r="N40" s="6" t="n">
         <v>6.641154026940387</v>
@@ -5452,10 +5452,10 @@
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5400520466405743</v>
+        <v>0.5404146852576648</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1647734682617721</v>
+        <v>0.1649876396295691</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5494,13 +5494,13 @@
         <v>0.01555763823805061</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.6974249401180137</v>
+        <v>0.697424970031328</v>
       </c>
       <c r="AJ40" s="4" t="n">
         <v>0.3523286318801636</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>1929638221.738618</v>
+        <v>1946576732.440821</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
         <v>11.83594864479315</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.63340516991205</v>
+        <v>10.63083041321805</v>
       </c>
       <c r="N41" s="6" t="n">
         <v>1.943389334262809</v>
@@ -5578,10 +5578,10 @@
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1130910988216443</v>
+        <v>0.1133606862994156</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2891645749529771</v>
+        <v>-0.2890798197180271</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5626,7 +5626,7 @@
         <v>0.2443852021271254</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1138961830.267982</v>
+        <v>1139280111.489665</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 17:47 ET</t>
+          <t>2026-09-26 11:25 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-27)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>38.93493150684932</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.52036130733035</v>
+        <v>35.5125142905931</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.7308691108193</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09612993995121033</v>
+        <v>0.09637214611872147</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.121704693985192</v>
+        <v>0.1219765024388257</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>28.67611111111111</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.01062080253352</v>
+        <v>24.9981838035207</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.55031850837304</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1465573500761037</v>
+        <v>0.1471277808219178</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2322711917691311</v>
+        <v>0.2328985216471497</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>16.93545183714002</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.75909794040633</v>
+        <v>20.77790607446563</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.283761507556081</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1841913417549715</v>
+        <v>-0.1849298107111804</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2991646553014995</v>
+        <v>0.2998677506040526</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>19.81507936507936</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.31307595972942</v>
+        <v>22.32481201364503</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.462413826577971</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1119521395955644</v>
+        <v>-0.1124189823874756</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.183423614078758</v>
+        <v>0.1838519169776447</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>28.31069182389937</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.55501180290884</v>
+        <v>16.53347663458033</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>17.99332760117372</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7100979546825186</v>
+        <v>0.7123253898509516</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9657347796573699</v>
+        <v>0.9759286917850041</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>27.93236714975846</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>22.61203173100634</v>
+        <v>22.59968127350366</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>8.389312305939155</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2352878096954334</v>
+        <v>0.2359628798175555</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2795409325493587</v>
+        <v>0.2806438403193861</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>315.3474576271187</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>173.2476662709221</v>
+        <v>174.58508291529</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>14.18336483445121</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8202118644067795</v>
+        <v>0.8062680520083585</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1277148676316173</v>
+        <v>0.126650182634036</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>43.77295285359801</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.0918516570777</v>
+        <v>19.07043911729104</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>18.83778281334171</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.292755759883069</v>
+        <v>1.295330096196336</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8727329956474132</v>
+        <v>0.874816190680922</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>33.39721317408615</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.2062941580495</v>
+        <v>40.1959343219621</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.349897739878082</v>
@@ -1754,10 +1754,10 @@
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1693536080991972</v>
+        <v>-0.1691395227542029</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.08879643901584977</v>
+        <v>0.08902543371459748</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>22.02631578947368</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>18.96959836222817</v>
+        <v>18.96671287722498</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.124433164400712</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1611376987997795</v>
+        <v>0.1613143475126173</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1467198881572687</v>
+        <v>0.1470469900626932</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.71461718493059</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.78654971920524</v>
+        <v>22.78652309657694</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.835764692303093</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.442012180799171</v>
+        <v>-0.4420115288742487</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06176934337546847</v>
+        <v>0.06181477376878597</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>14.74892519346518</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.69973006202843</v>
+        <v>13.69815216902652</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.088477086210198</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07658509523080359</v>
+        <v>0.07670910729219438</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2884346927984077</v>
+        <v>-0.2883398824562786</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.21325403568394</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.48756025996492</v>
+        <v>24.47952818339456</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.41799596243931</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2746575691623703</v>
+        <v>0.2750758021903843</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1411968549373943</v>
+        <v>0.141502921098748</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.17243272926963</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.497175305699</v>
+        <v>25.48735409066483</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.19061897215175</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.222583770771742</v>
+        <v>0.2230548772690002</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1608584032285862</v>
+        <v>0.1612253422845784</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>24.21644910295158</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.26707296067751</v>
+        <v>17.17097504369309</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7597779772065341</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4024640515563904</v>
+        <v>0.4103129869637951</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01247397052279386</v>
+        <v>0.01255437171809826</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.66409266409266</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.17577945234648</v>
+        <v>14.17885274983041</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.84300254140586</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.457704158953474</v>
+        <v>0.4573881983744998</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1135744714993598</v>
+        <v>0.113454193666366</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.35491329479769</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.85425218979131</v>
+        <v>21.84854512149763</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.674352320436235</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.434728263520469</v>
+        <v>0.4351030295351965</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09166935202478976</v>
+        <v>0.09188074283454162</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>38.98194945848376</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.70947884306728</v>
+        <v>34.69913177116059</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.167799356381822</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1230923297561941</v>
+        <v>0.1234272291182437</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05227112640504772</v>
+        <v>0.0523951647524068</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.66222222222222</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.6636269430437</v>
+        <v>20.66028914185039</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.993881454729295</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04832623439878225</v>
+        <v>0.04849559817351601</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.0262327244258449</v>
+        <v>0.02631252988562238</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>160.0583756345177</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.64730520466372</v>
+        <v>45.572538339599</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>24.8954189081225</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.506414560878937</v>
+        <v>2.512167227591961</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9293741779367319</v>
+        <v>0.931925107181226</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>55.24673439767779</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.34375703947268</v>
+        <v>35.33520862594448</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.61134903678438</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5631256840062882</v>
+        <v>0.5635038406739021</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3066425281046585</v>
+        <v>0.3063286695659782</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>74.18352059925091</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>74.73857231422116</v>
+        <v>74.35839310569898</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.665499078674398</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.007426576368580684</v>
+        <v>-0.002351752090708703</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1582034075201026</v>
+        <v>0.1586286042666216</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>14.25121876904327</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.01213384565608</v>
+        <v>13.01048873695455</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.339929777338749</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09522534413529993</v>
+        <v>0.09536382968954782</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3855268961990271</v>
+        <v>-0.3854877089420042</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>19.69519650655022</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.44672599750871</v>
+        <v>17.443633226404</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.074817117096256</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1288763581982413</v>
+        <v>0.1290765089429924</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.0471832149966267</v>
+        <v>0.04729073714399101</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.60254265640683</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.78272248176846</v>
+        <v>26.76382866800616</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.99292615551466</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4786600833192023</v>
+        <v>0.4797039372676986</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2376078234173944</v>
+        <v>0.2381190557818988</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>15.78054662379421</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.58531957976789</v>
+        <v>14.58297333306618</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.447153117467142</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08194726467867675</v>
+        <v>0.08212133858961379</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3271051416963593</v>
+        <v>-0.327006003572087</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>84.2360248447205</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.44205059960733</v>
+        <v>28.42663129835774</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.517537635080098</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.961671998638645</v>
+        <v>1.96327848208968</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2522933129255482</v>
+        <v>0.2528582116062696</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>37.88319238900635</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.827228116235348</v>
+        <v>9.827947640003091</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.565356455664406</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.854921442845145</v>
+        <v>2.854639216310928</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.0514940475070369</v>
+        <v>-0.05160085599039799</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>8.13560720204846</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.00443531895025063</v>
+        <v>0.004426792381163374</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.987077813549424</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1833.277826082549</v>
+        <v>1836.810880100593</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2432.935291707406</v>
+        <v>2437.392529054422</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-96.54545454545455</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>127.9699106279624</v>
+        <v>127.4350123282846</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>118.2423554885671</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.356256120994235</v>
+        <v>4.366449720035538</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
         <v>28.68899965225455</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6898227636857688</v>
+        <v>0.6894946981994463</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.45395915587732</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.58894307715698</v>
+        <v>40.60873133205129</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.679954423938</v>
+        <v>40.70264226981045</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
         <v>-24.29921259842519</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-103.5919722461546</v>
+        <v>-104.6929904706598</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>2.142329741769348</v>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02136127112348496</v>
+        <v>0.02143525284488845</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
         <v>18.7319587628866</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.83910591624148</v>
+        <v>15.8335122613649</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.481135511995528</v>
@@ -5200,10 +5200,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1826399079558387</v>
+        <v>0.1830577103599527</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.008237808786623502</v>
+        <v>0.008470672645869204</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
         <v>21.15432098765432</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.11533578334685</v>
+        <v>15.10218857739603</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>5.501133059336556</v>
@@ -5326,10 +5326,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.3995270294266873</v>
+        <v>0.4007453872822595</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4445965742942801</v>
+        <v>0.4461611315475387</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
         <v>31.75595238095238</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.61519711858666</v>
+        <v>20.61034510885216</v>
       </c>
       <c r="N40" s="6" t="n">
         <v>6.641154026940387</v>
@@ -5452,10 +5452,10 @@
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5404146852576648</v>
+        <v>0.5407773238747555</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1649876396295691</v>
+        <v>0.1652018109973663</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
         <v>11.83594864479315</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.63083041321805</v>
+        <v>10.62842102614351</v>
       </c>
       <c r="N41" s="6" t="n">
         <v>1.943389334262809</v>
@@ -5578,10 +5578,10 @@
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1133606862994156</v>
+        <v>0.1136130772086843</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2890798197180271</v>
+        <v>-0.2890835249581815</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 11:25 ET</t>
+          <t>2026-09-27 12:05 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-28)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -454,7 +454,7 @@
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="23" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>341.07</v>
+        <v>339.26511</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2585144006118605</v>
+        <v>0.2518545359022104</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.01236462616551803</v>
+        <v>-0.01759104071349971</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>345.34</v>
@@ -714,40 +714,40 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>5009416510920</v>
+        <v>4982907393154</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.93493150684932</v>
+        <v>38.72945205479452</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>35.5125142905931</v>
+        <v>35.32458752506711</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.7308691108193</v>
+        <v>10.67423685234018</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>46.60692048967635</v>
+        <v>46.36095204659598</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.189678462709283</v>
+        <v>1.183399923896498</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.99762301271322</v>
+        <v>29.84071240411666</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.82675770242683</v>
+        <v>10.77012544394771</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02728521369745268</v>
+        <v>0.02742997564120077</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09637214611872147</v>
+        <v>0.09638794868620182</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1219765024388257</v>
+        <v>0.1219926866181724</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003107866420382913</v>
+        <v>0.003124400266210693</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3019845712332221</v>
+        <v>0.3053550129780648</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2784776666105622</v>
+        <v>0.2784504892780152</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13396328030.79305</v>
+        <v>13316961441.30166</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>516.17</v>
+        <v>511.15</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.09140693816431744</v>
+        <v>0.0807924839542995</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.06781405764646409</v>
+        <v>-0.07688001155818835</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3832846143500</v>
+        <v>3795569882500</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.67611111111111</v>
+        <v>28.39722222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.9981838035207</v>
+        <v>24.74276071532097</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.55031850837304</v>
+        <v>11.43798613936276</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.668037103260266</v>
+        <v>8.583736298761039</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.9108490977055925</v>
+        <v>0.9019906548079385</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.98968019072953</v>
+        <v>18.81036689334471</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.8753957295556</v>
+        <v>11.76326027784558</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01747709078111604</v>
+        <v>0.01764842931098646</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1471277808219178</v>
+        <v>0.1476982115677321</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2328985216471497</v>
+        <v>0.2335258515251684</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007051940252242479</v>
+        <v>0.00712119730020542</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5559009439283675</v>
+        <v>0.5565954673503465</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4313552623124653</v>
+        <v>0.431926130511299</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10852564562.72502</v>
+        <v>10788865291.4251</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>343.92</v>
+        <v>342.465</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.09128988310552066</v>
+        <v>0.08667303389663905</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.158317221800739</v>
+        <v>-0.1618780744475172</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4162158113481</v>
+        <v>4144549541560</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.93545183714002</v>
+        <v>16.83862959285005</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.77790607446563</v>
+        <v>20.70876486849514</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.283761507556081</v>
+        <v>9.230685000755834</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.470870409692731</v>
+        <v>6.433875577691731</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1506079581764422</v>
+        <v>0.149746912326659</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.94056265366491</v>
+        <v>12.86758196576555</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.411254969717358</v>
+        <v>9.35817846291711</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01287000818029795</v>
+        <v>0.01294401082220859</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1849298107111804</v>
+        <v>-0.1868839257300587</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2998677506040526</v>
+        <v>0.2986293351088514</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002500581530588509</v>
+        <v>0.002511205524652154</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7623052681932441</v>
+        <v>0.7616226673120993</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3206523161285895</v>
+        <v>0.3202009018695926</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8500131780.098979</v>
+        <v>8422915453.875556</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>249.67</v>
+        <v>246.45</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1022958057395142</v>
+        <v>0.08807947019867535</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1306754874651811</v>
+        <v>-0.1418871866295265</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2685725157000</v>
+        <v>2651087295000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.81507936507936</v>
+        <v>19.56415079365079</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.32481201364503</v>
+        <v>22.04848526231589</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.462413826577971</v>
+        <v>3.418567494237315</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.868297958739712</v>
+        <v>4.806648190420941</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2243026750463299</v>
+        <v>0.2214622145677222</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.14479366685433</v>
+        <v>11.01089160080631</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.649371076990512</v>
+        <v>3.605524744649856</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004328439926066492</v>
+        <v>-0.004383956225169786</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1124189823874756</v>
+        <v>-0.1126759702133002</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1838519169776447</v>
+        <v>0.1845603721866091</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8343667953128601</v>
+        <v>0.8350052821193245</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4529088218280257</v>
+        <v>0.4516181906539232</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8738257341.305389</v>
+        <v>8663732596.239094</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>225.07</v>
+        <v>229.88</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1917923893347975</v>
+        <v>0.2172623382071501</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.04849074152363231</v>
+        <v>-0.02815591443307686</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5451420470000</v>
+        <v>5567923480000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.31069182389937</v>
+        <v>28.91320754716981</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.53347663458033</v>
+        <v>16.86487744704706</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.99332760117372</v>
+        <v>18.37626646548987</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>23.77652281382105</v>
+        <v>24.28254113824547</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2272558935523895</v>
+        <v>0.2320924143242203</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.40012697556779</v>
+        <v>23.89663955450705</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.04751466321637</v>
+        <v>18.43045352753252</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02329778095432804</v>
+        <v>0.02281228376171324</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7123253898509516</v>
+        <v>0.7144036556418816</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9759286917850041</v>
+        <v>0.9783060324384201</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.00231039232238859</v>
+        <v>0.002262049765094832</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.305861092676486</v>
+        <v>1.299673299187378</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.389194698065552</v>
+        <v>0.3787629634551394</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26600098382.11532</v>
+        <v>26855395627.53257</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>751.66</v>
+        <v>721.5073</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.1556710859858992</v>
+        <v>0.1093115570041694</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.03611089738657647</v>
+        <v>-0.07477712805519232</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>779.8200000000001</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1914843755206</v>
+        <v>1838030156907</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>27.93236714975846</v>
+        <v>26.78335154217763</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>22.59968127350366</v>
+        <v>21.68818711341582</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.389312305939155</v>
+        <v>8.044212635308963</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.317449133109513</v>
+        <v>7.016441230107841</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.726135265700479</v>
+        <v>-5.49058706614641</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>18.78828970418036</v>
+        <v>18.05263229961147</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.813657754749221</v>
+        <v>8.46855808411903</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02139913498874052</v>
+        <v>0.02231716572352874</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2359628798175555</v>
+        <v>0.2349280925195476</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2806438403193861</v>
+        <v>0.279900037238054</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.002793816353138387</v>
+        <v>0.002910573461973289</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8266593683881774</v>
+        <v>0.8330263853710935</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4905097236598456</v>
+        <v>0.5022334994072717</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>13481261198.45398</v>
+        <v>13788316349.27699</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>372.11</v>
+        <v>359.2917</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1505695578821065</v>
+        <v>-0.1798304061156928</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2540344405909829</v>
+        <v>-0.2797311709399996</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1469666080781</v>
+        <v>1419039597421</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>315.3474576271187</v>
+        <v>304.364406779661</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>174.58508291529</v>
+        <v>168.4449918181659</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14.18336483445121</v>
+        <v>13.68938077529218</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.8676929010569</v>
+        <v>13.38470319371848</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.394460491764141</v>
+        <v>-8.102094772021958</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>121.6984603243266</v>
+        <v>117.4428788289824</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>14.1266474370627</v>
+        <v>13.63266337790367</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.003920618482899188</v>
+        <v>0.004062094789562529</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8062680520083585</v>
+        <v>0.8069068334677367</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.126650182634036</v>
+        <v>0.1265784931824163</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.527550059420665</v>
+        <v>1.527582388187277</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.409613927618917</v>
+        <v>0.4126033222691708</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13786592185.9667</v>
+        <v>13608080286.87846</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>352.81</v>
+        <v>350.79</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.01493011033805147</v>
+        <v>0.009119167272710671</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2872525252525252</v>
+        <v>-0.2913333333333333</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1678521799800</v>
+        <v>1668911488200</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>43.77295285359801</v>
+        <v>43.52233250620348</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.07043911729104</v>
+        <v>18.94000981523482</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.83778281334171</v>
+        <v>18.72992781693302</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.86721296017655</v>
+        <v>16.7706403851941</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4355625506719404</v>
+        <v>0.4330687541458859</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>32.79501367697989</v>
+        <v>32.61568159500985</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.23556518001437</v>
+        <v>19.1303798617346</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02347482171795145</v>
+        <v>0.02360663507670292</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.295330096196336</v>
+        <v>1.297904432509603</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.874816190680922</v>
+        <v>0.8768993857144312</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007369405629092146</v>
+        <v>0.00741184184269791</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.596157977234559</v>
+        <v>1.59397456964459</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3896621793452344</v>
+        <v>0.3841590304293971</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9303515124.854837</v>
+        <v>9034004752.307709</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>922.765</v>
+        <v>921.55</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.07988882387361018</v>
+        <v>0.07846693973083663</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1584450524395805</v>
+        <v>-0.1595531235750114</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>409226899435</v>
+        <v>408688072450</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>33.39721317408615</v>
+        <v>33.35323923271807</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.1959343219621</v>
+        <v>40.13266767393613</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.349897739878082</v>
+        <v>1.348120336363696</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.44274476650001</v>
+        <v>11.42767816244449</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>0.6497858639947462</v>
+        <v>0.6489302942399835</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.41708332300299</v>
+        <v>27.65213959537572</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.298620171381542</v>
+        <v>1.309753697625629</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.0229457057025438</v>
+        <v>0.02297595803006655</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1691395227542029</v>
+        <v>-0.1689254374092086</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.08902543371459748</v>
+        <v>0.08925442841334497</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1766,7 +1766,7 @@
         <v>0.2802083491518731</v>
       </c>
       <c r="Y10" s="4" t="n">
-        <v>0.175339926242108</v>
+        <v>0.1282351544099699</v>
       </c>
       <c r="Z10" s="4" t="n">
         <v>0.03854476602650798</v>
@@ -1781,28 +1781,28 @@
         <v>0.6201765562431744</v>
       </c>
       <c r="AD10" s="6" t="n">
-        <v>0.1302125520207804</v>
+        <v>0.2395330000279306</v>
       </c>
       <c r="AE10" s="6" t="n">
-        <v>0.05235555056432141</v>
+        <v>0.09631085406255264</v>
       </c>
       <c r="AF10" s="6" t="n">
-        <v>-1.08259628107807</v>
+        <v>-0.810014624973884</v>
       </c>
       <c r="AG10" s="6" t="n">
         <v>80.58620689655173</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006003695415409124</v>
+        <v>0.006011610872985731</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1725160043142916</v>
+        <v>-0.1722264329796254</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1814114731558173</v>
+        <v>0.1800680736804853</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1975564704.342651</v>
+        <v>1978797307.883456</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>71.145</v>
+        <v>69.175</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2181008718505689</v>
+        <v>-0.2397516032084208</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.4302018260451707</v>
+        <v>-0.445979497036681</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>296243511229</v>
+        <v>288040549431</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>22.02631578947368</v>
+        <v>21.41640866873065</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>18.96671287722498</v>
+        <v>18.43872121120907</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.124433164400712</v>
+        <v>5.954848044802435</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.884831783090585</v>
+        <v>9.611121492659937</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6473587933247755</v>
+        <v>0.6294334742883034</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.852378038325147</v>
+        <v>9.584281440281899</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.232144384343402</v>
+        <v>6.062559264745127</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03711341373989126</v>
+        <v>0.03817034796565597</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1613143475126173</v>
+        <v>0.1614909962254547</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1470469900626932</v>
+        <v>0.1473740919681175</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.09973998985696915</v>
+        <v>0.1063714476291125</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3518610586434247</v>
+        <v>0.3554962435241693</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2374414112.674433</v>
+        <v>2372280575.627017</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>505.48</v>
+        <v>502.89</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01736941489477695</v>
+        <v>0.01215657406115844</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.05999181760702199</v>
+        <v>-0.06480827165544689</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1090246355201</v>
+        <v>1084660104390</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.71461718493059</v>
+        <v>12.66278688123384</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.78652309657694</v>
+        <v>22.66974205075438</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.835764692303093</v>
+        <v>2.824204883377915</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.45194349600161</v>
+        <v>1.446024743493869</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3502553243535411</v>
+        <v>0.3488275314779394</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.41734600449591</v>
+        <v>15.35922712146797</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.066500329327479</v>
+        <v>3.054940520402301</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02219763839625447</v>
+        <v>0.02228849598946987</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4420115288742487</v>
+        <v>-0.4414234245416804</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06181477376878597</v>
+        <v>0.06297813336129532</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02323224740464951</v>
+        <v>0.02371319949490255</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1347616100089321</v>
+        <v>0.134478536927243</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2220159570.140381</v>
+        <v>2186702107.65096</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>343.06</v>
+        <v>337.08</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.05401249975504752</v>
+        <v>0.03563963568306239</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.06395634379263304</v>
+        <v>-0.08027285129604367</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>919232700600</v>
+        <v>903209230800</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>14.74892519346518</v>
+        <v>14.49226139294927</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.69815216902652</v>
+        <v>13.45882688310635</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.088477086210198</v>
+        <v>3.034730778845088</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.553914922129857</v>
+        <v>2.509471174432325</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7722426515506036</v>
+        <v>0.7588039276254677</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.82924753756977</v>
+        <v>19.65753570094461</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.206612508021624</v>
+        <v>6.152866200656513</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1768148586249282</v>
+        <v>-0.179946321160129</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07670910729219438</v>
+        <v>0.0767848876294035</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2883398824562786</v>
+        <v>-0.2882671257918193</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01748965195592608</v>
+        <v>0.0177999288002848</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7718781883291154</v>
+        <v>0.7781210058911325</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1854938933482376</v>
+        <v>0.1689672064214316</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2478789947.98411</v>
+        <v>2458111994.999583</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>367.38</v>
+        <v>369.01001</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.06032090842463234</v>
+        <v>0.0650253933828262</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.04717690691703191</v>
+        <v>-0.04294937365458928</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>685915804377</v>
+        <v>688959109564</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.21325403568394</v>
+        <v>31.35174256584537</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.47952818339456</v>
+        <v>24.58007775824457</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.41799596243931</v>
+        <v>15.48640328996583</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>19.98304702882483</v>
+        <v>20.07170881359117</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.104841143853688</v>
+        <v>2.114180008552074</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.96779175122001</v>
+        <v>24.07237987366829</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.67647015772793</v>
+        <v>15.74487748525445</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03063495529030065</v>
+        <v>0.03049963300913147</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2750758021903843</v>
+        <v>0.2754940352183983</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.141502921098748</v>
+        <v>0.1418089872601016</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007294899014644238</v>
+        <v>0.007262675611428535</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3012001491799892</v>
+        <v>0.2956672953368226</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1766630962178798</v>
+        <v>0.1764161690778384</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2445815294.001974</v>
+        <v>2383703483.120117</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>567.65</v>
+        <v>567.875</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.008026557061416195</v>
+        <v>0.008426109559150463</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05585216971874329</v>
+        <v>-0.05547793689602987</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>497849485400</v>
+        <v>498046818500</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.17243272926963</v>
+        <v>31.18478857770456</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.48735409066483</v>
+        <v>25.48763899701708</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.19061897215175</v>
+        <v>14.19624372203061</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>89.22960256638746</v>
+        <v>89.2649705934771</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.377710196516827</v>
+        <v>1.37825628088962</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.11455441309459</v>
+        <v>23.12347705281244</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.5712021605906</v>
+        <v>14.57682691046946</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03303809782345112</v>
+        <v>0.03302500766802911</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2230548772690002</v>
+        <v>0.223525983766258</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1612253422845784</v>
+        <v>0.1615922813405704</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.00593675680436889</v>
+        <v>0.005934404578472375</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2869541046326143</v>
+        <v>0.2857759759030024</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1784708934114141</v>
+        <v>0.1784601725705013</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1564935163.187866</v>
+        <v>1534714772.482699</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>376.59</v>
+        <v>376.10001</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1194708883255293</v>
+        <v>0.1180143187390543</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1841991248212816</v>
+        <v>-0.1852605822971275</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>341998101102</v>
+        <v>341553115887</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.21644910295158</v>
+        <v>24.18494051829465</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.17097504369309</v>
+        <v>17.14290292604213</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7597779772065341</v>
+        <v>0.7587894045640249</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.465716682377319</v>
+        <v>3.46120735786738</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7337647306520968</v>
+        <v>-0.7328100123102071</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.01149326949501</v>
+        <v>14.99422101024726</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8591783713157783</v>
+        <v>0.8581897986732692</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.0690559389771474</v>
+        <v>0.06914590703899035</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4103129869637951</v>
+        <v>0.4107844291385925</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01255437171809826</v>
+        <v>0.01263477291340243</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02405799410499482</v>
+        <v>0.02408933730153318</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4377240790191192</v>
+        <v>0.4320372869996907</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.1949010994954906</v>
+        <v>0.190610229686095</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1859810112.65859</v>
+        <v>1841947650.677755</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>160.56</v>
+        <v>161.95</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3090908928046132</v>
+        <v>0.3204239542208962</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.08984751431324756</v>
+        <v>-0.08196814239555583</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>665434497600</v>
+        <v>671195297000</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.66409266409266</v>
+        <v>20.84298584298584</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.17885274983041</v>
+        <v>14.30470315906931</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.84300254140586</v>
+        <v>1.858957782640004</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.583674595419847</v>
+        <v>2.606041982612383</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.023359073359075</v>
+        <v>2.040875697125698</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.707128403759137</v>
+        <v>9.787334451792551</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.931021153270924</v>
+        <v>1.946976394505068</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04591436138371916</v>
+        <v>0.04552028319709755</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4573881983744998</v>
+        <v>0.4570722377955256</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.113454193666366</v>
+        <v>0.1133339158333719</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02566018933731938</v>
+        <v>0.02543995060203767</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.551556469350051</v>
+        <v>-0.5513607754075597</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2578079794257925</v>
+        <v>0.2520922083896671</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2337218226.222433</v>
+        <v>2322599007.543252</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>271.22</v>
+        <v>271.98</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.3080298626304283</v>
+        <v>0.3116951627395617</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.03504465079873331</v>
+        <v>-0.03234069804674988</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>179.8</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>653612648388</v>
+        <v>655444171184</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.35491329479769</v>
+        <v>31.44277456647399</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.84854512149763</v>
+        <v>21.90404802076957</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.674352320436235</v>
+        <v>6.693054878371065</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.788585776323687</v>
+        <v>7.810410587141495</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.882233343474299</v>
+        <v>-3.893111956191062</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.22490953361793</v>
+        <v>20.27920583374837</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.966543601874828</v>
+        <v>6.985246159809658</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02862245711759006</v>
+        <v>0.02854247672415136</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4351030295351965</v>
+        <v>0.4354777955499247</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09188074283454162</v>
+        <v>0.09209213364429392</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.0194675908856279</v>
+        <v>0.01941319214648136</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.157074155069618</v>
+        <v>-0.1560144923762522</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.191741468346202</v>
+        <v>0.191429999704316</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1708404011.753947</v>
+        <v>1691102364.546594</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>107.98</v>
+        <v>108.87</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.04239093690735773</v>
+        <v>-0.03449806724489746</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2010949985202722</v>
+        <v>-0.1945102101213376</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>859313478400</v>
+        <v>866396169600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.98194945848376</v>
+        <v>39.30324909747293</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.69913177116059</v>
+        <v>34.9747051456737</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.167799356381822</v>
+        <v>1.177424670580561</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.742776929497751</v>
+        <v>8.814837232028339</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.426544141778807</v>
+        <v>9.504240236298006</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.51169444664908</v>
+        <v>21.67702723219496</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.252363935638182</v>
+        <v>1.261989249836921</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01572068906117137</v>
+        <v>0.01559217419698066</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1234272291182437</v>
+        <v>0.1237621284802926</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.0523951647524068</v>
+        <v>0.05251920309976521</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009052602333765512</v>
+        <v>0.008978598328281436</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.05000685500234299</v>
+        <v>-0.05204501037438802</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3077459276137968</v>
+        <v>0.3074206349623856</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2821016151.449915</v>
+        <v>2799178446.674672</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>146.22</v>
+        <v>149.09</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.03124343693935727</v>
+        <v>0.05148463967507033</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1257399103139013</v>
+        <v>-0.1085799701046337</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>347595490768</v>
+        <v>354418071712</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.66222222222222</v>
+        <v>22.08740740740741</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.66028914185039</v>
+        <v>21.06240621062859</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.993881454729295</v>
+        <v>4.072273091644453</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.522029607261881</v>
+        <v>6.650043729631198</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.67194920634942</v>
+        <v>21.07769735449758</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.53455776644396</v>
+        <v>17.85555997515762</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.282097283390017</v>
+        <v>4.360488920305175</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04578022564343624</v>
+        <v>0.04489895202897808</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04849559817351601</v>
+        <v>0.04866496194824954</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02631252988562238</v>
+        <v>0.02639233534539964</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.0293434550677062</v>
+        <v>0.02877859011335435</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.03059475853779217</v>
+        <v>-0.03855578385837691</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1495866310155668</v>
+        <v>0.149951618700575</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1271269678.848826</v>
+        <v>1260428665.295301</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>293.2</v>
+        <v>290.65</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1521601012369582</v>
+        <v>-0.159533879346937</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2865312081761772</v>
+        <v>-0.2927363426207569</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>410.95</v>
@@ -3110,37 +3110,37 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>292354704400</v>
+        <v>289812056050</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20.47486033519553</v>
+        <v>20.2967877094972</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>19.53855165487934</v>
+        <v>19.36862223223288</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.728109805173311</v>
+        <v>1.713080200796803</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17.53871336583017</v>
+        <v>17.38617680688451</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.023353254514777</v>
+        <v>-6.962270202676396</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14.75378232908217</v>
+        <v>14.64746209701024</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.085619144559512</v>
+        <v>2.070589540183005</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05165300839263662</v>
+        <v>0.05210618290287652</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.0479210893854749</v>
+        <v>0.04792108938547468</v>
       </c>
       <c r="V21" s="4" t="n">
         <v>0.01423568777486173</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03168485675306958</v>
+        <v>0.0319628419060726</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7064666365582442</v>
+        <v>0.707618644338066</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2352095735933773</v>
+        <v>0.2328647584273901</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1385051008.94694</v>
+        <v>1378955705.126651</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>630.63</v>
+        <v>606.86</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.821989513380716</v>
+        <v>1.715621768850548</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.01309859154929582</v>
+        <v>-0.05029733959311422</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>639</v>
@@ -3236,40 +3236,40 @@
         <v>159.33</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>1028305278000</v>
+        <v>989545916000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>160.0583756345177</v>
+        <v>154.0253807106599</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.572538339599</v>
+        <v>43.78308356594623</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>24.8954189081225</v>
+        <v>23.95704917080257</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>15.30045117815066</v>
+        <v>14.72373943829585</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.292214408792437</v>
+        <v>1.243507660783309</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>95.86632562045158</v>
+        <v>92.25003881321142</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>24.87580869144172</v>
+        <v>23.93743895412178</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.008171697821432363</v>
+        <v>0.008491773715733267</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.512167227591961</v>
+        <v>2.517919894304986</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.931925107181226</v>
+        <v>0.9344760313425187</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.57633782396688</v>
+        <v>2.582398937832239</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6355259972551116</v>
+        <v>0.6256098503040556</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10754885318.6439</v>
+        <v>10652560696.52002</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1743.94</v>
+        <v>1781.895</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4985134270207767</v>
+        <v>0.5311269785893935</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.128012560251205</v>
+        <v>-0.1090346806936139</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>672145851225</v>
+        <v>686774391073</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>55.24673439767779</v>
+        <v>55.76923076923077</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.33520862594448</v>
+        <v>35.95417975840671</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.61134903678438</v>
+        <v>16.76845098484184</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.88656519468142</v>
+        <v>27.14084507042253</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.76084710361529</v>
+        <v>3.796415341032905</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>42.17102633901988</v>
+        <v>42.57307053257995</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.47866203657208</v>
+        <v>16.63576398462954</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01704373210688957</v>
+        <v>0.01688405107740257</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5635038406739021</v>
+        <v>0.5511195400359803</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3063286695659782</v>
+        <v>0.2957487901530362</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004461162654678487</v>
+        <v>0.004366138296588744</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.653708998784613</v>
+        <v>1.647003808595017</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.3971159842269665</v>
+        <v>0.3954846150389279</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2105351252.599284</v>
+        <v>2110010095.994548</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>198.07</v>
+        <v>185.5</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1303947127161375</v>
+        <v>-0.1855819619772984</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2212699036760369</v>
+        <v>-0.2706899941026145</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>156548585900</v>
+        <v>146613635000</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>74.18352059925091</v>
+        <v>69.47565543071158</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>74.35839310569898</v>
+        <v>69.28698197715714</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.665499078674398</v>
+        <v>1.559802489494122</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>25.68561291513443</v>
+        <v>24.05554195868853</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3970356682131908</v>
+        <v>0.3718388269477805</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>28.08627135251799</v>
+        <v>26.65678201438849</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.076701802223523</v>
+        <v>1.971005213043247</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001341436582085409</v>
+        <v>-0.001432336085248824</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.002351752090708703</v>
+        <v>0.002723072187162945</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1586286042666216</v>
+        <v>0.15905375185713</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.231298283538854</v>
+        <v>1.252261842346005</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3265156952935771</v>
+        <v>0.3531052046527953</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1266194328.628845</v>
+        <v>1325396639.736345</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>935.45</v>
+        <v>916.49</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.02308766161876474</v>
+        <v>0.00235139344377755</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1893777242437109</v>
+        <v>-0.2058076759763949</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>275964298150</v>
+        <v>270370965430</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>14.25121876904327</v>
+        <v>13.96237050578915</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.01048873695455</v>
+        <v>12.74517662948246</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.339929777338749</v>
+        <v>2.29250333169404</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.287143316876049</v>
+        <v>2.240786764106826</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.334028820969781</v>
+        <v>0.3272586179171463</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.45724518682509</v>
+        <v>26.2790738518141</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.042508272637085</v>
+        <v>6.995081826992377</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1504361262609216</v>
+        <v>-0.1535482921917087</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09536382968954782</v>
+        <v>0.09550231524379549</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3854877089420042</v>
+        <v>-0.3854485216849813</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01924207600620022</v>
+        <v>0.01964014882868335</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.579825351943071</v>
+        <v>1.587710706594825</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3111826575726561</v>
+        <v>0.2887961515648983</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2031486619.277751</v>
+        <v>2007468884.426805</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>225.51</v>
+        <v>220.99</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2263807890222985</v>
+        <v>-0.2418867924528302</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3216928352282982</v>
+        <v>-0.3352884557540756</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>212460638340</v>
+        <v>208202192660</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>19.69519650655022</v>
+        <v>19.30043668122271</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.443633226404</v>
+        <v>17.09097280604337</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.074817117096256</v>
+        <v>3.013187152264209</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.152236415882968</v>
+        <v>6.028924329501916</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2400829186554281</v>
+        <v>0.2352708269862226</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>16.67965220023427</v>
+        <v>16.41480225016953</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.915664042433102</v>
+        <v>3.853488679682186</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06415776638205502</v>
+        <v>0.06548186420826986</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1290765089429924</v>
+        <v>0.129276659687743</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04729073714399101</v>
+        <v>0.04739825929135577</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02988780985322159</v>
+        <v>0.03049911760713155</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8811376584612348</v>
+        <v>0.9058593328944763</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3064314291585977</v>
+        <v>0.3102287329692265</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1242825112.1433</v>
+        <v>1233075747.583923</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1183.72</v>
+        <v>1187.435</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.09567182795538565</v>
+        <v>0.09911049659396065</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.08426875024175151</v>
+        <v>-0.08139480911306241</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>716.08</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1114757656520</v>
+        <v>1118256224335</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>39.60254265640683</v>
+        <v>39.72683171629308</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.76382866800616</v>
+        <v>26.83063899981914</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.99292615551466</v>
+        <v>14.03684171043283</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>31.18013306177868</v>
+        <v>31.27798913781398</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4186476635942249</v>
+        <v>0.4199615520731326</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.8047804520515</v>
+        <v>26.89220260433024</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.57056423860678</v>
+        <v>14.61808524285201</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01798947052097705</v>
+        <v>0.01792858373473231</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4797039372676986</v>
+        <v>0.4806517174846585</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2381190557818988</v>
+        <v>0.2385892016199385</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.00565167438245531</v>
+        <v>0.005633992597489547</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.357598458182214</v>
+        <v>0.3437678339361285</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3139587734725938</v>
+        <v>0.3134771239229047</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2853729577.00765</v>
+        <v>2802525677.698893</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>196.31</v>
+        <v>193.66</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.07921938750430124</v>
+        <v>0.06465094281535833</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1547470398277718</v>
+        <v>-0.1661571582346609</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>309635836800</v>
+        <v>305456044800</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>15.78054662379421</v>
+        <v>15.56752411575563</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.58297333306618</v>
+        <v>14.33391310064549</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.447153117467142</v>
+        <v>2.41411885654672</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.79307543222511</v>
+        <v>2.755371546048163</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4014822830498072</v>
+        <v>0.3960626505803355</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>22.96922468395407</v>
+        <v>22.82679813268818</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.327457237471252</v>
+        <v>5.29442297655083</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.05065305153980161</v>
+        <v>-0.05134617653505347</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08212133858961379</v>
+        <v>0.08606240364709494</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.327006003572087</v>
+        <v>-0.3269007736940052</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02114003362029443</v>
+        <v>0.02142930909841992</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.37118413284995</v>
+        <v>1.377952525357693</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2609535691634336</v>
+        <v>0.2439544092628762</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>956808924.5290629</v>
+        <v>945784044.8358877</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1082.28</v>
+        <v>1054.2</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.431234398346002</v>
+        <v>2.342210243870676</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1376254980079682</v>
+        <v>-0.1599999999999999</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,31 +4120,31 @@
         <v>159.97</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1222316209200</v>
+        <v>1190602938000</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>24.15264449899576</v>
+        <v>23.52599866101317</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.831530326419744</v>
+        <v>6.654284723095405</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>13.54006922480448</v>
+        <v>13.18876905864368</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>12.12036694333029</v>
+        <v>11.80590127477066</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03442460039505005</v>
+        <v>0.03353144633224468</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>17.61181648084745</v>
+        <v>17.14780584086852</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>13.33381936327182</v>
+        <v>12.98251919711102</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02141180801089879</v>
+        <v>0.02198213960731886</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0004897069150312304</v>
+        <v>0.0005027509011572757</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.857958824207671</v>
+        <v>2.856747660887568</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.721414067327511</v>
+        <v>0.6709183133850734</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25155134915.873</v>
+        <v>24825561581.70271</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>135.62</v>
+        <v>131.3</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.08023056760316338</v>
+        <v>-0.1095286353509464</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2971964554075763</v>
+        <v>-0.3195833549256361</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>192.97</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>140212364440</v>
+        <v>135746080600</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>84.2360248447205</v>
+        <v>81.55279503105592</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.42663129835774</v>
+        <v>27.5062256980965</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.517537635080098</v>
+        <v>9.214368761878903</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.19330936401406</v>
+        <v>10.83676094598913</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>134.7776397515557</v>
+        <v>130.4844720496922</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>41.89233718543995</v>
+        <v>40.61223290341072</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>9.921420339397232</v>
+        <v>9.618251466196035</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03266473693880174</v>
+        <v>0.03373946400335333</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.96327848208968</v>
+        <v>1.964884965540714</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2528582116062696</v>
+        <v>0.2534231102869904</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.680908358701193</v>
+        <v>0.6872385142237319</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5513107222422996</v>
+        <v>0.5490531363555531</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2062078409.913101</v>
+        <v>2039521190.869481</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.67</v>
+        <v>28.765</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1386020513314628</v>
+        <v>0.1423748868695334</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.01848681958233478</v>
+        <v>-0.01523450872988708</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.62</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>163402944800</v>
+        <v>163944388121</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>37.88319238900635</v>
+        <v>38.00872093023256</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.827947640003091</v>
+        <v>9.861235228352442</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.565356455664406</v>
+        <v>2.573856884592439</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.917951989670149</v>
+        <v>1.924307254372579</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6336215364178938</v>
+        <v>-0.6357210845853056</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.87238155893536</v>
+        <v>17.91527155584601</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.542152486812359</v>
+        <v>3.550652915740392</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.0672325704622185</v>
+        <v>0.06701052793519059</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.854639216310928</v>
+        <v>2.85435698977671</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05160085599039799</v>
+        <v>-0.05170766447375896</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.05999302406696895</v>
+        <v>0.05979488962280549</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3469767748165458</v>
+        <v>0.3387368373408882</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.1918027931372212</v>
+        <v>0.1909987344683972</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>939924699.5058314</v>
+        <v>932767059.0948771</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>191.56</v>
+        <v>182.3387</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.1401702652410115</v>
+        <v>0.08528483995980984</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.04157702506629313</v>
+        <v>-0.08771351378395964</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1359798029200</v>
+        <v>1294340180136</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>8.13560720204846</v>
+        <v>7.724894486155574</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004426792381163374</v>
+        <v>0.004218367270065046</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.987077813549424</v>
+        <v>6.634346710180119</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>5.063261427740412</v>
+        <v>4.807651022687995</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01820647304199383</v>
+        <v>0.0172873492686601</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>8.21974583119084</v>
+        <v>7.802981027678777</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.956825509300162</v>
+        <v>6.604094405930858</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.06898723988018901</v>
+        <v>0.07265511349372848</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1836.810880100593</v>
+        <v>1830.252233766847</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2437.392529054422</v>
+        <v>2429.911947304836</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.566088953852579</v>
+        <v>1.64528978214718</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.7681477162484222</v>
+        <v>0.7769877379184571</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3391219023.770243</v>
+        <v>3346245713.156026</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>606.5599999999999</v>
+        <v>601.39</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6248594155765057</v>
+        <v>0.611009964279799</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.09715255347334906</v>
+        <v>-0.1048479526070584</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>315.05</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>76451276107</v>
+        <v>75799645440</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.817502989459575</v>
+        <v>1.817167845233825</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.3847343199442911</v>
+        <v>0.3630561549211155</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3828740338.151042</v>
+        <v>3806849109.297424</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>148.68</v>
+        <v>147.26</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.07623483802977593</v>
+        <v>-0.08505745391622832</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3410742776103527</v>
+        <v>-0.3473674880340365</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1959867042223</v>
+        <v>1941148914701</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-96.54545454545455</v>
+        <v>-95.62337662337661</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>127.4350123282846</v>
+        <v>125.6925379416786</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>118.2423554885671</v>
+        <v>117.1130566938763</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.852948500282966</v>
+        <v>6.787497956360435</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9654545454545455</v>
+        <v>-0.9562337662337661</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>457.3335834468443</v>
+        <v>452.8415922008639</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>114.974904508175</v>
+        <v>113.8456057134842</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01450251439901806</v>
+        <v>-0.01464235937013522</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.366449720035538</v>
+        <v>4.37664331907684</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.160248758681224</v>
+        <v>3.144973828814988</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7541715269041857</v>
+        <v>0.7487094037328906</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12673550841.14075</v>
+        <v>12535548702.00472</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>771.35</v>
+        <v>766.55</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1290747826978813</v>
+        <v>0.1220487128762053</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01029036272887074</v>
+        <v>-0.01644918331472867</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>821671505625</v>
+        <v>816558362140</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9959498199346021</v>
+        <v>0.9962899443173625</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1177761963223539</v>
+        <v>0.111851678327139</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>31467728797.33297</v>
+        <v>31305047649.19031</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>450.61</v>
+        <v>453.87</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.4098745992067205</v>
+        <v>0.4200745308403149</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.05926931106471811</v>
+        <v>-0.05246346555323589</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,13 +4914,13 @@
         <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2337079752800</v>
+        <v>2353987677600</v>
       </c>
       <c r="L36" s="6" t="n">
         <v>28.68899965225455</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6894946981994463</v>
+        <v>0.6923560128073691</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.45395915587732</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.60873133205129</v>
+        <v>40.43677403179649</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.70264226981045</v>
+        <v>40.53313743663112</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2663056745300814</v>
+        <v>0.2643928878313173</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.184512697624831</v>
+        <v>2.175950383264717</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3298638145831211</v>
+        <v>0.3058575138057339</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4147654996.64744</v>
+        <v>4138062089.982536</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>30.86</v>
+        <v>30.85</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.08242720982995699</v>
+        <v>0.08207645571141198</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.001940491591203131</v>
+        <v>-0.002263906856403652</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30.92</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>77370238624</v>
+        <v>77345167257</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-24.29921259842519</v>
+        <v>-24.29133858267716</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-104.6929904706598</v>
+        <v>-105.783374681721</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.142329741769348</v>
+        <v>2.141635532521113</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.359749680248493</v>
+        <v>2.358985017357939</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1808313495696759</v>
+        <v>0.180772752243179</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>17.52466754115702</v>
+        <v>17.52052351355372</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.935739682237298</v>
+        <v>2.935045472989063</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.02817620882099452</v>
+        <v>0.02818534211395997</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02143525284488845</v>
+        <v>0.02150923456629217</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2833935561927062</v>
+        <v>0.2829429283902015</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2881687054257782</v>
+        <v>0.2882801085457229</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>977437636.1167971</v>
+        <v>997389882.243656</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>308.89</v>
+        <v>306.27</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1712768199625058</v>
+        <v>-0.1783060366147065</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.2028439443598545</v>
+        <v>-0.2096054091718497</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>208596505900</v>
+        <v>206827193700</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.7319587628866</v>
+        <v>18.57307459066101</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.8335122613649</v>
+        <v>15.69367037200682</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.481135511995528</v>
+        <v>2.460090560584254</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.10931796966161</v>
+        <v>6.057498833138856</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.161545041192097</v>
+        <v>1.151692834879419</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>8.995409557514966</v>
+        <v>8.923847019090763</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.645349944690923</v>
+        <v>2.62430499327965</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07215844740570988</v>
+        <v>0.07277572997404161</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1830577103599527</v>
+        <v>0.1834755127640662</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.008470672645869204</v>
+        <v>0.008703536505114684</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01146039043025025</v>
+        <v>0.01155842883730042</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9613361264907827</v>
+        <v>0.963803936011258</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2074093233923537</v>
+        <v>0.2053983245864747</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>912131760.4375204</v>
+        <v>910012202.6841878</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>137.08</v>
+        <v>133.045</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2995759271501415</v>
+        <v>-0.3201931662364356</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5749984498046754</v>
+        <v>-0.5875085260742854</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>322.54</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>394854827600</v>
+        <v>383232131150</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>21.15432098765432</v>
+        <v>20.53163580246913</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.10218857739603</v>
+        <v>14.6449120911116</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.501133059336556</v>
+        <v>5.339205193167728</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.089068471814533</v>
+        <v>5.909834511471874</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4604175744371826</v>
+        <v>0.4468650145243284</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>13.63777379639449</v>
+        <v>13.32964292550371</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.166875567382309</v>
+        <v>7.004947701213481</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.07273559291288249</v>
+        <v>-0.07494152411964322</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4007453872822595</v>
+        <v>0.401963745137832</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4461611315475387</v>
+        <v>0.4477256888007968</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01459002042602859</v>
+        <v>0.01503250779811342</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.034944337151939</v>
+        <v>2.026299757667121</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5405225003117969</v>
+        <v>0.5440448578116766</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4277747868.814545</v>
+        <v>4269154024.027689</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>106.7</v>
+        <v>106.9875</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4032088205592315</v>
+        <v>0.4069897253006631</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1815601748868605</v>
+        <v>-0.1793549129400936</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>420551078756</v>
+        <v>421684241222</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>31.75595238095238</v>
+        <v>31.83633928571428</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.61034510885216</v>
+        <v>20.66101628151851</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.641154026940387</v>
+        <v>6.657965420592183</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.387891021179279</v>
+        <v>8.409124098637765</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.016190476190476</v>
+        <v>1.018762857142857</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>22.1222877644238</v>
+        <v>22.17546631994605</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>6.993542499107778</v>
+        <v>7.010353892759574</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.03232663209476083</v>
+        <v>0.03224500719837717</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5407773238747555</v>
+        <v>0.5408893179273189</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1652018109973663</v>
+        <v>0.1652264439794402</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01555763823805061</v>
+        <v>0.01551583128870195</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.697424970031328</v>
+        <v>0.6970592868970297</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3523286318801636</v>
+        <v>0.3467063374433904</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>1946576732.440821</v>
+        <v>1861820634.651652</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>82.97</v>
+        <v>81.06</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.1284663586164958</v>
+        <v>-0.1485293844697257</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1512888707037644</v>
+        <v>-0.1708265139116203</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>250901280000</v>
+        <v>245125440000</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>11.83594864479315</v>
+        <v>11.56348074179743</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.62842102614351</v>
+        <v>10.38123044175118</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>1.943389334262809</v>
+        <v>1.898651737864529</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.404170208391143</v>
+        <v>1.371845692324768</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6291179910295474</v>
+        <v>0.6146354628522973</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.29278560864447</v>
+        <v>15.11845198204099</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>3.924443514968436</v>
+        <v>3.879705918570156</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.07640455241997968</v>
+        <v>0.07820485942783612</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1136130772086843</v>
+        <v>0.1138834463486604</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2890835249581815</v>
+        <v>-0.2889987083306532</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.02229721586115464</v>
+        <v>0.0228226005428078</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.7232604328549544</v>
+        <v>0.7324395609256275</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.2443852021271254</v>
+        <v>0.2358072214064121</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1139280111.489665</v>
+        <v>1129453997.640034</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 12:05 ET</t>
+          <t>2026-09-28 15:00 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-29)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -784,13 +784,13 @@
         <v>0.003132387706855792</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3061103293173343</v>
+        <v>0.3019845712332221</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2788184607754385</v>
+        <v>0.2784776666105622</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13443672552.63886</v>
+        <v>13396328030.79305</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>28.29</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.6493370076411</v>
+        <v>24.63709184202832</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.39479859510184</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1476982115677321</v>
+        <v>0.1482686423135464</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2335258515251684</v>
+        <v>0.2341531814031865</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007148187423903224</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5575829483255803</v>
+        <v>0.5559009439283675</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4328774577883728</v>
+        <v>0.4313552623124653</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10895141814.20988</v>
+        <v>10852564562.72502</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>16.84011916583913</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.72599874053322</v>
+        <v>20.74481097457083</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.231501562397671</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1874881699714956</v>
+        <v>-0.1882249885775342</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2976642954022224</v>
+        <v>0.2983658194085921</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002509117432530999</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7606959957623504</v>
+        <v>0.7623052681932441</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3201306548172854</v>
+        <v>0.3206523161285895</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8498466011.197147</v>
+        <v>8500131780.098979</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>19.53571428571428</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.02164596193571</v>
+        <v>22.03324092907989</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.413598603805693</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1128858251793868</v>
+        <v>-0.1133526679712982</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.184280219876531</v>
+        <v>0.1847085227754175</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.835099635657726</v>
+        <v>0.8343667953128601</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4518679420447112</v>
+        <v>0.4529088218280257</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8746435772.460945</v>
+        <v>8738257341.305389</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>28.78742138364779</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.79004633953015</v>
+        <v>16.76826210740472</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>18.29632094372692</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7145528250193844</v>
+        <v>0.7167802601878173</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9784781585721893</v>
+        <v>0.9810276253593744</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1292,13 +1292,13 @@
         <v>0.002272131434064494</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.29790985299716</v>
+        <v>1.305861092676486</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.3777194801400032</v>
+        <v>0.389194698065552</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27065550813.90577</v>
+        <v>26600098382.11532</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>26.59308807134894</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>21.51121750549527</v>
+        <v>21.50634761136707</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>7.987068185583226</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2362428144550839</v>
+        <v>0.2365227490926125</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2812626365261797</v>
+        <v>0.2818814327329731</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.002934518319778654</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8366355973533384</v>
+        <v>0.8266593683881774</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.5066141380923777</v>
+        <v>0.4905097236598456</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>13926459563.90998</v>
+        <v>13481261198.45398</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>302.9237288135594</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>167.5815565052112</v>
+        <v>167.4563377261686</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.62458348357927</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8076197353146044</v>
+        <v>0.8089714186208503</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1270229764695137</v>
+        <v>0.1273957703049913</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.529113343916622</v>
+        <v>1.527550059420665</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.4155576749021161</v>
+        <v>0.409613927618917</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13712688120.15066</v>
+        <v>13786592185.9667</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>43.37096774193548</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>18.87413903221767</v>
+        <v>18.8530180455123</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>18.66478767058718</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.297904432509603</v>
+        <v>1.300478768822869</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8768993857144307</v>
+        <v>0.8789825807479386</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1670,13 +1670,13 @@
         <v>0.007437709185570845</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.593244013617408</v>
+        <v>1.596157977234559</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3845078458916448</v>
+        <v>0.3896621793452344</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9132935504.741922</v>
+        <v>9303515124.854837</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>33.40282301845821</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.19232993286218</v>
+        <v>40.1819790290682</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.350124486828477</v>
@@ -1754,10 +1754,10 @@
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1689254374092086</v>
+        <v>-0.1687113520642143</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.08925442841334497</v>
+        <v>0.08948342311209245</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1796,13 +1796,13 @@
         <v>0.006002687123477658</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1723598875534204</v>
+        <v>-0.1725160043142916</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1801045462565304</v>
+        <v>0.1814114731558173</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2000773443.407516</v>
+        <v>1975564704.342651</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>21.43343653250774</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>18.45338156056385</v>
+        <v>18.45057545150642</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>5.959582654741612</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1614909962254547</v>
+        <v>0.1616676449382926</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1473740919681175</v>
+        <v>0.1477011938735422</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1076954468673943</v>
+        <v>0.09973998985696915</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3551349845388983</v>
+        <v>0.3518610586434247</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2401718174.330054</v>
+        <v>2374414112.674433</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -1979,37 +1979,37 @@
         <v>1085242454860</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.64396285919557</v>
+        <v>12.63698906836538</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.68191336128691</v>
+        <v>22.68188686097226</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.820006526771115</v>
+        <v>2.81845114924601</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.443875137574199</v>
+        <v>1.443078766744382</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3483089776081094</v>
+        <v>0.3481168674302191</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.33811917771911</v>
+        <v>15.33029925569177</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.050742163795501</v>
+        <v>3.049186786270397</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.022321678556072</v>
+        <v>0.02233399689522718</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.442553074875241</v>
+        <v>-0.44285988437279</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06082839480209024</v>
+        <v>0.06028865501629332</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02424504518778726</v>
+        <v>0.02323224740464951</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.134452450792259</v>
+        <v>0.1347616100089321</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2198883716.304179</v>
+        <v>2220159570.140381</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>336.83</v>
+        <v>336.59</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.03487153935898268</v>
+        <v>0.0341341668878663</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.08095497953615283</v>
+        <v>-0.08160982264665761</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>902539353300</v>
+        <v>901896270900</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>14.4810834049871</v>
+        <v>14.4707652622528</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.44884495976241</v>
+        <v>13.4387151960241</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.032390068641582</v>
+        <v>3.030229413069115</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.507535600830757</v>
+        <v>2.505748917506233</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7582186565667516</v>
+        <v>0.7576784063587059</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.65005746350365</v>
+        <v>19.64315447509661</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.150525490453007</v>
+        <v>6.148364834880541</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1800852222185313</v>
+        <v>-0.1802136290438453</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07675294408650291</v>
+        <v>0.07679678088081165</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2882882398229152</v>
+        <v>-0.2882365971895516</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01781314015972449</v>
+        <v>0.01782584152826882</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7792694958452768</v>
+        <v>0.7718781883291154</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.169454896377173</v>
+        <v>0.1854938933482376</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2475532531.820114</v>
+        <v>2478789947.98411</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>367.82</v>
+        <v>367.74</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.06159082295374874</v>
+        <v>0.06135992940300028</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.04603573929506966</v>
+        <v>-0.04624322431724459</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>686737305150</v>
+        <v>686587941373</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.25063721325403</v>
+        <v>31.24384027187766</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.50081015698603</v>
+        <v>24.48745188007209</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.4364616334742</v>
+        <v>15.43310423873854</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.00698012450964</v>
+        <v>20.00262865256695</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.107362048920092</v>
+        <v>2.106903702544383</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.99602395869132</v>
+        <v>23.99089083005705</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.69493582876281</v>
+        <v>15.69157843402715</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03059830861439842</v>
+        <v>0.03060496512359274</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2754940352183983</v>
+        <v>0.2759122682464126</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1418089872601016</v>
+        <v>0.142115053421455</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007286172584416291</v>
+        <v>0.00728775765486485</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.2962731587847834</v>
+        <v>0.3012001491799892</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1760971385482051</v>
+        <v>0.1766630962178798</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2397844203.289577</v>
+        <v>2445815294.001974</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>568.21</v>
+        <v>568.26</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.009020998833554783</v>
+        <v>0.009109788277495534</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05492074580443418</v>
+        <v>-0.05483758295494245</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>498340625560</v>
+        <v>498384477360</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.20318506315211</v>
+        <v>31.20593080724876</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.50267462821056</v>
+        <v>25.49510211705682</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.20461834962802</v>
+        <v>14.20586829404555</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>89.31762965603281</v>
+        <v>89.32548921760826</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.379069339844669</v>
+        <v>1.379190691927512</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.13676187194791</v>
+        <v>23.1387446807741</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.58520153806687</v>
+        <v>14.58645148248439</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03300553708924874</v>
+        <v>0.03300263300158735</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.223525983766258</v>
+        <v>0.2239970902635162</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1615922813405704</v>
+        <v>0.1619592203965627</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005930905827070977</v>
+        <v>0.005930383979164467</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2849135101435682</v>
+        <v>0.2869541046326143</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.178471637592573</v>
+        <v>0.1784708934114141</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1543195946.455705</v>
+        <v>1564935163.187866</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>377.81</v>
+        <v>377.83</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1230975233497125</v>
+        <v>0.1231569763828957</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1815562583943503</v>
+        <v>-0.1815129327152204</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>343106037275</v>
+        <v>343124200163</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.29490064947592</v>
+        <v>24.29618674040255</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.22084547269216</v>
+        <v>17.21600401052094</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.762239351996872</v>
+        <v>0.7622797024030888</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.476944209269962</v>
+        <v>3.477128267087874</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7361418329952167</v>
+        <v>-0.7361808018860877</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.0544982057602</v>
+        <v>15.05520320471219</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8616397461061162</v>
+        <v>0.8616800965123331</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06883294793519165</v>
+        <v>0.0688293043416373</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4107844291385925</v>
+        <v>0.4112558713133903</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01263477291340243</v>
+        <v>0.01271517410870682</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02398030756200207</v>
+        <v>0.02397903819177937</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.429241246835034</v>
+        <v>0.4377240790191192</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.1911321691761181</v>
+        <v>0.1949010994954906</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1852677691.853762</v>
+        <v>1859810112.65859</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.91763191763192</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.35593334018854</v>
+        <v>14.35904704498654</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.865615365313244</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4570722377955256</v>
+        <v>0.4567562772165517</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1133339158333719</v>
+        <v>0.1132136380003781</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2678,13 +2678,13 @@
         <v>0.02534916630775857</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5530586325380339</v>
+        <v>-0.551556469350051</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2529274261554335</v>
+        <v>0.2578079794257925</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2335984415.416381</v>
+        <v>2337218226.222433</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>272.03</v>
+        <v>271.95</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.3119363009046359</v>
+        <v>0.3115504798405166</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.03216280641833003</v>
+        <v>-0.03244743302380193</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>179.8</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>655564666104</v>
+        <v>655371874231</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.44855491329479</v>
+        <v>31.4393063583815</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.90807479627158</v>
+        <v>21.89591549993266</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.694285309806084</v>
+        <v>6.692316619499842</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.811846429958456</v>
+        <v>7.809549081451318</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.893827654396111</v>
+        <v>-3.892682537268032</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.28277795873355</v>
+        <v>20.27706255872762</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.986476591244677</v>
+        <v>6.984507900938435</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02853723052400162</v>
+        <v>0.02854562537025499</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4354777955499247</v>
+        <v>0.4358525615646527</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09209213364429392</v>
+        <v>0.09230352445404599</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01940962393853619</v>
+        <v>0.01941533370104799</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1559413470019734</v>
+        <v>-0.157074155069618</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1914410238094823</v>
+        <v>0.191741468346202</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1701134739.90506</v>
+        <v>1708404011.753947</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>39.25270758122744</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.929729865795</v>
+        <v>34.91932334041608</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.17591057621222</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1237621284802926</v>
+        <v>0.1240970278423421</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05251920309976521</v>
+        <v>0.05264324144712451</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2930,13 +2930,13 @@
         <v>0.008990159109721329</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.05224564896969824</v>
+        <v>-0.05000685500234299</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3071875427482957</v>
+        <v>0.3077459276137968</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2822809296.026516</v>
+        <v>2821016151.449915</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>149.03</v>
+        <v>149.045</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.05106147864226807</v>
+        <v>0.05116726890046852</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1089387144992526</v>
+        <v>-0.108849028400598</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>354275447881</v>
+        <v>354311106015</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>22.07851851851852</v>
+        <v>22.08074074074074</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>21.0539298247366</v>
+        <v>21.05264883042422</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.070634340024359</v>
+        <v>4.071044052934553</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.647367476201874</v>
+        <v>6.648036539559205</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>21.06921481481504</v>
+        <v>21.07133544973567</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.84884952860638</v>
+        <v>17.85052724263668</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.358850168685081</v>
+        <v>4.359259881595276</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04491702740107784</v>
+        <v>0.04491250691793532</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04866496194824954</v>
+        <v>0.0488343257229833</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02639233534539964</v>
+        <v>0.02647214080517712</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02879017647453533</v>
+        <v>0.02878727900969506</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.04068520239235188</v>
+        <v>-0.03059475853779217</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1496939609533533</v>
+        <v>0.1495866310155668</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1268334515.048696</v>
+        <v>1271269678.848826</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -3182,13 +3182,13 @@
         <v>0.0320466383800752</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.708593383156998</v>
+        <v>0.7064666365582442</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2333296856658099</v>
+        <v>0.2352095735933773</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1388879348.295605</v>
+        <v>1385051008.94694</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>154.2817258883249</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>43.85595196129541</v>
+        <v>43.78435374362707</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>23.99692100229996</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.517919894304986</v>
+        <v>2.52367256101801</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9344760313425187</v>
+        <v>0.9370269555038113</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.581264143820687</v>
+        <v>2.57633782396688</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6248756710282831</v>
+        <v>0.6355259972551116</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10740613516.25956</v>
+        <v>10754885318.6439</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>55.76923076923077</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.74261870976642</v>
+        <v>35.7135487102158</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.76845098484184</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5603006377927262</v>
+        <v>0.5615706862890963</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3034183449517491</v>
+        <v>0.3042454989308816</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004391981528838609</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.645195224108735</v>
+        <v>1.653708998784613</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.3941800722814858</v>
+        <v>0.3971159842269665</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2128665778.871167</v>
+        <v>2105351252.599284</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>184.4</v>
+        <v>184.39</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.190411395086867</v>
+        <v>-0.1904552990242268</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.275014743463731</v>
+        <v>-0.275054059367014</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>145744228000</v>
+        <v>145736324300</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>69.063670411985</v>
+        <v>69.05992509363293</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>68.87611577675351</v>
+        <v>68.52556979516272</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.550552986861003</v>
+        <v>1.550468900473429</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>23.91289454006558</v>
+        <v>23.91159774535082</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3696338527718098</v>
+        <v>0.3696138075520282</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>26.53168748201439</v>
+        <v>26.5305502589928</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>1.961755710410128</v>
+        <v>1.961671624022554</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001440880389444994</v>
+        <v>-0.001440958532532442</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>0.002723072187162945</v>
+        <v>0.007797896465034926</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.15905375185713</v>
+        <v>0.1594789481710119</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.260302443640757</v>
+        <v>1.231298283538854</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.359388130186453</v>
+        <v>0.3265156952935771</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1348244443.427433</v>
+        <v>1266194328.628845</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>916.5</v>
+        <v>916.28</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.002362330294080728</v>
+        <v>0.00212171958740881</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.205799010390038</v>
+        <v>-0.2059896532898899</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>270373915500</v>
+        <v>270309013960</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>13.96252285191956</v>
+        <v>13.95917123705058</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.7453156945746</v>
+        <v>12.74064568139758</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.292528345642165</v>
+        <v>2.291978038783418</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.240811213765459</v>
+        <v>2.240273321275521</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3272621886993471</v>
+        <v>0.3271836314909305</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.27916782403721</v>
+        <v>26.27710043512885</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>6.995106840940502</v>
+        <v>6.994556534081755</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1535466168148162</v>
+        <v>-0.1535834835539126</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09550231524379549</v>
+        <v>0.09564080079804338</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3854485216849813</v>
+        <v>-0.3854093344279584</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01963993453355155</v>
+        <v>0.01964465010695421</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.587432553149905</v>
+        <v>1.579825351943071</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.2887983359912376</v>
+        <v>0.3111826575726561</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2015978941.950897</v>
+        <v>2031486619.277751</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>220.69</v>
+        <v>220.67</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2429159519725558</v>
+        <v>-0.2429845626072041</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3361908199482644</v>
+        <v>-0.3362509775612104</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>207919552460</v>
+        <v>207900709780</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>19.27423580786026</v>
+        <v>19.27248908296943</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.06777134062949</v>
+        <v>17.0632003286457</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.009096667872701</v>
+        <v>3.008823968913267</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.020739898989899</v>
+        <v>6.020194270289098</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2349514403710099</v>
+        <v>0.2349301479299957</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>16.39970115652549</v>
+        <v>16.39853953393749</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.849943593209546</v>
+        <v>3.849670894250112</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06555900990900007</v>
+        <v>0.06556495172346592</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1292766596877433</v>
+        <v>0.1294768104324941</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04739825929135555</v>
+        <v>0.04750578143871986</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.030540577280348</v>
+        <v>0.03054334526668782</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.9072151938617945</v>
+        <v>0.8811376584612348</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3107046690944907</v>
+        <v>0.3064314291585977</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1239209612.118459</v>
+        <v>1242825112.1433</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1185.7</v>
+        <v>1185.97</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.09750455040609318</v>
+        <v>0.097754467103917</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.08273701311259818</v>
+        <v>-0.08252813986771368</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>716.08</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1116622303700</v>
+        <v>1116876573770</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>39.66878554700569</v>
+        <v>39.67781866845099</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.79143587824644</v>
+        <v>26.78039424959482</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>14.01633202327724</v>
+        <v>14.01952373251759</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>31.23228784792939</v>
+        <v>31.23939986422267</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4193479325547195</v>
+        <v>0.419443423776605</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.84783912406939</v>
+        <v>26.85371076116273</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.59397010636936</v>
+        <v>14.59716181560971</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01795942991067804</v>
+        <v>0.0179553412355211</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4806517174846583</v>
+        <v>0.4815994977016183</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2385892016199385</v>
+        <v>0.2390593474579783</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005642236653453656</v>
+        <v>0.005640952132010085</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3437267738249194</v>
+        <v>0.357598458182214</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3133816624190013</v>
+        <v>0.3139587734725938</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2812960630.770133</v>
+        <v>2853729577.00765</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>15.56832797427653</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.33465325933085</v>
+        <v>14.33230260328399</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.4142435141351</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08606240364709494</v>
+        <v>0.08624052988591813</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3269007736940051</v>
+        <v>-0.3268008476699206</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4066,13 +4066,13 @@
         <v>0.0214282026126917</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.377219355648818</v>
+        <v>1.37118413284995</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2439301299427863</v>
+        <v>0.2609535691634336</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>952524127.3643148</v>
+        <v>956808924.5290629</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -4192,13 +4192,13 @@
         <v>0.0005028558416668249</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.855156016921367</v>
+        <v>2.857958824207671</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.6709770778068195</v>
+        <v>0.721414067327511</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>24959698438.01126</v>
+        <v>25155134915.873</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>131.44</v>
+        <v>131.45</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.1085791609331942</v>
+        <v>-0.1085113413319263</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.3188578535523656</v>
+        <v>-0.3188060320257036</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>192.97</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>135890821280</v>
+        <v>135901159900</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>81.63975155279503</v>
+        <v>81.64596273291926</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.53555449929782</v>
+        <v>27.52273658522398</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.224193679065978</v>
+        <v>9.224895458865056</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>10.84831575583253</v>
+        <v>10.84914109939278</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>130.6236024844748</v>
+        <v>130.6335403726736</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>40.65371776440241</v>
+        <v>40.65668096875896</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>9.628076383383112</v>
+        <v>9.628778163182188</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03370352726445749</v>
+        <v>0.03370096328368424</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.964884965540713</v>
+        <v>1.966491448991747</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2534231102869904</v>
+        <v>0.2539880089677118</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.689278771415385</v>
+        <v>0.680908358701193</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5486372136898701</v>
+        <v>0.5513107222422996</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2046580123.219203</v>
+        <v>2062078409.913101</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>37.96247357293869</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.849236506538002</v>
+        <v>9.849957747316838</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.570725182115047</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.85435698977671</v>
+        <v>2.854074763242492</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05170766447375896</v>
+        <v>-0.05181447295711994</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4444,13 +4444,13 @@
         <v>0.05986773407587887</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3384493604414484</v>
+        <v>0.3469767748165458</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.1910176898317054</v>
+        <v>0.1918027931372212</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>938226920.5015962</v>
+        <v>939924699.5058314</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>182.02</v>
+        <v>181.92</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.08338792899962888</v>
+        <v>0.0827927263136603</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.0893080502326512</v>
+        <v>-0.08980837544403875</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1292077872598</v>
+        <v>1291368017707</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.724894486155574</v>
+        <v>7.720525201943947</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004210994212952269</v>
+        <v>0.004205447726693081</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.634346710180119</v>
+        <v>6.630594251633637</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.807651022687995</v>
+        <v>4.804931763059778</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.0172873492686601</v>
+        <v>0.01727757135617783</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.802981027678777</v>
+        <v>7.798547359556308</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.604094405930858</v>
+        <v>6.600341947384376</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07265511349372848</v>
+        <v>0.07269623127159702</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1833.45858519472</v>
+        <v>1834.83906011713</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2434.16824681993</v>
+        <v>2436.325292862097</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.648170530710911</v>
+        <v>1.649076517150396</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.7777873271891454</v>
+        <v>0.7681477162484222</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3366368437.342227</v>
+        <v>3391219023.770243</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>600.35</v>
+        <v>600.01</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6082240011562836</v>
+        <v>0.6073132055197497</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1063959632645164</v>
+        <v>-0.1069020436717623</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>315.05</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>75668563062</v>
+        <v>75625709207</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.816067182406588</v>
+        <v>1.817502989459575</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.3635774948353487</v>
+        <v>0.3847343199442911</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3836216693.11176</v>
+        <v>3828740338.151042</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-94.46103896103897</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>124.1646984542712</v>
+        <v>123.6500081507184</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>115.6895039878733</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.37664331907684</v>
+        <v>4.386836918118143</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.151451198349944</v>
+        <v>3.160248758681224</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7508936452727831</v>
+        <v>0.7541715269041857</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12609510845.12123</v>
+        <v>12673550841.14075</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>765.5599999999999</v>
+        <v>765.61</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1205995859754845</v>
+        <v>0.1206727742027938</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01771944006056181</v>
+        <v>-0.01765528567945907</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>815503776297</v>
+        <v>815557038208</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9959960065625689</v>
+        <v>0.9959498199346021</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1124283774273622</v>
+        <v>0.1177761963223539</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>31592646838.55424</v>
+        <v>31467728797.33297</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>452.91</v>
+        <v>452.88</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.4170708699911583</v>
+        <v>0.416977005589622</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.05446764091858036</v>
+        <v>-0.05453027139874744</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,13 +4914,13 @@
         <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2349008656800</v>
+        <v>2348853062400</v>
       </c>
       <c r="L36" s="6" t="n">
         <v>28.68899965225455</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6908915807623011</v>
+        <v>0.6903728570621391</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.45395915587732</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.52460451262166</v>
+        <v>40.55580474924771</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.6211721718747</v>
+        <v>40.65528995494634</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2649533019805259</v>
+        <v>0.2649708532061473</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.172614709405229</v>
+        <v>2.184512697624831</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3057861047019841</v>
+        <v>0.3298638145831211</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4157110588.347372</v>
+        <v>4147654996.64744</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
         <v>-24.33070866141732</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-105.9548226147546</v>
+        <v>-107.1054120668128</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>2.145106578762287</v>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02150923456629217</v>
+        <v>0.02158321628769588</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2822536937753776</v>
+        <v>0.2833935561927062</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2881601771701584</v>
+        <v>0.2881687054257782</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>1008951394.669157</v>
+        <v>977437636.1167971</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
         <v>18.57216494845361</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.69290175263313</v>
+        <v>15.68736364206542</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.459970074221212</v>
@@ -5200,10 +5200,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1834755127640662</v>
+        <v>0.1838933151681801</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.008703536505114684</v>
+        <v>0.008936400364360608</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5242,13 +5242,13 @@
         <v>0.01155899495518441</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9630740660173449</v>
+        <v>0.9613361264907827</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2053884871577115</v>
+        <v>0.2074093233923537</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>915081046.4228109</v>
+        <v>912131760.4375204</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>132.62</v>
+        <v>132.63</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.3223647465615098</v>
+        <v>-0.3223136505538611</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5888261921002047</v>
+        <v>-0.5887951881937125</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>322.54</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>382007931400</v>
+        <v>382036736100</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>20.46604938271605</v>
+        <v>20.46759259259259</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>14.59813026812898</v>
+        <v>14.58655476643348</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.322149593881049</v>
+        <v>5.322550902099558</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>5.890956089378782</v>
+        <v>5.891400287545677</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.445437545388526</v>
+        <v>0.4454711328976037</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>13.29718800106045</v>
+        <v>13.29795164634146</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>6.987892101926802</v>
+        <v>6.988293410145311</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.07518168508896043</v>
+        <v>-0.07517601656109427</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4019637451378317</v>
+        <v>0.4031821029934042</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4477256888007968</v>
+        <v>0.4492902460540551</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01508068164681044</v>
+        <v>0.01507954459775315</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.027558669345245</v>
+        <v>2.034944337151939</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5453209634813888</v>
+        <v>0.5405225003117969</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4287957960.210384</v>
+        <v>4277747868.814545</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
         <v>31.76785714285714</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.61322002934255</v>
+        <v>20.60837076758986</v>
       </c>
       <c r="N40" s="6" t="n">
         <v>6.643643681673905</v>
@@ -5452,10 +5452,10 @@
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5411399624918463</v>
+        <v>0.5415026011089366</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1654159823651633</v>
+        <v>0.1656301537329605</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5494,13 +5494,13 @@
         <v>0.01555180813190931</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.6967470967267494</v>
+        <v>0.697424970031328</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.346593307189622</v>
+        <v>0.3523286318801636</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>1887802169.979013</v>
+        <v>1946576732.440821</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
         <v>11.52853067047076</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.34985366580461</v>
+        <v>10.34734209065619</v>
       </c>
       <c r="N41" s="6" t="n">
         <v>1.892913210177762</v>
@@ -5578,10 +5578,10 @@
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1138834463486604</v>
+        <v>0.1141538154886368</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2889986869158109</v>
+        <v>-0.2889138488734401</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5620,13 +5620,13 @@
         <v>0.02289178989049063</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.7353912728038535</v>
+        <v>0.7232604328549544</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.2376897609219769</v>
+        <v>0.2443852021271254</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1138873836.146473</v>
+        <v>1139280111.489665</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 16:12 ET</t>
+          <t>2026-09-28 20:30 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-30)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>329.4</v>
+        <v>335.67001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.215453260508244</v>
+        <v>0.2385889742238461</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.0461574100886083</v>
+        <v>-0.02800136097758721</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>345.34</v>
@@ -714,31 +714,31 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4838015066400</v>
+        <v>4930104985738</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>37.60273972602739</v>
+        <v>38.31849429223745</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.29742342428641</v>
+        <v>34.95026248878097</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.36370330167965</v>
+        <v>10.5609727578504</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.01222508370536</v>
+        <v>45.86901652692662</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.148972602739725</v>
+        <v>1.170842881151698</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>28.98031923364552</v>
+        <v>29.52601946132023</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.45959189328718</v>
+        <v>10.65654630333124</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02825187563992163</v>
+        <v>0.02772498312515696</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003217972070431087</v>
+        <v>0.003157863283645745</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3059734413934497</v>
+        <v>0.3088872491216167</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2845157292199745</v>
+        <v>0.2151277349327726</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13505220892.73459</v>
+        <v>13189992830.64099</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>508.96</v>
+        <v>517.24</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.0761618754443516</v>
+        <v>0.09366938159155236</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.0808350791013509</v>
+        <v>-0.06588167304774983</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3779307928000</v>
+        <v>3840791482000</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.27555555555555</v>
+        <v>28.73555555555555</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.62451251702354</v>
+        <v>25.01268996625673</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.38898058395788</v>
+        <v>11.57426186192702</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.546959652973527</v>
+        <v>8.686005601430422</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8981261149780855</v>
+        <v>0.9127372518690368</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.73168831769621</v>
+        <v>19.02796747285791</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.71405780514045</v>
+        <v>11.89933908310958</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01772467374349392</v>
+        <v>0.01744093640957518</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1482686423135464</v>
+        <v>0.1488390730593609</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2341533287192044</v>
+        <v>0.2347806602160802</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007151839044325684</v>
+        <v>0.007037352099605599</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5569667205637707</v>
+        <v>0.5584985789112304</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.2604336440530852</v>
+        <v>0.2538404719516619</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10783704426.08385</v>
+        <v>10582988437.42306</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>340.92</v>
+        <v>351.118</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.08177060638617739</v>
+        <v>0.1141298010474652</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1656591860209001</v>
+        <v>-0.1407014023151661</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4125851779623</v>
+        <v>4249269110518</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.74875868917577</v>
+        <v>17.24528301886792</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.60297710550509</v>
+        <v>21.23846478660302</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.181419114956062</v>
+        <v>9.453606329320916</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.399536784911317</v>
+        <v>6.589253872095928</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1489476851532704</v>
+        <v>0.1533633048957485</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.79984091699664</v>
+        <v>13.17410085494843</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.308912577117338</v>
+        <v>9.581099791482194</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01301346611566308</v>
+        <v>0.01263878380207152</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1870709459410834</v>
+        <v>-0.1880164977957329</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2994194454752559</v>
+        <v>0.2998068897256299</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002522585943916461</v>
+        <v>0.0024493190323481</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7605668214202917</v>
+        <v>0.7651051310912055</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3195767803420648</v>
+        <v>0.2843108725665713</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8540046283.51343</v>
+        <v>8510481795.666606</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1079,55 +1079,55 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>246.67</v>
+        <v>250.9</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.08905077262693162</v>
+        <v>0.1077262693156733</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1411211699164345</v>
+        <v>-0.1263927576601671</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>196</v>
+        <v>165.29</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2653453857000</v>
+        <v>2698956390000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.57698412698413</v>
+        <v>19.91269841269841</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.07978687782302</v>
+        <v>22.47025143811045</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.420809943533416</v>
+        <v>3.479471418626238</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.80980116747036</v>
+        <v>4.892281643160146</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2216074852953026</v>
+        <v>0.2254077028442511</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.01773980401343</v>
+        <v>11.1968857506191</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.607767193945957</v>
+        <v>3.666428669038779</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004381082402971668</v>
+        <v>-0.004307220391953054</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1133526679712979</v>
+        <v>-0.1138195107632095</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1847085227754173</v>
+        <v>0.1851368256743036</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8347722388044967</v>
+        <v>0.8358358199063929</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.442579640311021</v>
+        <v>0.2686099560691078</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8644899733.382998</v>
+        <v>8522539501.465707</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>227.21</v>
+        <v>230.37</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.2031241337395449</v>
+        <v>0.2198569899633773</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.03944364589498595</v>
+        <v>-0.02608438319100359</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5503253410000</v>
+        <v>5579791770000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.57987421383647</v>
+        <v>28.97735849056603</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.64736884306312</v>
+        <v>16.85702662579455</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18.16441091332777</v>
+        <v>18.41703860791038</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>24.00259363099605</v>
+        <v>24.33641782831988</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.229416677362769</v>
+        <v>0.232607367475292</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.62195093872904</v>
+        <v>23.94950408059332</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.21859797537042</v>
+        <v>18.47122566995303</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02307834848550069</v>
+        <v>0.02276178130568482</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7167802601878173</v>
+        <v>0.7190076953562501</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9810276253593739</v>
+        <v>0.9835770921465585</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002288631662338806</v>
+        <v>0.002257238355688675</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.297877359638944</v>
+        <v>1.297340310734804</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.3747687255987011</v>
+        <v>0.3703380218585207</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27160328553.68591</v>
+        <v>26816682332.50897</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>738.79</v>
+        <v>734.55</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.1358835665267839</v>
+        <v>0.1293646012970522</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.05261470595778528</v>
+        <v>-0.05805185812110503</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>779.8200000000001</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1882057603050</v>
+        <v>1871256259994</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>27.45410628019324</v>
+        <v>27.29654403567447</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>22.19460100788056</v>
+        <v>22.05585246360579</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.245669635878519</v>
+        <v>8.198346798193194</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.192159014780588</v>
+        <v>7.15088239460074</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.628091787439608</v>
+        <v>-5.595791527313261</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>18.48208311276524</v>
+        <v>18.38120386276524</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.670015084688584</v>
+        <v>8.622692247003259</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02177191597833969</v>
+        <v>0.02189758873545807</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2369722830541174</v>
+        <v>0.2376100212275316</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2818989216908505</v>
+        <v>0.2825167857362312</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.002842485686054224</v>
+        <v>0.002858893199918318</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8384075541928585</v>
+        <v>0.8371236672662691</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4604514332222305</v>
+        <v>0.457290369884492</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>14218013122.43755</v>
+        <v>13977726593.3773</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>352.84</v>
+        <v>351.22</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.194557960826429</v>
+        <v>-0.1982559998907673</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2926648357155744</v>
+        <v>-0.2959124350981296</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1393558302499</v>
+        <v>1387160035721</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>299.0169491525424</v>
+        <v>297.6440677966102</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>165.2966686342183</v>
+        <v>164.8610271540053</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.44886847488395</v>
+        <v>13.38712046749148</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.14954385318566</v>
+        <v>13.08917013976836</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-7.959746956314153</v>
+        <v>-7.923201241346381</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>115.3709097521616</v>
+        <v>114.8586634305786</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.39215107749544</v>
+        <v>13.33268998680744</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004134739098943537</v>
+        <v>0.004153101083867806</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8089714186208501</v>
+        <v>0.805424077083817</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1273957703049913</v>
+        <v>0.1278156307669018</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.525622938082992</v>
+        <v>1.523604535268877</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.4105096893097155</v>
+        <v>0.4107655256103137</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13817283351.96726</v>
+        <v>13784381332.93909</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>355.1</v>
+        <v>352.75</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.02151776361509605</v>
+        <v>0.01475750806878384</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2826262626262626</v>
+        <v>-0.2873737373737374</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1689416658000</v>
+        <v>1678236345000</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>44.05707196029777</v>
+        <v>43.76550868486352</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.15126214481053</v>
+        <v>19.00325641091827</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.96005407164661</v>
+        <v>18.834579199587</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.97669375062694</v>
+        <v>16.86434446785034</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4383896764366261</v>
+        <v>0.4354884775078001</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>33.00347584333085</v>
+        <v>32.78955178615847</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.35783643831927</v>
+        <v>19.23236156625965</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02332343523038708</v>
+        <v>0.02347881460045486</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.300478768822869</v>
+        <v>1.303053105136136</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8789825807479386</v>
+        <v>0.8810657757814475</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007321881160236553</v>
+        <v>0.007370659107016301</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.594569904090648</v>
+        <v>1.594415181868662</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3682056355982011</v>
+        <v>0.3680750378351958</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9129361093.127928</v>
+        <v>8930063988.395027</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>924.59</v>
+        <v>919.015</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.08202457577530731</v>
+        <v>0.07550029256875357</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.156780665754674</v>
+        <v>-0.1618650250797994</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>410036248610</v>
+        <v>407563853185</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>33.4632645674991</v>
+        <v>33.26149113282665</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.24924750771873</v>
+        <v>39.99716955799227</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.352567502358537</v>
+        <v>1.344411926562077</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.46537567382622</v>
+        <v>11.39624290213111</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>0.6510709790584844</v>
+        <v>0.6471452166035033</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.74603026742809</v>
+        <v>27.57384589351626</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.31420086362047</v>
+        <v>1.30604528782401</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02290041437026989</v>
+        <v>0.02303933463828973</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1685990014824068</v>
+        <v>-0.1684038770643382</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.09026779948728092</v>
+        <v>0.09059323239914874</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1793,16 +1793,16 @@
         <v>80.58620689655173</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005991845034015077</v>
+        <v>0.006028193228619773</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1698189454904585</v>
+        <v>-0.1707209971646982</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1735782749346297</v>
+        <v>0.174038469471881</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2048119472.376538</v>
+        <v>2010068239.805599</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>70.3</v>
+        <v>70.095</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2273876068746221</v>
+        <v>-0.2296406017621143</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.4369694057344226</v>
+        <v>-0.4386112445939452</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>292724981930</v>
+        <v>291871374230</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>21.76470588235294</v>
+        <v>21.70123839009288</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>18.73574251395207</v>
+        <v>18.67826739665441</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.051692338992207</v>
+        <v>6.034045156491636</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.767428130596221</v>
+        <v>9.738945587683386</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6396700143472025</v>
+        <v>0.637804689269803</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.737382289422916</v>
+        <v>9.709483912462375</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.159403558934898</v>
+        <v>6.141756376434327</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03755951380545022</v>
+        <v>0.03766936044689346</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1616676449382928</v>
+        <v>0.1618442936511302</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1477011938735422</v>
+        <v>0.1480282957789663</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1078861492275607</v>
+        <v>0.1078142502568853</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3572766946838056</v>
+        <v>0.3540629440493743</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2404734313.844937</v>
+        <v>2347846836.540981</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>502.35</v>
+        <v>500.76</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01106972693754682</v>
+        <v>0.00786956596246835</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.06581247443002192</v>
+        <v>-0.06876929371071527</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1083495403448</v>
+        <v>1080066006232</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.62849037367772</v>
+        <v>12.58504880128174</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.64537297203556</v>
+        <v>22.57367118656871</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.816555669580724</v>
+        <v>2.80686681498205</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.442108259784024</v>
+        <v>1.437147456986818</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3478827500343815</v>
+        <v>0.3466860453433419</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.32076941297018</v>
+        <v>15.27205706739943</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.04729130660511</v>
+        <v>3.037602452006436</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02234902718112448</v>
+        <v>0.02242617244274642</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4423368345810663</v>
+        <v>-0.4424899389528708</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06128406666346264</v>
+        <v>0.06103684670283682</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02115239581216902</v>
+        <v>0.02068475063196762</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1343838331266105</v>
+        <v>0.134177081925943</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2192730452.879674</v>
+        <v>2165337394.610005</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>334.98</v>
+        <v>332.16</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.02918762656079354</v>
+        <v>0.02052350002517511</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.08600272851296042</v>
+        <v>-0.09369713506139143</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>897582259800</v>
+        <v>890026041600</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>14.40154772141015</v>
+        <v>14.28030954428203</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.36327228961263</v>
+        <v>13.23315832712553</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.015735015270484</v>
+        <v>2.990347312293999</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.493763250204219</v>
+        <v>2.472769721141063</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.754054227879733</v>
+        <v>0.7477062879351964</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.59684692786604</v>
+        <v>19.5157368140833</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.133870437081909</v>
+        <v>6.108482734105425</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1810797820761475</v>
+        <v>-0.1826171284918951</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07769619665720451</v>
+        <v>0.07913086137645919</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2874313181555164</v>
+        <v>-0.2867343905451731</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01791151710549883</v>
+        <v>0.0180635838150289</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7788621670721908</v>
+        <v>0.7769548578312206</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1639170144984192</v>
+        <v>0.1645627726493883</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2538923673.655523</v>
+        <v>2506022829.960525</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>365.88</v>
+        <v>360.13269</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.0559916543480985</v>
+        <v>0.03940394418369664</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.0510672510828124</v>
+        <v>-0.06597326036776707</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>683115233561</v>
+        <v>672384735257</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.08581138487681</v>
+        <v>30.59750977060323</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.36359627421758</v>
+        <v>23.97303029274264</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.35504481120752</v>
+        <v>15.1138449752068</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>19.90145692989937</v>
+        <v>19.5888412022625</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.096247149309128</v>
+        <v>2.063318915451864</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.87154558942195</v>
+        <v>23.50277459815107</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.61351900649613</v>
+        <v>15.37231917049541</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03076054956418068</v>
+        <v>0.0312514530716828</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2759122682464126</v>
+        <v>0.2763305012744266</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.142115053421455</v>
+        <v>0.1424590110366841</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007324805947305128</v>
+        <v>0.007441701557278791</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.2953774063644165</v>
+        <v>0.2910269077725071</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1757573407672058</v>
+        <v>0.1799743232598947</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2305387426.122729</v>
+        <v>2249768166.9255</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>563.58</v>
+        <v>554.635</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.000799096324624271</v>
+        <v>-0.01508533519640876</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.06262162566738183</v>
+        <v>-0.07749945944147829</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>494279948880</v>
+        <v>486434861860</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>30.9489291598023</v>
+        <v>30.45771554091158</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.28513295169621</v>
+        <v>24.87433728669638</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.08887349656529</v>
+        <v>13.86525844027022</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>88.58983425414365</v>
+        <v>87.18375868829085</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.367832136973405</v>
+        <v>1.346122249352788</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>22.95315377464279</v>
+        <v>22.59426537710255</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.46945668500413</v>
+        <v>14.24321674543226</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03327668872117894</v>
+        <v>0.03381976850572923</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2239970902635162</v>
+        <v>0.2244633973505448</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1619592203965627</v>
+        <v>0.1623261594525547</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005979630221086624</v>
+        <v>0.006076068044750151</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2876542968088208</v>
+        <v>0.2835773572004795</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1687571204193007</v>
+        <v>0.1723955204557923</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1566540909.684357</v>
+        <v>1524548858.420665</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>374.94</v>
+        <v>371.67499</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1145660130879045</v>
+        <v>0.1048602756942092</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1877734933495082</v>
+        <v>-0.1948464321303237</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>340499662836</v>
+        <v>337534560271</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.11034660150473</v>
+        <v>23.90039161468716</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.08431978324834</v>
+        <v>16.92989247026221</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7564490686803116</v>
+        <v>0.7498618402080292</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.450531912399565</v>
+        <v>3.420484381596493</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7305497971552543</v>
+        <v>-0.7241881062361474</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.95333085572332</v>
+        <v>14.83823934600008</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8558494627895559</v>
+        <v>0.8492622343172734</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06935983373168569</v>
+        <v>0.0699691314010582</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4112558713133903</v>
+        <v>0.4117273134881871</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01271517410870682</v>
+        <v>0.01279557530401076</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02416386621859498</v>
+        <v>0.02437613572008168</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4324553090402653</v>
+        <v>0.4300623024283645</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.191174214517866</v>
+        <v>0.1884907552110039</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1843282330.494529</v>
+        <v>1819731386.663517</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>161.36</v>
+        <v>163.98</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.315613518080172</v>
+        <v>0.3369751158576262</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.08531262400090689</v>
+        <v>-0.07046085822799164</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>668750065600</v>
+        <v>679608550800</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.76705276705277</v>
+        <v>21.10489060489061</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.16835141027581</v>
+        <v>14.40178146114802</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.852185414058605</v>
+        <v>1.882316714950424</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.596547911789652</v>
+        <v>2.638788481128075</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.033440583440585</v>
+        <v>2.06652053839554</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.753290158022972</v>
+        <v>9.905046925165333</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.940204025923669</v>
+        <v>1.970392719769567</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04568672449039383</v>
+        <v>0.04495402075596042</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4657352973325575</v>
+        <v>0.4654361102357856</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1148270956981992</v>
+        <v>0.1147296643147926</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02553296975706495</v>
+        <v>0.02512501524576168</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5565803905971521</v>
+        <v>-0.5500635065089082</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2536789978491606</v>
+        <v>0.2550513864692091</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2332019893.740789</v>
+        <v>2249756253.679039</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2717,55 +2717,55 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>267.57</v>
+        <v>267.14</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2904267765799855</v>
+        <v>0.2883529883603444</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.048030739673391</v>
+        <v>-0.04956060767780268</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>181.07</v>
+        <v>182.94</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>644816519169</v>
+        <v>643780262850</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>30.93294797687861</v>
+        <v>30.88323699421965</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.54326203462763</v>
+        <v>21.50302838636993</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.584530825077352</v>
+        <v>6.573949114664706</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.683769250685527</v>
+        <v>7.671421002459661</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.829987374505634</v>
+        <v>-3.823832369942202</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.9641444079509</v>
+        <v>19.93342413287086</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.876722106515945</v>
+        <v>6.866140396103299</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.0290129043593823</v>
+        <v>0.02905960477443053</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4358525615646527</v>
+        <v>0.4362273275793809</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09230352445404599</v>
+        <v>0.09251491526379829</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01973315394102478</v>
+        <v>0.01976491727184248</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1565436065024367</v>
+        <v>-0.158241417295156</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1718143810475347</v>
+        <v>0.1719295494781324</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1731637733.257947</v>
+        <v>1675123763.984172</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>106.8</v>
+        <v>105.32</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.05285564050477687</v>
+        <v>-0.06598086196594666</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2098253921278485</v>
+        <v>-0.2207753773305712</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>849922944000</v>
+        <v>838144985600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.55595667870036</v>
+        <v>38.02166064981949</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.29949170198139</v>
+        <v>33.83714905757169</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.155037703848663</v>
+        <v>1.139031560082355</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.647236303670676</v>
+        <v>8.527405688226551</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.323531342303912</v>
+        <v>9.194328848047267</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.29248918041971</v>
+        <v>21.01755370505848</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.239602283105023</v>
+        <v>1.223596139338715</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01589438206765248</v>
+        <v>0.01611773651485768</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1240970278423421</v>
+        <v>0.1236661985065033</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05264324144712451</v>
+        <v>0.05301533483059595</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009152621722846442</v>
+        <v>0.009281238131409041</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.05008695128125387</v>
+        <v>-0.05279685340668275</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3028996400639239</v>
+        <v>0.3045169860525633</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2846465021.9608</v>
+        <v>2805616475.203291</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>148.36</v>
+        <v>146.75</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.04633618044264165</v>
+        <v>0.03498135939577818</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1129446935724961</v>
+        <v>-0.1225710014947683</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>352682717893</v>
+        <v>348855411505</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.97925925925926</v>
+        <v>21.74074074074074</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.95589238472768</v>
+        <v>20.72513276969562</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.052333830005056</v>
+        <v>4.008357977582958</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.617482646241093</v>
+        <v>6.545669845887574</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.97449312169335</v>
+        <v>20.74687830687853</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.7739116351275</v>
+        <v>17.59495547162887</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.340549658665778</v>
+        <v>4.29684694817998</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04511987458605167</v>
+        <v>0.04561177837001127</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.0488343257229833</v>
+        <v>0.04900368949771683</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02647214080517712</v>
+        <v>0.02655194626495438</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02892019412240496</v>
+        <v>0.02923747870528109</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.04078922667700036</v>
+        <v>-0.04371699442517538</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1453352250664473</v>
+        <v>0.1477200347600763</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1268881493.553874</v>
+        <v>1221709761.412506</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3095,52 +3095,52 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>288.04</v>
+        <v>285.53</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1670811581183268</v>
+        <v>-0.1743392691206982</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2922850122850122</v>
+        <v>-0.2952138819638142</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>407</v>
+        <v>405.13</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>287.34</v>
+        <v>285.32</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>287209580680</v>
+        <v>284706815793</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20.11452513966481</v>
+        <v>19.93924581005586</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>19.19469447023003</v>
+        <v>19.02743060715449</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.697696958670261</v>
+        <v>1.682903105600085</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17.23005115243425</v>
+        <v>17.079907323825</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-6.89974990255947</v>
+        <v>-6.839625016240122</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14.53864021241898</v>
+        <v>14.43398769780472</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.055206298056462</v>
+        <v>2.040412444986286</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05257832960950236</v>
+        <v>0.05304052858003719</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.0479210893854749</v>
+        <v>0.04792108938547468</v>
       </c>
       <c r="V21" s="4" t="n">
         <v>0.01423568777486173</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03225246493542563</v>
+        <v>0.03253598571078346</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7076158122226198</v>
+        <v>0.7066022678294781</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2317279633769414</v>
+        <v>0.2320858509246742</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1397489734.963623</v>
+        <v>1344186830.675214</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3221,55 +3221,55 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>607.5700000000001</v>
+        <v>605.51</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.718798929078416</v>
+        <v>1.709580689544039</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.04918622848200305</v>
+        <v>-0.05241001564945225</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>639</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>159.33</v>
+        <v>160.49</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>990703642000</v>
+        <v>987344606000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>154.2055837563452</v>
+        <v>153.6827411167513</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>43.76274500142382</v>
+        <v>43.59036692734633</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>23.98507788403341</v>
+        <v>23.90375513860307</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>14.74096557776985</v>
+        <v>14.69098551112698</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.244962511060401</v>
+        <v>1.240741396171937</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>92.35805579399141</v>
+        <v>92.06291080425453</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>23.96546766735262</v>
+        <v>23.88888216922891</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.008481850317049707</v>
+        <v>0.008509020023991365</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.52367256101801</v>
+        <v>2.52561246783951</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9370269555038113</v>
+        <v>0.937563268337078</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.583289320099062</v>
+        <v>2.579967763401005</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.5558474031970515</v>
+        <v>0.5528777622897511</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10757840417.85991</v>
+        <v>10553616032.69704</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1834.39</v>
+        <v>1813.20959</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.576234300143722</v>
+        <v>0.558034632279687</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.08278665573311461</v>
+        <v>-0.09337707254145089</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>707006908510</v>
+        <v>698843599261</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>58.09869375907112</v>
+        <v>57.93904208998548</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.94546222874737</v>
+        <v>36.48920179305509</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>17.46886383664284</v>
+        <v>17.42086046363315</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>28.27450951643497</v>
+        <v>28.1968128877363</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.954990399519771</v>
+        <v>3.944122326975499</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>44.36551756231663</v>
+        <v>44.24267072541562</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>17.33617683643054</v>
+        <v>17.28817346342085</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01620708625154644</v>
+        <v>0.01625174505633725</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5725528997134688</v>
+        <v>0.5878407650181292</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3134180231863319</v>
+        <v>0.3259493126548507</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.00424119189485333</v>
+        <v>0.004290733979627805</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.646651735766883</v>
+        <v>1.642844138302287</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.373499193296834</v>
+        <v>0.3729825143044539</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2149056360.34242</v>
+        <v>2105405728.12286</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>187.68</v>
+        <v>187.34</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1760109036328806</v>
+        <v>-0.1775036375031109</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2621191271869471</v>
+        <v>-0.2634558678985649</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>148336641600</v>
+        <v>148067915800</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>70.29213483146066</v>
+        <v>70.16479400749061</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>70.85960498556889</v>
+        <v>70.09352739976468</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.578133321985212</v>
+        <v>1.575274384807702</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>24.33824320650492</v>
+        <v>24.29415218620328</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3762086848601587</v>
+        <v>0.375527147387586</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>26.90469663309353</v>
+        <v>26.86603105035971</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>1.989336045534337</v>
+        <v>1.986477108356827</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001415698762860491</v>
+        <v>-0.001418268089108876</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.008008373095275023</v>
+        <v>0.001016735929402879</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1592629606567237</v>
+        <v>0.1596882802827024</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,23 +3562,23 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.248066032696376</v>
+        <v>1.249457789977497</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3527143431145178</v>
+        <v>0.3498645376209936</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1382887230.448431</v>
+        <v>1390752080.666682</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (C)</t>
+          <t>2026-10-27 (C)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>916.24</v>
+        <v>904.6</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.002077972186195876</v>
+        <v>-0.01065252156680263</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.2060243156353174</v>
+        <v>-0.2161110581547501</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>270297213680</v>
+        <v>266863332200</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>13.95856185252895</v>
+        <v>13.7812309567337</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.75202988078092</v>
+        <v>12.58833110244731</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.291877982990919</v>
+        <v>2.262761747373597</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.240175522640987</v>
+        <v>2.211716119991527</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3271693483621275</v>
+        <v>0.3230129578804467</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.27672454623642</v>
+        <v>26.1673408785398</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>6.994456478289256</v>
+        <v>6.965340242671934</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1535901884994969</v>
+        <v>-0.1555665203523978</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09461489527768752</v>
+        <v>0.09476235130600275</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3857500158595004</v>
+        <v>-0.3857093404968824</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01964550772723304</v>
+        <v>0.01989829759009507</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.586993502018283</v>
+        <v>1.583424573865802</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.2653619887134868</v>
+        <v>0.2663575133905691</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2037521288.635612</v>
+        <v>1990551061.599198</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>219.99</v>
+        <v>218.69</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2453173241852487</v>
+        <v>-0.2497770154373928</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3382963364013716</v>
+        <v>-0.3422065812428563</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>207260058660</v>
+        <v>206035284460</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>19.21310043668123</v>
+        <v>19.0995633187773</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.01061965966723</v>
+        <v>16.90710174249592</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>2.999552204292517</v>
+        <v>2.981826771929317</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.001642894461861</v>
+        <v>5.966177028909788</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2342062049355135</v>
+        <v>0.2328221962695915</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>16.35904436594538</v>
+        <v>16.28353889772517</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.840399129629362</v>
+        <v>3.822673697266162</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06576761624081652</v>
+        <v>0.06615857102207337</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1294768104324941</v>
+        <v>0.129676961177245</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04750578143872008</v>
+        <v>0.04761330358608418</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.03063775626164826</v>
+        <v>0.03081988202478394</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.905469763940283</v>
+        <v>0.9058709974537258</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3066002902580111</v>
+        <v>0.3060858035085073</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1215368151.321643</v>
+        <v>1192548014.347941</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3853,55 +3853,55 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1186.1</v>
+        <v>1187.48</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.09787479736583204</v>
+        <v>0.0991521493769314</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.0824275712683249</v>
+        <v>-0.0813599969055816</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>725.3099999999999</v>
+        <v>763.3</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1116999000100</v>
+        <v>1118298602680</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>39.68216794914687</v>
+        <v>39.72833723653396</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.79551659656742</v>
+        <v>26.80961036533049</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>14.02106048141109</v>
+        <v>14.03737366197289</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>31.24282416836388</v>
+        <v>31.27917447386286</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.419489401031587</v>
+        <v>0.4199774672767802</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.85653784568916</v>
+        <v>26.88654843527738</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.59869856450321</v>
+        <v>14.61501174506501</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.0179533732780465</v>
+        <v>0.01793250921707393</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4809256543398857</v>
+        <v>0.4818692511812721</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2387200868361141</v>
+        <v>0.2391881117809029</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005640333867296182</v>
+        <v>0.005633779095226867</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.341333460032751</v>
+        <v>0.3410318485374041</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.2912509698532731</v>
+        <v>0.2908820118271814</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2835035375.960787</v>
+        <v>2790380833.679606</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>192.83</v>
+        <v>189.59</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.06008799598825543</v>
+        <v>0.04227601078366083</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1697308934337998</v>
+        <v>-0.1836813778256189</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>304146902400</v>
+        <v>299036515200</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>15.5008038585209</v>
+        <v>15.2403536977492</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.28190103940102</v>
+        <v>14.03961633047045</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.403772276711268</v>
+        <v>2.363383218076489</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.743562404339912</v>
+        <v>2.697464068033002</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.3943651807880104</v>
+        <v>0.3877389131649582</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>22.78218906191434</v>
+        <v>22.60805244829114</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.284076396715378</v>
+        <v>5.243687338080599</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.05156718637026632</v>
+        <v>-0.05244844426276942</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08534597850504344</v>
+        <v>0.08552494163766888</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3268008476699207</v>
+        <v>-0.3267009216458363</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02152154747705233</v>
+        <v>0.02188934015507147</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.377893481990983</v>
+        <v>1.373099053402035</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.228013327070826</v>
+        <v>0.2305096063471255</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>965546990.5944591</v>
+        <v>955827127.3068771</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4105,46 +4105,46 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1065.08</v>
+        <v>1070.8</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.376703933353993</v>
+        <v>2.394838483339707</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1513306772908367</v>
+        <v>-0.1467729083665339</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>163.96</v>
+        <v>165.5</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1202890701200</v>
+        <v>1209350812000</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>23.7688016067842</v>
+        <v>23.89645168489176</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.65480305418146</v>
+        <v>6.690542598131135</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>13.32488536234132</v>
+        <v>13.3964465073</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>11.92774552241769</v>
+        <v>11.99180334379095</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03387751172410089</v>
+        <v>0.03405945051467235</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>17.32759343926492</v>
+        <v>17.42541904427472</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>13.11863550080865</v>
+        <v>13.19269878370295</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02175758776245497</v>
+        <v>0.02163732173112562</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0004976152026138882</v>
+        <v>0.0004949570414643258</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.856497770012539</v>
+        <v>2.851517923471014</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.5376498652022783</v>
+        <v>0.511890203576345</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>24571308524.90171</v>
+        <v>23866380614.68683</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>129.94</v>
+        <v>133.5</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.1187521011233967</v>
+        <v>-0.09460832307198286</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.3266310825516919</v>
+        <v>-0.3081826190599575</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>192.97</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>134340028280</v>
+        <v>138020577000</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>80.7080745341615</v>
+        <v>82.9192546583851</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.2065758226246</v>
+        <v>27.93683245826782</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.118926709204453</v>
+        <v>9.368760317675807</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>10.7245142217961</v>
+        <v>11.01833652924257</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>129.1329192546611</v>
+        <v>132.670807453419</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>40.20923711092004</v>
+        <v>41.26413786185153</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>9.522809413521585</v>
+        <v>9.772643021992941</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03409259368662684</v>
+        <v>0.03318345785498347</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.966491448991747</v>
+        <v>1.968097932442781</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2539880089677118</v>
+        <v>0.2545529076484327</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6854485474489103</v>
+        <v>0.6901390010051707</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5333955272617895</v>
+        <v>0.5361732647125566</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2016376601.182604</v>
+        <v>1968823058.448287</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.725</v>
+        <v>28.835</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1407863245377141</v>
+        <v>0.1451548709502173</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.01660390277302293</v>
+        <v>-0.01283806915439922</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.62</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>163716414000</v>
+        <v>164343352400</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>37.955866807611</v>
+        <v>38.1012156448203</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.848243518679991</v>
+        <v>9.88668053142387</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.57027778824416</v>
+        <v>2.580120453403667</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.92163135344524</v>
+        <v>1.928990080995422</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6348370643042901</v>
+        <v>-0.6372681200770829</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.89721276932826</v>
+        <v>17.94687519011407</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.547073819392113</v>
+        <v>3.55691648455162</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06710383969196883</v>
+        <v>0.06684785140113766</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.854074763242492</v>
+        <v>2.853792536708274</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05181447295711994</v>
+        <v>-0.05192128144048103</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.0598781549173194</v>
+        <v>0.0596497312294087</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3373397537756896</v>
+        <v>0.3374733370618643</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.1885259553380176</v>
+        <v>0.188525750457862</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>948195572.7969369</v>
+        <v>929219563.0473415</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>186.68</v>
+        <v>185.2998</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.111124374165755</v>
+        <v>0.1029093866940194</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.06599289538199826</v>
+        <v>-0.07289838394956727</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1325157110519</v>
+        <v>1315359693313</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.711786633520695</v>
+        <v>7.759848759848586</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004291315930027319</v>
+        <v>0.004272153437124404</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.623089334540674</v>
+        <v>6.664366378551975</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.799493243803344</v>
+        <v>4.829405099713733</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01725801553121328</v>
+        <v>0.01736557256851829</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.789680023311371</v>
+        <v>7.838450372658528</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.592837030291411</v>
+        <v>6.634114074302713</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.0727786066044827</v>
+        <v>0.07232783820772069</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1796.06802278517</v>
+        <v>1815.378759343381</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2383.407955811916</v>
+        <v>2409.733422196111</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.607028069423613</v>
+        <v>1.618997969776546</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.6786386644967608</v>
+        <v>0.6714003556830267</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3314950147.904968</v>
+        <v>3234733303.550244</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>606.9</v>
+        <v>608.1396999999999</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6257702112130399</v>
+        <v>0.6290911328324842</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.09664647306610308</v>
+        <v>-0.09480121459297752</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>315.05</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>76494129961</v>
+        <v>76650382676</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.816841519415415</v>
+        <v>1.815746513096696</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.3288703072317768</v>
+        <v>0.3288753281644395</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3797601502.165019</v>
+        <v>3632315471.819092</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>149.24</v>
+        <v>151.114</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.07275549655342861</v>
+        <v>-0.06111212882722339</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3385924481474915</v>
+        <v>-0.3302871831235596</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,50 +4706,50 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1967248838992</v>
+        <v>1991951494609</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-96.90909090909092</v>
+        <v>-80.37978723404255</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>126.8545213199506</v>
+        <v>127.9171826804889</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>118.6877127596983</v>
+        <v>96.48123097011528</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.87875998239326</v>
+        <v>6.965136263598064</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9690909090909092</v>
+        <v>0.3965621780801078</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>459.1050729522439</v>
+        <v>370.161125999809</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>115.4202617793062</v>
+        <v>93.85805941145985</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.0144480959584979</v>
+        <v>-0.01426892174680144</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.386836918118143</v>
+        <v>3.332838362003187</v>
       </c>
       <c r="W34" s="4" t="n">
-        <v>-0.027727343466307</v>
+        <v>-0.03295637287959745</v>
       </c>
       <c r="X34" s="4" t="n">
-        <v>-0.07630954023918413</v>
+        <v>-0.0907005629821397</v>
       </c>
       <c r="Y34" s="4" t="n">
-        <v>0.5266968325791855</v>
+        <v>0.509493364332074</v>
       </c>
       <c r="Z34" s="4" t="n">
-        <v>-0.1242232277526395</v>
+        <v>-0.1467112273563886</v>
       </c>
       <c r="AA34" s="5" t="n">
         <v>-13952000000</v>
@@ -4767,7 +4767,7 @@
         <v>0.2042018986356798</v>
       </c>
       <c r="AF34" s="6" t="n">
-        <v>-12.99688024958003</v>
+        <v>-10.34536771728749</v>
       </c>
       <c r="AG34" s="6" t="n">
         <v>-1.240102827763496</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.134053967888129</v>
+        <v>3.136168062978704</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7520169410975485</v>
+        <v>0.7449138916836571</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12455811312.28988</v>
+        <v>12277534068.88478</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>764.2</v>
+        <v>767.10999</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1186088661926765</v>
+        <v>0.1228684063844221</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01946443922655472</v>
+        <v>-0.01573066707725468</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>814055052309</v>
+        <v>817154879943</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9960295656979709</v>
+        <v>0.9959686650764419</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1056649077836969</v>
+        <v>0.1047157061180461</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>31793398402.79096</v>
+        <v>31066820219.15649</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>456.94</v>
+        <v>458.76</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.4296799879308468</v>
+        <v>0.4353744282907062</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.04605427974947807</v>
+        <v>-0.0422546972860125</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2369910171200</v>
+        <v>2379349564800</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.68899965225455</v>
+        <v>28.74695722730961</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6962857555200989</v>
+        <v>0.6980100197934923</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.45395915587732</v>
+        <v>14.48315907336394</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.97683540489121</v>
+        <v>9.996990627931394</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5389358293032802</v>
+        <v>0.5400245885543979</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>19.03058039802561</v>
+        <v>19.07035964288201</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.9693797444067</v>
+        <v>13.99857966189332</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01742632511974802</v>
+        <v>0.01739119139974853</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.20291047865106</v>
+        <v>40.18416127581443</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.30652973760859</v>
+        <v>40.29647952314902</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.262616536087889</v>
+        <v>0.2615746795710175</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.179106668016557</v>
+        <v>2.178806369054419</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.2522400942994752</v>
+        <v>0.2522464925104009</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4190796147.326589</v>
+        <v>4078462211.593518</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>30.85</v>
+        <v>30.8056</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.08207645571141198</v>
+        <v>0.08051910742507196</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.002263906856403652</v>
+        <v>-0.003699870633893987</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30.92</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>77345167257</v>
+        <v>77233850387</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-24.29133858267716</v>
+        <v>-24.25590551181102</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-106.9321023385494</v>
+        <v>-107.9504639110789</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.141635532521113</v>
+        <v>2.138511590890212</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.358985017357939</v>
+        <v>2.355544034350448</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.180772752243179</v>
+        <v>0.1805090642739426</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>17.52052351355372</v>
+        <v>17.5018753892562</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.935045472989063</v>
+        <v>2.931921531358161</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.02818534211395997</v>
+        <v>0.02822651531310749</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02158321628769588</v>
+        <v>0.0216372992143945</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2835875613935903</v>
+        <v>0.2860193723353814</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2872313097064008</v>
+        <v>0.2791243957583453</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>1045842390.490458</v>
+        <v>1044968946.401364</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>305.4</v>
+        <v>304.465</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1806401658083761</v>
+        <v>-0.1831486839647911</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.2118506284033137</v>
+        <v>-0.2142635938991975</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>206239674000</v>
+        <v>205608256677</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.5203153426319</v>
+        <v>18.46422073984233</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.6530901253734</v>
+        <v>15.59965247599748</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.453102351527839</v>
+        <v>2.445672359140271</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.040291715285881</v>
+        <v>6.021996791131856</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.148421300722155</v>
+        <v>1.144942945440007</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>8.900083886102573</v>
+        <v>8.874818486086394</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.617316784223235</v>
+        <v>2.609886791835667</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.0729830478688596</v>
+        <v>0.07320477155480655</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1831731111424941</v>
+        <v>0.1836302615236101</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.008936249840769683</v>
+        <v>0.009202681175526584</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01159135559921415</v>
+        <v>0.01162695219483356</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9631508871593408</v>
+        <v>0.9619024125563305</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.19919787637864</v>
+        <v>0.1991751810864952</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>934167187.6384217</v>
+        <v>914578081.7725372</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>137.895</v>
+        <v>137.3</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2954116025267637</v>
+        <v>-0.2984518149818677</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5724716314255596</v>
+        <v>-0.5743163638618466</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>322.54</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>397202410650</v>
+        <v>395488531000</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>21.28009259259259</v>
+        <v>21.18827160493827</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.16559578916794</v>
+        <v>15.08705828259962</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.533839679145131</v>
+        <v>5.509961840143779</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.125270622416582</v>
+        <v>6.098840831486251</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4631549564270155</v>
+        <v>0.461156499636892</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>13.70001088679746</v>
+        <v>13.65457399257688</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.199582187190884</v>
+        <v>7.175704348189532</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.07230570416982438</v>
+        <v>-0.07261904644208254</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4031821029934042</v>
+        <v>0.4044004608489769</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4492902460540553</v>
+        <v>0.4508548033073136</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01450378911490627</v>
+        <v>0.01456664238892935</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.032428724699586</v>
+        <v>2.031282291236527</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.517901727989547</v>
+        <v>0.5164672568029839</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4435255553.332789</v>
+        <v>4403288586.384299</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>106.94</v>
+        <v>107.7428</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4063650540825137</v>
+        <v>0.4169226552178928</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1797192605660812</v>
+        <v>-0.1735614021630744</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>421497023075</v>
+        <v>424661206824</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>31.82738095238095</v>
+        <v>32.06630952380952</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.64698491555237</v>
+        <v>20.79708958839189</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.656091955388868</v>
+        <v>6.706059326079748</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.406757880083525</v>
+        <v>8.469867523118227</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.018476190476191</v>
+        <v>1.026121904761905</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>22.16954009066387</v>
+        <v>22.32759912203407</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>7.008480427556258</v>
+        <v>7.058447798247138</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.03225408307944548</v>
+        <v>0.03201375539262389</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5415026011089366</v>
+        <v>0.5418652397260271</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1656301537329607</v>
+        <v>0.1658443251007578</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01552272302225547</v>
+        <v>0.01540706200321506</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.6979180570223241</v>
+        <v>0.6978725670872156</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3456309775632626</v>
+        <v>0.3417436466534221</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>1861966719.518946</v>
+        <v>1800655363.733928</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>80.5</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.1544117375994687</v>
+        <v>-0.1603991327493853</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1765548281505729</v>
+        <v>-0.1823854337152209</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>243432000000</v>
+        <v>241708320923</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>11.48359486447932</v>
+        <v>11.40228245363766</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.3019006476392</v>
+        <v>10.22644617951259</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>1.885535029627048</v>
+        <v>1.872184043398784</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.362368347300072</v>
+        <v>1.352721763971364</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6103892765804335</v>
+        <v>0.6060672655537149</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.06733874618937</v>
+        <v>15.01531257502037</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>3.866589210332675</v>
+        <v>3.853238224104411</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.0787488908606921</v>
+        <v>0.07931046778528947</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1147064272174783</v>
+        <v>0.11497995036445</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2887870760114656</v>
+        <v>-0.2887014992540743</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.02298136645962733</v>
+        <v>0.02314525209558364</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.734372634318827</v>
+        <v>0.7331764408829589</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.232834626588816</v>
+        <v>0.2307741317164961</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1140123538.570048</v>
+        <v>1133007790.231356</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:08 ET</t>
+          <t>2026-09-30 13:18 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-10-01)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -454,7 +454,7 @@
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>333.02</v>
+        <v>329.66</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2288107007117652</v>
+        <v>0.2164126346665083</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.03567498696936355</v>
+        <v>-0.04540452887009894</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>345.34</v>
@@ -714,31 +714,31 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4891183295120</v>
+        <v>4841833778960</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.01598173515982</v>
+        <v>37.63242009132421</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.67434107090425</v>
+        <v>34.32449485746891</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.47759706595433</v>
+        <v>10.3718835167933</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.50689495256697</v>
+        <v>45.04775385881698</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.16159944190766</v>
+        <v>1.149879502790461</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.29588390204527</v>
+        <v>29.00298409933169</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.57348565756186</v>
+        <v>10.46777210840083</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02794477159266767</v>
+        <v>0.02822959362916394</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003182992012491742</v>
+        <v>0.003215434083601286</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3068487682520522</v>
+        <v>0.3051403160021482</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.212175917752888</v>
+        <v>0.2085307084076333</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13514494020.59031</v>
+        <v>13191382862.89308</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>512.9</v>
+        <v>516.1724</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.08449274189603884</v>
+        <v>0.09141201280378053</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.07371956945748759</v>
+        <v>-0.06780972332586865</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3808564595000</v>
+        <v>3832863964820</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.49444444444444</v>
+        <v>28.67624444444445</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.80281626264998</v>
+        <v>24.94863930936713</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.47714582975479</v>
+        <v>11.55037221309129</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.613124029413159</v>
+        <v>8.668077406433733</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.9050787574117023</v>
+        <v>0.910853332817735</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.87267139394465</v>
+        <v>18.9875332403298</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.80222305093735</v>
+        <v>11.8740531115993</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01758851617954506</v>
+        <v>0.01747912256784147</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1488390730593607</v>
+        <v>0.1494111598173515</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2347806602160802</v>
+        <v>0.2354083608742514</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007096899980503023</v>
+        <v>0.007051907463475381</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5568474062169736</v>
+        <v>0.5570193613606674</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.2519126472208998</v>
+        <v>0.2244909465623531</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10881269501.79647</v>
+        <v>10739441009.97441</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>344.08</v>
+        <v>339.39001</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.09179757786388554</v>
+        <v>0.0769158069902347</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1579256503756639</v>
+        <v>-0.1694035632999682</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4164094451287</v>
+        <v>4107335726633</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.91857000993049</v>
+        <v>16.69364399205561</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.81274945680474</v>
+        <v>20.5497359329893</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.274507142266959</v>
+        <v>9.151206101579847</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.464420028728454</v>
+        <v>6.378477998516738</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.150457827105198</v>
+        <v>0.1484575469462356</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.92783781577357</v>
+        <v>12.75904658375891</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.402000604428236</v>
+        <v>9.279244170750854</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01288285023811811</v>
+        <v>0.01305565354113498</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1871054785412338</v>
+        <v>-0.1876467879445279</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.3012652310592596</v>
+        <v>0.3025963703161056</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002499418739827947</v>
+        <v>0.002533957908778753</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7620537900204533</v>
+        <v>0.759735705892704</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.2764777821993065</v>
+        <v>0.2499728850446888</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8744889434.43535</v>
+        <v>8769797447.543859</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>249.15</v>
+        <v>249.315</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1000000000000001</v>
+        <v>0.100728476821192</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1324860724233983</v>
+        <v>-0.1319115598885794</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2680131465000</v>
+        <v>2681906386500</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.77380952380952</v>
+        <v>19.78690476190476</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.31352389719098</v>
+        <v>22.33886037231659</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.455202486850248</v>
+        <v>3.457490700417698</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.85815851491969</v>
+        <v>4.861375838439505</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2238355088228185</v>
+        <v>0.223983744259125</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.12277099729524</v>
+        <v>11.12912369043729</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.642159737262789</v>
+        <v>3.644239931415017</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004337473796271408</v>
+        <v>-0.0043348640045769</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1138195107632095</v>
+        <v>-0.1142383974777125</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1851368256743036</v>
+        <v>0.1854659482523509</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8344139214362121</v>
+        <v>0.8344538430922581</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.2661377280656054</v>
+        <v>0.2389634618802327</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8719928484.368526</v>
+        <v>8568416938.536662</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>228.38</v>
+        <v>231.398</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.2093195267084955</v>
+        <v>0.2253004634437885</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.03449733660268872</v>
+        <v>-0.02173839519742959</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5531591980000</v>
+        <v>5604690958000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.72704402515723</v>
+        <v>29.10666666666666</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.71141095107418</v>
+        <v>16.90963657246951</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18.25794711670171</v>
+        <v>18.4992225541227</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>24.12619309646088</v>
+        <v>24.4450163330189</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2305980404740512</v>
+        <v>0.2336453514739229</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.74322852606487</v>
+        <v>24.05212357756979</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.31213417874436</v>
+        <v>18.55037168819252</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02296011717046419</v>
+        <v>0.02266438260455831</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7190076953562501</v>
+        <v>0.7213064598948906</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9835770921465588</v>
+        <v>0.9863018805345292</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002276906909536737</v>
+        <v>0.002247210433970907</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.296646808595956</v>
+        <v>1.296250411553451</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.3694232280577041</v>
+        <v>0.3645904288530423</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27333212314.89771</v>
+        <v>27090516658.48847</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>725.1799999999999</v>
+        <v>730.21</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.1149583031360646</v>
+        <v>0.1226918868873741</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.07006745146315829</v>
+        <v>-0.06361724500525767</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>779.8200000000001</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1847386310833</v>
+        <v>1860200168280</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>26.94834633965069</v>
+        <v>27.1352657004831</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>21.77450560146708</v>
+        <v>21.92042895962305</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.093767791319092</v>
+        <v>8.149907855841015</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.059664958024048</v>
+        <v>7.108632269227972</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.524410999628386</v>
+        <v>-5.56272946859903</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>18.15827023715817</v>
+        <v>18.27794538516138</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.518113240129159</v>
+        <v>8.574253304651082</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02218052594615342</v>
+        <v>0.02202773696009699</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2376100212275316</v>
+        <v>0.2378984804752526</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.282516785736231</v>
+        <v>0.283112003985319</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.002895832758763342</v>
+        <v>0.002875885019377987</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8380449193485922</v>
+        <v>0.8389659360756477</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4604925114039621</v>
+        <v>0.4414972467298536</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>14203641080.5146</v>
+        <v>14084996005.08432</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>354.81</v>
+        <v>357.06</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1900609627049802</v>
+        <v>-0.1849247973378434</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2887155944911092</v>
+        <v>-0.2842050397931158</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1401338910865</v>
+        <v>1410225392502</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>300.6864406779661</v>
+        <v>302.5932203389831</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>166.5461563820757</v>
+        <v>167.4773441442511</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.52395710115905</v>
+        <v>13.60971822254606</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.22296127011905</v>
+        <v>13.3068136498653</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.004188350441629</v>
+        <v>-8.05494628789687</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>116.0177844084636</v>
+        <v>116.7434661295311</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.46723970377055</v>
+        <v>13.55147618299733</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004111781921793144</v>
+        <v>0.004086329459613342</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.805424077083817</v>
+        <v>0.8067710703505921</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1278156307669018</v>
+        <v>0.1281899177260426</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.525623185771236</v>
+        <v>1.525392922851457</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.4104042602334315</v>
+        <v>0.4029839855604745</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13967999262.07737</v>
+        <v>13785761058.8828</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>351.19</v>
+        <v>350.0567</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.01026984906782769</v>
+        <v>0.007009679871812446</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2905252525252525</v>
+        <v>-0.2928147474747476</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1670814520200</v>
+        <v>1665422754786</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>43.57196029776674</v>
+        <v>43.43135235732009</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>18.91921649596141</v>
+        <v>18.83710766819184</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.75128524196445</v>
+        <v>18.69077431749416</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.78976366736884</v>
+        <v>16.73558262814726</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.433562575240154</v>
+        <v>0.4321634566248185</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>32.64754262480148</v>
+        <v>32.57562772898608</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.1490676086371</v>
+        <v>19.10688669420004</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02358310843221747</v>
+        <v>0.02363627811161659</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.303053105136136</v>
+        <v>1.305627441449403</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.881065775781448</v>
+        <v>0.8831489708149565</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007403399869016771</v>
+        <v>0.007427368194923852</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.596383269191508</v>
+        <v>1.594686849800867</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3685526223399482</v>
+        <v>0.3676984476875576</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9058902903.545204</v>
+        <v>8776937685.47164</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>910.34</v>
+        <v>916.35</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.06534815681685191</v>
+        <v>0.07238150965476886</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1697765617875057</v>
+        <v>-0.1642954856361148</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>403716672860</v>
+        <v>406381981650</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>32.947520810713</v>
+        <v>33.16503800217156</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.61961810789017</v>
+        <v>39.87095827211687</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.331721411757721</v>
+        <v>1.340513341898837</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.28866858922437</v>
+        <v>11.36319557718627</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>0.6410365189717613</v>
+        <v>0.6452685965241267</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.3059177421826</v>
+        <v>27.49153713002298</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.293354773019653</v>
+        <v>1.30214670316077</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02325888582574405</v>
+        <v>0.0231063394146427</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1684038770643383</v>
+        <v>-0.1681905968795083</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.09059323239914874</v>
+        <v>0.09081742447519536</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1793,16 +1793,16 @@
         <v>80.58620689655173</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006085638332930553</v>
+        <v>0.006045724886779069</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1704786040300559</v>
+        <v>-0.1699432286041341</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1772869727130852</v>
+        <v>0.1780574776663853</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2056162838.365721</v>
+        <v>2034095867.947713</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>69.58</v>
+        <v>68.37</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2353005645282533</v>
+        <v>-0.248598729473939</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.442735864167868</v>
+        <v>-0.452426717924075</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>289726945130</v>
+        <v>284688577732</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>21.54179566563468</v>
+        <v>21.1671826625387</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>18.54103495911568</v>
+        <v>18.21503589624932</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5.989711990697522</v>
+        <v>5.885550572076968</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.667391882316998</v>
+        <v>9.499275409514418</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6331186287095071</v>
+        <v>0.6221086611794913</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.639397745951747</v>
+        <v>9.474729277128066</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.097423210640213</v>
+        <v>5.993261792019659</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.0379481721835252</v>
+        <v>0.03861977212991699</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1618442936511304</v>
+        <v>0.1620719708214939</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1480282957789665</v>
+        <v>0.148286854895888</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1077640275762283</v>
+        <v>0.1057975058626026</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3548273029831461</v>
+        <v>0.352317512650331</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2394368118.816971</v>
+        <v>2368467738.460869</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -1961,55 +1961,55 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>498.41</v>
+        <v>499.06</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.003139768294899481</v>
+        <v>0.00444801020295027</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.07313943541488444</v>
+        <v>-0.07934399616285726</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>537.74</v>
+        <v>542.0700000000001</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>464.01</v>
+        <v>455.19</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1074997400284</v>
+        <v>1076399349855</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.525435905929</v>
+        <v>12.56173589275351</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.46773595354603</v>
+        <v>22.49701090395791</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.793571240182278</v>
+        <v>2.801667293682916</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.430339972779757</v>
+        <v>1.434485243455878</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3450438618867944</v>
+        <v>0.3460438340821285</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.20521132958674</v>
+        <v>15.24591559982487</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.024306877206664</v>
+        <v>3.032402930707302</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02253290637846866</v>
+        <v>0.02246779243150705</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4425145492262142</v>
+        <v>-0.4416264477809574</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06099000915039721</v>
+        <v>0.06272444301054314</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02297296342200343</v>
+        <v>0.02192497685697011</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1355645843353423</v>
+        <v>0.135429333337595</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2252679003.910805</v>
+        <v>2225212255.372571</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>330.83</v>
+        <v>332.14</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.01643722758107136</v>
+        <v>0.02046205231924869</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.0973260572987722</v>
+        <v>-0.09375170532060029</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>886462293300</v>
+        <v>889972451400</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>14.22312983662941</v>
+        <v>14.27944969905417</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.18017151181038</v>
+        <v>13.23180770621369</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2.978373679329913</v>
+        <v>2.990167257662961</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.46286851771766</v>
+        <v>2.472620830864019</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.74471240136561</v>
+        <v>0.7476612670845258</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.47748275332761</v>
+        <v>19.51516156504938</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.096509101141338</v>
+        <v>6.108302679474386</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1833512843450349</v>
+        <v>-0.1826281248866981</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07913086137645919</v>
+        <v>0.07917602916406574</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2867343905451732</v>
+        <v>-0.2866847194180255</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01813620288365626</v>
+        <v>0.01806467152405612</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7811401801186869</v>
+        <v>0.7822032551753771</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1659556661977021</v>
+        <v>0.1662463925064663</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2586235229.721713</v>
+        <v>2555827335.200446</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>359.33</v>
+        <v>359.34</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.03708724488056814</v>
+        <v>0.03711610657441167</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.06805508727338749</v>
+        <v>-0.06802915164561563</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,31 +2228,31 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>670886074329</v>
+        <v>670904744801</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>30.52931180968564</v>
+        <v>30.53016142735769</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>23.91959745473596</v>
+        <v>23.92026312688843</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.0801581174474</v>
+        <v>15.08057779178655</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>19.54518016459151</v>
+        <v>19.54572409858434</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.058720039797882</v>
+        <v>2.058777333094845</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.45127068283043</v>
+        <v>23.45191232390542</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.33863231273602</v>
+        <v>15.33905198707517</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03132126422659252</v>
+        <v>0.03132039259348621</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007458325216374921</v>
+        <v>0.007458117660154729</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.2977042484457705</v>
+        <v>0.2970169115867151</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1812295212635588</v>
+        <v>0.1812215205559704</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2312416234.605637</v>
+        <v>2267617901.336808</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>551.47</v>
+        <v>550.105</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-0.02070570699786978</v>
+        <v>-0.02312965881745721</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.08276366781431399</v>
+        <v>-0.08503401360544216</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>483659042920</v>
+        <v>482461888780</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>30.28390993959363</v>
+        <v>30.20895112575508</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>24.73239298546694</v>
+        <v>24.66168698520733</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>13.78613695864094</v>
+        <v>13.75201347604253</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>86.68624844056319</v>
+        <v>86.47168240955267</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.338440662508825</v>
+        <v>1.33512775064721</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>22.47291747693977</v>
+        <v>22.41878679598481</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.16672014707978</v>
+        <v>14.13259666448137</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03400742783738377</v>
+        <v>0.03409181198040743</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2244633973505448</v>
+        <v>0.2249344963252164</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1623261594525547</v>
+        <v>0.1626930985085466</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.006110939851669175</v>
+        <v>0.00612610319848029</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2909050054694113</v>
+        <v>0.2902733303024938</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1758186944194425</v>
+        <v>0.1757165652840637</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1591873912.521012</v>
+        <v>1559745833.644694</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>367.08</v>
+        <v>364.51999</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.09120097104685532</v>
+        <v>0.08359095307287245</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.2048004852476063</v>
+        <v>-0.2103461938390884</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>333361647820</v>
+        <v>331036788169</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>23.60491286733972</v>
+        <v>23.44029258568581</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>16.72058948056702</v>
+        <v>16.59843735996022</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7405913589659853</v>
+        <v>0.735426484783251</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.37819718996008</v>
+        <v>3.354637697238412</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7152350230430221</v>
+        <v>-0.7102469855271117</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.67626626635097</v>
+        <v>14.58602601284788</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8399917530752294</v>
+        <v>0.8348268788924952</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.07084498218208982</v>
+        <v>0.07134252398541009</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4117273134881871</v>
+        <v>0.4121987556629845</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01279557530401099</v>
+        <v>0.01287597649931516</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02468126838836221</v>
+        <v>0.02485460399579184</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4359744422742588</v>
+        <v>0.4347054606515424</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.1933871522682629</v>
+        <v>0.193193026554665</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1854571643.720571</v>
+        <v>1810919208.778081</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>162.88</v>
+        <v>162.69</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3280065061037332</v>
+        <v>0.3264573826007882</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.07669633240745988</v>
+        <v>-0.07777336885664077</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>675049644800</v>
+        <v>674262197400</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.96267696267696</v>
+        <v>20.93822393822394</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.30517236487248</v>
+        <v>14.29183906562992</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.86963287209882</v>
+        <v>1.867451939843793</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.621007212892281</v>
+        <v>2.617949800254453</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.052595452595454</v>
+        <v>2.050201093951095</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.840997491124261</v>
+        <v>9.830034074486599</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.957651483963884</v>
+        <v>1.955470551708857</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04526037490035578</v>
+        <v>0.04531323292009311</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4653914282188254</v>
+        <v>0.4650475591050935</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1146956755455664</v>
+        <v>0.1145642553929336</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02529469548133595</v>
+        <v>0.02532423627758313</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5544397865553242</v>
+        <v>-0.5518803669329927</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2530294200857307</v>
+        <v>0.2529040726143827</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2298307119.035201</v>
+        <v>2248242158.256643</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>264.74</v>
+        <v>259.035</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2767783564367656</v>
+        <v>0.2492644918017588</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.05809940584196105</v>
+        <v>-0.07839684064467911</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>182.94</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>637996506652</v>
+        <v>624248036189</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>30.60578034682081</v>
+        <v>29.94624277456647</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.30984403311962</v>
+        <v>21.04134212284668</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.514888405395746</v>
+        <v>6.374496177730805</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.602500547245531</v>
+        <v>7.438670881830272</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.789478856099793</v>
+        <v>-3.707817690903565</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.76196213245583</v>
+        <v>19.35438266894936</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.80707968683434</v>
+        <v>6.666687459169398</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02932304456990455</v>
+        <v>0.02996885679322487</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4362273275793809</v>
+        <v>0.4232097268192254</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09251491526379829</v>
+        <v>0.09309168674187629</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01994409609428118</v>
+        <v>0.0203833458799004</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.15533107673842</v>
+        <v>-0.1636439217449586</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1741611840506237</v>
+        <v>0.1816119153214505</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1716568337.70457</v>
+        <v>1672953093.817291</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>103.92</v>
+        <v>104.81</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.07839661199678283</v>
+        <v>-0.07050374233432266</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2311334714412547</v>
+        <v>-0.2245486830423202</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>827003673600</v>
+        <v>834086364800</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>37.51624548736462</v>
+        <v>37.8375451263538</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.38735786235141</v>
+        <v>33.69249127215929</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.123890619699935</v>
+        <v>1.133515933898674</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.414052403346973</v>
+        <v>8.486112705877563</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.072110272399089</v>
+        <v>9.149806366918288</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>20.75747971708023</v>
+        <v>20.92281250262611</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.208455198956295</v>
+        <v>1.218080513155034</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01633487302564746</v>
+        <v>0.01619616453415976</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1236661985065033</v>
+        <v>0.123026042233322</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05301533788230439</v>
+        <v>0.05283438718430467</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009406274056966897</v>
+        <v>0.009326400152657189</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.04490988064009223</v>
+        <v>-0.04330916797200763</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3096666356200337</v>
+        <v>0.3105569809702414</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2872147876.01436</v>
+        <v>2775568942.802483</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>145.335</v>
+        <v>144.16</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.02500181170552263</v>
+        <v>0.01671490814647614</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1310313901345291</v>
+        <v>-0.1380568011958146</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>345491660859</v>
+        <v>342698449064</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.53111111111111</v>
+        <v>21.35703703703703</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.52529588472717</v>
+        <v>20.3607985950792</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.969708392993382</v>
+        <v>3.937614315010571</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.482554869179356</v>
+        <v>6.430144906188433</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.54683174603197</v>
+        <v>20.38071534391556</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.4355726385151</v>
+        <v>17.30415211555472</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.257924221654104</v>
+        <v>4.225830143671294</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04605899882050791</v>
+        <v>0.04643440915318586</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04900368949771683</v>
+        <v>0.04892924200913229</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02655194626495438</v>
+        <v>0.02675350702871682</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02952213850758592</v>
+        <v>0.02976276359600444</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.03782615212094106</v>
+        <v>-0.03941639359100356</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1542765398304741</v>
+        <v>0.1552466703012699</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1251620585.066966</v>
+        <v>1199437921.297251</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -3095,55 +3095,55 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>284.49</v>
+        <v>282.54999</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1773466139184933</v>
+        <v>-0.1829564975542345</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.297780959198282</v>
+        <v>-0.2894148077358348</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>405.13</v>
+        <v>397.63</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>284.01</v>
+        <v>277.2</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>283669815330</v>
+        <v>281735396178</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>19.86662011173184</v>
+        <v>19.73114455307262</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>18.95812605831045</v>
+        <v>18.83251029272873</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.676773391793162</v>
+        <v>1.665339032593276</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17.01769633507853</v>
+        <v>16.90164831558043</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-6.814712712745255</v>
+        <v>-6.768241445530755</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14.39062577169141</v>
+        <v>14.30973849793017</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.034282731179363</v>
+        <v>2.022848371979477</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05323442673106633</v>
+        <v>0.0535999388250783</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.0479210893854749</v>
+        <v>0.04771717877094983</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01423568777486173</v>
+        <v>0.01440173331914685</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03265492635945024</v>
+        <v>0.03287913759968634</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7102518473241516</v>
+        <v>0.7099127354309843</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2327537363263104</v>
+        <v>0.2222454860174952</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1377386035.222257</v>
+        <v>1368960499.087616</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -3221,55 +3221,55 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>611.76</v>
+        <v>618.47</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.737548649296397</v>
+        <v>1.767575050886529</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.04262910798122066</v>
+        <v>-0.03212832550860711</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>639</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>160.49</v>
+        <v>163.14</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>997535856000</v>
+        <v>1008477182000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>155.2690355329949</v>
+        <v>156.9720812182741</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>44.04030135170912</v>
+        <v>44.45099821194754</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>24.15048676915628</v>
+        <v>24.41537784771819</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>14.8426240628347</v>
+        <v>15.00542321194811</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.253548176780142</v>
+        <v>1.267297536441112</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>92.99550811718605</v>
+        <v>94.01634465385334</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>24.13087655247549</v>
+        <v>24.3957676310374</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.008423757351134254</v>
+        <v>0.008332365025191021</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.52561246783951</v>
+        <v>2.531351095195049</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.937563268337078</v>
+        <v>0.9401069202616024</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.583484606611615</v>
+        <v>2.582637978538599</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.5524237278395616</v>
+        <v>0.55179727045751</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10716961620.88514</v>
+        <v>10640661218.46899</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1811.67</v>
+        <v>1820.54004</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.5567117104549071</v>
+        <v>0.564333460078295</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.09414688293765872</v>
+        <v>-0.08971177423548471</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>698250211755</v>
+        <v>701668884391</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>57.93904208998548</v>
+        <v>57.94629898403483</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.45821893784718</v>
+        <v>36.51594316603593</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>17.42086046363315</v>
+        <v>17.42304243512844</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>28.1968128877363</v>
+        <v>28.20034455267715</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.944122326975499</v>
+        <v>3.944616330272966</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>44.24267072541562</v>
+        <v>44.24825467253432</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>17.28817346342085</v>
+        <v>17.29035543491614</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01625174505633725</v>
+        <v>0.01624970977205244</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5891901408776479</v>
+        <v>0.5868766889179415</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3270761318701876</v>
+        <v>0.3248561960587237</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004294380323127281</v>
+        <v>0.004273457231954096</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.645783240630152</v>
+        <v>1.644857893878017</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.3731865298021549</v>
+        <v>0.3729590043622481</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2131057152.7186</v>
+        <v>2108913662.624479</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>186.05</v>
+        <v>189.69</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1831672454225141</v>
+        <v>-0.1671862122235781</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2685276194220562</v>
+        <v>-0.2542166306270887</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>147048338500</v>
+        <v>149925285300</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>69.68164794007488</v>
+        <v>71.04494382022469</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>69.61087206536895</v>
+        <v>70.84862577139003</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.564427240810681</v>
+        <v>1.595034685887547</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>24.126865668</v>
+        <v>24.59889894417049</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3729413140357658</v>
+        <v>0.3802377740362505</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>26.71932928057554</v>
+        <v>27.13327846043165</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>1.975629964359806</v>
+        <v>2.006237409436672</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.00142810182108926</v>
+        <v>-0.001400697684715361</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>0.001016735929402879</v>
+        <v>0.002770950695192287</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1596882802827024</v>
+        <v>0.1601138351317724</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.251442240843674</v>
+        <v>1.256437239124566</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3500806613467961</v>
+        <v>0.2918652563784824</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1420912361.516076</v>
+        <v>1408430052.535917</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>900.36</v>
+        <v>895.12</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>-0.01528974609538625</v>
+        <v>-0.02102065565429623</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.219785266770076</v>
+        <v>-0.2243260340210921</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>265612502520</v>
+        <v>264066665840</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>13.71663619744059</v>
+        <v>13.63680682510664</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.52932764912608</v>
+        <v>12.499638088009</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.252155833368663</v>
+        <v>2.239048524551243</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.201349464730899</v>
+        <v>2.188537843606915</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3214989462273259</v>
+        <v>0.3196278563541294</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.12749665594241</v>
+        <v>26.07825521103431</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>6.954734328667</v>
+        <v>6.94162701984958</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1562991184756976</v>
+        <v>-0.1572140878438411</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09476235130600275</v>
+        <v>0.0909761329960852</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3857093404968824</v>
+        <v>-0.3861435826282921</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01999200319872051</v>
+        <v>0.02010903566002324</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.589653643641105</v>
+        <v>1.590887144771518</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.2677032645613989</v>
+        <v>0.2662432084664404</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2024669591.666178</v>
+        <v>1975066246.807218</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>219.93</v>
+        <v>228.47</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2455231560891938</v>
+        <v>-0.2162264150943396</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3384768092402093</v>
+        <v>-0.3127895085123021</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>207203530620</v>
+        <v>215249356130</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>19.20786026200874</v>
+        <v>19.95371179039302</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.0029671508854</v>
+        <v>17.6600725688216</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>2.998734107414215</v>
+        <v>3.115176579735734</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.000006008359457</v>
+        <v>6.232989463601533</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2341423276124709</v>
+        <v>0.2432341999255273</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>16.35555949818137</v>
+        <v>16.85157241415449</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.83958103275106</v>
+        <v>3.956023505072579</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06578555857235131</v>
+        <v>0.06332655411878467</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1296769611772448</v>
+        <v>0.1298771119219957</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04761330358608418</v>
+        <v>0.04772082573344871</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.03064611467285045</v>
+        <v>0.0295005908872062</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.9070029786662263</v>
+        <v>0.9125149324049799</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3058105343151351</v>
+        <v>0.3187614738602288</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1213577878.945264</v>
+        <v>1212875814.23144</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -3853,55 +3853,55 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1157.08</v>
+        <v>1143.92</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.07101338043677341</v>
+        <v>0.05883225546136295</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1048775770703595</v>
+        <v>-0.1150582137469539</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>763.3</v>
+        <v>783.85</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1089669676280</v>
+        <v>1077276364720</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.71127467380395</v>
+        <v>38.27099364335899</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.12327278060818</v>
+        <v>25.80972622026686</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.67801084379997</v>
+        <v>13.52244457119617</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.47841412084182</v>
+        <v>30.13176917854718</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4092258630348442</v>
+        <v>0.404571550145901</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.22544559217454</v>
+        <v>25.93925765088397</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.25564892689209</v>
+        <v>14.10008265428829</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01840365060764248</v>
+        <v>0.01861537174373291</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4818692511812721</v>
+        <v>0.4828128480226588</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2391881117809029</v>
+        <v>0.2396561367256922</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005781795554326409</v>
+        <v>0.005848311070704245</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3458608969860252</v>
+        <v>0.3335022959767971</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.2968887648257696</v>
+        <v>0.2918808697664217</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2864832999.314466</v>
+        <v>2711412188.275171</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>188.12</v>
+        <v>186.545</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.03419464712602083</v>
+        <v>0.02553604320712077</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.190010764262648</v>
+        <v>-0.1967922497308935</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>296717913600</v>
+        <v>294233697600</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>15.12218649517685</v>
+        <v>14.99557877813505</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>13.93075913333035</v>
+        <v>13.81268631344078</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.345058552584783</v>
+        <v>2.325424982415099</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.676549082115979</v>
+        <v>2.654140168633453</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.3847325510026475</v>
+        <v>0.381511448685886</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>22.52904602173987</v>
+        <v>22.44439627900637</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.225362672588893</v>
+        <v>5.205729102419209</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.05285828485954951</v>
+        <v>-0.05330456751871374</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08552494163766888</v>
+        <v>0.08563811831035562</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3267009216458363</v>
+        <v>-0.3267940645807226</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02206038698702956</v>
+        <v>0.02224664290117666</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.381400002363678</v>
+        <v>1.383031124690246</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2343556203387864</v>
+        <v>0.234135553122507</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>988741985.4159322</v>
+        <v>987493345.5499654</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -4105,110 +4105,110 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1065.11</v>
+        <v>1090.335</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.376799044630141</v>
+        <v>2.456771775991969</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1513067729083666</v>
+        <v>-0.131207171314741</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>165.5</v>
+        <v>179.61</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1202924582900</v>
+        <v>1231413445650</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>23.76947110020084</v>
+        <v>14.47795777453194</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.572466190528623</v>
+        <v>6.424802146796563</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>13.32526068303166</v>
+        <v>9.245678632083973</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>11.92808149001231</v>
+        <v>8.903716992585526</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03387846594852696</v>
+        <v>0.01636955024758636</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>17.32808917712814</v>
+        <v>11.28083628099329</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>13.11901082149899</v>
+        <v>8.990925105114576</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02175697493595548</v>
+        <v>0.04297412900682402</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>2.563272513243084</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.616522384619381</v>
+        <v>1.253448035244278</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.863123077493117</v>
+        <v>1.023493644986467</v>
       </c>
       <c r="W29" s="4" t="n">
-        <v>0.3763197924123121</v>
+        <v>0.4337631707914727</v>
       </c>
       <c r="X29" s="4" t="n">
-        <v>0.7054802658708248</v>
+        <v>0.9176735508293126</v>
       </c>
       <c r="Y29" s="4" t="n">
-        <v>0.7256906750559408</v>
+        <v>0.8071598041865633</v>
       </c>
       <c r="Z29" s="4" t="n">
-        <v>0.6573653543655981</v>
+        <v>0.7458629906598192</v>
       </c>
       <c r="AA29" s="5" t="n">
         <v>89675000000</v>
       </c>
       <c r="AB29" s="6" t="n">
-        <v>3.424517651888341</v>
+        <v>3.313805399898115</v>
       </c>
       <c r="AC29" s="6" t="n">
-        <v>2.984913793103448</v>
+        <v>2.936394731096718</v>
       </c>
       <c r="AD29" s="6" t="n">
-        <v>0.06330169572296573</v>
+        <v>0.03387821763575135</v>
       </c>
       <c r="AE29" s="6" t="n">
-        <v>0.0475423526604629</v>
+        <v>0.02393204279996733</v>
       </c>
       <c r="AF29" s="6" t="n">
-        <v>-0.2724226728703947</v>
+        <v>-0.3172431984324365</v>
       </c>
       <c r="AG29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0004976011867318869</v>
+        <v>0.0004860891377420701</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.853997286556701</v>
+        <v>2.85374468512457</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.5121165569229071</v>
+        <v>0.5140364271475639</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>24452984900.25945</v>
+        <v>24760510839.87468</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30 (C)</t>
+          <t>2026-12-23 (E)</t>
         </is>
       </c>
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>134.01</v>
+        <v>137.81</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.09114952340731408</v>
+        <v>-0.06537807492546788</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.3055397212001866</v>
+        <v>-0.2858475410685599</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>192.97</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>138547846620</v>
+        <v>142476522220</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>83.2360248447205</v>
+        <v>85.59627329192547</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.04355743619828</v>
+        <v>28.82316261302488</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.404551087428727</v>
+        <v>9.671227411077925</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.06042905081495</v>
+        <v>11.37405960370725</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>133.1776397515556</v>
+        <v>136.9540372670837</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>41.41526128403554</v>
+        <v>42.54127893952422</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>9.808433791745859</v>
+        <v>10.07511011539506</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03305717202925373</v>
+        <v>0.03214564707670193</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.968097932442781</v>
+        <v>1.969704415893815</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2545529076484327</v>
+        <v>0.2551178063291539</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6785598901997032</v>
+        <v>0.6884406865580344</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5372449985023826</v>
+        <v>0.5376849211732968</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>1988892933.177476</v>
+        <v>1923228618.083366</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.52</v>
+        <v>28.255</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1326449425871403</v>
+        <v>0.1221207171388377</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.02362204724409456</v>
+        <v>-0.03269428277986997</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.62</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>162548028800</v>
+        <v>161037677200</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>37.68498942917548</v>
+        <v>37.33483086680761</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.778676218353</v>
+        <v>9.688524971176543</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.551934639537805</v>
+        <v>2.528222764380809</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.907917361192628</v>
+        <v>1.890189517549008</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6303064603640854</v>
+        <v>-0.6244498260023574</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.80466007604563</v>
+        <v>17.6850187896071</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.528730670685757</v>
+        <v>3.505018795528762</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06758617795062427</v>
+        <v>0.06822005999475507</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.853792536708274</v>
+        <v>2.853510310174057</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05192128144048103</v>
+        <v>-0.052028089923842</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06030855539971949</v>
+        <v>0.0608741815607857</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.338316783869119</v>
+        <v>0.3223900301829781</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.1902204621090411</v>
+        <v>0.1925877696936527</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>947960025.794668</v>
+        <v>905870574.2831416</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>184.15</v>
+        <v>190.65</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.09606574621075525</v>
+        <v>0.1347539207986992</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.0786511232300996</v>
+        <v>-0.04612998448991845</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1307197781777</v>
+        <v>1353338349692</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.759848759848586</v>
+        <v>8.008897959911293</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004245644385187998</v>
+        <v>0.004385383245184843</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.664366378551975</v>
+        <v>6.878256515701447</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.829405099713733</v>
+        <v>4.984402898522113</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01736557256851829</v>
+        <v>0.01792291358000789</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.838450372658528</v>
+        <v>8.091169455639246</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.634114074302713</v>
+        <v>6.848004211452185</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07232783820772069</v>
+        <v>0.07007869102941186</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1826.719906763924</v>
+        <v>1825.270935089897</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2424.785614911811</v>
+        <v>2424.302104925622</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.629106706489275</v>
+        <v>1.573564122738002</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.6724402774954298</v>
+        <v>0.6752922748419871</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3267254655.9271</v>
+        <v>3150753977.074224</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>609</v>
+        <v>620.9400000000001</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6313957136739847</v>
+        <v>0.6633807133804994</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.09352068231546673</v>
+        <v>-0.07574832919042018</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>315.05</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>76758815532</v>
+        <v>78263742063</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.817352172208363</v>
+        <v>1.818044444023989</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.3288735733796376</v>
+        <v>0.3310172881589163</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3672351914.168245</v>
+        <v>3578836429.003666</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>150.86</v>
+        <v>150.81</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.06269025871113798</v>
+        <v>-0.06300091420009768</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3314128700585002</v>
+        <v>-0.3316344619748272</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1988603322503</v>
+        <v>1987944233505</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-80.24468085106383</v>
+        <v>-80.21808510638297</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>127.7021730559615</v>
+        <v>112.443620541733</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>96.31906047190739</v>
+        <v>96.28713714545191</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.953428912783752</v>
+        <v>6.951124316166761</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>0.3958956164562189</v>
+        <v>0.3957644035381305</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>369.5215515765043</v>
+        <v>369.3956510993314</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>93.69588891325196</v>
+        <v>93.66396558679648</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01429294604829723</v>
+        <v>-0.01429768477453043</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.332838362003187</v>
+        <v>3.341142733542203</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.03295637287959745</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.119591424151587</v>
+        <v>3.110620299420498</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7447999627796515</v>
+        <v>0.7354507581214247</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12453287560.05933</v>
+        <v>12330258673.27295</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>762.63</v>
+        <v>765.23</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1163107558551699</v>
+        <v>0.1201165436752445</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.02147888679317911</v>
+        <v>-0.01814285897583945</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>812382628294</v>
+        <v>815152247682</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9959243097873951</v>
+        <v>0.9959589553705406</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1046089992970697</v>
+        <v>0.09917698537730722</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32232130205.14278</v>
+        <v>31928152121.89176</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>456.19</v>
+        <v>460.3</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.4273333778924433</v>
+        <v>0.4401928009028948</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.04762004175365342</v>
+        <v>-0.03903966597077246</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2366020311200</v>
+        <v>2387336744000</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.74695722730961</v>
+        <v>29.09470267763997</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6940997273729036</v>
+        <v>0.6986371688890247</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.48315907336394</v>
+        <v>14.65835857828367</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.996990627931394</v>
+        <v>10.1179219661725</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5400245885543979</v>
+        <v>0.5465571440611043</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>19.07035964288201</v>
+        <v>19.30903511202044</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.99857966189332</v>
+        <v>14.17377916681305</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01739119139974853</v>
+        <v>0.01718332855433321</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.41617709045053</v>
+        <v>40.64493956699508</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.52912809583692</v>
+        <v>40.75068185275771</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2630482912821412</v>
+        <v>0.2606995437757984</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.179477856782658</v>
+        <v>2.176918780201253</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.2524898499849076</v>
+        <v>0.25289983493492</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4134132941.88371</v>
+        <v>4090494344.555532</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>30.95</v>
+        <v>30.94</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.08558399689686214</v>
+        <v>0.08523324277831734</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.0006457862447529772</v>
+        <v>-0.0009686793671294103</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30.97</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>77595880927</v>
+        <v>77570809560</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-24.37007874015748</v>
+        <v>-24.36220472440945</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-108.4564773303521</v>
+        <v>-109.6249483477212</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.148577625003461</v>
+        <v>2.147883415755226</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.366631646263475</v>
+        <v>2.365866983372922</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1813587255081487</v>
+        <v>0.1813001281816518</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>17.56196378958678</v>
+        <v>17.55781976198347</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.941987565471411</v>
+        <v>2.941293356223176</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.02809427477279216</v>
+        <v>0.02810335501673215</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.0216571980090996</v>
+        <v>0.02173075752146403</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2868151651243249</v>
+        <v>0.2846782922371406</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2788210310385767</v>
+        <v>0.2774699397218678</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>1107559587.036933</v>
+        <v>1133786275.630823</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5155,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>304.1</v>
+        <v>300.94</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1841279450632847</v>
+        <v>-0.192605931559832</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.2152055536917081</v>
+        <v>-0.2233606028542672</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5170,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>205361771000</v>
+        <v>203227791400</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.44147968465737</v>
+        <v>18.24984839296544</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.58095123561275</v>
+        <v>15.42236662925884</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.44266020006423</v>
+        <v>2.417277739583457</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.014579929988332</v>
+        <v>5.952080513418903</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.143532801406704</v>
+        <v>1.131649987686069</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>8.864575756350106</v>
+        <v>8.778263753801975</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.606874632759625</v>
+        <v>2.58149219189276</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07329504379858508</v>
+        <v>0.07406467281948405</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1835913870589896</v>
+        <v>0.1833364380238751</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.009169523370997412</v>
+        <v>0.009193245173364506</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01164090759618546</v>
+        <v>0.01176314215458231</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9633034634819719</v>
+        <v>0.9677494818052128</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.1992228317946164</v>
+        <v>0.1879756685577179</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>941277744.6016307</v>
+        <v>935306404.6005554</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>137.31</v>
+        <v>138.96</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2984007189742189</v>
+        <v>-0.2899698777121656</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5742853599553543</v>
+        <v>-0.5691697153841384</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>322.54</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>395517335700</v>
+        <v>400270111200</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>21.18981481481481</v>
+        <v>21.44444444444444</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.08815712151313</v>
+        <v>15.25622467857401</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.510363148362289</v>
+        <v>5.576579004416457</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.099285029653148</v>
+        <v>6.172577727191038</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4611900871459697</v>
+        <v>0.4667320261437911</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>13.6553376378579</v>
+        <v>13.78133910922588</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.176105656408042</v>
+        <v>7.24232151246221</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.07261375774887432</v>
+        <v>-0.07175154775833285</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4044004608489769</v>
+        <v>0.4056193387451377</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4508548033073139</v>
+        <v>0.4524194152468428</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01456558153084262</v>
+        <v>0.01439263097294185</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.032036045927392</v>
+        <v>2.035665938551664</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5164672568029839</v>
+        <v>0.4692162200095287</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4446397968.056055</v>
+        <v>4376393352.200984</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>107.63</v>
+        <v>108.69</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4154392254619501</v>
+        <v>0.4293792568564467</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1744266318938407</v>
+        <v>-0.1662959269770653</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>424216612994</v>
+        <v>428394543361</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>32.03273809523809</v>
+        <v>32.34821428571428</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.77531633110165</v>
+        <v>20.97244762822168</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.699038499707857</v>
+        <v>6.765014502345046</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.46100009943323</v>
+        <v>8.544328726260316</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.025047619047619</v>
+        <v>1.035142857142857</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>22.30539052869774</v>
+        <v>22.51408830306209</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>7.051426971875247</v>
+        <v>7.117402822566127</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.03204730692664383</v>
+        <v>0.03173476533732518</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5418652397260273</v>
+        <v>0.5424148320287019</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1658443251007578</v>
+        <v>0.1665946223574193</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01542320914243241</v>
+        <v>0.01527279418529764</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.6977772324081493</v>
+        <v>0.6979968636446052</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3415681093384201</v>
+        <v>0.3427434253204347</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>1847524622.555676</v>
+        <v>1799795847.880576</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>80.11</v>
+        <v>79.58</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.1585083763862538</v>
+        <v>-0.1640756034554747</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1805441898527005</v>
+        <v>-0.1859656301145663</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>242252640000</v>
+        <v>240649920000</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>11.42796005706134</v>
+        <v>11.35235378031384</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.24947583436448</v>
+        <v>10.17437971274635</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>1.876400139421401</v>
+        <v>1.863986057859881</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.355768053443587</v>
+        <v>1.346798423330928</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6074321111410996</v>
+        <v>0.6034133991337999</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.03174187317014</v>
+        <v>14.98336663547735</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>3.857454320127028</v>
+        <v>3.845040238565509</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.07913226456479483</v>
+        <v>0.07965928266254982</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.11497995036445</v>
+        <v>0.1157784652062612</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2887014992540743</v>
+        <v>-0.2883792807334584</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.0230932467856697</v>
+        <v>0.02324704699673285</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.7356140782002376</v>
+        <v>0.7367073273432854</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.2306039263147308</v>
+        <v>0.2261326981038017</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1164059443.797344</v>
+        <v>1156476370.210965</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 18:32 ET</t>
+          <t>2026-10-01 13:46 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-10-02)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="23" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>330.32</v>
+        <v>333.6712</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.218847969068255</v>
+        <v>0.2312135639881556</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.04349336885388311</v>
+        <v>-0.03378930908669708</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>345.34</v>
@@ -714,40 +714,40 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4851527433920</v>
+        <v>4900747701347</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>37.70776255707763</v>
+        <v>38.0903196347032</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.39321464939371</v>
+        <v>34.7511904117179</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.39264867823565</v>
+        <v>10.49808535857702</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.13794228794644</v>
+        <v>45.59588086930804</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.152181633688482</v>
+        <v>1.163870877727041</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.06051798915043</v>
+        <v>29.35265067333191</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.48853726984317</v>
+        <v>10.59397395018454</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02817318913717058</v>
+        <v>0.02789023396622353</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09637214611872147</v>
+        <v>0.09608675799086774</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1219765024388257</v>
+        <v>0.1220643675525841</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003209009445386292</v>
+        <v>0.00317678001577601</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3063535615180512</v>
+        <v>0.3077718284507744</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.207894563384302</v>
+        <v>0.2043115893786129</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13367931219.07394</v>
+        <v>13138304503.45512</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>512.8</v>
+        <v>514.46</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.08428129858508226</v>
+        <v>0.08779125754696082</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.07390016614895623</v>
+        <v>-0.07090226107057718</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3807822040000</v>
+        <v>3820148453000</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.48888888888888</v>
+        <v>28.58111111111111</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.78563797259107</v>
+        <v>24.85255278627491</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.47490813316096</v>
+        <v>11.51205389661854</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.611444730518752</v>
+        <v>8.639321092165909</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.9049022944057729</v>
+        <v>0.9078315803042005</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.86909314327845</v>
+        <v>18.92849210433744</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.79998535434352</v>
+        <v>11.8371311178011</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01759194607739599</v>
+        <v>0.01753518242135183</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1494111598173515</v>
+        <v>0.1500271765601218</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2354083608742514</v>
+        <v>0.2360808167417217</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007098283931357256</v>
+        <v>0.007075380010107686</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.556510696569168</v>
+        <v>0.5557707620697911</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.2241802053750376</v>
+        <v>0.2230201907642496</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10885672148.26014</v>
+        <v>10705386743.68614</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>338.24</v>
+        <v>344.2</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.07326671918356409</v>
+        <v>0.0921783489326593</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1722180073909106</v>
+        <v>-0.1576319718068574</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4093418121377</v>
+        <v>4165546704641</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.63008937437935</v>
+        <v>16.93346573982125</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.48010394287769</v>
+        <v>20.85992527715845</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.116366370721249</v>
+        <v>9.282672758698801</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.354194401074195</v>
+        <v>6.470111541343993</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1478923520348182</v>
+        <v>0.1505902956974723</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.71039279182395</v>
+        <v>12.93906561391336</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.243859832882524</v>
+        <v>9.410166220860079</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01310632785995953</v>
+        <v>0.01287151768160902</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.187988038500032</v>
+        <v>-0.1882297987728968</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.3020491922915698</v>
+        <v>0.3035481490800602</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002542573320719016</v>
+        <v>0.002498547356188263</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7612833798177663</v>
+        <v>0.7631672123965487</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.2510376874904931</v>
+        <v>0.2536740107473829</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8899837216.70809</v>
+        <v>8842405746.833708</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>248.23</v>
+        <v>251.11501</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.09593818984547453</v>
+        <v>0.1086755408388522</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1356894150417828</v>
+        <v>-0.1256441155988857</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2670234933000</v>
+        <v>2701269225591</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.70079365079365</v>
+        <v>19.93095238095238</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.24164334364216</v>
+        <v>22.51201406519194</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.442443962716584</v>
+        <v>3.482661049659654</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.840219498930423</v>
+        <v>4.896766397157463</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2230089839658368</v>
+        <v>0.2256143340584965</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.0838078126907</v>
+        <v>11.20662654677024</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.629401213129126</v>
+        <v>3.669618300072195</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004353549515936918</v>
+        <v>-0.004303275579743644</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1142383974777125</v>
+        <v>-0.1146526328903817</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1854659482523509</v>
+        <v>0.1859650526009251</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8347412718534323</v>
+        <v>0.8353152336340126</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.2387817715757208</v>
+        <v>0.2358857430370868</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8676940352.255217</v>
+        <v>8579026440.113382</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -1205,55 +1205,55 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>230.86</v>
+        <v>234.97501</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.2224516417196045</v>
+        <v>0.2442414742163237</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.02401285194893032</v>
+        <v>-0.0121704712658175</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>236.54</v>
+        <v>237.87</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5591660060000</v>
+        <v>5691329622833</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>29.03899371069182</v>
+        <v>29.55534591194968</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.87032169301511</v>
+        <v>17.13853034166713</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18.45621188966528</v>
+        <v>18.78438776343454</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>24.38818170701883</v>
+        <v>24.82183624183349</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2331021263851452</v>
+        <v>0.2372469943952424</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>24.00029554879379</v>
+        <v>24.42580328544467</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.51039895170793</v>
+        <v>18.8385748254772</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02271346945937196</v>
+        <v>0.02231664988877777</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7213064598948906</v>
+        <v>0.724497102303739</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9863018805345292</v>
+        <v>0.9898076485366889</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002252447370700857</v>
+        <v>0.002213001288945578</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.295957692682088</v>
+        <v>1.297166381591739</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.3642614908562415</v>
+        <v>0.3617829757755868</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27405038892.52246</v>
+        <v>27434752931.51926</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>725.9299999999999</v>
+        <v>730.21997</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.1161114219856634</v>
+        <v>0.1227072156806146</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.06910569105691067</v>
+        <v>-0.06360446000359066</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>779.8200000000001</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1849296925760</v>
+        <v>1860225568512</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>26.97621701969528</v>
+        <v>27.13563619472315</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>21.79194614516257</v>
+        <v>21.91562140107403</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.102138576285444</v>
+        <v>8.150019139322142</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.066966246970956</v>
+        <v>7.108729327695706</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.530124489037528</v>
+        <v>-5.562805419918241</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>18.17611444411237</v>
+        <v>18.27818261087866</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.526484025095511</v>
+        <v>8.574364588132207</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02215760997015675</v>
+        <v>0.0220274361849444</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2378984804752524</v>
+        <v>0.238186939722973</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.283112003985319</v>
+        <v>0.2837307908993967</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.002892840907525519</v>
+        <v>0.002875845753711721</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8386528847524404</v>
+        <v>0.8406150340619335</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4415869424661695</v>
+        <v>0.4410330504521152</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>14194738249.17449</v>
+        <v>14100271728.62915</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>354.11</v>
+        <v>371.87</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1916588808192005</v>
+        <v>-0.1511174155212677</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2901188781749293</v>
+        <v>-0.2545155664254355</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1398574227689</v>
+        <v>1468718189407</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>300.0932203389831</v>
+        <v>315.1737288135593</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>166.0936602669601</v>
+        <v>175.2208793062194</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.49727586339378</v>
+        <v>14.17555099686351</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.19687386308688</v>
+        <v>13.8600530175689</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-7.988396992122222</v>
+        <v>-8.389835879684885</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>115.7879304696541</v>
+        <v>121.6311455557034</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.44055846600527</v>
+        <v>14.118833599475</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.00411991003832604</v>
+        <v>0.003922779603555132</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8067710703505921</v>
+        <v>0.7987224471277508</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1281899177260426</v>
+        <v>0.1291337573683964</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,23 +1544,23 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.525314912177723</v>
+        <v>1.531488365839634</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.4030029545405748</v>
+        <v>0.4176873572575144</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13904298742.98586</v>
+        <v>13982361790.162</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
-          <t>2026-10-21 (E)</t>
+          <t>2026-10-21 (C)</t>
         </is>
       </c>
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>343.64</v>
+        <v>353.619</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-0.01144926981500538</v>
+        <v>0.01725736426867552</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.3057777777777778</v>
+        <v>-0.2856181818181818</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1634894791200</v>
+        <v>1682370682020</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>42.63523573200992</v>
+        <v>43.87332506203474</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>18.49181483770328</v>
+        <v>18.9580838612542</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.34816384449632</v>
+        <v>18.88097820546777</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.42881171632059</v>
+        <v>16.90588979837496</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4242417020858411</v>
+        <v>0.4365613038350979</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>31.96025469643916</v>
+        <v>32.8686581715554</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>18.74594621116897</v>
+        <v>19.27876057214042</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02410124505386583</v>
+        <v>0.02342111665467764</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.305627441449403</v>
+        <v>1.314227818756586</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8831489708149565</v>
+        <v>0.8912125520033845</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007566057502037016</v>
+        <v>0.007352546101878009</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.594873252828962</v>
+        <v>1.597709879672603</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3706423119362034</v>
+        <v>0.3401814548898847</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8905628518.060604</v>
+        <v>8847275334.765457</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>914.9400000000001</v>
+        <v>913.205</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.07073142188414283</v>
+        <v>0.06870099473376245</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1655813953488372</v>
+        <v>-0.1671637026903784</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>405756676260</v>
+        <v>404987240195</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>33.11400651465799</v>
+        <v>33.04958378574015</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>39.8096082954009</v>
+        <v>39.72278138937377</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.338450676092019</v>
+        <v>1.335846743371356</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.34571087618356</v>
+        <v>11.32363799122978</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>0.6442757131050194</v>
+        <v>0.643022285809976</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.4479891538408</v>
+        <v>27.39301369454698</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.300084037353952</v>
+        <v>1.297480104633289</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02314194823989315</v>
+        <v>0.02318705826208751</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1681905968795082</v>
+        <v>-0.1679942181848014</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.09081742447519536</v>
+        <v>0.09121305791329148</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1793,16 +1793,16 @@
         <v>80.58620689655173</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006055041860668459</v>
+        <v>0.00606654584677044</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1706532525404282</v>
+        <v>-0.1698776800680873</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1777331675221044</v>
+        <v>0.1772041324540218</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2068375501.252238</v>
+        <v>2019387397.985254</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>67.84999999999999</v>
+        <v>66.9499</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2543136433348949</v>
+        <v>-0.2642059394238302</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.45659138234823</v>
+        <v>-0.4638002562870415</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>282523328932</v>
+        <v>278775357237</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>21.00619195046439</v>
+        <v>20.72752321981424</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>18.07649825304251</v>
+        <v>17.83237683040873</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5.840786987197474</v>
+        <v>5.763302751161839</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.427027007979424</v>
+        <v>9.301967803707026</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6173771048856</v>
+        <v>0.6091869629238089</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.403962662398889</v>
+        <v>9.280801534874062</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>5.948498207140164</v>
+        <v>5.870592352707103</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03891575269752776</v>
+        <v>0.03944183763576634</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1620719708214937</v>
+        <v>0.1623533652826668</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1482868548958878</v>
+        <v>0.1485215357132694</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1067164251712059</v>
+        <v>0.1057580335817361</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3549388053060822</v>
+        <v>0.3558288240316629</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2406036674.994924</v>
+        <v>2379006997.819509</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -1961,55 +1961,55 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>500.93</v>
+        <v>501.59</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.008211721538420091</v>
+        <v>0.009540090245056421</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.0758942571992548</v>
+        <v>-0.06722579685349805</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>542.0700000000001</v>
+        <v>537.74</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>455.19</v>
+        <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1080432671343</v>
+        <v>1081856194716</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.60128449305035</v>
+        <v>12.61631863366469</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.58130820366216</v>
+        <v>22.61103377435201</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.810487891480606</v>
+        <v>2.813840983792018</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.439001488981934</v>
+        <v>1.440718310052161</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.347133297305694</v>
+        <v>0.3475474495936208</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.2902626383407</v>
+        <v>15.30712087372246</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.041223528504992</v>
+        <v>3.044576620816404</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02239727821187954</v>
+        <v>0.02237058866481509</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4419595012211599</v>
+        <v>-0.4420282257074181</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06209055386684414</v>
+        <v>0.06200394202778137</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02194511571651328</v>
+        <v>0.02435061344218852</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.135989858117545</v>
+        <v>0.1345100739642211</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2269941147.227409</v>
+        <v>2242672800.274588</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>333.18</v>
+        <v>331.11</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.0236573330274199</v>
+        <v>0.01729749546404058</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.09091405184174628</v>
+        <v>-0.09656207366984992</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>892759141800</v>
+        <v>887212556100</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>14.32416165090284</v>
+        <v>14.23516766981943</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.27323927125994</v>
+        <v>13.18770918160008</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2.999530098476983</v>
+        <v>2.980894444164457</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.48036312527029</v>
+        <v>2.464952981596271</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7500023513193904</v>
+        <v>0.7453426932749966</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.54507451481323</v>
+        <v>19.48553623980249</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.117665520288408</v>
+        <v>6.099029865975883</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1820580629085416</v>
+        <v>-0.1831962350876382</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07917602916406574</v>
+        <v>0.07942687193017584</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2866847194180255</v>
+        <v>-0.2863068383680573</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01800828381055285</v>
+        <v>0.01812086617740328</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7824185125479436</v>
+        <v>0.780216351472049</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.16701531897634</v>
+        <v>0.1630238087010308</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2596061186.30586</v>
+        <v>2545635934.397392</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>359.85</v>
+        <v>360.63</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.03858805296043322</v>
+        <v>0.04083926508023072</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.06670643462925008</v>
+        <v>-0.06468345566304434</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,37 +2228,37 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>671856938878</v>
+        <v>673313235703</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>30.57349192863212</v>
+        <v>30.63976210705183</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>23.95421240666444</v>
+        <v>24.00613483455717</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.10198118319547</v>
+        <v>15.13471578185129</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>19.573464732219</v>
+        <v>19.61589158366024</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.061699291239996</v>
+        <v>2.066168168403167</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.48463601890164</v>
+        <v>23.53468402306</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.36045537848409</v>
+        <v>15.3931899771399</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03127600354190235</v>
+        <v>0.03120835724855538</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2763305012744264</v>
+        <v>0.2763305012744266</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>0.1424590110366841</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007447547589273309</v>
+        <v>0.007431439425449908</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.2972963889504869</v>
+        <v>0.2943303559357441</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.181276151816512</v>
+        <v>0.179303865791111</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2304156000.309708</v>
+        <v>2248665737.100283</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>550</v>
+        <v>553.01</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-0.02331611664973321</v>
+        <v>-0.01797099212448905</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.08520865558937518</v>
+        <v>-0.08020225204996423</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>482369800000</v>
+        <v>485009678360</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>30.20318506315211</v>
+        <v>30.36847885777045</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>24.65697974361991</v>
+        <v>24.78238958125413</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>13.74938859276573</v>
+        <v>13.82463524670068</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>86.45517733024417</v>
+        <v>86.92832293708787</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.33487291127324</v>
+        <v>1.34217830666039</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>22.41462289744981</v>
+        <v>22.5339879887864</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.12997178120457</v>
+        <v>14.20521843513953</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03409832041724005</v>
+        <v>0.03391272532048611</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2249344963252164</v>
+        <v>0.2254055952998879</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1626930985085466</v>
+        <v>0.1630600375645386</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.006127272727272728</v>
+        <v>0.006093922352217862</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2906183498816045</v>
+        <v>0.2907418511268744</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1757341543849963</v>
+        <v>0.17640054933796</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1588943086.333008</v>
+        <v>1556811865.792562</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>365.2</v>
+        <v>368.8</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.08561238592762233</v>
+        <v>0.09631393190062187</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.2088730990858282</v>
+        <v>-0.2010744768424245</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>331654336341</v>
+        <v>334923656195</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>23.48402032023664</v>
+        <v>23.71551668702978</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>16.62940165190247</v>
+        <v>16.78772350639838</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7367984207660471</v>
+        <v>0.7440614939161884</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.360895755076335</v>
+        <v>3.394026162300527</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.711571947301165</v>
+        <v>-0.7185863476579126</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.60999636459263</v>
+        <v>14.73689617649342</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8361988148752912</v>
+        <v>0.8434618880254326</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.07120968252837044</v>
+        <v>0.07051457716754907</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4121987556629845</v>
+        <v>0.4126701978377818</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01287597649931516</v>
+        <v>0.01295637769461933</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02480832420591457</v>
+        <v>0.02456616052060738</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4358161641400222</v>
+        <v>0.4373028020738027</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.1930162444934698</v>
+        <v>0.1912884220594798</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1834271373.937758</v>
+        <v>1791614725.487882</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>163.87</v>
+        <v>164.03</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3360782548822372</v>
+        <v>0.3373827799373488</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.07108440564593843</v>
+        <v>-0.07017742758347034</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>679152660200</v>
+        <v>679815773800</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.09009009009009</v>
+        <v>21.11068211068211</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.39549860277076</v>
+        <v>14.32403094755036</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.880996677006592</v>
+        <v>1.882833251537141</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.636937941899915</v>
+        <v>2.639512605173876</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.065071321321323</v>
+        <v>2.067087623337625</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.898122662025758</v>
+        <v>9.907355012878524</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.969015288871656</v>
+        <v>1.970851863402205</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.044986940036431</v>
+        <v>0.04494305836596933</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4650475591050933</v>
+        <v>0.4737947850002644</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1145642553929336</v>
+        <v>0.1137141050512229</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02514188075913834</v>
+        <v>0.02511735658111321</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.551351629467426</v>
+        <v>-0.5486907574939983</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2532154849883972</v>
+        <v>0.2523317196535113</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2287474654.602138</v>
+        <v>2236361975.435644</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>258.66</v>
+        <v>255.865</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2474559555636995</v>
+        <v>0.2339763321360318</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.07973102785782893</v>
+        <v>-0.08967516988650504</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>182.94</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>623344324283</v>
+        <v>616608658210</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>29.90289017341041</v>
+        <v>29.57976878612717</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.01088097552655</v>
+        <v>20.79422126686764</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.365267941906891</v>
+        <v>6.296486824229799</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.427902060703063</v>
+        <v>7.347638447234939</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.702449954365689</v>
+        <v>-3.662442424703383</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.32759173138266</v>
+        <v>19.12790994337721</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.657459223345485</v>
+        <v>6.588678105668392</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.03001230503144281</v>
+        <v>0.03034015132760035</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4232097268192254</v>
+        <v>0.422499472642331</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09309168674187629</v>
+        <v>0.09250494653255203</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.02041289723961958</v>
+        <v>0.02063588220350576</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1614964188606702</v>
+        <v>-0.1665457894924392</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1827754330129731</v>
+        <v>0.1847339737292962</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1717069267.542791</v>
+        <v>1687764949.119389</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>104.26</v>
+        <v>104.215</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.07538135841786542</v>
+        <v>-0.07578043609742802</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2286179343000887</v>
+        <v>-0.2289508730393607</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>829709420800</v>
+        <v>829351307200</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>37.63898916967509</v>
+        <v>37.62274368231047</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.51568686227772</v>
+        <v>33.49138514036138</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.127567706023048</v>
+        <v>1.127081032833225</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.4415810582463</v>
+        <v>8.437937559803741</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.101791926485074</v>
+        <v>9.097863472267811</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>20.82064055650225</v>
+        <v>20.81228103363757</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.212132285279409</v>
+        <v>1.211645612089585</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01628160372938121</v>
+        <v>0.01628863412009101</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.123026042233322</v>
+        <v>0.1233558577716236</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05283438718430467</v>
+        <v>0.05295807679061038</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009375599462881258</v>
+        <v>0.009379647843400661</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.04460743944237326</v>
+        <v>-0.04289150431402575</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3098108219402948</v>
+        <v>0.309006095600626</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2811512129.639375</v>
+        <v>2564819258.219067</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>143.95</v>
+        <v>144.48</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.01523384453166776</v>
+        <v>0.01897176698808867</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1393124065769806</v>
+        <v>-0.1361434977578476</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>342199226481</v>
+        <v>343459147218</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.32592592592592</v>
+        <v>21.40444444444444</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.33113871921234</v>
+        <v>20.40235607147015</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.931878234224194</v>
+        <v>3.946354757077856</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.420778019185799</v>
+        <v>6.444418257811492</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.35102645502667</v>
+        <v>20.42595555555577</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.28066370946645</v>
+        <v>17.33994293864684</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.220094062884916</v>
+        <v>4.234570585738579</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04650215070221247</v>
+        <v>0.04633156557015417</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04892924200913229</v>
+        <v>0.04911630644342946</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02675350702871682</v>
+        <v>0.02710308467428768</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.0298061827023272</v>
+        <v>0.0296968438538206</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.03878189077509722</v>
+        <v>-0.03660249797253431</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1557259715758914</v>
+        <v>0.1469799867332665</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1219674764.1295</v>
+        <v>1155755368.855778</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -3095,46 +3095,46 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>282.46</v>
+        <v>283.77</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1832167196295744</v>
+        <v>-0.1794286218554285</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2896411236576717</v>
+        <v>-0.286346603626487</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>397.63</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>277.2</v>
+        <v>277.15</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>281645667820</v>
+        <v>282951891090</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>19.72486033519553</v>
+        <v>19.8163407821229</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>18.82651228295623</v>
+        <v>18.91382634898565</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.664808647916962</v>
+        <v>1.672529738792736</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>16.89626527050611</v>
+        <v>16.97462718902329</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-6.76608581265431</v>
+        <v>-6.797465733402653</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14.30598652812043</v>
+        <v>14.36060594145933</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.022317987303163</v>
+        <v>2.030039078178938</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05361701501352779</v>
+        <v>0.05336949663713944</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3143,7 +3143,7 @@
         <v>0.04771717877094983</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01440173331914685</v>
+        <v>0.01416228040029321</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03288961268852227</v>
+        <v>0.03273778059696233</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7107755743350802</v>
+        <v>0.7146054769759254</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2222683010546592</v>
+        <v>0.2119521663400371</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1393959263.753872</v>
+        <v>1368973230.123559</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -3221,55 +3221,55 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>615.73</v>
+        <v>630.09</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.755313897331095</v>
+        <v>1.819573081658112</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.03641627543035986</v>
+        <v>-0.02381232358509011</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>639</v>
+        <v>645.4598999999999</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>163.14</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>1004009338000</v>
+        <v>1027424754000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>156.2766497461929</v>
+        <v>159.9213197969543</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>44.25406750374708</v>
+        <v>45.21268396936095</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>24.30721070088367</v>
+        <v>24.87410129524271</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>14.93894487087945</v>
+        <v>15.28734960728312</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.261683043822475</v>
+        <v>1.291107902947888</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>93.59949038999814</v>
+        <v>95.77047956708341</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>24.28760048420288</v>
+        <v>24.85093814308195</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.008369444069851868</v>
+        <v>0.008179869519253796</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.531351095195049</v>
+        <v>2.537089722550588</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9401069202616024</v>
+        <v>0.9426505721861265</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.583595990975924</v>
+        <v>2.581644622612572</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.5516455589468467</v>
+        <v>0.5312464617300725</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10762942582.409</v>
+        <v>10801504179.53471</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1808.49</v>
+        <v>1867.65</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.5539792353136028</v>
+        <v>0.6048135841688096</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.09573691473829482</v>
+        <v>-0.06615632312646247</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>697024582544</v>
+        <v>719825910891</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>57.94629898403483</v>
+        <v>59.97822931785196</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.27424643532933</v>
+        <v>37.35641325036137</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>17.42304243512844</v>
+        <v>18.03399445539594</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>28.20034455267715</v>
+        <v>29.1892107361148</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.944616330272966</v>
+        <v>4.08293725356369</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>44.24825467253432</v>
+        <v>45.81175986982505</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>17.29035543491614</v>
+        <v>17.90130745518364</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01624970977205244</v>
+        <v>0.01569920538776029</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5974501107098944</v>
+        <v>0.6055671329011156</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3336837643145056</v>
+        <v>0.3402218340302536</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004301931445570614</v>
+        <v>0.004165662731239793</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.645351458491849</v>
+        <v>1.646034826764518</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.3730473536893661</v>
+        <v>0.3677776716130242</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2131666144.904175</v>
+        <v>2134334011.587874</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>192.28</v>
+        <v>192.95</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1558150924474121</v>
+        <v>-0.1528735286443113</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2440338116768233</v>
+        <v>-0.2413996461568705</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>151972343600</v>
+        <v>152501891500</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>72.01498127340821</v>
+        <v>72.26591760299623</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>71.81598272614728</v>
+        <v>71.96842154206331</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.616813060269163</v>
+        <v>1.622446848236608</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>24.9347687752918</v>
+        <v>25.02165402118033</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3854294859596724</v>
+        <v>0.3867725156850363</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>27.42781922302158</v>
+        <v>27.50401316546763</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.028015783818288</v>
+        <v>2.033649571785733</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001381830371404498</v>
+        <v>-0.001377032100614962</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>0.002770950695192287</v>
+        <v>0.004133702734595124</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1601138351317726</v>
+        <v>0.1588534294136892</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.256124660868292</v>
+        <v>1.254916727473262</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3005850100738784</v>
+        <v>0.2970194914455552</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1464791636.289649</v>
+        <v>1434717902.393649</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>896.67</v>
+        <v>902.96</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>-0.0193254438572904</v>
+        <v>-0.01244616501653772</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.2229828681357724</v>
+        <v>-0.2175322143172818</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>264523926690</v>
+        <v>266379520720</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>13.66042047531993</v>
+        <v>13.75624619134674</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.52128260386879</v>
+        <v>12.63705625365651</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.242925686510595</v>
+        <v>2.258659459881123</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.192327540695116</v>
+        <v>2.207706375975623</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3201813275952466</v>
+        <v>0.3224273495995226</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.09282090561591</v>
+        <v>26.15192943395025</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>6.945504181808931</v>
+        <v>6.96123795517946</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1569423247245688</v>
+        <v>-0.1558490678554743</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.0909761329960852</v>
+        <v>0.0885641335470353</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3861435826282921</v>
+        <v>-0.3860561277925144</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.02007427481682224</v>
+        <v>0.01993443784885266</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.592418781777549</v>
+        <v>1.593408725162392</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.2661742243727342</v>
+        <v>0.2580197491355951</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2008853751.420162</v>
+        <v>1975907382.037516</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>225.62</v>
+        <v>221.95</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2260034305317324</v>
+        <v>-0.2385934819897084</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3213619683570955</v>
+        <v>-0.3324008903326716</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>212564273080</v>
+        <v>209106641300</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>19.70480349344978</v>
+        <v>19.38427947598253</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.43977578228008</v>
+        <v>17.153056800948</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.076316961373142</v>
+        <v>3.026276702317033</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.155237373737375</v>
+        <v>6.055114507140369</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2402000270810062</v>
+        <v>0.2362928641549034</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>16.68604112446828</v>
+        <v>16.47288337956969</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.917163886709988</v>
+        <v>3.867123627653878</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06412648655623272</v>
+        <v>0.0651868344078271</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1298771119219957</v>
+        <v>0.1300772626667468</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04772082573344871</v>
+        <v>0.04782834788081303</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02987323818810389</v>
+        <v>0.03036719981977923</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.9078606610292855</v>
+        <v>0.8960668704818062</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.3109835651049289</v>
+        <v>0.2981374028746708</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1238213523.097524</v>
+        <v>1223167102.181099</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1151.42</v>
+        <v>1139.215</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.0657743859564679</v>
+        <v>0.05447722559743395</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1092561791668278</v>
+        <v>-0.1186980234402198</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>783.85</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1084339422220</v>
+        <v>1072845473315</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.52191368350619</v>
+        <v>38.1135831381733</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>25.9789451749595</v>
+        <v>25.6872233108754</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.61110316120594</v>
+        <v>13.46682608239671</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.32932518669382</v>
+        <v>30.00783570943652</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.407224084087168</v>
+        <v>0.402907527186746</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>26.10235868125474</v>
+        <v>25.83693893783137</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.18874124429806</v>
+        <v>14.04446416548883</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01849411686881499</v>
+        <v>0.01869225391615363</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4828128480226583</v>
+        <v>0.483756444864045</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2396561367256922</v>
+        <v>0.2401241616704812</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005810216949505827</v>
+        <v>0.005872464811295498</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3353007432765417</v>
+        <v>0.316631481857006</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.2910276862764735</v>
+        <v>0.2915845549426211</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2754602708.328646</v>
+        <v>2677737469.277344</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>188.03</v>
+        <v>190.705</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.03369986975922656</v>
+        <v>0.04840575260561253</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1903982777179763</v>
+        <v>-0.178880516684607</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>296575958400</v>
+        <v>300795182400</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>15.11495176848875</v>
+        <v>15.32556270096463</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>13.92264283425592</v>
+        <v>14.13932901298379</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.343936634289372</v>
+        <v>2.376596922444657</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.67526857277412</v>
+        <v>2.712545622503781</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.3845484880131183</v>
+        <v>0.3899067661527469</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>22.52420889358367</v>
+        <v>22.6650230687975</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.224240754293483</v>
+        <v>5.256901042448767</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.052883585320313</v>
+        <v>-0.05215683476411463</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08563811831035562</v>
+        <v>0.08389603826967718</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3267940645807226</v>
+        <v>-0.3270177364966708</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02207094612561825</v>
+        <v>0.02176135916730028</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.385192280764841</v>
+        <v>1.389783573782485</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2338624383149912</v>
+        <v>0.2258270437588209</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1012973427.956974</v>
+        <v>995563912.7746317</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1097.39</v>
+        <v>1078</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.479138777766308</v>
+        <v>2.417665189615432</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1255856573705179</v>
+        <v>-0.1410358565737052</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,40 +4120,40 @@
         <v>179.61</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1239381292100</v>
+        <v>1217482420000</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>14.57163723277121</v>
+        <v>14.31416810516532</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.466373754738755</v>
+        <v>6.21221055791666</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>9.305502688680663</v>
+        <v>9.14108192930294</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>8.961328390351067</v>
+        <v>8.802988914422812</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.01647546923303278</v>
+        <v>0.01618436092292561</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>11.35829086687015</v>
+        <v>10.81991061146147</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>9.052657086974804</v>
+        <v>8.888236327597081</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.0426890419738005</v>
+        <v>0.0434568903261864</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>2.563272513243084</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>1.253448035244278</v>
+        <v>1.3041987987551</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.023493644986467</v>
+        <v>1.059878965778603</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.4337631707914727</v>
@@ -4165,7 +4165,7 @@
         <v>0.8071598041865633</v>
       </c>
       <c r="Z29" s="4" t="n">
-        <v>0.7458629906598192</v>
+        <v>0.7501201309427276</v>
       </c>
       <c r="AA29" s="5" t="n">
         <v>89675000000</v>
@@ -4183,22 +4183,22 @@
         <v>0.02393204279996733</v>
       </c>
       <c r="AF29" s="6" t="n">
-        <v>-0.3172431984324365</v>
+        <v>-0.3077963623069189</v>
       </c>
       <c r="AG29" s="6" t="n">
-        <v>0</v>
+        <v>942.5188679245283</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0004829641239668668</v>
+        <v>0.0004916512059369203</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.854515602388947</v>
+        <v>2.833836470107001</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.5153952182212441</v>
+        <v>0.4906260841666388</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25339970985.36523</v>
+        <v>25194013042.00367</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>137.76</v>
+        <v>135.73</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.06571717293180801</v>
+        <v>-0.07948455198921534</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2861066487018707</v>
+        <v>-0.2966264186142924</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>192.97</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>142424829120</v>
+        <v>140326084843</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>85.56521739130434</v>
+        <v>84.30434782608695</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.81270504005737</v>
+        <v>28.37242082112788</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.667718512082542</v>
+        <v>9.52525691304643</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.36993288590604</v>
+        <v>11.20238814317673</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>136.9043478260899</v>
+        <v>134.886956521742</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>42.52646291774147</v>
+        <v>41.9249311673832</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.07160121639967</v>
+        <v>9.929139617363562</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03215731434117518</v>
+        <v>0.03263826540250309</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.969704415893815</v>
+        <v>1.971348421679572</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2551178063291542</v>
+        <v>0.2556827048211145</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6857718607876562</v>
+        <v>0.6792902704653833</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5375882213176902</v>
+        <v>0.5343982816266427</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>1940259472.197003</v>
+        <v>1885910294.587726</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.12</v>
+        <v>27.565</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1167593192689478</v>
+        <v>0.09471801691495529</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.03731598767545363</v>
+        <v>-0.05631633002396441</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.62</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>160268252800</v>
+        <v>157105063600</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>37.15644820295984</v>
+        <v>36.42309725158563</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.642234018385574</v>
+        <v>9.452967652002901</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.516143129866868</v>
+        <v>2.466482410198442</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.881158351919239</v>
+        <v>1.844030226552412</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6214662575539299</v>
+        <v>-0.6092004761548393</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.62406945500634</v>
+        <v>17.37349996831432</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.49293916101482</v>
+        <v>3.443278441346395</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06854757450753216</v>
+        <v>0.06992772701439523</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.853510310174057</v>
+        <v>2.853085992933476</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.052028089923842</v>
+        <v>-0.05213500470277488</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06116642958748222</v>
+        <v>0.06239796843823689</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3231524583688886</v>
+        <v>0.3024030625798646</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.1948002945206406</v>
+        <v>0.2001088390732026</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>920980661.4170207</v>
+        <v>908421410.9012306</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>193.5</v>
+        <v>193.74</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.1517171973487978</v>
+        <v>0.1531456837951219</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.03187071596537749</v>
+        <v>-0.03066993545804775</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1373569214085</v>
+        <v>1375272865823</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>8.008897959911293</v>
+        <v>8.043852233604305</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004450939721706096</v>
+        <v>0.004462943158488125</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.878256515701447</v>
+        <v>6.908276184073303</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.984402898522113</v>
+        <v>5.00615697554785</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01792291358000789</v>
+        <v>0.01800113687986609</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>8.091169455639246</v>
+        <v>8.126638800618997</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.848004211452185</v>
+        <v>6.878023879824041</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07007869102941186</v>
+        <v>0.06977416657083756</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1798.372370929658</v>
+        <v>1801.364930036271</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2388.580601055508</v>
+        <v>2393.868204169602</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.550387596899225</v>
+        <v>1.548467017652524</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>0.679981290788235</v>
+        <v>0.6561127664429871</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3203660537.088507</v>
+        <v>3137780403.970642</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>617.8099999999999</v>
+        <v>631.3200000000001</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6549960359029956</v>
+        <v>0.6911867684017405</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.08040724588065451</v>
+        <v>-0.06029799205156061</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>315.05</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>77869234522</v>
+        <v>79572045027</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.817524582240243</v>
+        <v>1.816564604692817</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.3297431638599451</v>
+        <v>0.3078543264676102</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3615282533.510901</v>
+        <v>3600779151.151469</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>148.07</v>
+        <v>157.645</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.08002483499508306</v>
+        <v>-0.02053430885932228</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3437776989895408</v>
+        <v>-0.3013428470129409</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1951826156456</v>
+        <v>2078041699430</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-87.09999999999998</v>
+        <v>-92.71764705882352</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>110.4006822731544</v>
+        <v>117.1187156523509</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>117.7288229963206</v>
+        <v>125.3219226087822</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.824832421555681</v>
+        <v>7.265010375400868</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>0.4297170582226761</v>
+        <v>0.4574323138857176</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>533.952773341587</v>
+        <v>569.3737070711874</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>114.4621603508052</v>
+        <v>122.0552599632668</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01281364117253739</v>
+        <v>-0.01203727857135753</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.406069900278203</v>
+        <v>4.522632508010068</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.03021735747263578</v>
@@ -4776,13 +4776,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.110569095749032</v>
+        <v>3.183811896982828</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7378633222176418</v>
+        <v>0.7213379472880888</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12438207396.78692</v>
+        <v>12316035887.03485</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4819,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>763.99</v>
+        <v>769.205</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1183014756379781</v>
+        <v>0.1259350077463199</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01973388762718609</v>
+        <v>-0.01304258567817596</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4834,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>813831352282</v>
+        <v>819386569630</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4860,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9959763388905098</v>
+        <v>0.9955955776748456</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.09892233949713872</v>
+        <v>0.09009247783997112</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32427147548.92735</v>
+        <v>31907863083.13456</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -4899,13 +4899,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>459.2</v>
+        <v>472.59</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.436751106179903</v>
+        <v>0.4786459173988682</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.04133611691022965</v>
+        <v>-0.01338204592901882</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4914,40 +4914,40 @@
         <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2381631616000</v>
+        <v>2451078564207</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>29.09470267763997</v>
+        <v>28.97878752752985</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6969676036364113</v>
+        <v>0.7148852323143976</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.65835857828367</v>
+        <v>14.59995874331043</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>10.1179219661725</v>
+        <v>10.07761152009213</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5465571440611043</v>
+        <v>0.5443796255588689</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>19.30903511202044</v>
+        <v>19.22947662230763</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>14.17377916681305</v>
+        <v>14.11537933183981</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01718332855433321</v>
+        <v>0.01725206186855054</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.74469878634111</v>
+        <v>39.53627941608583</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.85069437461754</v>
+        <v>39.6123560650974</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4981,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2613240418118467</v>
+        <v>0.2539198882752492</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.17702766076417</v>
+        <v>2.177761992641401</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.2526194683032298</v>
+        <v>0.2537825105946789</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4144036484.329987</v>
+        <v>4085984616.660311</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -5027,13 +5027,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>30.95</v>
+        <v>30.9458</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.08558399689686214</v>
+        <v>0.08543668016707318</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.0006457862447529772</v>
+        <v>-0.0007814013561511235</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30.97</v>
@@ -5042,38 +5042,38 @@
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>77595880927</v>
+        <v>77585350953</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-24.37007874015748</v>
+        <v>-24.36220472440945</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-109.6603798113113</v>
+        <v>-110.8762614754603</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.148577625003461</v>
+        <v>2.147883415755226</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.366631646263475</v>
+        <v>2.365866983372922</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1813587255081487</v>
+        <v>0.1813001281816518</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>17.56196378958678</v>
+        <v>17.55781976198347</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.941987565471411</v>
+        <v>2.941293356223176</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.02809427477279216</v>
+        <v>0.02810335501673215</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02173075752146403</v>
+        <v>0.02161322525767528</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2851046332542647</v>
+        <v>0.2850469312803105</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2774071758774403</v>
+        <v>0.274868551048402</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>1145414698.517874</v>
+        <v>1142202668.104479</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -5155,55 +5155,55 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>302.09</v>
+        <v>302.95</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1895205883727974</v>
+        <v>-0.1872132882503194</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.2203927843299183</v>
+        <v>-0.2181733722160573</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>239.27</v>
+        <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>204004397900</v>
+        <v>204585164500</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.31958762886598</v>
+        <v>18.37174044875682</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.48130104018343</v>
+        <v>15.51664349953506</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.42651502741665</v>
+        <v>2.433422912231037</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>5.974825554259043</v>
+        <v>5.991834889148191</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.135974429388198</v>
+        <v>1.139208359704574</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>8.809674724963598</v>
+        <v>8.833164718492155</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.590729460112045</v>
+        <v>2.597637344926433</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07378272309295152</v>
+        <v>0.07357327222033248</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1833364380238751</v>
+        <v>0.1840022263389187</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.009193245173364506</v>
+        <v>0.009352068397343594</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5239,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01171836207752657</v>
+        <v>0.01168509655058591</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9695386603479144</v>
+        <v>0.9701999360810932</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.1873072519185823</v>
+        <v>0.1866277989829302</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>953019564.5416056</v>
+        <v>924190243.9739217</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5281,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>138.08</v>
+        <v>140.711</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2944663263852607</v>
+        <v>-0.2810229667728593</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5718980591554536</v>
+        <v>-0.563740931357351</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>322.54</v>
@@ -5296,40 +5296,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>397735297600</v>
+        <v>405313814170</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>21.30864197530864</v>
+        <v>21.71466049382716</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.15961070536484</v>
+        <v>15.43508571104995</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.541263881187567</v>
+        <v>5.646848073477576</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.133488288504163</v>
+        <v>6.250356826214581</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4637763253449531</v>
+        <v>0.4726131989832973</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>13.71413832449629</v>
+        <v>13.91505339793213</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.20700638923332</v>
+        <v>7.312590581523329</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.07220882876953891</v>
+        <v>-0.07085867541626406</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4056193387451377</v>
+        <v>0.4068377008286823</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4524194152468424</v>
+        <v>0.4539839729447046</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5365,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01448435689455388</v>
+        <v>0.01421352985907285</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.034604224734208</v>
+        <v>2.033459025156892</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.468426769372298</v>
+        <v>0.4659002321944846</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4426270924.07277</v>
+        <v>4455294754.157512</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5407,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>108.76</v>
+        <v>111.6</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4302998249674042</v>
+        <v>0.4676485883262438</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1657589936335047</v>
+        <v>-0.1439748408376161</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5422,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>428670434165</v>
+        <v>439864108614</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>32.36904761904762</v>
+        <v>33.21428571428572</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>20.9859545868561</v>
+        <v>21.52887802432403</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.769371246190289</v>
+        <v>6.946136732949073</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.549831560107389</v>
+        <v>8.773089390474297</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.035809523809524</v>
+        <v>1.062857142857143</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>22.52787023153004</v>
+        <v>23.08702275907887</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>7.121759718357679</v>
+        <v>7.298525205116463</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.0317143402401462</v>
+        <v>0.03090727280031435</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5424148320287019</v>
+        <v>0.5427782941943899</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1665946223574193</v>
+        <v>0.1668121081832903</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5491,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01526296432511953</v>
+        <v>0.01496415770609319</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.69782371734385</v>
+        <v>0.702131283720284</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.34287773930855</v>
+        <v>0.325675495569452</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>1827710326.509302</v>
+        <v>1804148582.309812</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>80.27</v>
+        <v>80.3</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.1568277040634702</v>
+        <v>-0.1565125780029483</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1789075286415712</v>
+        <v>-0.1786006546644845</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5548,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>242736480000</v>
+        <v>242827200000</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>11.45078459343795</v>
+        <v>11.45506419400856</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.26259687788576</v>
+        <v>10.25888946974585</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>1.880147786685256</v>
+        <v>1.880850470547229</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.358475866307786</v>
+        <v>1.358983581219824</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6086453072187751</v>
+        <v>0.6088727814833391</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.04634571851136</v>
+        <v>15.04908393951284</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>3.861201967390883</v>
+        <v>3.861904651252856</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.07897453238178291</v>
+        <v>0.07894502757516456</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1157784652062612</v>
+        <v>0.1165988509565592</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2883792807334585</v>
+        <v>-0.2882053521359116</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5617,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.02304721564719073</v>
+        <v>0.02303860523038605</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.7383234713803694</v>
+        <v>0.7426084983822193</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.226262174389647</v>
+        <v>0.2255306843255055</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1177355383.56677</v>
+        <v>1151087192.0286</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 19:23 ET</t>
+          <t>2026-10-02 13:06 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-10-03)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -443,7 +443,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
@@ -720,7 +720,7 @@
         <v>38.09246575342466</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.75314839424603</v>
+        <v>34.72978233130519</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.4986768510549</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09608675799086774</v>
+        <v>0.09682420091324206</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1220643675525841</v>
+        <v>0.1237555839879354</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003176601036890527</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3077125671403584</v>
+        <v>0.3077125615899974</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.2043191108382786</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13311682602.84147</v>
+        <v>13326888489.19373</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>28.75166666666667</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.00085846029011</v>
+        <v>24.98845597279366</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.58075118204913</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1500271765601218</v>
+        <v>0.1505979680365297</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2360808167417217</v>
+        <v>0.2367082903413673</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007033408691283598</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5573272470191897</v>
+        <v>0.5573272488331004</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.2238603879860033</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10875132685.60161</v>
+        <v>10885893929.01479</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>16.89920556107249</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.81750241924442</v>
+        <v>20.84077342420278</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.263891840907357</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1882212755046789</v>
+        <v>-0.1891277153156355</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.3035618358234407</v>
+        <v>0.3042680008145242</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002503639010189229</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.762634282349573</v>
+        <v>0.7626342821504202</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.2527090373726006</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8951048482.341259</v>
+        <v>8962545782.29126</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>19.96190476190476</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.54832069846035</v>
+        <v>22.56022348728764</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.488069554455446</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1147054794520548</v>
+        <v>-0.1151725614263971</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.185894240826008</v>
+        <v>0.186322533399665</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8357984276955277</v>
+        <v>0.8357984321047139</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.2365027694000736</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8712945476.449318</v>
+        <v>8715845460.178579</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -1211,10 +1211,10 @@
         <v>0.238813833406833</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.0164795896918486</v>
+        <v>-0.01652093492517237</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>237.87</v>
+        <v>237.88</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>164.27</v>
@@ -1226,7 +1226,7 @@
         <v>29.42767295597483</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.06376849790548</v>
+        <v>17.04222654675353</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>18.70324340114005</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7245705694839317</v>
+        <v>0.7267504850521234</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9898924165170029</v>
+        <v>0.992392935564365</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1292,13 +1292,13 @@
         <v>0.002222697157512289</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.296333330673191</v>
+        <v>1.296333349165572</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3608323955500798</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27793480930.01773</v>
+        <v>27796943015.65257</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>27.05611296915645</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>21.85139586047473</v>
+        <v>21.84634935909594</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>8.126134826530791</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2381869397229732</v>
+        <v>0.2384729606043485</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2837307908993965</v>
+        <v>0.2843621815581034</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.002884298428744094</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8401949107559736</v>
+        <v>0.8401949314511553</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.4410630741729306</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>14258457322.96835</v>
+        <v>14260191925.07039</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>314.0593220338983</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>174.6177579855645</v>
+        <v>174.4853752506838</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>14.12542843244965</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7985531692593453</v>
+        <v>0.7999177385651266</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.129027498234642</v>
+        <v>0.129399336556381</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.530193244730398</v>
+        <v>1.530193213701677</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.4154194997610596</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>14228418822.09464</v>
+        <v>14241949087.56693</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>44.06203473945409</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.03962711982619</v>
+        <v>19.01832682853388</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>18.96218981414976</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.314227818756586</v>
+        <v>1.316819725347564</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8912125520033847</v>
+        <v>0.8933135152237064</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1670,13 +1670,13 @@
         <v>0.007321056484766572</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.598741744427964</v>
+        <v>1.598741738467171</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.3427865039122595</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8982847951.902552</v>
+        <v>8984006560.68634</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>33.32066594281579</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.04662555080947</v>
+        <v>40.03636686274647</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.346803741167855</v>
@@ -1754,10 +1754,10 @@
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1679532174180337</v>
+        <v>-0.1677400185424814</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.09126683226565691</v>
+        <v>0.09149087184076876</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1796,13 +1796,13 @@
         <v>0.006017487644598925</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.168025413883796</v>
+        <v>-0.1680254288398988</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1780334448745785</v>
+        <v>0.1780334448745784</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2052733794.217427</v>
+        <v>2053114789.885864</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>20.76160990712075</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>17.86170241101495</v>
+        <v>17.85358713525227</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>5.772780771728145</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.162353365282667</v>
+        <v>0.1628817082997582</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1485215357132692</v>
+        <v>0.1489503391999123</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1064516788901533</v>
+        <v>0.1064516977890281</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3555075668048129</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2421761065.757981</v>
+        <v>2422396161.935526</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.65232694931057</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.6588172146136</v>
+        <v>22.65801789655555</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.821871985328332</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4416157370672217</v>
+        <v>-0.4415960386705334</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06278904368001603</v>
+        <v>0.06283450603239404</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2054,7 +2054,7 @@
         <v>0.1348785802685299</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2285548458.463979</v>
+        <v>2286357423.364156</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>14.28976784178848</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.23829173924144</v>
+        <v>13.23121441259915</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>2.992327913235427</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07942687193017584</v>
+        <v>0.08000425328920269</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2863068383680573</v>
+        <v>-0.2860120708933945</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.1626722303349957</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2589931148.260856</v>
+        <v>2591247550.349528</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
         <v>0.1792858342637725</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2277117361.534969</v>
+        <v>2277374055.281576</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>30.3272926963207</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>24.74877935325474</v>
+        <v>24.73926850715404</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>13.80588608043782</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2254055952998879</v>
+        <v>0.2258766942745591</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1630600375645386</v>
+        <v>0.1634269766205307</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.1761412792400913</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1584438650.433724</v>
+        <v>1584446418.891195</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>23.91486078065719</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>16.92883506515606</v>
+        <v>16.92318738866425</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7503158069086862</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4126701978377818</v>
+        <v>0.4131416400125791</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01295637769461955</v>
+        <v>0.01303677888992372</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.1956266165552836</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1817490922.689262</v>
+        <v>1817665616.513062</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.10810810810811</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.32228443399216</v>
+        <v>14.32563412067245</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.882603679720822</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4737947850002646</v>
+        <v>0.4734501754200384</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1137141050512229</v>
+        <v>0.1135807288891308</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2523323921237285</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2272081414.47892</v>
+        <v>2272752630.84844</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>146.12</v>
+        <v>182.94</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>617006291448</v>
@@ -2738,7 +2738,7 @@
         <v>29.59884393063583</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>20.80763086376066</v>
+        <v>20.82414835057152</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.300547247985786</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.422499472642331</v>
+        <v>0.4213711616121625</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09250494653255203</v>
+        <v>0.0927931659382244</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2807,10 +2807,10 @@
         <v>-0.166112224755526</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1845552652087571</v>
+        <v>0.184555265208757</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1747350939.131608</v>
+        <v>1753868643.604533</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>37.63898916967509</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.50584670857437</v>
+        <v>33.49601233128282</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.127567706023048</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1233558577716236</v>
+        <v>0.1236856733099252</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05295807679061038</v>
+        <v>0.05308176639691631</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2936,7 +2936,7 @@
         <v>0.3090152315932373</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2613472057.316089</v>
+        <v>2614601902.107239</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.46814814814815</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.4630773693019</v>
+        <v>20.45976788294378</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.958099860522566</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04911630644342946</v>
+        <v>0.04928600710299325</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02710308467428768</v>
+        <v>0.02718330971115024</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.1477048353764854</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1174526136.898394</v>
+        <v>1174667535.249634</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v>19.75209497206704</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>18.85250654688866</v>
+        <v>18.85402710287227</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1.667107293292193</v>
@@ -3140,7 +3140,7 @@
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04771717877094961</v>
+        <v>0.0476326815642456</v>
       </c>
       <c r="V21" s="4" t="n">
         <v>0.01416228040029321</v>
@@ -3188,7 +3188,7 @@
         <v>0.2112150781700568</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1393718870.277472</v>
+        <v>1394353830.82784</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -3227,13 +3227,13 @@
         <v>1.836667098658753</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.01789406282249284</v>
+        <v>-0.01789421497846511</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>645.4598999999999</v>
+        <v>645.46</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>163.14</v>
+        <v>188.22</v>
       </c>
       <c r="K22" s="5" t="n">
         <v>1033653646000</v>
@@ -3242,7 +3242,7 @@
         <v>160.8908629441624</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.48679156155088</v>
+        <v>45.399470818286</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>25.02490366783682</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.537089722550587</v>
+        <v>2.543892914261873</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9426505721861265</v>
+        <v>0.9479036686977758</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.583796302406725</v>
+        <v>2.583796341276141</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.532768801593928</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10944009702.88475</v>
+        <v>10954613474.22119</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>59.97822931785196</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.34961262898953</v>
+        <v>37.35445693150112</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>18.03399445539594</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.605859474732513</v>
+        <v>0.6056512192865573</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3404658617620062</v>
+        <v>0.339390097152966</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004166421215545357</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.646024390430644</v>
+        <v>1.64602439098886</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.3676876579045484</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2166731709.925147</v>
+        <v>2167307401.616211</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>72.49438202247188</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>72.19594544535774</v>
+        <v>71.83892179813952</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.627576117878611</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>0.004133702734594902</v>
+        <v>0.009124026473756652</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1588534294136892</v>
+        <v>0.1592739976984785</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,7 +3568,7 @@
         <v>0.2976674614795599</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1489960463.697768</v>
+        <v>1490290186.701609</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>13.75015234613041</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.63145819560137</v>
+        <v>12.63317384445917</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.257658901956129</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.0885641335470353</v>
+        <v>0.08841630103595377</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3860561277925143</v>
+        <v>-0.3856799360090674</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.2579039776544408</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1999159994.921871</v>
+        <v>1999831319.048055</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>19.44454148471616</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.20638236613229</v>
+        <v>17.20333544136481</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.0356848164175</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1300772626667466</v>
+        <v>0.1302774134114975</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04782834788081303</v>
+        <v>0.04793587002817756</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.2972153427664984</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1256791537.408262</v>
+        <v>1256909083.906606</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>38.23519571763131</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>25.76918594017279</v>
+        <v>25.75279440123893</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.50979594568811</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.483756444864045</v>
+        <v>0.4847008492325742</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2401241616704812</v>
+        <v>0.2405922671077951</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3946,7 +3946,7 @@
         <v>0.2911618053174975</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2722880618.300155</v>
+        <v>2724107353.463949</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
         <v>232.25</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>151.84</v>
+        <v>107.97</v>
       </c>
       <c r="K28" s="5" t="n">
         <v>300172156800</v>
@@ -4000,7 +4000,7 @@
         <v>15.29823151125402</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.11004275955504</v>
+        <v>14.11361365170655</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.372358564439773</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08420872792142009</v>
+        <v>0.08393441175175087</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.326823590026738</v>
+        <v>-0.3266710464831442</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.2247928906658313</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1019447190.290145</v>
+        <v>1019891354.793447</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>14.27287212853539</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.194288503338626</v>
+        <v>6.156758758247687</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>9.114710162326936</v>
@@ -4150,10 +4150,10 @@
         <v>2.563272513243084</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>1.3041987987551</v>
+        <v>1.318244499902685</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.059878965778603</v>
+        <v>1.066155043275526</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.4337631707914727</v>
@@ -4192,13 +4192,13 @@
         <v>0.0004930737098679865</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.834859152839396</v>
+        <v>2.834859283550031</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>0.4915022541449128</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25507144651.083</v>
+        <v>25532252576.97917</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>83.46583850931678</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.09022257380951</v>
+        <v>28.07504164703675</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.43051693999457</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.971348421679572</v>
+        <v>1.972955109333788</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2556827048211143</v>
+        <v>0.256247603500162</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.5370393532678653</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>1906519268.630121</v>
+        <v>1906916088.305206</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.73361522198732</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.533557073306026</v>
+        <v>9.534630356278514</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.487509922130118</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.853085992933476</v>
+        <v>2.852652263314895</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05213500470277488</v>
+        <v>-0.05224180804050416</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.1953388323706219</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>926781767.8938206</v>
+        <v>926857018.7850889</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>8.043852233604305</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004494962829130731</v>
+        <v>0.004494530107998797</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.908276184073303</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1788.525862477462</v>
+        <v>1788.698153159298</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2376.808465514192</v>
+        <v>2378.499116531139</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4574,7 +4574,7 @@
         <v>0.6560713248816935</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3186911878.90683</v>
+        <v>3187987916.814423</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.816574062332065</v>
+        <v>1.816574087056346</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.3073465589163391</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3651739771.57959</v>
+        <v>3652328457.676798</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-93.50588235294117</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>118.0956645634032</v>
+        <v>117.6741167403561</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>126.3873418214006</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.523508448962088</v>
+        <v>4.534087932662793</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.03021735747263578</v>
@@ -4782,7 +4782,7 @@
         <v>0.7258596652729258</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12536837084.65302</v>
+        <v>12537749128.28888</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -4831,7 +4831,7 @@
         <v>779.37</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>508.46</v>
+        <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
         <v>819849948259</v>
@@ -4866,7 +4866,7 @@
         <v>0.09036762064446385</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32458232048.746</v>
+        <v>32469748762.34253</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
         <v>28.97878752752985</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.7151726446467359</v>
+        <v>0.7140361805050256</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.59995874331043</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>39.51998876696984</v>
+        <v>39.58448061698169</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>39.59603452785877</v>
+        <v>39.63284482563324</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4990,7 +4990,7 @@
         <v>0.2540021808144101</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4153240841.159297</v>
+        <v>4156301666.149394</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
         <v>-24.36220472440945</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-110.8554805515043</v>
+        <v>-112.1139516391971</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>2.147883415755226</v>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02180473646513503</v>
+        <v>0.02187871540880648</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2852111246281611</v>
+        <v>0.2852111368464148</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.274868551048402</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>1181137121.303196</v>
+        <v>1191154992.248116</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
         <v>18.36143117040631</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.50793635513856</v>
+        <v>15.50246610586962</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.432057400116566</v>
@@ -5200,10 +5200,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1840022263389187</v>
+        <v>0.1844200171129038</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.009352068397343594</v>
+        <v>0.009584754252444316</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5248,7 +5248,7 @@
         <v>0.1864841376668144</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>938589003.1375732</v>
+        <v>940276214.402771</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
         <v>21.95987654320988</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.60938872357106</v>
+        <v>15.59588223908579</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>5.710615949398833</v>
@@ -5326,10 +5326,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4068377008286823</v>
+        <v>0.4080560629122274</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4539839729447048</v>
+        <v>0.4555485306425668</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5374,7 +5374,7 @@
         <v>0.469622517849374</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4508890669.372356</v>
+        <v>4533255223.718211</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
         <v>33.39285714285715</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>21.64462468036878</v>
+        <v>21.63952663793074</v>
       </c>
       <c r="N40" s="6" t="n">
         <v>6.98348155409396</v>
@@ -5452,10 +5452,10 @@
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5427782941943899</v>
+        <v>0.5431417563600782</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1668121081832903</v>
+        <v>0.1670295940091615</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5494,13 +5494,13 @@
         <v>0.01488413547237077</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.703181388236128</v>
+        <v>0.7031813612060062</v>
       </c>
       <c r="AJ40" s="4" t="n">
         <v>0.3287439176769288</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>1843492235.829197</v>
+        <v>1847504683.500061</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
         <v>11.47646219686163</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.27805302417252</v>
+        <v>10.27552203924642</v>
       </c>
       <c r="N41" s="6" t="n">
         <v>1.884363889857093</v>
@@ -5578,10 +5578,10 @@
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1165988509565592</v>
+        <v>0.1168738827115863</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2882053521359115</v>
+        <v>-0.2882789051785076</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5626,7 +5626,7 @@
         <v>0.225718041828961</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1169047403.136974</v>
+        <v>1169156892.901154</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 19:11 ET</t>
+          <t>2026-10-03 11:27 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-10-04)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>28.75166666666667</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.98845597279366</v>
+        <v>24.97606578450893</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.58075118204913</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1505979680365297</v>
+        <v>0.1511687595129376</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2367082903413673</v>
+        <v>0.2373359161143793</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>16.89920556107249</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.84077342420278</v>
+        <v>20.85969755197966</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.263891840907357</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1891277153156355</v>
+        <v>-0.1898633468216948</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.3042680008145242</v>
+        <v>0.3049741658056075</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>19.96190476190476</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.56022348728764</v>
+        <v>22.5721388492206</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.488069554455446</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1151725614263971</v>
+        <v>-0.1156396434007392</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.186322533399665</v>
+        <v>0.1867508259733222</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>29.42767295597483</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.04222654675353</v>
+        <v>17.02022952446262</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>18.70324340114005</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7267504850521234</v>
+        <v>0.7289821452571721</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.992392935564365</v>
+        <v>0.9949470770639905</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>27.05611296915645</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>21.84634935909594</v>
+        <v>21.84126237540952</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>8.126134826530791</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2384729606043485</v>
+        <v>0.2387614096709989</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2843621815581034</v>
+        <v>0.284980965184829</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>314.0593220338983</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>174.4853752506838</v>
+        <v>175.4100547120006</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>14.12542843244965</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7999177385651266</v>
+        <v>0.790429417227769</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.129399336556381</v>
+        <v>0.1308952031679547</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>44.06203473945409</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.01832682853388</v>
+        <v>18.9970741427331</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>18.96218981414976</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.316819725347564</v>
+        <v>1.319411631938543</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8933135152237064</v>
+        <v>0.8954144784440283</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>33.32066594281579</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.03636686274647</v>
+        <v>40.02611342924497</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.346803741167855</v>
@@ -1754,10 +1754,10 @@
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1677400185424814</v>
+        <v>-0.1675268196669294</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.09149087184076876</v>
+        <v>0.09171491141588062</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1799,7 +1799,7 @@
         <v>-0.1680254288398988</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1780334448745784</v>
+        <v>0.1780334448745785</v>
       </c>
       <c r="AK10" s="5" t="n">
         <v>2053114789.885864</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>20.76160990712075</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>17.85358713525227</v>
+        <v>17.85085621266557</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>5.772780771728145</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1628817082997582</v>
+        <v>0.1630596123669368</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1489503391999123</v>
+        <v>0.1492768419716088</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.65232694931057</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.65801789655555</v>
+        <v>22.65798840312266</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.821871985328332</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4415960386705334</v>
+        <v>-0.4415953118076953</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06283450603239404</v>
+        <v>0.06287996838477183</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>14.28976784178848</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.23121441259915</v>
+        <v>13.23067393795742</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>2.992327913235427</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.08000425328920269</v>
+        <v>0.08004837159448286</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2860120708933945</v>
+        <v>-0.2859581534976812</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>30.3272926963207</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>24.73926850715404</v>
+        <v>24.72976496819714</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>13.80588608043782</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2258766942745591</v>
+        <v>0.2263477932492308</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1634269766205307</v>
+        <v>0.1637939156765229</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>23.91486078065719</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>16.92318738866425</v>
+        <v>16.91754347919033</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7503158069086862</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4131416400125791</v>
+        <v>0.4136130821873767</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01303677888992372</v>
+        <v>0.01311718008522811</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.10810810810811</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.32563412067245</v>
+        <v>14.26860233665699</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.882603679720822</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4734501754200384</v>
+        <v>0.4793395744080677</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1135807288891308</v>
+        <v>0.1134473474597095</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>29.59884393063583</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>20.82414835057152</v>
+        <v>20.81894085979369</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.300547247985786</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4213711616121625</v>
+        <v>0.4217266925330587</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.0927931659382244</v>
+        <v>0.09300206382958187</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2807,7 +2807,7 @@
         <v>-0.166112224755526</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.184555265208757</v>
+        <v>0.1845552652087571</v>
       </c>
       <c r="AK18" s="5" t="n">
         <v>1753868643.604533</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>37.63898916967509</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.49601233128282</v>
+        <v>33.48618372531821</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.127567706023048</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1236856733099252</v>
+        <v>0.1240154888482272</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05308176639691631</v>
+        <v>0.05320545600322202</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.46814814814815</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.45976788294378</v>
+        <v>20.45645946689671</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.958099860522566</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04928600710299325</v>
+        <v>0.04945570776255681</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02718330971115024</v>
+        <v>0.0272635347480128</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v>19.75209497206704</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>18.85402710287227</v>
+        <v>18.85250654688866</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1.667107293292193</v>
@@ -3140,7 +3140,7 @@
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.0476326815642456</v>
+        <v>0.04771717877094961</v>
       </c>
       <c r="V21" s="4" t="n">
         <v>0.01416228040029321</v>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>160.8908629441624</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.399470818286</v>
+        <v>45.32604738217059</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>25.02490366783682</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.543892914261873</v>
+        <v>2.549633648564077</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9479036686977758</v>
+        <v>0.9504554714666873</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>59.97822931785196</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.35445693150112</v>
+        <v>37.29483644772574</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>18.03399445539594</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.6056512192865573</v>
+        <v>0.6082180545802998</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.339390097152966</v>
+        <v>0.3409127564138461</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>72.49438202247188</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>71.83892179813952</v>
+        <v>71.48322031232634</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.627576117878611</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>0.009124026473756652</v>
+        <v>0.01414544148581354</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1592739976984785</v>
+        <v>0.1596944710258705</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>13.75015234613041</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.63317384445917</v>
+        <v>12.63119439827465</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.257658901956129</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.08841630103595377</v>
+        <v>0.08858686776355884</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3856799360090674</v>
+        <v>-0.3856347422544031</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>19.44454148471616</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.20333544136481</v>
+        <v>17.20028959551173</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.0356848164175</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1302774134114975</v>
+        <v>0.1304775641562483</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04793587002817756</v>
+        <v>0.0480433921755421</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>38.23519571763131</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>25.75279440123893</v>
+        <v>25.73643791348252</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.50979594568811</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4847008492325742</v>
+        <v>0.4856444332415204</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2405922671077951</v>
+        <v>0.2410602916704396</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
         <v>232.25</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>107.97</v>
+        <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
         <v>300172156800</v>
@@ -4000,7 +4000,7 @@
         <v>15.29823151125402</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.11361365170655</v>
+        <v>14.11114666591346</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.372358564439773</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08393441175175087</v>
+        <v>0.08412391093688054</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3266710464831442</v>
+        <v>-0.3265664528255312</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>14.27287212853539</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.156758758247687</v>
+        <v>6.153523367181669</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>9.114710162326936</v>
@@ -4138,10 +4138,10 @@
         <v>0.01613766949206263</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>10.7878074865186</v>
+        <v>10.79229519330957</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>8.861864560621077</v>
+        <v>8.86555107892603</v>
       </c>
       <c r="S29" s="4" t="n">
         <v>0.04358262498639762</v>
@@ -4150,10 +4150,10 @@
         <v>2.563272513243084</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>1.318244499902685</v>
+        <v>1.319463383312446</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.066155043275526</v>
+        <v>1.067138005986326</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.4337631707914727</v>
@@ -4168,7 +4168,7 @@
         <v>0.7501201309427276</v>
       </c>
       <c r="AA29" s="5" t="n">
-        <v>89675000000</v>
+        <v>58963000000</v>
       </c>
       <c r="AB29" s="6" t="n">
         <v>3.313805399898115</v>
@@ -4177,13 +4177,13 @@
         <v>2.936394731096718</v>
       </c>
       <c r="AD29" s="6" t="n">
-        <v>0.03387821763575135</v>
+        <v>0.03742646952550261</v>
       </c>
       <c r="AE29" s="6" t="n">
-        <v>0.02393204279996733</v>
+        <v>0.02643857714612432</v>
       </c>
       <c r="AF29" s="6" t="n">
-        <v>-0.3077963623069189</v>
+        <v>-0.3033086555159492</v>
       </c>
       <c r="AG29" s="6" t="n">
         <v>942.5188679245283</v>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>83.46583850931678</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.07504164703675</v>
+        <v>28.05987711999563</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.43051693999457</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.972955109333788</v>
+        <v>1.974561796988004</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.256247603500162</v>
+        <v>0.2568125021792091</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.73361522198732</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.534630356278514</v>
+        <v>9.535328419987623</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.487509922130118</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.852652263314895</v>
+        <v>2.852370217787947</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05224180804050416</v>
+        <v>-0.05234861553023273</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>8.043852233604305</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004494530107998797</v>
+        <v>0.004497064964814552</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.908276184073303</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1788.698153159298</v>
+        <v>1787.689355510792</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2378.499116531139</v>
+        <v>2378.052114203247</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-93.50588235294117</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>117.6741167403561</v>
+        <v>117.255567681177</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>126.3873418214006</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.534087932662793</v>
+        <v>4.544667416363497</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.03021735747263578</v>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
         <v>28.97878752752985</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.7140361805050256</v>
+        <v>0.7134948287703539</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.59995874331043</v>
@@ -4944,10 +4944,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>39.58448061698169</v>
+        <v>39.6152733825307</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>39.63284482563324</v>
+        <v>39.66718435954637</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5004,7 +5004,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5048,7 @@
         <v>-24.36220472440945</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-112.1139516391971</v>
+        <v>-113.4013240534189</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>2.147883415755226</v>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02187871540880648</v>
+        <v>0.02195269435247749</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
         <v>18.36143117040631</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.50246610586962</v>
+        <v>15.4969997143771</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.432057400116566</v>
@@ -5200,10 +5200,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1844200171129038</v>
+        <v>0.1848378078868889</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.009584754252444316</v>
+        <v>0.009817440107545261</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5258,7 +5258,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
         <v>21.95987654320988</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.59588223908579</v>
+        <v>15.58239910816217</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>5.710615949398833</v>
@@ -5326,10 +5326,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4080560629122274</v>
+        <v>0.409274424995772</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4555485306425668</v>
+        <v>0.4571130883404291</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5384,7 +5384,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
         <v>33.39285714285715</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>21.63952663793074</v>
+        <v>21.63443099645063</v>
       </c>
       <c r="N40" s="6" t="n">
         <v>6.98348155409396</v>
@@ -5452,10 +5452,10 @@
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5431417563600782</v>
+        <v>0.5435052185257663</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1670295940091615</v>
+        <v>0.1672470798350325</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5510,7 +5510,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
         <v>11.47646219686163</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.27552203924642</v>
+        <v>10.2730255449039</v>
       </c>
       <c r="N41" s="6" t="n">
         <v>1.884363889857093</v>
@@ -5578,10 +5578,10 @@
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1168738827115863</v>
+        <v>0.1171452992789166</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2882789051785076</v>
+        <v>-0.2881927399867689</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5636,7 +5636,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:27 ET</t>
+          <t>2026-10-04 12:12 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-10-05)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>333.69</v>
+        <v>332.89</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2312829341195992</v>
+        <v>0.2283310136326333</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.03373486998320485</v>
+        <v>-0.03605142757861812</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>345.34</v>
@@ -714,31 +714,31 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4901023823640</v>
+        <v>4889273938840</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.09246575342466</v>
+        <v>38.00114155251141</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.72978233130519</v>
+        <v>34.64651994446398</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.4986768510549</v>
+        <v>10.47350695839751</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.59844987304688</v>
+        <v>45.48913056501117</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.163936453576863</v>
+        <v>1.161145991882292</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.35428951746733</v>
+        <v>29.28455146920219</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.59456544266242</v>
+        <v>10.56939555000503</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02788866263834753</v>
+        <v>0.02795568456784579</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003176601036890527</v>
+        <v>0.00318423503259335</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3077125615899974</v>
+        <v>0.3062230826324607</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2043191108382786</v>
+        <v>0.2043876846169409</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13326888489.19373</v>
+        <v>13224435610.94145</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>517.53</v>
+        <v>525.1799999999999</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.09428256719332606</v>
+        <v>0.1104579804815007</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.06535794264249084</v>
+        <v>-0.05154229574514213</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3842944891500</v>
+        <v>3899750349000</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.75166666666667</v>
+        <v>29.17666666666666</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.97606578450893</v>
+        <v>25.33269491492575</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.58075118204913</v>
+        <v>11.75193497147713</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.6908755682242</v>
+        <v>8.819341933646331</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.9132489945862319</v>
+        <v>0.926748414539828</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>19.0383443997899</v>
+        <v>19.31208057575451</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.90582840323169</v>
+        <v>12.07701219265969</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01743116331128372</v>
+        <v>0.01717725341499803</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1511687595129376</v>
+        <v>0.1517395509893456</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2373359161143793</v>
+        <v>0.2379635418873909</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007033408691283598</v>
+        <v>0.00693095700521726</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5573272488331004</v>
+        <v>0.5599944147792565</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.2238603879860033</v>
+        <v>0.2241475897157378</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10885893929.01479</v>
+        <v>10983486115.98458</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>343.5</v>
+        <v>346.47</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.08995718436481259</v>
+        <v>0.09938126831696259</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1593450967915616</v>
+        <v>-0.1520765522136022</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4157075226741</v>
+        <v>4193018497260</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.89920556107249</v>
+        <v>17.07199602780536</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.85969755197966</v>
+        <v>21.05917895637294</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.263891840907357</v>
+        <v>9.358612991506417</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.457021062328255</v>
+        <v>6.523042608668499</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1502856179352413</v>
+        <v>0.1518222536056237</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.91324167819431</v>
+        <v>13.04348413660166</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.391385303068635</v>
+        <v>9.486106453667695</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01289761242878234</v>
+        <v>0.01276707207089557</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1898633468216948</v>
+        <v>-0.1893323066786027</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.3049741658056075</v>
+        <v>0.3077236544566671</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002503639010189229</v>
+        <v>0.002482177389095737</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7626342821504202</v>
+        <v>0.7628946847043234</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.2527090373726006</v>
+        <v>0.2343807526217414</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8962545782.29126</v>
+        <v>9011340087.929232</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>251.52</v>
+        <v>251.4</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1104635761589405</v>
+        <v>0.1099337748344371</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.124233983286908</v>
+        <v>-0.1246518105849581</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2705625792000</v>
+        <v>2704334940000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>19.96190476190476</v>
+        <v>19.95238095238095</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.5721388492206</v>
+        <v>22.57329196315899</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.488069554455446</v>
+        <v>3.486405399133663</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.904370980022479</v>
+        <v>4.902031108371705</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2259647087261301</v>
+        <v>0.225856901136089</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.22314354893956</v>
+        <v>11.21806139442592</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.675026804867987</v>
+        <v>3.673362649546205</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004296603038887648</v>
+        <v>-0.004298653923393084</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1156396434007392</v>
+        <v>-0.1161067253750815</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1867508259733222</v>
+        <v>0.1871791185469789</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8357984321047139</v>
+        <v>0.8339322282519522</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.2365027694000736</v>
+        <v>0.233512964243589</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8715845460.178579</v>
+        <v>8724807454.709829</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -1205,55 +1205,55 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>233.95</v>
+        <v>238.9</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.238813833406833</v>
+        <v>0.2650251113523934</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.01652093492517237</v>
+        <v>-0.004990872488476517</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>237.88</v>
+        <v>240.0983</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5666502950000</v>
+        <v>5786396900000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>29.42767295597483</v>
+        <v>30.0503144654088</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.02022952446262</v>
+        <v>17.35794525817428</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18.70324340114005</v>
+        <v>19.0989734923375</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>24.71461106452852</v>
+        <v>25.23753187995668</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2362221366534035</v>
+        <v>0.2412202113549822</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>24.32059276662943</v>
+        <v>24.83369025151177</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.7574304631827</v>
+        <v>19.15316055438015</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02241347108096008</v>
+        <v>0.02194906471071834</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7289821452571721</v>
+        <v>0.7312138054622206</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9949470770639905</v>
+        <v>0.9975012185636154</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002222697157512289</v>
+        <v>0.002176642946839682</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.296333349165572</v>
+        <v>1.297998671862829</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.3608323955500798</v>
+        <v>0.3552901619867762</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27796943015.65257</v>
+        <v>28095743849.35992</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>728.08</v>
+        <v>741.9</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.1194170293545134</v>
+        <v>0.1406651660231204</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.0663486445590008</v>
+        <v>-0.04862660613987857</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>779.8200000000001</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1854774021886</v>
+        <v>1889980286283</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>27.05611296915645</v>
+        <v>27.56967670011148</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>21.84126237540952</v>
+        <v>22.25065965319557</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.126134826530791</v>
+        <v>8.280380490882724</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.087896608618756</v>
+        <v>7.222435026280429</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.546503158677067</v>
+        <v>-5.651783723522849</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>18.22726783739913</v>
+        <v>18.55607709095749</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.550480275340858</v>
+        <v>8.704725939692791</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02209217916387148</v>
+        <v>0.021680649421263</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2387614096709989</v>
+        <v>0.2390498587376491</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.284980965184829</v>
+        <v>0.2855997488115547</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.002884298428744094</v>
+        <v>0.002830570157703195</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8401949314511553</v>
+        <v>0.8418095609082045</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4410630741729306</v>
+        <v>0.442227340370012</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>14260191925.07039</v>
+        <v>14371731718.12439</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>370.59</v>
+        <v>378.73</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1540393229301278</v>
+        <v>-0.1354578180019085</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2570815708758495</v>
+        <v>-0.2407633863239981</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1463662768742</v>
+        <v>1495812084530</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>314.0593220338983</v>
+        <v>320.9576271186441</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>175.4100547120006</v>
+        <v>176.5122845949596</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14.12542843244965</v>
+        <v>14.4356931115915</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.81104596007276</v>
+        <v>14.11440523613254</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.360170685127711</v>
+        <v>-8.543801623299114</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>121.1993489143665</v>
+        <v>123.8722218598271</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>14.06871103506114</v>
+        <v>14.37897571420299</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.003936699165308664</v>
+        <v>0.003852088146359963</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.790429417227769</v>
+        <v>0.8183302530763872</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1308952031679547</v>
+        <v>0.1319383062031652</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.530193213701677</v>
+        <v>1.536072125235094</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.4154194997610596</v>
+        <v>0.4145394575207418</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>14241949087.56693</v>
+        <v>14055916580.71307</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>355.14</v>
+        <v>362.51</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.02163283179460773</v>
+        <v>0.04283414386963802</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2825454545454545</v>
+        <v>-0.2676565656565657</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1689606961200</v>
+        <v>1724670325800</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>44.06203473945409</v>
+        <v>44.97642679900744</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>18.9970741427331</v>
+        <v>19.36966333285181</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18.96218981414976</v>
+        <v>19.35570037035374</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.97860607884442</v>
+        <v>17.33095255291403</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4384390585460529</v>
+        <v>0.4475377122079451</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>33.00711710387846</v>
+        <v>33.67801935977651</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.35997218082241</v>
+        <v>19.7534827370264</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.023320808273668</v>
+        <v>0.02284668519574757</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.319411631938543</v>
+        <v>1.322003538529522</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8954144784440283</v>
+        <v>0.8975154416643503</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007321056484766572</v>
+        <v>0.007172215938870652</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.598741738467171</v>
+        <v>1.599598061922649</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3427865039122595</v>
+        <v>0.3478554888596226</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8984006560.68634</v>
+        <v>9008274438.345057</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>920.65</v>
+        <v>923.52</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.07741369221767114</v>
+        <v>0.08077238150965482</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.160373917008664</v>
+        <v>-0.1577564979480164</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>408288941350</v>
+        <v>409561726080</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>33.32066594281579</v>
+        <v>33.42453854505973</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.02611342924497</v>
+        <v>40.14060921331039</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.346803741167855</v>
+        <v>1.351002216959037</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.41651771499595</v>
+        <v>11.45210714185962</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>0.6482965388660852</v>
+        <v>0.6503175143361831</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.6243430148339</v>
+        <v>27.71298322167282</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.308437102429788</v>
+        <v>1.31263557822097</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02299841864183765</v>
+        <v>0.02292694703158333</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1675268196669294</v>
+        <v>-0.1673136207913769</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.09171491141588062</v>
+        <v>0.09193895099099247</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1793,16 +1793,16 @@
         <v>80.58620689655173</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.006017487644598925</v>
+        <v>0.005998787248787249</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1680254288398988</v>
+        <v>-0.1671570464253578</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1780334448745785</v>
+        <v>0.1777237822791485</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2053114789.885864</v>
+        <v>2038392417.119718</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -1835,55 +1835,55 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>67.06</v>
+        <v>67.5</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2629959163159624</v>
+        <v>-0.2581602199720767</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.4629184686849271</v>
+        <v>-0.4967193558007754</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>124.86</v>
+        <v>134.12</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>279233816333</v>
+        <v>281065949933</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>20.76160990712075</v>
+        <v>20.89783281733746</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>17.85085621266557</v>
+        <v>17.96523282828722</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5.772780771728145</v>
+        <v>5.810657651241565</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.317265013339723</v>
+        <v>9.378398276177025</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6101887789775733</v>
+        <v>0.6141924035339427</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.296451843900707</v>
+        <v>9.356331287133086</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>5.880491991670837</v>
+        <v>5.918368871184255</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03937419953064851</v>
+        <v>0.03911753808179495</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1630596123669368</v>
+        <v>0.1632375164341151</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1492768419716088</v>
+        <v>0.1496033447433052</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1064516977890281</v>
+        <v>0.1083430508822622</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3555075668048129</v>
+        <v>0.3551720408742266</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2422396161.935526</v>
+        <v>2440523236.437602</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>502.65</v>
+        <v>504.26</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01167353089510881</v>
+        <v>0.01491394546735814</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.06525458399970252</v>
+        <v>-0.06226057202365454</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1084142459527</v>
+        <v>1087614993815</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.65232694931057</v>
+        <v>12.67891260961556</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.65798840312266</v>
+        <v>22.73053289533251</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.821871985328332</v>
+        <v>2.827801434537689</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.444830273388814</v>
+        <v>1.447866218239162</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3485393869907546</v>
+        <v>0.349271754229016</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.34749808427216</v>
+        <v>15.37730938714484</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.052607622352718</v>
+        <v>3.058537071562075</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02230692233520501</v>
+        <v>0.02226014827200941</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4415953118076953</v>
+        <v>-0.4422078590062861</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06287996838477183</v>
+        <v>0.06175806276693296</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02512494823908186</v>
+        <v>0.02618883219267291</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1348785802685299</v>
+        <v>0.1348876056111173</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2286357423.364156</v>
+        <v>2268606657.845821</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>14.28976784178848</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.23067393795742</v>
+        <v>13.22351115075698</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>2.992327913235427</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.08004837159448286</v>
+        <v>0.08063340204242686</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2859581534976812</v>
+        <v>-0.2859042361019679</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2174,13 +2174,13 @@
         <v>0.01805162765509357</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.782125038505104</v>
+        <v>0.780306905241485</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1626722303349957</v>
+        <v>0.1619101237589091</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2591247550.349528</v>
+        <v>2555214514.393022</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>360.66</v>
+        <v>369.71</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.04092585016176131</v>
+        <v>0.06704568309018111</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.06460564877972863</v>
+        <v>-0.04113390564618624</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,37 +2228,37 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>673369247119</v>
+        <v>690266024379</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>30.64231096006797</v>
+        <v>31.41121495327102</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.00813185101459</v>
+        <v>24.60786232216857</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.13597480486873</v>
+        <v>15.51578008404514</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>19.61752338563875</v>
+        <v>20.10978364915572</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.066340048294058</v>
+        <v>2.118190482046238</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.53660894628497</v>
+        <v>24.11729412258574</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.39444900015735</v>
+        <v>15.77425427933375</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03120576131135153</v>
+        <v>0.03044188654498012</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2763305012744264</v>
+        <v>0.2764706881903143</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>0.1424590110366841</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007430821272112239</v>
+        <v>0.007248924832977199</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.2943031843606881</v>
+        <v>0.3025519909360619</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1792858342637725</v>
+        <v>0.1896176699762527</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2277374055.281576</v>
+        <v>2250640022.281311</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>552.26</v>
+        <v>564.59</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-0.01930283378360309</v>
+        <v>0.002592643092231173</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.08144969479234243</v>
+        <v>-0.06094173610764597</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>484351901360</v>
+        <v>495165755240</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>30.3272926963207</v>
+        <v>31.00439319055464</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>24.72976496819714</v>
+        <v>25.27218433549859</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>13.80588608043782</v>
+        <v>14.11412237379928</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>86.81042951345572</v>
+        <v>88.74859739796828</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.340358025417745</v>
+        <v>1.370283449046834</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>22.50424585639356</v>
+        <v>22.99320651293181</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.18646926887666</v>
+        <v>14.49470556223812</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03395878070018112</v>
+        <v>0.03321715976103372</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2263477932492308</v>
+        <v>0.2268188922239023</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1637939156765229</v>
+        <v>0.1641608547325148</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.00610219823995944</v>
+        <v>0.005968933208168759</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2901665804490863</v>
+        <v>0.2975368089026829</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1761412792400913</v>
+        <v>0.1848354848168007</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1584446418.891195</v>
+        <v>1587113364.765224</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>371.9</v>
+        <v>378.58</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1055291520440382</v>
+        <v>0.1253864651272707</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1943589965772714</v>
+        <v>-0.1798882197478446</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>337738903848</v>
+        <v>343805308466</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>23.91486078065719</v>
+        <v>24.34441515015112</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>16.91754347919033</v>
+        <v>17.21567185747381</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7503158069086862</v>
+        <v>0.7637928426428867</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.422555124076914</v>
+        <v>3.484030435259581</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7246265257428895</v>
+        <v>-0.7376421352937433</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>14.84617101455576</v>
+        <v>15.08164066552808</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8497162010179303</v>
+        <v>0.863193236752131</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06992679768579126</v>
+        <v>0.06869294748639856</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4136130821873767</v>
+        <v>0.414084524362174</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01311718008522811</v>
+        <v>0.01319758128053206</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02436138746974994</v>
+        <v>0.02393153362565376</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4406443709033275</v>
+        <v>0.4459285900293961</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.1956266165552836</v>
+        <v>0.1984014911807933</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1817665616.513062</v>
+        <v>1824761635.629409</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>164.01</v>
+        <v>164.02</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3372197143054598</v>
+        <v>0.3373012471214043</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.07029079984127884</v>
+        <v>-0.07023411371237454</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>679732884600</v>
+        <v>679774329200</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.10810810810811</v>
+        <v>21.10939510939511</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.26860233665699</v>
+        <v>14.23194144714753</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.882603679720822</v>
+        <v>1.882718465628981</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.639190772264631</v>
+        <v>2.639351688719254</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.066835585585587</v>
+        <v>2.066961604461606</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.906200969021929</v>
+        <v>9.906777990950227</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.970622291585886</v>
+        <v>1.970737077494045</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04494853889256721</v>
+        <v>0.04494579846219942</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4793395744080677</v>
+        <v>0.4832407221311332</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1134473474597095</v>
+        <v>0.1133139660302882</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02512041948661667</v>
+        <v>0.02511888794049506</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5489003382477062</v>
+        <v>-0.5483235866955304</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2523323921237285</v>
+        <v>0.2488523261859908</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2272752630.84844</v>
+        <v>2262086423.857214</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>256.03</v>
+        <v>252.93</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2347720880807775</v>
+        <v>0.2198215218461552</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.08908812751271933</v>
+        <v>-0.1001174084747571</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>182.94</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>617006291448</v>
+        <v>609535606359</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>29.59884393063583</v>
+        <v>29.24046242774567</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>20.81894085979369</v>
+        <v>20.56172417142406</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.300547247985786</v>
+        <v>6.22426049851423</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.352376728530909</v>
+        <v>7.263354473879323</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.664804228780048</v>
+        <v>-3.620430940066936</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.13969795588758</v>
+        <v>18.91822620535396</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.592738529424379</v>
+        <v>6.516451779952823</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.03032059844332506</v>
+        <v>0.03069221847719507</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4217266925330587</v>
+        <v>0.4220822234539554</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09300206382958187</v>
+        <v>0.09321096172093912</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.02062258329102059</v>
+        <v>0.02087534100343969</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.166112224755526</v>
+        <v>-0.1705593645121297</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1845552652087571</v>
+        <v>0.1851065406483072</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1753868643.604533</v>
+        <v>1774367434.11205</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>104.26</v>
+        <v>105.07</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.07538135841786542</v>
+        <v>-0.06819796018573887</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2286179343000887</v>
+        <v>-0.2226250369931932</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>829709420800</v>
+        <v>836155465600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>37.63898916967509</v>
+        <v>37.93140794223827</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.48618372531821</v>
+        <v>33.73644003692851</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.127567706023048</v>
+        <v>1.136327823439878</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.4415810582463</v>
+        <v>8.507164030212341</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.101791926485074</v>
+        <v>9.172504102395806</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>20.82064055650225</v>
+        <v>20.97111196806648</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.212132285279409</v>
+        <v>1.220892402696238</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01628160372938121</v>
+        <v>0.01615608646450256</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1240154888482272</v>
+        <v>0.124345304386529</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05320545600322202</v>
+        <v>0.05332914560952795</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009375599462881258</v>
+        <v>0.009303321595127059</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.04276608151476034</v>
+        <v>-0.03997715754408303</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3090152315932373</v>
+        <v>0.3091372774375272</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2614601902.107239</v>
+        <v>2528180255.535717</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>144.91</v>
+        <v>145.94</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.0220044210565058</v>
+        <v>0.02926868545294625</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1335724962630792</v>
+        <v>-0.1274140508221225</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>344481347061</v>
+        <v>346929872266</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.46814814814815</v>
+        <v>21.62074074074074</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.45645946689671</v>
+        <v>20.59853026351823</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.958099860522566</v>
+        <v>3.986233480398015</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.463598074054979</v>
+        <v>6.509540424591703</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.4867470899473</v>
+        <v>20.63236402116424</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.38803740759386</v>
+        <v>17.50324043784699</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.246315689183289</v>
+        <v>4.274449309058737</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04619408317972631</v>
+        <v>0.0458680594324812</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04945570776255681</v>
+        <v>0.04962540842212082</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.0272635347480128</v>
+        <v>0.02734375978487513</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02960872265544131</v>
+        <v>0.02939975332328354</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.03546233801581527</v>
+        <v>-0.03279234046625135</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1477048353764854</v>
+        <v>0.1475513773023727</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1174667535.249634</v>
+        <v>1161688220.001583</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>282.85</v>
+        <v>281.15</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1820889653304011</v>
+        <v>-0.1870048174037204</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2886603123506777</v>
+        <v>-0.2929356436888565</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>397.63</v>
@@ -3110,31 +3110,31 @@
         <v>277.15</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>282034543450</v>
+        <v>280339444550</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>19.75209497206704</v>
+        <v>19.63337988826815</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>18.85250654688866</v>
+        <v>18.73919821692679</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.667107293292193</v>
+        <v>1.657087557041188</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>16.91959439128603</v>
+        <v>16.81790335198892</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-6.775427926464886</v>
+        <v>-6.734705891905965</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14.32224726949613</v>
+        <v>14.25136711478152</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.024616632678394</v>
+        <v>2.014596896427389</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05354308665625264</v>
+        <v>0.05386683998122375</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03284426374403394</v>
+        <v>0.033042859683443</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7134102446323061</v>
+        <v>0.7101562422204377</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2112150781700568</v>
+        <v>0.2058133877973638</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1394353830.82784</v>
+        <v>1395990288.477343</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>633.91</v>
+        <v>631.75</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.836667098658753</v>
+        <v>1.827001371768338</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.01789421497846511</v>
+        <v>-0.02124066557184034</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>645.46</v>
@@ -3236,40 +3236,40 @@
         <v>188.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>1033653646000</v>
+        <v>1030131550000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>160.8908629441624</v>
+        <v>160.3426395939086</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.32604738217059</v>
+        <v>45.098665380112</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>25.02490366783682</v>
+        <v>24.93963321631764</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>15.38003109008687</v>
+        <v>15.32762480661668</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.298935407255623</v>
+        <v>1.294509383877427</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>96.36533364433663</v>
+        <v>96.0367186042172</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>25.00529345115604</v>
+        <v>24.92002299963685</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.008129415527645708</v>
+        <v>0.008157210600917912</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.549633648564077</v>
+        <v>2.555374382866281</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9504554714666873</v>
+        <v>0.9530072742355977</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.583796341276141</v>
+        <v>2.576437009299936</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.532768801593928</v>
+        <v>0.4963026772194564</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10954613474.22119</v>
+        <v>11014892081.08786</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1867.31</v>
+        <v>1859.86</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.604521432738607</v>
+        <v>0.5981198793415263</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.06632632652653059</v>
+        <v>-0.07005140102802065</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>719694868774</v>
+        <v>716823504741</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>59.97822931785196</v>
+        <v>60.09433962264151</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.29483644772574</v>
+        <v>37.05328524314731</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>18.03399445539594</v>
+        <v>18.06890599940556</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>29.1892107361148</v>
+        <v>29.24571737516838</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>4.08293725356369</v>
+        <v>4.09084130632316</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>45.81175986982505</v>
+        <v>45.90110302394147</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>17.90130745518364</v>
+        <v>17.93621899919326</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01569920538776029</v>
+        <v>0.01566887242239819</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.6082180545802998</v>
+        <v>0.6218356679656478</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3409127564138461</v>
+        <v>0.352027069356613</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004166421215545357</v>
+        <v>0.00418311055670857</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.64602439098886</v>
+        <v>1.640809670201554</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.3676876579045484</v>
+        <v>0.3639048581074436</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2167307401.616211</v>
+        <v>2196041211.50776</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>193.56</v>
+        <v>192.72</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1501953884653686</v>
+        <v>-0.1538833192035847</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2390013760566149</v>
+        <v>-0.2423039119323767</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>152984017200</v>
+        <v>152320106400</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>72.49438202247188</v>
+        <v>72.17977528089885</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>71.48322031232634</v>
+        <v>70.82233377263448</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.627576117878611</v>
+        <v>1.620512861322411</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>25.10075849878033</v>
+        <v>24.99182774274098</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.387995274091711</v>
+        <v>0.3863114756300607</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>27.57338376978417</v>
+        <v>27.47785703597122</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.038778841427735</v>
+        <v>2.031715584871536</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001372692414825671</v>
+        <v>-0.001378675507542844</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>0.01414544148581354</v>
+        <v>0.01916685649787042</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1596944710258705</v>
+        <v>0.1601149443639016</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.256519670019414</v>
+        <v>1.252319545467326</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.2976674614795599</v>
+        <v>0.2944072639186791</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1490290186.701609</v>
+        <v>1486790165.699441</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>902.5599999999999</v>
+        <v>893.46</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>-0.0128836390286684</v>
+        <v>-0.0228361728046379</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.2178788377715579</v>
+        <v>-0.2257645213563375</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>266261517920</v>
+        <v>263576954220</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>13.75015234613041</v>
+        <v>13.61151736745887</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.63119439827465</v>
+        <v>12.52755682656454</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.257658901956129</v>
+        <v>2.234896209162519</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.206728389630281</v>
+        <v>2.184479200273745</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3222845183114924</v>
+        <v>0.3190351065088038</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.14817054502596</v>
+        <v>26.06265582199854</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>6.960237397254466</v>
+        <v>6.937474704460856</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.155918137642682</v>
+        <v>-0.157506183053275</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.08858686776355884</v>
+        <v>0.08652609250957899</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3856347422544031</v>
+        <v>-0.3855895484997388</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01994327246942032</v>
+        <v>0.02014639715264253</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.593599860345509</v>
+        <v>1.58628654557469</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.2579039776544408</v>
+        <v>0.2569593001747523</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1999831319.048055</v>
+        <v>1961241579.969781</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>222.64</v>
+        <v>221.58</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2362264150943396</v>
+        <v>-0.2398627787307032</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3303254526860374</v>
+        <v>-0.333513806172171</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>209756713760</v>
+        <v>208758051720</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>19.44454148471616</v>
+        <v>19.35196506550218</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.20028959551173</v>
+        <v>17.11536789879743</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.0356848164175</v>
+        <v>3.021231771567507</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.073938697318008</v>
+        <v>6.045020376175549</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2370274533698928</v>
+        <v>0.2358989539961411</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>16.51295935885581</v>
+        <v>16.45139336169164</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.876531741754345</v>
+        <v>3.862078696904352</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06498480909457971</v>
+        <v>0.06529568506551686</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1304775641562483</v>
+        <v>0.130677714900999</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.0480433921755421</v>
+        <v>0.04815091432290641</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.03027308659719727</v>
+        <v>0.03041790775340735</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8980446870703808</v>
+        <v>0.8945836124477378</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.2972153427664984</v>
+        <v>0.2971079409963645</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1256909083.906606</v>
+        <v>1272958322.921071</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1142.85</v>
+        <v>1143.12</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.05784184484406119</v>
+        <v>0.058091761541885</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1158859706803854</v>
+        <v>-0.1156770974355008</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>783.85</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1076268701850</v>
+        <v>1076522971920</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.23519571763131</v>
+        <v>38.24422883907661</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>25.73643791348252</v>
+        <v>25.72617860179689</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.50979594568811</v>
+        <v>13.51298765492846</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.10358452138492</v>
+        <v>30.1106965376782</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4041931219702801</v>
+        <v>0.4042886131921657</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>25.91598857055107</v>
+        <v>25.92186020764442</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.08743402878023</v>
+        <v>14.09062573802058</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01863280049445767</v>
+        <v>0.01862839950756785</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4856444332415204</v>
+        <v>0.4865880172504664</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2410602916704396</v>
+        <v>0.2415283162330844</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3937,16 +3937,16 @@
         <v>37.33936879165095</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005853786586166164</v>
+        <v>0.005852403947092169</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3179878922120574</v>
+        <v>0.3168426369667163</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.2911618053174975</v>
+        <v>0.2663851431851464</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2724107353.463949</v>
+        <v>2694881208.867427</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>190.31</v>
+        <v>190.19</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.04623422971801516</v>
+        <v>0.04557452656228955</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.1805812701829924</v>
+        <v>-0.1810979547900969</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>151.84</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>300172156800</v>
+        <v>299982883200</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>15.29823151125402</v>
+        <v>15.28858520900322</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.11114666591346</v>
+        <v>14.102701535104</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.372358564439773</v>
+        <v>2.370862673379226</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.707708142767871</v>
+        <v>2.706000796978726</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.389211417081192</v>
+        <v>0.3889659997618197</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>22.64674947354074</v>
+        <v>22.64029996933247</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.252662684443883</v>
+        <v>5.251166793383335</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.0522500160148098</v>
+        <v>-0.05228298305788135</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08412391093688054</v>
+        <v>0.08408911377351003</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3265664528255312</v>
+        <v>-0.3264618591679181</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.02180652619410436</v>
+        <v>0.02182028497817972</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.388979387405049</v>
+        <v>1.385425394784406</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2247928906658313</v>
+        <v>0.2238092465301521</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1019891354.793447</v>
+        <v>1014485525.113043</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>1074.89</v>
+        <v>1063.96</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.407805320654668</v>
+        <v>2.37315311237777</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1435139442231075</v>
+        <v>-0.1522231075697211</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,40 +4120,40 @@
         <v>179.61</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1213970017100</v>
+        <v>1201625784400</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>14.27287212853539</v>
+        <v>14.12773868012216</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.153523367181669</v>
+        <v>6.019550265434241</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>9.114710162326936</v>
+        <v>9.022027392858217</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>8.777592536385843</v>
+        <v>8.688337741548512</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.01613766949206263</v>
+        <v>0.01597357388456024</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>10.79229519330957</v>
+        <v>10.67946974133991</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>8.86555107892603</v>
+        <v>8.772868309457309</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.04358262498639762</v>
+        <v>0.044030346790884</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>2.563272513243084</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>1.319463383312446</v>
+        <v>1.346975780108883</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.067138005986326</v>
+        <v>1.104774028100335</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.4337631707914727</v>
@@ -4189,16 +4189,16 @@
         <v>942.5188679245283</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0004930737098679865</v>
+        <v>0.0004981390277829994</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.834859283550031</v>
+        <v>2.827404797581972</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.4915022541449128</v>
+        <v>0.4927318589452093</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25532252576.97917</v>
+        <v>25463007573.82243</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>134.38</v>
+        <v>136.08</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.08864019816039748</v>
+        <v>-0.07711086594483463</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.3036223247136861</v>
+        <v>-0.2948126651811162</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>192.97</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>138930375560</v>
+        <v>140687940960</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>83.46583850931678</v>
+        <v>84.5217391304348</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.05987711999563</v>
+        <v>28.3995141963865</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.43051693999457</v>
+        <v>9.549819505837633</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.09096676254394</v>
+        <v>11.23127516778523</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>133.5453416149097</v>
+        <v>135.2347826086986</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>41.52489984522786</v>
+        <v>42.02864458584121</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>9.834399644311702</v>
+        <v>9.953702210154765</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03296615287721605</v>
+        <v>0.03255431822193042</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.974561796988004</v>
+        <v>1.976168484642219</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2568125021792091</v>
+        <v>0.2573774008582563</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6759201268917027</v>
+        <v>0.6791808288802959</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5370393532678653</v>
+        <v>0.5368216663377353</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>1906916088.305206</v>
+        <v>1885565812.847365</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.8</v>
+        <v>27.41</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1040508206143935</v>
+        <v>0.08856233787915557</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.04827114002054089</v>
+        <v>-0.06162273194111612</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.62</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>158444432000</v>
+        <v>156221650400</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.73361522198732</v>
+        <v>36.21828752642706</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.535328419987623</v>
+        <v>9.402247795685476</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.487509922130118</v>
+        <v>2.452613200200954</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.859751144500528</v>
+        <v>1.833661110458974</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6143940953058056</v>
+        <v>-0.605774897565904</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.47959695817491</v>
+        <v>17.30352110266159</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.464305953278071</v>
+        <v>3.429409231348907</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06933661133639585</v>
+        <v>0.07032315925398776</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.852370217787947</v>
+        <v>2.852088172260998</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05234861553023273</v>
+        <v>-0.05245542301996131</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.0618705035971223</v>
+        <v>0.06275082086829624</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3063910587600985</v>
+        <v>0.300653142743155</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.1953388323706219</v>
+        <v>0.196310438670456</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>926857018.7850889</v>
+        <v>921925909.049744</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>195.13</v>
+        <v>195.02</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.1614190011300822</v>
+        <v>0.1607642781755172</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.02371541501976293</v>
+        <v>-0.02426577275228892</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>199.87</v>
@@ -4498,13 +4498,13 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1385139848808</v>
+        <v>1384359008428</v>
       </c>
       <c r="L32" s="6" t="n">
         <v>8.043852233604305</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004497064964814552</v>
+        <v>0.004490535459339664</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.908276184073303</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1787.689355510792</v>
+        <v>1790.290216153233</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2378.052114203247</v>
+        <v>2381.773333670841</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,28 +4567,26 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.537436580741044</v>
-      </c>
-      <c r="AI32" s="6" t="inlineStr"/>
+        <v>1.538303763716542</v>
+      </c>
+      <c r="AI32" s="6" t="n">
+        <v>3.253007235326781</v>
+      </c>
       <c r="AJ32" s="4" t="n">
-        <v>0.6560713248816935</v>
+        <v>0.6526415180611447</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3187987916.814423</v>
+        <v>3183027552.931372</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
           <t>2026-10-27 (E)</t>
         </is>
       </c>
-      <c r="AM32" s="2" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
+      <c r="AM32" s="2" t="inlineStr"/>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4609,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>630.6</v>
+        <v>633.9</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.6892580247008453</v>
+        <v>0.6980980999966155</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.06136969173749318</v>
+        <v>-0.05645773484363614</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4624,7 @@
         <v>315.05</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>79481295689</v>
+        <v>79897230157</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4650,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.816574087056346</v>
+        <v>1.813866769877098</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.3073465589163391</v>
+        <v>0.3057736200990498</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3652328457.676798</v>
+        <v>3546228875.394332</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4666,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4689,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>158.96</v>
+        <v>171.09</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.01236406949968516</v>
+        <v>0.06300095212191037</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.2955149796135437</v>
+        <v>-0.2417567807126395</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4704,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>2095375740057</v>
+        <v>2255270730790</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-93.50588235294117</v>
+        <v>-100.6411764705882</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>117.255567681177</v>
+        <v>125.7558701518386</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>126.3873418214006</v>
+        <v>136.0317709626636</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>7.326773564736214</v>
+        <v>7.88586870401811</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>0.461321156041579</v>
+        <v>0.4965238839151594</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>574.343764788126</v>
+        <v>619.3339141221159</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>123.1206791758852</v>
+        <v>132.7651083171482</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01193580679678942</v>
+        <v>-0.01108957769838978</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.544667416363497</v>
+        <v>4.5552469000642</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.03021735747263578</v>
@@ -4776,13 +4774,13 @@
         <v>0</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <v>3.197675613882407</v>
+        <v>3.279602813511894</v>
       </c>
       <c r="AJ34" s="4" t="n">
-        <v>0.7258596652729258</v>
+        <v>0.6372956378194149</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12537749128.28888</v>
+        <v>12944539204.17569</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4796,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -4819,13 +4817,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>769.64</v>
+        <v>774.88</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1265717453239092</v>
+        <v>0.1342418715459057</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01248444256258263</v>
+        <v>-0.005761063423021184</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4834,7 +4832,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>819849948259</v>
+        <v>825431796563</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4860,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9960059598209436</v>
+        <v>0.9960528761662092</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.09036762064446385</v>
+        <v>0.09172704642134921</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32469748762.34253</v>
+        <v>32608291371.94629</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4876,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -4899,55 +4897,55 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>472.78</v>
+        <v>485.8</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.4792403919419306</v>
+        <v>0.5199775422086168</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.01298538622129441</v>
+        <v>-0.003364516658460492</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>479</v>
+        <v>487.44</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>266.82</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2452064014400</v>
+        <v>2519591984000</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.97878752752985</v>
+        <v>29.84815115335574</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.7134948287703539</v>
+        <v>0.7330616877901778</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.59995874331043</v>
+        <v>15.03795750560974</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>10.07761152009213</v>
+        <v>10.3799398656949</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5443796255588689</v>
+        <v>0.560711014325635</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>19.22947662230763</v>
+        <v>19.8261652951537</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>14.11537933183981</v>
+        <v>14.55337809413912</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01725206186855054</v>
+        <v>0.01674957462966072</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>39.6152733825307</v>
+        <v>39.7171069645357</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>39.66718435954637</v>
+        <v>39.77368483680704</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4981,16 +4979,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2538178433943906</v>
+        <v>0.2470152326060107</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.17798594784254</v>
+        <v>2.182310732562592</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.2540021808144101</v>
+        <v>0.2593148190334965</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4156301666.149394</v>
+        <v>4207553751.047943</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5004,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -5027,53 +5025,53 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>30.94</v>
+        <v>30.95</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.08523324277831734</v>
+        <v>0.08558399689686214</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.0009686793671294103</v>
+        <v>-0.001290738948047765</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>30.97</v>
+        <v>30.99</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>17.08</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>77570809560</v>
+        <v>77595880927</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-24.36220472440945</v>
+        <v>-24.37007874015748</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-113.4013240534189</v>
+        <v>-114.7556827211154</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.147883415755226</v>
+        <v>2.148577625003461</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.365866983372922</v>
+        <v>2.366631646263475</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1813001281816518</v>
+        <v>0.1813587255081487</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>17.55781976198347</v>
+        <v>17.56196378958678</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.941293356223176</v>
+        <v>2.941987565471411</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.02810335501673215</v>
+        <v>0.02809427477279216</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02195269435247749</v>
+        <v>0.02202667329614871</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5112,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2852111368464148</v>
+        <v>0.2850346966975765</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.274868551048402</v>
+        <v>0.2749599954111459</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>1191154992.248116</v>
+        <v>1623976462.528148</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -5155,13 +5153,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>302.78</v>
+        <v>304.01</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1876693824605766</v>
+        <v>-0.1843694067040091</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.2186120932153088</v>
+        <v>-0.2154378177501355</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5170,40 +5168,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>204470361800</v>
+        <v>205300993100</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>18.36143117040631</v>
+        <v>18.43602183141298</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.4969997143771</v>
+        <v>15.56064782601201</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.432057400116566</v>
+        <v>2.44193728188598</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>5.988472578763127</v>
+        <v>6.012799883313885</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.138569094409476</v>
+        <v>1.143194366838711</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>8.82852134767837</v>
+        <v>8.862117501213396</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.596271832811961</v>
+        <v>2.606151714581376</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.07361458094705636</v>
+        <v>0.07331674227541767</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1848378078868889</v>
+        <v>0.1847849805195345</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.009817440107545261</v>
+        <v>0.01005012596264576</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5239,16 +5237,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01169165730893718</v>
+        <v>0.01164435380415118</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9701464405544634</v>
+        <v>0.9695784172145332</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.1864841376668144</v>
+        <v>0.1857853558059747</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>940276214.402771</v>
+        <v>939630011.0632203</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5258,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -5281,13 +5279,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>142.3</v>
+        <v>142.55</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2729038111574638</v>
+        <v>-0.2716264109662435</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5588144106157376</v>
+        <v>-0.5580393129534321</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>322.54</v>
@@ -5296,40 +5294,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>409890881000</v>
+        <v>410610998500</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>21.95987654320988</v>
+        <v>21.99845679012346</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.58239910816217</v>
+        <v>15.59629158804511</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>5.710615949398833</v>
+        <v>5.720648654861585</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>6.320939914934404</v>
+        <v>6.332044869106811</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.4779502541757446</v>
+        <v>0.4787899419026872</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>14.0363966330859</v>
+        <v>14.05548776511135</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.376358457444586</v>
+        <v>7.386391162907338</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.07006742850666151</v>
+        <v>-0.06994454631005215</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.409274424995772</v>
+        <v>0.4104927870793167</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4571130883404291</v>
+        <v>0.4586776460382909</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5365,16 +5363,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.0140548137737175</v>
+        <v>0.01403016485443704</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.038236988172801</v>
+        <v>2.03506585768156</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.469622517849374</v>
+        <v>0.469127236293663</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4533255223.718211</v>
+        <v>4518167471.051721</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5384,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5405,13 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="3" t="n">
-        <v>112.2</v>
+        <v>112.82</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0.4755391721344495</v>
+        <v>0.4836927754029285</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>-0.1393725550356677</v>
+        <v>-0.1346168597069879</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>130.37</v>
@@ -5422,40 +5420,40 @@
         <v>66.81</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>442228969413</v>
+        <v>444672658905</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>33.39285714285715</v>
+        <v>33.57738095238095</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>21.63443099645063</v>
+        <v>21.74885815893526</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>6.98348155409396</v>
+        <v>7.022071202605606</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>8.820256537734911</v>
+        <v>8.868995923237547</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>1.068571428571429</v>
+        <v>1.07447619047619</v>
       </c>
       <c r="Q40" s="6" t="n">
-        <v>23.20515357475398</v>
+        <v>23.32722208426994</v>
       </c>
       <c r="R40" s="6" t="n">
-        <v>7.33587002626135</v>
+        <v>7.374459674772997</v>
       </c>
       <c r="S40" s="4" t="n">
-        <v>0.03074199326662283</v>
+        <v>0.0305730512720919</v>
       </c>
       <c r="T40" s="4" t="n">
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5435052185257663</v>
+        <v>0.5438686806914546</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1672470798350325</v>
+        <v>0.1674645656609037</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5491,16 +5489,16 @@
         <v>11.89047619047619</v>
       </c>
       <c r="AH40" s="4" t="n">
-        <v>0.01488413547237077</v>
+        <v>0.01480234001063641</v>
       </c>
       <c r="AI40" s="6" t="n">
-        <v>0.7031813612060062</v>
+        <v>0.70349627467822</v>
       </c>
       <c r="AJ40" s="4" t="n">
-        <v>0.3287439176769288</v>
+        <v>0.3292504072903227</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>1847504683.500061</v>
+        <v>1845855544.685794</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5510,7 +5508,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5531,13 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="n">
-        <v>80.45</v>
+        <v>81.44</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.1549369477003385</v>
+        <v>-0.1445377877031147</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-0.1770662847790507</v>
+        <v>-0.1669394435351883</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>97.76000000000001</v>
@@ -5548,40 +5546,40 @@
         <v>72.78</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>243280800000</v>
+        <v>246274560000</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>11.47646219686163</v>
+        <v>11.61768901569187</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.2730255449039</v>
+        <v>10.39899179847634</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>1.884363889857093</v>
+        <v>1.907552457302196</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>1.36152215578001</v>
+        <v>1.378276747877241</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0.6100101528061599</v>
+        <v>0.6175168035367764</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>15.06277504452024</v>
+        <v>15.15313633756904</v>
       </c>
       <c r="R41" s="6" t="n">
-        <v>3.86541807056272</v>
+        <v>3.888606638007823</v>
       </c>
       <c r="S41" s="4" t="n">
-        <v>0.07879783361448993</v>
+        <v>0.07783995228739826</v>
       </c>
       <c r="T41" s="4" t="n">
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1171452992789166</v>
+        <v>0.1171937857854728</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2881927399867689</v>
+        <v>-0.2879548508939894</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5617,16 +5615,16 @@
         <v>0.6326638212402712</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>0.02299564947172157</v>
+        <v>0.02271611001964637</v>
       </c>
       <c r="AI41" s="6" t="n">
-        <v>0.743557623481363</v>
+        <v>0.7463081266237687</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>0.225718041828961</v>
+        <v>0.2269070286678308</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1169156892.901154</v>
+        <v>1166611264.123555</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5636,7 +5634,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 12:12 ET</t>
+          <t>2026-10-05 17:13 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-10-06)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -790,7 +790,7 @@
         <v>0.2043876846169409</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13224435610.94145</v>
+        <v>13225047768.43221</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>29.17666666666666</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.33269491492575</v>
+        <v>25.32014648435197</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.75193497147713</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1517395509893456</v>
+        <v>0.1523103424657535</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2379635418873909</v>
+        <v>0.2385911676604024</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -920,7 +920,7 @@
         <v>0.2241475897157378</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>10983486115.98458</v>
+        <v>10988853687.27285</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.07199602780536</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>21.05917895637294</v>
+        <v>21.07833619460823</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.358612991506417</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1893323066786027</v>
+        <v>-0.1900690894107513</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.3077236544566671</v>
+        <v>0.308430924560235</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1046,7 +1046,7 @@
         <v>0.2343807526217414</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9011340087.929232</v>
+        <v>9018837945.942282</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>19.95238095238095</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.57329196315899</v>
+        <v>22.58522683430643</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.486405399133663</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1161067253750815</v>
+        <v>-0.1165738073494238</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1871791185469789</v>
+        <v>0.1876074111206358</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1172,7 +1172,7 @@
         <v>0.233512964243589</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8724807454.709829</v>
+        <v>8736446530.601196</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>30.0503144654088</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.35794525817428</v>
+        <v>17.33559841401834</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>19.0989734923375</v>
@@ -1238,7 +1238,7 @@
         <v>0.2412202113549822</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>24.83369025151177</v>
+        <v>24.80958853155703</v>
       </c>
       <c r="R6" s="6" t="n">
         <v>19.15316055438015</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7312138054622206</v>
+        <v>0.7334454656672695</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9975012185636154</v>
+        <v>1.000055360063241</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1283,7 +1283,7 @@
         <v>0.1213343657890793</v>
       </c>
       <c r="AF6" s="6" t="n">
-        <v>0.07025810234222205</v>
+        <v>0.07018991508974151</v>
       </c>
       <c r="AG6" s="6" t="n">
         <v>547.1389961389962</v>
@@ -1298,7 +1298,7 @@
         <v>0.3552901619867762</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>28095743849.35992</v>
+        <v>28099752724.30552</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>27.56967670011148</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>22.25065965319557</v>
+        <v>22.24548093648125</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>8.280380490882724</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2390498587376491</v>
+        <v>0.2393383078042994</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2855997488115547</v>
+        <v>0.2862185324382802</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1424,7 +1424,7 @@
         <v>0.442227340370012</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>14371731718.12439</v>
+        <v>14382633502.37874</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>320.9576271186441</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>176.5122845949596</v>
+        <v>176.3784436529894</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>14.4356931115915</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8183302530763872</v>
+        <v>0.8197100534014394</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1319383062031652</v>
+        <v>0.1323063458301601</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1550,7 +1550,7 @@
         <v>0.4145394575207418</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>14055916580.71307</v>
+        <v>14058340814.69645</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>44.97642679900744</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.36966333285181</v>
+        <v>19.34806630264046</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>19.35570037035374</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.322003538529522</v>
+        <v>1.3245954451205</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8975154416643503</v>
+        <v>0.8996164048846722</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1676,7 +1676,7 @@
         <v>0.3478554888596226</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9008274438.345057</v>
+        <v>9009515179.931335</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>33.42453854505973</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.14060921331039</v>
+        <v>40.13033434587927</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.351002216959037</v>
@@ -1754,10 +1754,10 @@
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>-0.1673136207913769</v>
+        <v>-0.1671004219158249</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.09193895099099247</v>
+        <v>0.09216299056610389</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1802,7 +1802,7 @@
         <v>0.1777237822791485</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2038392417.119718</v>
+        <v>2038491172.193807</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>20.89783281733746</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>17.96523282828722</v>
+        <v>17.96248566856109</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>5.810657651241565</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1632375164341151</v>
+        <v>0.1634154205012937</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1496033447433052</v>
+        <v>0.1499298475150013</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1928,7 +1928,7 @@
         <v>0.3551720408742266</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2440523236.437602</v>
+        <v>2442124513.164774</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.67891260961556</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.73053289533251</v>
+        <v>22.7305033075855</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.827801434537689</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422078590062861</v>
+        <v>-0.442207132941732</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06175806276693296</v>
+        <v>0.06180347518984974</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2054,7 +2054,7 @@
         <v>0.1348876056111173</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2268606657.845821</v>
+        <v>2269539656.524557</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>14.28976784178848</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.22351115075698</v>
+        <v>13.22306703179552</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>2.992327913235427</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.08063340204242686</v>
+        <v>0.08066969693400394</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2859042361019679</v>
+        <v>-0.2858503187062545</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.1619101237589091</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2555214514.393022</v>
+        <v>2555254156.248271</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
         <v>0.1896176699762527</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2250640022.281311</v>
+        <v>2250661465.460815</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.00439319055464</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.27218433549859</v>
+        <v>25.26248353111369</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.11412237379928</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2268188922239023</v>
+        <v>0.2272899911985737</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1641608547325148</v>
+        <v>0.164527793788507</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.1848354848168007</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1587113364.765224</v>
+        <v>1587118615.452474</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>24.34441515015112</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.21567185747381</v>
+        <v>17.20993423098671</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7637928426428867</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.414084524362174</v>
+        <v>0.4145559665369714</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01319758128053206</v>
+        <v>0.01327798247583623</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.1984014911807933</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1824761635.629409</v>
+        <v>1827699088.222554</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.10939510939511</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.23194144714753</v>
+        <v>14.23530031953235</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.882718465628981</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4832407221311332</v>
+        <v>0.4828907459318419</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1133139660302882</v>
+        <v>0.1131805846008669</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2488523261859908</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2262086423.857214</v>
+        <v>2262100921.457214</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>29.24046242774567</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>20.56172417142406</v>
+        <v>20.55658487537585</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.22426049851423</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4220822234539554</v>
+        <v>0.4224377543748514</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.09321096172093912</v>
+        <v>0.0934198596122966</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2810,7 +2810,7 @@
         <v>0.1851065406483072</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1774367434.11205</v>
+        <v>1782673899.570516</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>37.93140794223827</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.73644003692851</v>
+        <v>33.72654668912162</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.136327823439878</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.124345304386529</v>
+        <v>0.1246751199248308</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05332914560952795</v>
+        <v>0.05345283521583388</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2936,7 +2936,7 @@
         <v>0.3091372774375272</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2528180255.535717</v>
+        <v>2528326405.368601</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.62074074074074</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.59853026351823</v>
+        <v>20.5952004859821</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.986233480398015</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04962540842212082</v>
+        <v>0.04979510908168439</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02734375978487513</v>
+        <v>0.02742398482173769</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.1475513773023727</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1161688220.001583</v>
+        <v>1161707007.344564</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
         <v>0.2058133877973638</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1395990288.477343</v>
+        <v>1396000325.532125</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>160.3426395939086</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.098665380112</v>
+        <v>45.02596358676556</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>24.93963321631764</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.555374382866281</v>
+        <v>2.561115117168486</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.9530072742355977</v>
+        <v>0.9555590770045088</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3314,7 +3314,7 @@
         <v>0.4963026772194564</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>11014892081.08786</v>
+        <v>11017468022.28556</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>60.09433962264151</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.05328524314731</v>
+        <v>37.02334385468461</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>18.06890599940556</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.6218356679656478</v>
+        <v>0.623147273204435</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.352027069356613</v>
+        <v>0.3528807826717835</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3438,7 +3438,7 @@
         <v>0.3639048581074436</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2196041211.50776</v>
+        <v>2196069791.356201</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>72.17977528089885</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>70.82233377263448</v>
+        <v>70.47510432284737</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.620512861322411</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>0.01916685649787042</v>
+        <v>0.02418827150992731</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1601149443639016</v>
+        <v>0.1605354176912936</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,7 +3568,7 @@
         <v>0.2944072639186791</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1486790165.699441</v>
+        <v>1487556157.998606</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>13.61151736745887</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.52755682656454</v>
+        <v>12.52557813154398</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.234896209162519</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.08652609250957899</v>
+        <v>0.08669773359044353</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3855895484997388</v>
+        <v>-0.3855443547450745</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.2569593001747523</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1961241579.969781</v>
+        <v>1961277229.024658</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>19.35196506550218</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.11536789879743</v>
+        <v>17.11233870021136</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.021231771567507</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.130677714900999</v>
+        <v>0.1308778656457499</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04815091432290641</v>
+        <v>0.04825843647027073</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.2971079409963645</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1272958322.921071</v>
+        <v>1272975458.441213</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>38.24422883907661</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>25.72617860179689</v>
+        <v>25.70985974798606</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.51298765492846</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470394955930999</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4865880172504664</v>
+        <v>0.4875316012594124</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2415283162330844</v>
+        <v>0.2419963407957288</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877328985191485</v>
@@ -3946,7 +3946,7 @@
         <v>0.2663851431851464</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>2694881208.867427</v>
+        <v>2694920036.843262</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>15.28858520900322</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>14.102701535104</v>
+        <v>14.10023932871881</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.370862673379226</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.08408911377351003</v>
+        <v>0.08427841915165413</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3264618591679181</v>
+        <v>-0.3263572655103053</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.2238092465301521</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1014485525.113043</v>
+        <v>1014492460.708466</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>14.12773868012216</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.019550265434241</v>
+        <v>6.016381322269832</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>9.022027392858217</v>
@@ -4150,10 +4150,10 @@
         <v>2.563272513243084</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>1.346975780108883</v>
+        <v>1.348211977161068</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.104774028100335</v>
+        <v>1.105775433266254</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.4337631707914727</v>
@@ -4198,7 +4198,7 @@
         <v>0.4927318589452093</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>25463007573.82243</v>
+        <v>25478741266.48193</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>84.5217391304348</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>28.3995141963865</v>
+        <v>28.38419096135198</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.549819505837633</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.976168484642219</v>
+        <v>1.977775172296435</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2573774008582563</v>
+        <v>0.257942299537304</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.5368216663377353</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>1885565812.847365</v>
+        <v>1888896119.498596</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.21828752642706</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.402247795685476</v>
+        <v>9.402936268014242</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.452613200200954</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.852088172260998</v>
+        <v>2.851806126734049</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05245542301996131</v>
+        <v>-0.05256223050968989</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.196310438670456</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>921925909.049744</v>
+        <v>922276728.6278852</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1384359008428</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>8.043852233604305</v>
+        <v>7.882188717774126</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.004490535459339664</v>
+        <v>0.004487100520791956</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.908276184073303</v>
+        <v>6.76943521785347</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>5.00615697554785</v>
+        <v>4.905544369303814</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01800113687986609</v>
+        <v>0.01763935411802195</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>8.126638800618997</v>
+        <v>7.962593080087653</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.878023879824041</v>
+        <v>6.739182913604208</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.06977416657083756</v>
+        <v>0.07120523318010641</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1790.290216153233</v>
+        <v>1755.632970723587</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2381.773333670841</v>
+        <v>2335.980854486084</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4576,7 +4576,7 @@
         <v>0.6526415180611447</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3183027552.931372</v>
+        <v>3183391406.60553</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4586,7 +4586,7 @@
       <c r="AM32" s="2" t="inlineStr"/>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -4656,7 +4656,7 @@
         <v>0.3057736200990498</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>3546228875.394332</v>
+        <v>3546351873.129069</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -4710,7 +4710,7 @@
         <v>-100.6411764705882</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>125.7558701518386</v>
+        <v>125.3117349600674</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>136.0317709626636</v>
@@ -4735,7 +4735,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.5552469000642</v>
+        <v>4.565826383764905</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.03021735747263578</v>
@@ -4780,7 +4780,7 @@
         <v>0.6372956378194149</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12944539204.17569</v>
+        <v>12948297211.46525</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -4817,13 +4817,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>774.88</v>
+        <v>774.83</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1342418715459057</v>
+        <v>0.1341686833185967</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.005761063423021184</v>
+        <v>-0.005825217804123817</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4832,7 +4832,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>825431796563</v>
+        <v>825378534652</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4864,7 +4864,7 @@
         <v>0.09172704642134921</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32608291371.94629</v>
+        <v>32627056474.44194</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
         <v>29.84815115335574</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.7330616877901778</v>
+        <v>0.7325573588556409</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>15.03795750560974</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>39.7171069645357</v>
+        <v>39.74513864686693</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>39.77368483680704</v>
+        <v>39.80439486687898</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4988,7 +4988,7 @@
         <v>0.2593148190334965</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4207553751.047943</v>
+        <v>4207966958.009237</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-24.37007874015748</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-114.7556827211154</v>
+        <v>-116.1043623821393</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>2.148577625003461</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02202667329614871</v>
+        <v>0.02210065223981994</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5116,7 +5116,7 @@
         <v>0.2749599954111459</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>1623976462.528148</v>
+        <v>1626197623.377902</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>18.43602183141298</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>15.56064782601201</v>
+        <v>15.55515848715297</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.44193728188598</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1847849805195345</v>
+        <v>0.1852030853069939</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.01005012596264576</v>
+        <v>0.01028281181774693</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5246,7 +5246,7 @@
         <v>0.1857853558059747</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>939630011.0632203</v>
+        <v>939634632.1670532</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>21.99845679012346</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>15.59629158804511</v>
+        <v>15.58283137677877</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>5.720648654861585</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4104927870793167</v>
+        <v>0.4117111491628613</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4586776460382909</v>
+        <v>0.4602422037361531</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06238891508578476</v>
@@ -5372,7 +5372,7 @@
         <v>0.469127236293663</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4518167471.051721</v>
+        <v>4523321719.095103</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
         <v>33.57738095238095</v>
       </c>
       <c r="M40" s="6" t="n">
-        <v>21.74885815893526</v>
+        <v>21.74373918305831</v>
       </c>
       <c r="N40" s="6" t="n">
         <v>7.022071202605606</v>
@@ -5450,10 +5450,10 @@
         <v>0.1177498499664631</v>
       </c>
       <c r="U40" s="4" t="n">
-        <v>0.5438686806914546</v>
+        <v>0.5442321428571428</v>
       </c>
       <c r="V40" s="4" t="n">
-        <v>0.1674645656609037</v>
+        <v>0.1676820514867747</v>
       </c>
       <c r="W40" s="4" t="n">
         <v>0.1023396098336123</v>
@@ -5498,7 +5498,7 @@
         <v>0.3292504072903227</v>
       </c>
       <c r="AK40" s="5" t="n">
-        <v>1845855544.685794</v>
+        <v>1849097047.549693</v>
       </c>
       <c r="AL40" s="7" t="inlineStr">
         <is>
@@ -5508,7 +5508,7 @@
       <c r="AM40" s="2" t="inlineStr"/>
       <c r="AN40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>
@@ -5552,7 +5552,7 @@
         <v>11.61768901569187</v>
       </c>
       <c r="M41" s="6" t="n">
-        <v>10.39899179847634</v>
+        <v>10.39645439411117</v>
       </c>
       <c r="N41" s="6" t="n">
         <v>1.907552457302196</v>
@@ -5576,10 +5576,10 @@
         <v>-0.01489668811853551</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>0.1171937857854728</v>
+        <v>0.1174664530123308</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>-0.2879548508939894</v>
+        <v>-0.2878672749517781</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>0.009923315255755299</v>
@@ -5624,7 +5624,7 @@
         <v>0.2269070286678308</v>
       </c>
       <c r="AK41" s="5" t="n">
-        <v>1166611264.123555</v>
+        <v>1166617385.697072</v>
       </c>
       <c r="AL41" s="7" t="inlineStr">
         <is>
@@ -5634,7 +5634,7 @@
       <c r="AM41" s="2" t="inlineStr"/>
       <c r="AN41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 17:13 ET</t>
+          <t>2026-10-05 21:51 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-10-07)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>333.63</v>
+        <v>337.04001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2310615400830769</v>
+        <v>0.2436441380577754</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.03390861180286087</v>
+        <v>-0.02403425609544207</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>345.34</v>
@@ -714,40 +714,40 @@
         <v>243.42</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4900142582280</v>
+        <v>4950226591742</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.08561643835617</v>
+        <v>38.47488584474886</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.72353765229211</v>
+        <v>35.07870018140925</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.49678910910559</v>
+        <v>10.60407577655771</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>45.5902509249442</v>
+        <v>46.05622447544644</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.163727168949771</v>
+        <v>1.175621511922881</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.34905916384744</v>
+        <v>29.64631759457759</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.59267770071312</v>
+        <v>10.69996436816523</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02789367813383145</v>
+        <v>0.02761146402738603</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.09682420091324229</v>
+        <v>0.09681617750305072</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1237555839879354</v>
+        <v>0.1237555641539942</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,20 +781,20 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003177172316638192</v>
+        <v>0.003145027203150155</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3067423947880809</v>
+        <v>0.3071851536336922</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2042643751178725</v>
+        <v>0.2053282718030524</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13205426144.30081</v>
+        <v>13145542543.87055</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
-          <t>2026-10-29 (C)</t>
+          <t>2026-11-02 (C)</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>529.3</v>
+        <v>530.13</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.1191694448929097</v>
+        <v>0.120924424373849</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.04410171205663527</v>
+        <v>-0.04260275951744574</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3930343615000</v>
+        <v>3936506857758</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>29.40555555555555</v>
+        <v>29.450555</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.50563546490485</v>
+        <v>25.53202921864816</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.84412807114293</v>
+        <v>11.86225308576448</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.888529048095897</v>
+        <v>8.902131201210704</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.9340186903841178</v>
+        <v>0.9354480230858453</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>19.45950450320212</v>
+        <v>19.48848780943914</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>12.1692052923255</v>
+        <v>12.18733030694704</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01704354798505321</v>
+        <v>0.01701750617375491</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1529042511415524</v>
+        <v>0.1534749058836975</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2394069641717078</v>
+        <v>0.2401662961436741</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.006877007368222181</v>
+        <v>0.00686624035613906</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5612920553734346</v>
+        <v>0.5579059338986809</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.2169626029058913</v>
+        <v>0.2169453127628976</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>11081725772.67283</v>
+        <v>10909893222.33997</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>347.68</v>
+        <v>348.165</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.1032207099270976</v>
+        <v>0.1047596596633915</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1491152933114706</v>
+        <v>-0.1479283424292112</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>235.84</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4207662051916</v>
+        <v>4213531575890</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>17.10973187686196</v>
+        <v>17.13356504468719</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>21.15194945634943</v>
+        <v>21.19615010677283</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.379299219799224</v>
+        <v>9.392364206088825</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.537461107294529</v>
+        <v>6.54656752747939</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.152157840706052</v>
+        <v>0.152369790453691</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>13.07192789188748</v>
+        <v>13.08989236890928</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.5067926819605</v>
+        <v>9.519857668250102</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01273891404316875</v>
+        <v>0.01272119393205865</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.191103783971745</v>
+        <v>-0.1916661771888245</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.3067593914168005</v>
+        <v>0.3082997201941258</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002473538886332259</v>
+        <v>0.002470093202935389</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7629452788845049</v>
+        <v>0.7602540302386704</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.2326978850756171</v>
+        <v>0.2316413800258776</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8930467375.7146</v>
+        <v>8818968244.400261</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>256.29</v>
+        <v>258.84</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1315231788079472</v>
+        <v>0.1427814569536423</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1076253481894149</v>
+        <v>-0.09874651810584967</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2756937159000</v>
+        <v>2784367764000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.34047619047619</v>
+        <v>20.54285714285714</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.01478273460146</v>
+        <v>23.25898376419948</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.554219728496288</v>
+        <v>3.589583029084159</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.997380878140749</v>
+        <v>5.047103150719697</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2302500604302635</v>
+        <v>0.2325409717186367</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.42515919085659</v>
+        <v>11.53315497427135</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.741176978908828</v>
+        <v>3.7765402794967</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004216635827933283</v>
+        <v>-0.004175095025270519</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1161995129375951</v>
+        <v>-0.1167775277234181</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1876074111206361</v>
+        <v>0.1880706079165892</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8341626175839107</v>
+        <v>0.8329756942034598</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.2392186225052658</v>
+        <v>0.2396949742197649</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>8783156581.508448</v>
+        <v>8739499772.368645</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>239.24</v>
+        <v>236.99</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.266825481958755</v>
+        <v>0.2549112647107732</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.01697004560956561</v>
+        <v>-0.02621522784237995</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>243.37</v>
@@ -1220,40 +1220,40 @@
         <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5794632040000</v>
+        <v>5740134790000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>30.09308176100629</v>
+        <v>29.81006289308176</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.340041219498</v>
+        <v>17.1552227630903</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>19.12615495314702</v>
+        <v>18.94627763896636</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>25.27344967333962</v>
+        <v>25.03575839359955</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2415635134556967</v>
+        <v>0.2392916613186155</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>24.84479738685046</v>
+        <v>24.61179760917339</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>19.18034201518967</v>
+        <v>19.00046470100902</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02191787142363573</v>
+        <v>0.02212596126161699</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7354677177565259</v>
+        <v>0.7376669079004043</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>1.001536105882264</v>
+        <v>1.004094575413815</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.002173549573649891</v>
+        <v>0.002194185408667032</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.297397898396789</v>
+        <v>1.301612234660254</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.3552093280747284</v>
+        <v>0.3525673467058537</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27973816735.84153</v>
+        <v>27488226286.09902</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>738.88</v>
+        <v>725.22</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.136021940788736</v>
+        <v>0.1150198028080434</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.05249929470903547</v>
+        <v>-0.07001615757482493</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>779.8200000000001</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1882286876842</v>
+        <v>1847488210295</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>27.45745076179859</v>
+        <v>26.94983277591973</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>22.15492782632062</v>
+        <v>21.74562593582311</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8.24667413007781</v>
+        <v>8.094214233180576</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.193035169454217</v>
+        <v>7.060054360101217</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-5.628777406168706</v>
+        <v>-5.524715719063541</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>18.48422441760684</v>
+        <v>18.15922192818851</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>8.671019578887877</v>
+        <v>8.518559681990642</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02176926402884312</v>
+        <v>0.02217930256424051</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2393383078042997</v>
+        <v>0.2393220068925845</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2862185324382802</v>
+        <v>0.2865729026465684</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.002842139454309225</v>
+        <v>0.002895673037147348</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8385634083243936</v>
+        <v>0.8399389819667411</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4427698636480967</v>
+        <v>0.4466610266502127</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>14450324925.00989</v>
+        <v>14457898627.6732</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>380.68</v>
+        <v>376.415</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1310064746837233</v>
+        <v>-0.1407423614796514</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2368542389190705</v>
+        <v>-0.2454042459354889</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1503513701948</v>
+        <v>1486668882313</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>322.6101694915255</v>
+        <v>318.9957627118645</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>177.2865786439416</v>
+        <v>175.1217212907629</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14.5100194167865</v>
+        <v>14.34745444670379</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>14.18707729857929</v>
+        <v>14.02813045430473</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.587791835760322</v>
+        <v>-8.491577345428501</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>124.512529260725</v>
+        <v>123.1120620479714</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>14.45330201939799</v>
+        <v>14.29073704931528</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.003832356161792587</v>
+        <v>0.003875778977115148</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.8197100534014399</v>
+        <v>0.8215659391687955</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1323063458301601</v>
+        <v>0.1327147364283829</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.535222300350033</v>
+        <v>1.52807857288433</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.4137558901177404</v>
+        <v>0.411052063324842</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13955532583.09162</v>
+        <v>13831046891.02012</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>375.81</v>
+        <v>373.372</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.08109431355727748</v>
+        <v>0.07408090801603961</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2407878787878788</v>
+        <v>-0.2457131313131313</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1787946139800</v>
+        <v>1776347159760</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>46.62655086848635</v>
+        <v>46.32406947890819</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.05786191238663</v>
+        <v>19.90554545560042</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>20.06583475264859</v>
+        <v>19.93566124708206</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>17.96680168522419</v>
+        <v>17.85024528036914</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4639572635923639</v>
+        <v>0.460947424022799</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>34.88873849185848</v>
+        <v>34.66680366148135</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>20.46361711932124</v>
+        <v>20.33344361375471</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02203813589396358</v>
+        <v>0.02218203788797888</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.324602246847276</v>
+        <v>1.327194177232401</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8996164048846722</v>
+        <v>0.9017173681049937</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.006918389611771906</v>
+        <v>0.006963564487963747</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.603569703009585</v>
+        <v>1.607176200719476</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.3604767884264293</v>
+        <v>0.3571870928075244</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>9172303637.810804</v>
+        <v>9077237517.543905</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>935.6799999999999</v>
+        <v>946.4819</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.09500292568753643</v>
+        <v>0.1076441193680515</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1466666666666667</v>
+        <v>-0.1368154126766986</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>414954430720</v>
+        <v>419744846530</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>45.0279114533205</v>
+        <v>45.54773339749759</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.65817898703663</v>
+        <v>41.11702859766119</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.368790880938401</v>
+        <v>1.384592802766911</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.60289718738653</v>
+        <v>11.7368461177136</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.24806080641541</v>
+        <v>3.285557843890635</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>28.0885459098823</v>
+        <v>28.42216355804722</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.330424242200334</v>
+        <v>1.346226164028843</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02262899081161063</v>
+        <v>0.02237073326242465</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.1014369538757789</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1074748691444618</v>
+        <v>0.1077583899165424</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.09216299056610389</v>
+        <v>0.09238703014121574</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1036105339996631</v>
@@ -1793,16 +1793,16 @@
         <v>80.58620689655173</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005920827633378934</v>
+        <v>0.005853255091301799</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1661833097202909</v>
+        <v>-0.1665530910125246</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.1797568683804935</v>
+        <v>0.1819937176324787</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2026428869.844566</v>
+        <v>2014322256.472473</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>68.69</v>
+        <v>69.42</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.2450818594056585</v>
+        <v>-0.2370589995623935</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.4498638475092104</v>
+        <v>-0.4440172993753003</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>124.86</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>286021038531</v>
+        <v>289060714731</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>21.26625386996904</v>
+        <v>21.49226006191951</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>18.29831151159781</v>
+        <v>18.49917660729498</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5.913097393520599</v>
+        <v>5.975938579986043</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.543735964305183</v>
+        <v>9.645161604921617</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6250203881295781</v>
+        <v>0.6316627652344636</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.51827796308257</v>
+        <v>9.617623402990837</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.02080861346329</v>
+        <v>6.083649799928734</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03843985762889384</v>
+        <v>0.03803563555923394</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1621976080410534</v>
+        <v>0.1617954959921963</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1496456283741519</v>
+        <v>0.149634792722009</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.10943732332623</v>
+        <v>0.1065031065387648</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3582180103473409</v>
+        <v>0.3589527853854795</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2466600959.473044</v>
+        <v>2423515492.365225</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>505.54</v>
+        <v>505.81</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.0174901756862893</v>
+        <v>0.01803359924809511</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.05988023952095811</v>
+        <v>-0.05937813813367054</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1090375766416</v>
+        <v>1090958116887</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.70891786304932</v>
+        <v>12.72522999278198</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.78820180485617</v>
+        <v>22.80034290300732</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.834493561955564</v>
+        <v>2.838131686555563</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.451292662931548</v>
+        <v>1.453155423746663</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3500983225496263</v>
+        <v>0.350547680183231</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.41095518294691</v>
+        <v>15.42924646608464</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.06522919897995</v>
+        <v>3.06886732357995</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02220759294058213</v>
+        <v>0.02217912562507079</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4423027331475955</v>
+        <v>-0.4418842713499916</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06162149252839355</v>
+        <v>0.06246212386303385</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.02707944474230121</v>
+        <v>0.02656991393592922</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1319219865343907</v>
+        <v>0.1314791271073162</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2270573589.231171</v>
+        <v>2243219589.663155</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>331.28</v>
+        <v>328.82</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.0178198009644146</v>
+        <v>0.01026173313547107</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.09609822646657584</v>
+        <v>-0.1028103683492497</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>887668072800</v>
+        <v>881076478200</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>14.24247635425623</v>
+        <v>14.13671539122958</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>13.17740839034349</v>
+        <v>13.07638874929365</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2.982424908528288</v>
+        <v>2.960278188910504</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.466218548951142</v>
+        <v>2.447905044874772</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7457253705056957</v>
+        <v>0.7401878058732276</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>19.49042585659081</v>
+        <v>19.41967022541863</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.100560330339714</v>
+        <v>6.078413610721929</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>-0.1831022259112167</v>
+        <v>-0.1844720680003281</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.08082529829562191</v>
+        <v>0.08108711527815426</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2847902309114806</v>
+        <v>-0.2847343576633796</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01856435643564357</v>
+        <v>0.01870324189526185</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7782144299613685</v>
+        <v>0.7801234254831549</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1611687472663854</v>
+        <v>0.1612487715354581</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2572636712.294358</v>
+        <v>2559969779.344228</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>370.64</v>
+        <v>374.41</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.069729820617632</v>
+        <v>0.08061067919665366</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.03872189226340228</v>
+        <v>-0.0289441605934071</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>692002378285</v>
+        <v>699041153108</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.49022939677145</v>
+        <v>31.80968564146134</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.66976303342771</v>
+        <v>24.92069387369326</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.55480979781065</v>
+        <v>15.71260735025175</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.16036951048951</v>
+        <v>20.36488869179601</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.123518758663865</v>
+        <v>2.145061038322229</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.17696674290329</v>
+        <v>24.4182237885078</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.81328399309926</v>
+        <v>15.97108154554037</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03036550257540565</v>
+        <v>0.03006054987861682</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2764706881903145</v>
+        <v>0.2764365953325327</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1424590110366841</v>
+        <v>0.1424284862799992</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007230736024174402</v>
+        <v>0.007157928474132635</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3031070682442013</v>
+        <v>0.301867595804079</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.1892813075289345</v>
+        <v>0.1827651329703194</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2186263822.633028</v>
+        <v>2124251360.586749</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>566.58</v>
+        <v>573.08</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.006126462961080437</v>
+        <v>0.01766909067340161</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05763185469786936</v>
+        <v>-0.0468206842639256</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.23</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>496911056880</v>
+        <v>502611790880</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.11367380560132</v>
+        <v>31.47062053816584</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.34570509943894</v>
+        <v>25.62877657946632</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.16387016161674</v>
+        <v>14.32636293589488</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>89.06140794867225</v>
+        <v>90.08315095348424</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.375113261943986</v>
+        <v>1.390889032713579</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.07212230421414</v>
+        <v>23.32988745161873</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.54445335005558</v>
+        <v>14.70694612433372</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03310049106830815</v>
+        <v>0.03272505798401974</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2275718384449308</v>
+        <v>0.2279408047663107</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.164527793788507</v>
+        <v>0.164894732844499</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005947968512831374</v>
+        <v>0.005880505339568646</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2983277942338674</v>
+        <v>0.2970065701103723</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.1834582224423093</v>
+        <v>0.1767386998166109</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1567870877.882924</v>
+        <v>1520463348.008948</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>376.32</v>
+        <v>381.345</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1186682723775543</v>
+        <v>0.1336058469648662</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1847840214895369</v>
+        <v>-0.1738984446081192</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>341752902113</v>
+        <v>346316327743</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>24.1990868754421</v>
+        <v>24.52221722075751</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.1071964969225</v>
+        <v>17.32985316735481</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7592332467203845</v>
+        <v>0.7693712863268085</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.463231901835505</v>
+        <v>3.50947642858594</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7332386506253407</v>
+        <v>-0.7430295844566341</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.0019757836044</v>
+        <v>15.17910677106704</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8586336408296288</v>
+        <v>0.8687716804360527</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06910548485171629</v>
+        <v>0.06819487880896589</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4145559665369714</v>
+        <v>0.4150274087117687</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.01325224556094806</v>
+        <v>0.01333267693532125</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02407525510204082</v>
+        <v>0.0237580143964127</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4438573143085862</v>
+        <v>0.4425506202725809</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.1926113333976813</v>
+        <v>0.1948379764874802</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1828633723.367757</v>
+        <v>1822838639.219849</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>164.48</v>
+        <v>163.755</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3410517566548503</v>
+        <v>0.3351406274988755</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.06762655178277877</v>
+        <v>-0.07173629612833743</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>110.39</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>681680780800</v>
+        <v>678676067537</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.16859716859717</v>
+        <v>21.07528957528957</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.27522373220754</v>
+        <v>14.13135121819847</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.88799861740431</v>
+        <v>1.879676695111616</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.646753845631891</v>
+        <v>2.635087402671755</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.072758472758474</v>
+        <v>2.063622104247105</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.933320999651933</v>
+        <v>9.891487191604595</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.976017229269373</v>
+        <v>1.96769530697668</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.0448200988799243</v>
+        <v>0.04501853161093575</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4828907459318417</v>
+        <v>0.4913853070291425</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.1131805846008669</v>
+        <v>0.1215007435639657</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02504863813229572</v>
+        <v>0.02515953711337059</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5465419280448265</v>
+        <v>-0.5468121846286893</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2442310721497457</v>
+        <v>0.2424706871364872</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2253789904.667857</v>
+        <v>2185473696.022074</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -2717,55 +2717,55 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>254.78</v>
+        <v>259.885</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2287436339539137</v>
+        <v>0.2533638406080261</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.09353541822321843</v>
+        <v>-0.07537268296153987</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>182.94</v>
+        <v>184.66</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>613993918428</v>
+        <v>626296449842</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>29.45433526011561</v>
+        <v>30.04450867052023</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>20.70694142469561</v>
+        <v>21.22801707857505</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.269786461906075</v>
+        <v>6.395413512258881</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.316480658106883</v>
+        <v>7.463080209718609</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.646911773653793</v>
+        <v>-3.719984560389419</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.05039483066524</v>
+        <v>19.41510879408277</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.561977743344668</v>
+        <v>6.687604793697474</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.0304693571687124</v>
+        <v>0.02987083833018627</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4224377543748514</v>
+        <v>0.4153233700213792</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.0934198596122966</v>
+        <v>0.09380698265615139</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.02072376167674072</v>
+        <v>0.02031667853088866</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1680144479123665</v>
+        <v>-0.1704184612478871</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.1859953605717556</v>
+        <v>0.1912471798308693</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1781293138.604381</v>
+        <v>1760001786.665754</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>107.2</v>
+        <v>108.15</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.04930828335310933</v>
+        <v>-0.04088331011789903</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2068659366676531</v>
+        <v>-0.1998372299496892</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>853106176000</v>
+        <v>860666352000</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.70036101083033</v>
+        <v>39.043321299639</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.41025797157931</v>
+        <v>34.71030154812706</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.159363687758208</v>
+        <v>1.169637899543379</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.679622956493414</v>
+        <v>8.756541256947413</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.35845093534625</v>
+        <v>9.441384968821801</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.36679605032797</v>
+        <v>21.54327486636009</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.243928267014568</v>
+        <v>1.254202478799739</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01583507467187766</v>
+        <v>0.01569597785321576</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1246751199248308</v>
+        <v>0.1248338262202664</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05345283521583388</v>
+        <v>0.05341541079966006</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009118470149253731</v>
+        <v>0.00903837263060564</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.03369398028887385</v>
+        <v>-0.036143838150693</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3136432430731917</v>
+        <v>0.3145719869101938</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2480633287.031174</v>
+        <v>2417678024.507946</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>148.41</v>
+        <v>148.34</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.04668881463664354</v>
+        <v>0.04619512676504089</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1126457399103139</v>
+        <v>-0.1130642750373692</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>352801578340</v>
+        <v>352635173715</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.98666666666666</v>
+        <v>21.9762962962963</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.9444915499856</v>
+        <v>20.93269448680185</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.053699539709532</v>
+        <v>4.051787546132458</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.619712857432195</v>
+        <v>6.616590561764651</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.98156190476213</v>
+        <v>20.97166560846583</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.77950401524419</v>
+        <v>17.77167468311847</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.341915368370254</v>
+        <v>4.34000337479318</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04510467349628581</v>
+        <v>0.04512595789114587</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04975891222729545</v>
+        <v>0.04985511111111118</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02787853336486523</v>
+        <v>0.0279918342541936</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02912404824472745</v>
+        <v>0.02892409329917757</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.02749665852485781</v>
+        <v>-0.02524559440116231</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1532500564830009</v>
+        <v>0.1518444462521102</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1193161405.41285</v>
+        <v>1172340674.178595</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>286.69</v>
+        <v>284.48</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.1709849230000803</v>
+        <v>-0.1773755306953951</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2790030933279682</v>
+        <v>-0.2845610240676005</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>397.63</v>
@@ -3110,40 +3110,40 @@
         <v>277.15</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>285863472730</v>
+        <v>283659844160</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20.02025139664804</v>
+        <v>19.8659217877095</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>19.10999126788916</v>
+        <v>18.96082065801673</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.689740109294463</v>
+        <v>1.676714452168156</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17.14929650358067</v>
+        <v>17.01709815249443</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-6.867411816292091</v>
+        <v>-6.814473171365496</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>14.48235303073385</v>
+        <v>14.39020882960485</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.047249448680664</v>
+        <v>2.034223791554358</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.05282591670696941</v>
+        <v>0.05323629801996998</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.0476326815642456</v>
+        <v>0.04773533519553053</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01416228040029321</v>
+        <v>0.01414159188655595</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.03240433918169451</v>
+        <v>0.0326560742407199</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7154807261325346</v>
+        <v>0.7190175289207321</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2142576359557458</v>
+        <v>0.2070999572177213</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1401922867.3355</v>
+        <v>1397170142.204433</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>649.42</v>
+        <v>645.385</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.906072387580204</v>
+        <v>1.888016272764082</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.01381886654923159</v>
+        <v>-0.0199462430905667</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>658.52</v>
@@ -3236,40 +3236,40 @@
         <v>188.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>1058944252000</v>
+        <v>1052364781000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>164.8274111675127</v>
+        <v>163.8032994923858</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45.91903673816037</v>
+        <v>45.55970838145967</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>25.63719288221765</v>
+        <v>25.4779029415325</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>15.75633732000476</v>
+        <v>15.65843947102226</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.330716714012946</v>
+        <v>1.322448656452289</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>98.72497219630529</v>
+        <v>98.11110104497108</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>25.61758266553686</v>
+        <v>25.45829272485171</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.007935261921606804</v>
+        <v>0.007984873830550587</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.589522404561575</v>
+        <v>2.595354432932341</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.96907958985197</v>
+        <v>0.9716698986931498</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.574552235095028</v>
+        <v>2.537848733662965</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.4986006807308233</v>
+        <v>0.4974002825214326</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>11289678492.03703</v>
+        <v>11270283182.9106</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1834.1</v>
+        <v>1802.9765</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.5759851121591375</v>
+        <v>0.5492416561653068</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.08293165863317276</v>
+        <v>-0.09849371987439748</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>935.41</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>706895137293</v>
+        <v>694899580450</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>59.37590711175617</v>
+        <v>58.42525399129173</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.56911357098868</v>
+        <v>35.90478558768867</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>17.85289082080532</v>
+        <v>17.56705255418583</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>28.89608254602435</v>
+        <v>28.43343443877317</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>4.041934979873941</v>
+        <v>3.97722054790578</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>45.34829225774204</v>
+        <v>44.61679518330979</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>17.72020382059302</v>
+        <v>17.43436555397353</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01585846156562222</v>
+        <v>0.01611649888583785</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.6236627392264922</v>
+        <v>0.6272274861133014</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.3536137082734963</v>
+        <v>0.3540038848881726</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004241862493866202</v>
+        <v>0.004315086746832252</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.639677814115044</v>
+        <v>1.641515363014149</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.3645695946622249</v>
+        <v>0.3640334775127934</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2225792566.120178</v>
+        <v>2229226046.859033</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>189.82</v>
+        <v>187.9869</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.1666154610379018</v>
+        <v>-0.174663491795311</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.2537055238844113</v>
+        <v>-0.2609125221151957</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>150028033400</v>
+        <v>148579206153</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>71.09363295880146</v>
+        <v>70.40707865168537</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>69.55452838486389</v>
+        <v>70.22002699698919</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.596127808926007</v>
+        <v>1.580713933219852</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>24.6157572754623</v>
+        <v>24.37804183630072</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.3804983618934107</v>
+        <v>0.3768238726552545</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>27.14806235971223</v>
+        <v>26.9395980076259</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.007330532475132</v>
+        <v>1.991916656768977</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001399738403822869</v>
+        <v>-0.00141338754888589</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>0.02212802832076277</v>
+        <v>0.002663793545738757</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1596356731723851</v>
+        <v>0.1583879403910291</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.24568007953254</v>
+        <v>1.24441618050236</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.2866889995043072</v>
+        <v>0.2846359693347141</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1486203678.915458</v>
+        <v>1476643500.776843</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>897.1799999999999</v>
+        <v>884.5</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>-0.01876766449182399</v>
+        <v>-0.03263559067636179</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.2225409232315705</v>
+        <v>-0.2335288867321207</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>740.01</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>264674380260</v>
+        <v>260933691500</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>13.66819012797075</v>
+        <v>13.47501523461304</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>12.61127930183583</v>
+        <v>12.44502882635926</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.244201397864962</v>
+        <v>2.212483711642657</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.193574473285428</v>
+        <v>2.162572306138078</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3203634374874852</v>
+        <v>0.3158356856569258</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>26.09761348899436</v>
+        <v>25.97845671009461</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>6.946779893163299</v>
+        <v>6.915062206940994</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1568531112048631</v>
+        <v>-0.1591017233587101</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.08380678921138962</v>
+        <v>0.08276287846535268</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3856501985115806</v>
+        <v>-0.3869265294003613</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.02006286363940346</v>
+        <v>0.02035048049745619</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.585290808645695</v>
+        <v>1.586430631700645</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.2513923352242851</v>
+        <v>0.2514578718899778</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1953892846.433563</v>
+        <v>1911178472.293774</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 19:12 ET</t>
+          <t>2026-10-07 14:11 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>221.29</v>
+        <v>221.265</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2408576329331047</v>
+        <v>-0.2409433962264151</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3343860915598869</v>
+        <v>-0.3344612885760693</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>208484832860</v>
+        <v>208461278935</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>19.32663755458515</v>
+        <v>19.32445414847162</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.08994237282142</v>
+        <v>17.08498783323529</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.017277636655716</v>
+        <v>3.016936754634789</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.037108760013933</v>
+        <v>6.036426724137931</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2355902136014354</v>
+        <v>0.2355635980501676</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>16.43454983416559</v>
+        <v>16.43309777048271</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.858124561992561</v>
+        <v>3.857783679971634</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06538125489998295</v>
+        <v>0.065388642291935</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1308778656457499</v>
+        <v>0.1310780163905008</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04825843647027073</v>
+        <v>0.04836595861763526</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.030457770346604</v>
+        <v>0.03046121166926536</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8931623292511017</v>
+        <v>0.8924160083765384</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.2962258282558146</v>
+        <v>0.2929297535926072</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1270585192.998852</v>
+        <v>1261568442.574663</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
       